<commit_message>
reglas: G08 (solo prestacion/subsidio) es dato de origen; 7 reglas la excluyen
1.180 personas tienen solo episodios TRL 7xx/400: sin primer empleo ni historia
de empleo por diseno, igual que ya se excluyo en A-045/A-046/C-282/C-283.
16 reglas excluyen ese colectivo via tabla auxiliar solo_prestaciones (creada en
ejecutar_reglas.py). 7 pasan; los residuos (episodios con baja anterior al alta)
pasan a G20 (baja calidad) y B-046/B-076/C-265 a G21 (pendiente, sin investigar).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/reglas_consistencia_resultados_sin_ipf.xlsx
+++ b/tests/reglas_consistencia_resultados_sin_ipf.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -955,51 +955,51 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Con afiliación pero sin primer empleo ni historia</t>
+          <t>Con afiliación pero solo prestación/subsidio: sin primer empleo ni historia de empleo</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>1189</v>
+        <v>0</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>0.08699999999999999</v>
+        <v>0</v>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>A-043, C-132, A-039, A-046, C-128, C-136, C-280, B-046, B-047, B-076, B-077, C-265, A-042, C-130, C-138, C-080</t>
+          <t>A-039, A-046, B-047, B-077, C-128, C-136, C-280</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>1.180-1.194 personas con afiliación (no Nunca_ha_cotizado) sin fecha_ini_primer_empleo, num_altas, edad_ultimo_empleo ni tiempo total; lo mismo aparece en Parado_LD (289) y Parado_NoLD (156).</t>
+          <t>VERIFICADO 2026-09-24 con datos reales: 1.180 personas (no Nunca_ha_cotizado) cuyos episodios de Afiliación son TODOS TRL 7xx (2.530 episodios; 755: 1.037 personas, 751: 156, 753: 115) o 400, sin ningún episodio de empleo real. 77 % mujeres, mediana 74 años, cohortes 1930-1959 (78 %), régimen 111; 758 con pensión en 2024. 604 tienen Bases de cotización (CA), todas dentro del año de un episodio 7xx suyo (cotización durante el subsidio); ninguna anterior. Ya se había excluido a este mismo colectivo (1.189 personas) en A-045, A-046, C-282 y C-283 (commit a3018a1) y en C-278.</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Personas cuyos episodios no cuentan como 'empleo' (p. ej. solo situaciones asimiladas).</t>
+          <t>Dato de origen: quien cobra prestación/subsidio tuvo algún trabajo previo (p. ej. agrarios con trabajo temporal mal registrado o fuera de la muestra), pero no consta en Afiliación. El ETL no inventa valores: sus campos de empleo quedan a NULL por diseño (TRL 7xx/400 no cuentan como empleo, decisión ya tomada).</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>A investigar / decisión</t>
+          <t>Dato de origen</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>Definir si eso es correcto o si deben tener valores - sin decidir.</t>
+          <t>Ninguna acción sobre el ETL. Las 7 reglas afectadas ya no incumplen (excluyen a quien solo tiene TRL 7xx/400 vía tabla auxiliar solo_prestaciones en tests/ejecutar_reglas.py).</t>
         </is>
       </c>
     </row>
@@ -1608,6 +1608,118 @@
       <c r="L20" s="2" t="inlineStr">
         <is>
           <t>Ninguna acción sobre el ETL. Dejar las reglas como detección informativa de baja confianza, sin tratarlas como error pendiente de resolver.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>G20</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Episodios con baja anterior al alta (duración de empleo nula)</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Baja calidad de los datos</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>0.0007</v>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>A-042, A-043, C-080, C-130, C-132, C-138</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Residuo de G08: 6-9 personas con episodios de 1979-1984 (TRL 0/901/902/930) cuya baja es anterior al alta; DURACION_EMPLEO sale NULL (duración negativa) y arrastra t_total_empleo, num_altas y tiempo total. Verificado: el 100 % de las personas de A-042, A-043, C-080, C-138 tiene un episodio con duración nula.</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Fechas incoherentes en el dato de origen (Afiliación cruda).</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Dato de origen</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>Ninguna acción sobre el ETL; volumen insignificante.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>G21</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Residuo tras G08 sin investigar</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>0.0061</v>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>B-046, B-076, C-265</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>B-046/B-076: 26 personas Parado_LD/Parado_NoLD sin empleo real que no son del colectivo solo-prestaciones (ninguna con episodio de duración nula). C-265: 83 con duración del primer empleo significativo mayor que el tiempo total de empleo.</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Por investigar.</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>A investigar</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>Investigar cuando haya tiempo; volumen muy pequeño.</t>
         </is>
       </c>
     </row>
@@ -4280,27 +4392,27 @@
       </c>
       <c r="I40" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J40" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pasan</t>
         </is>
       </c>
       <c r="K40" s="2" t="n">
-        <v>1180</v>
+        <v>0</v>
       </c>
       <c r="L40" s="2" t="n">
-        <v>0.0868</v>
-      </c>
-      <c r="M40" s="2" t="inlineStr">
-        <is>
-          <t>G08</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M40" s="2" t="n"/>
       <c r="N40" s="2" t="n"/>
-      <c r="O40" s="2" t="inlineStr"/>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>Regla ajustada 2026-09-24 (G08): excluye a quien solo tiene episodios TRL 7xx/400 (dato de origen, p. ej. agrarios con trabajo temporal mal registrado).</t>
+        </is>
+      </c>
       <c r="P40" s="2" t="inlineStr">
         <is>
           <t>situacion_actual_afiliacion &lt;&gt; 'Nunca_ha_cotizado' AND fecha_ini_primer_empleo IS NULL</t>
@@ -4487,22 +4599,26 @@
       </c>
       <c r="J43" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K43" s="2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L43" s="2" t="n">
-        <v>0.0007</v>
+        <v>0.0005</v>
       </c>
       <c r="M43" s="2" t="inlineStr">
         <is>
-          <t>G08</t>
+          <t>G20</t>
         </is>
       </c>
       <c r="N43" s="2" t="n"/>
-      <c r="O43" s="2" t="inlineStr"/>
+      <c r="O43" s="2" t="inlineStr">
+        <is>
+          <t>Regla ajustada 2026-09-24 (G08): excluye a quien solo tiene episodios TRL 7xx/400 (dato de origen, p. ej. agrarios con trabajo temporal mal registrado).</t>
+        </is>
+      </c>
       <c r="P43" s="2" t="inlineStr">
         <is>
           <t>situacion_actual_afiliacion &lt;&gt; 'Nunca_ha_cotizado' AND t_total_empleo IS NULL</t>
@@ -4557,22 +4673,26 @@
       </c>
       <c r="J44" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K44" s="2" t="n">
-        <v>1189</v>
+        <v>9</v>
       </c>
       <c r="L44" s="2" t="n">
-        <v>0.08749999999999999</v>
+        <v>0.0007</v>
       </c>
       <c r="M44" s="2" t="inlineStr">
         <is>
-          <t>G08</t>
+          <t>G20</t>
         </is>
       </c>
       <c r="N44" s="2" t="n"/>
-      <c r="O44" s="2" t="inlineStr"/>
+      <c r="O44" s="2" t="inlineStr">
+        <is>
+          <t>Regla ajustada 2026-09-24 (G08): excluye a quien solo tiene episodios TRL 7xx/400 (dato de origen, p. ej. agrarios con trabajo temporal mal registrado).</t>
+        </is>
+      </c>
       <c r="P44" s="2" t="inlineStr">
         <is>
           <t>situacion_actual_afiliacion &lt;&gt; 'Nunca_ha_cotizado' AND num_altas_anual_promedio IS NULL</t>
@@ -4754,27 +4874,27 @@
       </c>
       <c r="I47" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J47" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pasan</t>
         </is>
       </c>
       <c r="K47" s="2" t="n">
-        <v>1180</v>
+        <v>0</v>
       </c>
       <c r="L47" s="2" t="n">
-        <v>0.0868</v>
-      </c>
-      <c r="M47" s="2" t="inlineStr">
-        <is>
-          <t>G08</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M47" s="2" t="n"/>
       <c r="N47" s="2" t="n"/>
-      <c r="O47" s="2" t="inlineStr"/>
+      <c r="O47" s="2" t="inlineStr">
+        <is>
+          <t>Regla ajustada 2026-09-24 (G08): excluye a quien solo tiene episodios TRL 7xx/400 (dato de origen, p. ej. agrarios con trabajo temporal mal registrado).</t>
+        </is>
+      </c>
       <c r="P47" s="2" t="inlineStr">
         <is>
           <t>situacion_actual_afiliacion &lt;&gt; 'Nunca_ha_cotizado' AND edad_ultimo_empleo IS NULL</t>
@@ -12273,20 +12393,20 @@
         </is>
       </c>
       <c r="K158" s="2" t="n">
-        <v>291</v>
+        <v>26</v>
       </c>
       <c r="L158" s="2" t="n">
-        <v>0.0214</v>
+        <v>0.0019</v>
       </c>
       <c r="M158" s="2" t="inlineStr">
         <is>
-          <t>G08</t>
+          <t>G21</t>
         </is>
       </c>
       <c r="N158" s="2" t="n"/>
       <c r="O158" s="2" t="inlineStr">
         <is>
-          <t>Alguien puede haber tenido solo prestaciones</t>
+          <t>Alguien puede haber tenido solo prestaciones | Regla ajustada 2026-09-24 (G08): excluye a quien solo tiene episodios TRL 7xx/400 (dato de origen, p. ej. agrarios con trabajo temporal mal registrado).</t>
         </is>
       </c>
       <c r="P158" s="2" t="inlineStr">
@@ -12338,27 +12458,27 @@
       </c>
       <c r="I159" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J159" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pasan</t>
         </is>
       </c>
       <c r="K159" s="2" t="n">
-        <v>265</v>
+        <v>0</v>
       </c>
       <c r="L159" s="2" t="n">
-        <v>0.0195</v>
-      </c>
-      <c r="M159" s="2" t="inlineStr">
-        <is>
-          <t>G08</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M159" s="2" t="n"/>
       <c r="N159" s="2" t="n"/>
-      <c r="O159" s="2" t="inlineStr"/>
+      <c r="O159" s="2" t="inlineStr">
+        <is>
+          <t>Regla ajustada 2026-09-24 (G08): excluye a quien solo tiene episodios TRL 7xx/400 (dato de origen, p. ej. agrarios con trabajo temporal mal registrado).</t>
+        </is>
+      </c>
       <c r="P159" s="2" t="inlineStr">
         <is>
           <t>situacion_paro_ocupacion = 'Parado_LD' AND fecha_ini_primer_empleo IS NULL</t>
@@ -14341,20 +14461,20 @@
         </is>
       </c>
       <c r="K188" s="2" t="n">
-        <v>158</v>
+        <v>26</v>
       </c>
       <c r="L188" s="2" t="n">
-        <v>0.0116</v>
+        <v>0.0019</v>
       </c>
       <c r="M188" s="2" t="inlineStr">
         <is>
-          <t>G08</t>
+          <t>G21</t>
         </is>
       </c>
       <c r="N188" s="2" t="n"/>
       <c r="O188" s="2" t="inlineStr">
         <is>
-          <t>Alguien puede haber tenido solo prestaciones</t>
+          <t>Alguien puede haber tenido solo prestaciones | Regla ajustada 2026-09-24 (G08): excluye a quien solo tiene episodios TRL 7xx/400 (dato de origen, p. ej. agrarios con trabajo temporal mal registrado).</t>
         </is>
       </c>
       <c r="P188" s="2" t="inlineStr">
@@ -14406,27 +14526,27 @@
       </c>
       <c r="I189" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J189" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pasan</t>
         </is>
       </c>
       <c r="K189" s="2" t="n">
-        <v>132</v>
+        <v>0</v>
       </c>
       <c r="L189" s="2" t="n">
-        <v>0.0097</v>
-      </c>
-      <c r="M189" s="2" t="inlineStr">
-        <is>
-          <t>G08</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M189" s="2" t="n"/>
       <c r="N189" s="2" t="n"/>
-      <c r="O189" s="2" t="inlineStr"/>
+      <c r="O189" s="2" t="inlineStr">
+        <is>
+          <t>Regla ajustada 2026-09-24 (G08): excluye a quien solo tiene episodios TRL 7xx/400 (dato de origen, p. ej. agrarios con trabajo temporal mal registrado).</t>
+        </is>
+      </c>
       <c r="P189" s="2" t="inlineStr">
         <is>
           <t>situacion_paro_ocupacion = 'Parado_NoLD' AND fecha_ini_primer_empleo IS NULL</t>
@@ -22109,7 +22229,7 @@
       </c>
       <c r="J304" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K304" s="2" t="n">
@@ -22120,11 +22240,15 @@
       </c>
       <c r="M304" s="2" t="inlineStr">
         <is>
-          <t>G08</t>
+          <t>G20</t>
         </is>
       </c>
       <c r="N304" s="2" t="n"/>
-      <c r="O304" s="2" t="inlineStr"/>
+      <c r="O304" s="2" t="inlineStr">
+        <is>
+          <t>Regla ajustada 2026-09-24 (G08): excluye a quien solo tiene episodios TRL 7xx/400 (dato de origen, p. ej. agrarios con trabajo temporal mal registrado).</t>
+        </is>
+      </c>
       <c r="P304" s="2" t="inlineStr">
         <is>
           <t>fecha_ultima_baja &lt; fecha_ini_primer_empleo</t>
@@ -25284,27 +25408,27 @@
       </c>
       <c r="I352" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J352" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pasan</t>
         </is>
       </c>
       <c r="K352" s="2" t="n">
-        <v>1180</v>
+        <v>0</v>
       </c>
       <c r="L352" s="2" t="n">
-        <v>0.0868</v>
-      </c>
-      <c r="M352" s="2" t="inlineStr">
-        <is>
-          <t>G08</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M352" s="2" t="n"/>
       <c r="N352" s="2" t="n"/>
-      <c r="O352" s="2" t="inlineStr"/>
+      <c r="O352" s="2" t="inlineStr">
+        <is>
+          <t>Regla ajustada 2026-09-24 (G08): excluye a quien solo tiene episodios TRL 7xx/400 (dato de origen, p. ej. agrarios con trabajo temporal mal registrado).</t>
+        </is>
+      </c>
       <c r="P352" s="2" t="inlineStr">
         <is>
           <t>fecha_ini_primer_empleo IS NULL AND tiempo_total_desde_inicio_vl IS NOT NULL</t>
@@ -25425,22 +25549,26 @@
       </c>
       <c r="J354" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K354" s="2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L354" s="2" t="n">
-        <v>0.0007</v>
+        <v>0.0005</v>
       </c>
       <c r="M354" s="2" t="inlineStr">
         <is>
-          <t>G08</t>
+          <t>G20</t>
         </is>
       </c>
       <c r="N354" s="2" t="n"/>
-      <c r="O354" s="2" t="inlineStr"/>
+      <c r="O354" s="2" t="inlineStr">
+        <is>
+          <t>Regla ajustada 2026-09-24 (G08): excluye a quien solo tiene episodios TRL 7xx/400 (dato de origen, p. ej. agrarios con trabajo temporal mal registrado).</t>
+        </is>
+      </c>
       <c r="P354" s="2" t="inlineStr">
         <is>
           <t>t_total_empleo IS NULL AND tiempo_total_desde_inicio_vl IS NOT NULL</t>
@@ -25561,22 +25689,26 @@
       </c>
       <c r="J356" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K356" s="2" t="n">
-        <v>1189</v>
+        <v>9</v>
       </c>
       <c r="L356" s="2" t="n">
-        <v>0.08749999999999999</v>
+        <v>0.0007</v>
       </c>
       <c r="M356" s="2" t="inlineStr">
         <is>
-          <t>G08</t>
+          <t>G20</t>
         </is>
       </c>
       <c r="N356" s="2" t="n"/>
-      <c r="O356" s="2" t="inlineStr"/>
+      <c r="O356" s="2" t="inlineStr">
+        <is>
+          <t>Regla ajustada 2026-09-24 (G08): excluye a quien solo tiene episodios TRL 7xx/400 (dato de origen, p. ej. agrarios con trabajo temporal mal registrado).</t>
+        </is>
+      </c>
       <c r="P356" s="2" t="inlineStr">
         <is>
           <t>num_altas_anual_promedio IS NULL AND tiempo_total_desde_inicio_vl IS NOT NULL</t>
@@ -25824,27 +25956,27 @@
       </c>
       <c r="I360" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J360" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pasan</t>
         </is>
       </c>
       <c r="K360" s="2" t="n">
-        <v>1180</v>
+        <v>0</v>
       </c>
       <c r="L360" s="2" t="n">
-        <v>0.0868</v>
-      </c>
-      <c r="M360" s="2" t="inlineStr">
-        <is>
-          <t>G08</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M360" s="2" t="n"/>
       <c r="N360" s="2" t="n"/>
-      <c r="O360" s="2" t="inlineStr"/>
+      <c r="O360" s="2" t="inlineStr">
+        <is>
+          <t>Regla ajustada 2026-09-24 (G08): excluye a quien solo tiene episodios TRL 7xx/400 (dato de origen, p. ej. agrarios con trabajo temporal mal registrado).</t>
+        </is>
+      </c>
       <c r="P360" s="2" t="inlineStr">
         <is>
           <t>edad_ultimo_empleo IS NULL AND tiempo_total_desde_inicio_vl IS NOT NULL</t>
@@ -25965,22 +26097,26 @@
       </c>
       <c r="J362" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K362" s="2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L362" s="2" t="n">
-        <v>0.0007</v>
+        <v>0.0005</v>
       </c>
       <c r="M362" s="2" t="inlineStr">
         <is>
-          <t>G08</t>
+          <t>G20</t>
         </is>
       </c>
       <c r="N362" s="2" t="n"/>
-      <c r="O362" s="2" t="inlineStr"/>
+      <c r="O362" s="2" t="inlineStr">
+        <is>
+          <t>Regla ajustada 2026-09-24 (G08): excluye a quien solo tiene episodios TRL 7xx/400 (dato de origen, p. ej. agrarios con trabajo temporal mal registrado).</t>
+        </is>
+      </c>
       <c r="P362" s="2" t="inlineStr">
         <is>
           <t>t_total_desempleo IS NULL AND tiempo_total_desde_inicio_vl IS NOT NULL</t>
@@ -34350,11 +34486,15 @@
       </c>
       <c r="M489" s="2" t="inlineStr">
         <is>
-          <t>G08</t>
+          <t>G21</t>
         </is>
       </c>
       <c r="N489" s="2" t="n"/>
-      <c r="O489" s="2" t="inlineStr"/>
+      <c r="O489" s="2" t="inlineStr">
+        <is>
+          <t>Regla ajustada 2026-09-24 (G08): excluye a quien solo tiene episodios TRL 7xx/400 (dato de origen, p. ej. agrarios con trabajo temporal mal registrado).</t>
+        </is>
+      </c>
       <c r="P489" s="2" t="inlineStr">
         <is>
           <t>duracion_1er_empleo_signif &gt; COALESCE(t_total_empleo,0) + COALESCE(t_total_mixto_empl_desempl,0) + 1</t>
@@ -35368,27 +35508,27 @@
       </c>
       <c r="I504" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J504" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pasan</t>
         </is>
       </c>
       <c r="K504" s="2" t="n">
-        <v>1180</v>
+        <v>0</v>
       </c>
       <c r="L504" s="2" t="n">
-        <v>0.0868</v>
-      </c>
-      <c r="M504" s="2" t="inlineStr">
-        <is>
-          <t>G08</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M504" s="2" t="n"/>
       <c r="N504" s="2" t="n"/>
-      <c r="O504" s="2" t="inlineStr"/>
+      <c r="O504" s="2" t="inlineStr">
+        <is>
+          <t>Regla ajustada 2026-09-24 (G08): excluye a quien solo tiene episodios TRL 7xx/400 (dato de origen, p. ej. agrarios con trabajo temporal mal registrado).</t>
+        </is>
+      </c>
       <c r="P504" s="2" t="inlineStr">
         <is>
           <t>situacion_actual_afiliacion &lt;&gt; 'Nunca_ha_cotizado' AND fecha_ini_primer_empleo IS NULL</t>
@@ -39324,10 +39464,10 @@
         <v>111</v>
       </c>
       <c r="C2" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D2" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3">
@@ -39340,10 +39480,10 @@
         <v>112</v>
       </c>
       <c r="C3" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D3" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4">
@@ -39356,10 +39496,10 @@
         <v>338</v>
       </c>
       <c r="C4" t="n">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="D4" t="n">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="5">
@@ -39372,12 +39512,13 @@
         <v>561</v>
       </c>
       <c r="C5" t="n">
-        <v>391</v>
+        <v>398</v>
       </c>
       <c r="D5" t="n">
-        <v>170</v>
-      </c>
-    </row>
+        <v>163</v>
+      </c>
+    </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
@@ -39410,10 +39551,10 @@
         <v>381</v>
       </c>
       <c r="C8" t="n">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="D8" t="n">
-        <v>49</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9">
@@ -39426,10 +39567,10 @@
         <v>120</v>
       </c>
       <c r="C9" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D9" t="n">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="10">
@@ -39448,6 +39589,7 @@
         <v>47</v>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -39467,7 +39609,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>391</v>
+        <v>398</v>
       </c>
     </row>
     <row r="14">
@@ -39487,7 +39629,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>119</v>
+        <v>106</v>
       </c>
     </row>
     <row r="16">
@@ -39497,9 +39639,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>29</v>
-      </c>
-    </row>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
reglas: G16 - corrige C-259, C-279 y C-180; clasifica el resto como dato de origen
C-259 comparaba con bajas de empleo (otro universo que causas_baja_distintas):
ahora recuenta desde Afiliacion. C-279 excluye solo-prestaciones y empleo abierto.
C-180 trata 'N99 No consta' como pais desconocido. Las reglas de 1-1.088 casos
por cotizacion previa fuera de la muestra o errores puntuales pasan a G22 (baja
calidad); A-092 a G20. G16 queda con C-124, C-153 y C-314.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/reglas_consistencia_resultados_sin_ipf.xlsx
+++ b/tests/reglas_consistencia_resultados_sin_ipf.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1399,7 +1399,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Casos puntuales y fechas incoherentes</t>
+          <t>Provincia "NO CONSTA" con tiempo (código 56/53 del Mar), orfandad en mayores y clave fiscal</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -1408,32 +1408,32 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>4140</v>
+        <v>2615</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>0.305</v>
+        <v>0.1924</v>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>C-259, C-153, C-279, C-088, C-124, A-106, C-314, C-087, C-180, A-092, A-052, B-004, A-078, C-086, C-156, A-074, A-098</t>
+          <t>C-124, C-153, C-314</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>4.140 con más causas distintas que bajas + 2 (C-259), 2.619 orfandad con más de 60 años (C-154), 1.363 con desempleo &gt; 0 sin bajas (C-279), 1.081 con racha antes de 360 días tras el primer empleo (C-088), 524 con discapacidad por pensión sin pensión de incapacidad (C-151), 224 nacidos después de su primer empleo (C-078).</t>
+          <t>C-153: 2.615 con orfandad y más de 60 años; la pensión empieza a edad mediana 46 (95 %: 22 o más), 50/50 por sexo, 65 % Nunca_ha_cotizado; discapacidad no lo explica. C-124: 503 con prov_trabajo_ppal NO CONSTA y tiempo; en 502 el código de provincia del CCC (dígitos 5-6 de CCC_2) es 56 (y 53 en 79 episodios), que no está en provincias_dict.csv: 100 % de esos episodios son Régimen del Mar (08xx), domicilio A Coruña (15) o Pontevedra (36). C-314: 278, pendiente de reformular (desfasada tras clave_subclave_ppal).</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>Casos sueltos de la MCVL o reglas de baja confianza. C-278 (sin bajas con situacion Baja_*) SI se corrigio como regla (excluye a quien nunca tuvo empleo real) y ya no incumple.</t>
+          <t>C-124: el 56/53 parece un código especial del Mar en Galicia, no un error; la provincia real se podría sacar de domic_cc_2 (11.6k de 14.1k episodios; 2.4k con domic 0). C-153: por decidir (¿huérfanos adultos incapacitados o régimen antiguo?).</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>A revisar</t>
+          <t>A decidir</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1443,7 +1443,7 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>Revisar caso a caso solo los de confianza alta - sin decidir la mayoria.</t>
+          <t>C-124: decidir si se usa domic_cc_2 cuando el CCC es 56/53. C-153: seguir hablando. C-314: reformular.</t>
         </is>
       </c>
     </row>
@@ -1628,7 +1628,7 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>9</v>
@@ -1638,7 +1638,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>A-042, A-043, C-080, C-130, C-132, C-138</t>
+          <t>A-042, A-043, C-080, C-130, C-132, C-138, A-092</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1720,6 +1720,62 @@
       <c r="L22" s="2" t="inlineStr">
         <is>
           <t>Investigar cuando haya tiempo; volumen muy pequeño.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>G22</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Casos sueltos y cotización previa fuera de la muestra</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Baja calidad de los datos</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>1088</v>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>0.0801</v>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>C-279, C-088, C-087, A-106, A-052, B-004, A-078, C-086, C-156, A-074, A-098</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>C-088 (1.088) y C-087 (24): racha sin empleo a menos de 360 días del primer empleo o antes (88 % subsidio/asimilado, mediana 184 días). A-106 (486): Nunca_ha_cotizado con incapacidad, sobre todo Incapacidad&gt;65, edad mediana 89. C-279 (8) tras excluir solo-prestaciones y empleo abierto. Resto (1-5 personas cada una): A-052, B-004, A-078, C-086, C-156, A-074, A-098.</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Cotización previa fuera de la muestra (mismo motivo que G08) y errores puntuales del dato de origen.</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Dato de origen</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>Ninguna acción sobre el ETL.</t>
         </is>
       </c>
     </row>
@@ -5279,7 +5335,7 @@
       </c>
       <c r="J53" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K53" s="2" t="n">
@@ -5290,7 +5346,7 @@
       </c>
       <c r="M53" s="2" t="inlineStr">
         <is>
-          <t>G16</t>
+          <t>G22</t>
         </is>
       </c>
       <c r="N53" s="2" t="n"/>
@@ -6759,7 +6815,7 @@
       </c>
       <c r="J75" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K75" s="2" t="n">
@@ -6770,7 +6826,7 @@
       </c>
       <c r="M75" s="2" t="inlineStr">
         <is>
-          <t>G16</t>
+          <t>G22</t>
         </is>
       </c>
       <c r="N75" s="2" t="n"/>
@@ -7031,7 +7087,7 @@
       </c>
       <c r="J79" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K79" s="2" t="n">
@@ -7042,7 +7098,7 @@
       </c>
       <c r="M79" s="2" t="inlineStr">
         <is>
-          <t>G16</t>
+          <t>G22</t>
         </is>
       </c>
       <c r="N79" s="2" t="n"/>
@@ -7959,7 +8015,7 @@
       </c>
       <c r="J93" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K93" s="2" t="n">
@@ -7970,7 +8026,7 @@
       </c>
       <c r="M93" s="2" t="inlineStr">
         <is>
-          <t>G16</t>
+          <t>G20</t>
         </is>
       </c>
       <c r="N93" s="2" t="n"/>
@@ -8379,7 +8435,7 @@
       </c>
       <c r="J99" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K99" s="2" t="n">
@@ -8390,7 +8446,7 @@
       </c>
       <c r="M99" s="2" t="inlineStr">
         <is>
-          <t>G16</t>
+          <t>G22</t>
         </is>
       </c>
       <c r="N99" s="2" t="n"/>
@@ -8919,7 +8975,7 @@
       </c>
       <c r="J107" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K107" s="2" t="n">
@@ -8930,7 +8986,7 @@
       </c>
       <c r="M107" s="2" t="inlineStr">
         <is>
-          <t>G16</t>
+          <t>G22</t>
         </is>
       </c>
       <c r="N107" s="2" t="n"/>
@@ -9525,7 +9581,7 @@
       </c>
       <c r="J116" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K116" s="2" t="n">
@@ -9536,7 +9592,7 @@
       </c>
       <c r="M116" s="2" t="inlineStr">
         <is>
-          <t>G16</t>
+          <t>G22</t>
         </is>
       </c>
       <c r="N116" s="2" t="n"/>
@@ -22629,7 +22685,7 @@
       </c>
       <c r="J310" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K310" s="2" t="n">
@@ -22640,7 +22696,7 @@
       </c>
       <c r="M310" s="2" t="inlineStr">
         <is>
-          <t>G16</t>
+          <t>G22</t>
         </is>
       </c>
       <c r="N310" s="2" t="n"/>
@@ -22699,7 +22755,7 @@
       </c>
       <c r="J311" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K311" s="2" t="n">
@@ -22710,7 +22766,7 @@
       </c>
       <c r="M311" s="2" t="inlineStr">
         <is>
-          <t>G16</t>
+          <t>G22</t>
         </is>
       </c>
       <c r="N311" s="2" t="n"/>
@@ -22769,7 +22825,7 @@
       </c>
       <c r="J312" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K312" s="2" t="n">
@@ -22780,7 +22836,7 @@
       </c>
       <c r="M312" s="2" t="inlineStr">
         <is>
-          <t>G16</t>
+          <t>G22</t>
         </is>
       </c>
       <c r="N312" s="2" t="n"/>
@@ -27313,7 +27369,7 @@
       </c>
       <c r="J380" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K380" s="2" t="n">
@@ -27324,7 +27380,7 @@
       </c>
       <c r="M380" s="2" t="inlineStr">
         <is>
-          <t>G16</t>
+          <t>G22</t>
         </is>
       </c>
       <c r="N380" s="2" t="n"/>
@@ -28908,27 +28964,27 @@
       </c>
       <c r="I404" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J404" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pasan</t>
         </is>
       </c>
       <c r="K404" s="2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L404" s="2" t="n">
-        <v>0.0005</v>
-      </c>
-      <c r="M404" s="2" t="inlineStr">
-        <is>
-          <t>G16</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M404" s="2" t="n"/>
       <c r="N404" s="2" t="n"/>
-      <c r="O404" s="2" t="inlineStr"/>
+      <c r="O404" s="2" t="inlineStr">
+        <is>
+          <t>Regla ajustada 2026-09-24 (G16): 'N99 No consta' también es país desconocido.</t>
+        </is>
+      </c>
       <c r="P404" s="2" t="inlineStr">
         <is>
           <t>(prov_nacimiento IS NOT NULL AND prov_nacimiento NOT IN ('NO CONSTA','No consta','0 NO CONSTA','00 No consta')) AND pais_nacimiento NOT LIKE 'N00%' AND pais_nacimiento &lt;&gt; 'NO CONSTA'</t>
@@ -34058,27 +34114,27 @@
       </c>
       <c r="I483" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J483" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pasan</t>
         </is>
       </c>
       <c r="K483" s="2" t="n">
-        <v>4140</v>
+        <v>0</v>
       </c>
       <c r="L483" s="2" t="n">
-        <v>0.3046</v>
-      </c>
-      <c r="M483" s="2" t="inlineStr">
-        <is>
-          <t>G16</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M483" s="2" t="n"/>
       <c r="N483" s="2" t="n"/>
-      <c r="O483" s="2" t="inlineStr"/>
+      <c r="O483" s="2" t="inlineStr">
+        <is>
+          <t>Regla reformulada 2026-09-24 (G16): compara con las causas distintas de todos sus episodios en Afiliación; la anterior usaba num_bajas de empleo real (otro universo).</t>
+        </is>
+      </c>
       <c r="P483" s="2" t="inlineStr">
         <is>
           <t>tiempo_total_desde_inicio_vl &gt; 0 AND causas_baja_distintas &gt; ROUND(COALESCE(num_bajas_anual_promedio,0) * tiempo_total_desde_inicio_vl) + 2</t>
@@ -35443,22 +35499,26 @@
       </c>
       <c r="J503" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K503" s="2" t="n">
-        <v>1363</v>
+        <v>8</v>
       </c>
       <c r="L503" s="2" t="n">
-        <v>0.1003</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="M503" s="2" t="inlineStr">
         <is>
-          <t>G16</t>
+          <t>G22</t>
         </is>
       </c>
       <c r="N503" s="2" t="n"/>
-      <c r="O503" s="2" t="inlineStr"/>
+      <c r="O503" s="2" t="inlineStr">
+        <is>
+          <t>Regla ajustada 2026-09-24 (G16): excluye solo-prestaciones (G08) y empleo abierto (Alta_ocupado).</t>
+        </is>
+      </c>
       <c r="P503" s="2" t="inlineStr">
         <is>
           <t>t_total_desempleo &gt; 0 AND num_bajas_anual_promedio IS NULL</t>
@@ -39496,10 +39556,10 @@
         <v>338</v>
       </c>
       <c r="C4" t="n">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D4" t="n">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5">
@@ -39512,10 +39572,10 @@
         <v>561</v>
       </c>
       <c r="C5" t="n">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="D5" t="n">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="6"/>
@@ -39567,10 +39627,10 @@
         <v>120</v>
       </c>
       <c r="C9" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D9" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="10">
@@ -39583,10 +39643,10 @@
         <v>60</v>
       </c>
       <c r="C10" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D10" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="11"/>
@@ -39609,7 +39669,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>398</v>
+        <v>400</v>
       </c>
     </row>
     <row r="14">
@@ -39629,7 +39689,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>106</v>
+        <v>92</v>
       </c>
     </row>
     <row r="16">
@@ -39639,7 +39699,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>35</v>
+        <v>47</v>
       </c>
     </row>
     <row r="17"/>

</xml_diff>

<commit_message>
ETL: provincia "MAR" para los codigos 53/56 del CCC (Regimen del Mar)
Prov_trabajo_ppal etiquetaba como NO CONSTA los codigos 56 (y 53) de los digitos
5-6 de CCC_2: el 100 % de sus episodios son del Regimen del Mar, domicilio A Coruna
o Pontevedra. Ahora "MAR", solo en esta columna (en Prov_fiscal_actual el 53 es
otro codigo). Verificado con Grupo H regenerado: 503 personas, solo cambia esa
columna. C-124 pasa; C-201 admite 'MAR'.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/reglas_consistencia_resultados_sin_ipf.xlsx
+++ b/tests/reglas_consistencia_resultados_sin_ipf.xlsx
@@ -1399,7 +1399,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Provincia "NO CONSTA" con tiempo (código 56/53 del Mar), orfandad en mayores y clave fiscal</t>
+          <t>Orfandad en mayores, clave fiscal y provincia del Mar</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -1408,7 +1408,7 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E17" s="2" t="n">
         <v>2615</v>
@@ -1418,17 +1418,17 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>C-124, C-153, C-314</t>
+          <t>C-153, C-314</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>C-153: 2.615 con orfandad y más de 60 años; la pensión empieza a edad mediana 46 (95 %: 22 o más), 50/50 por sexo, 65 % Nunca_ha_cotizado; discapacidad no lo explica. C-124: 503 con prov_trabajo_ppal NO CONSTA y tiempo; en 502 el código de provincia del CCC (dígitos 5-6 de CCC_2) es 56 (y 53 en 79 episodios), que no está en provincias_dict.csv: 100 % de esos episodios son Régimen del Mar (08xx), domicilio A Coruña (15) o Pontevedra (36). C-314: 278, pendiente de reformular (desfasada tras clave_subclave_ppal).</t>
+          <t>C-153: 2.615 con orfandad y más de 60 años; la pensión empieza a edad mediana 46 (95 %: 22 o más), 50/50 por sexo, 65 % Nunca_ha_cotizado; discapacidad no lo explica. C-124 CORREGIDO 2026-09-24: 503 con prov_trabajo_ppal NO CONSTA y tiempo; en 502 el código de provincia del CCC (dígitos 5-6 de CCC_2) es 56 (y 53 en 79 episodios), que no está en provincias_dict.csv: 100 % de esos episodios son Régimen del Mar (08xx), domicilio A Coruña (15) o Pontevedra (36). C-314: 278, pendiente de reformular (desfasada tras clave_subclave_ppal). Resuelto: el código 56/53 se etiqueta 'MAR' (solo en Prov_trabajo_ppal; en Prov_fiscal_actual el 53 es Isla de La Palma).</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>C-124: el 56/53 parece un código especial del Mar en Galicia, no un error; la provincia real se podría sacar de domic_cc_2 (11.6k de 14.1k episodios; 2.4k con domic 0). C-153: por decidir (¿huérfanos adultos incapacitados o régimen antiguo?).</t>
+          <t>C-153: por decidir (¿huérfanos adultos incapacitados o régimen antiguo?). C-314: reformular.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
@@ -1443,7 +1443,7 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>C-124: decidir si se usa domic_cc_2 cuando el CCC es 56/53. C-153: seguir hablando. C-314: reformular.</t>
+          <t>C-153: seguir hablando. C-314: reformular.</t>
         </is>
       </c>
     </row>
@@ -25196,19 +25196,19 @@
       </c>
       <c r="I348" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J348" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Corregido</t>
         </is>
       </c>
       <c r="K348" s="2" t="n">
-        <v>503</v>
+        <v>0</v>
       </c>
       <c r="L348" s="2" t="n">
-        <v>0.037</v>
+        <v>0</v>
       </c>
       <c r="M348" s="2" t="inlineStr">
         <is>
@@ -25216,7 +25216,11 @@
         </is>
       </c>
       <c r="N348" s="2" t="n"/>
-      <c r="O348" s="2" t="inlineStr"/>
+      <c r="O348" s="2" t="inlineStr">
+        <is>
+          <t>Corregido 2026-09-24 (G16): los codigos 53/56 del CCC (Regimen del Mar, A Coruña/Pontevedra) se etiquetan 'MAR' en Prov_trabajo_ppal en vez de NO CONSTA (503 personas).</t>
+        </is>
+      </c>
       <c r="P348" s="2" t="inlineStr">
         <is>
           <t>t_tot_prov_ppal IS NOT NULL AND (prov_trabajo_ppal = 'NO CONSTA') AND t_tot_prov_ppal &gt; 0</t>
@@ -30271,7 +30275,7 @@
       <c r="E425" s="2" t="inlineStr"/>
       <c r="F425" s="2" t="inlineStr">
         <is>
-          <t>prov_trabajo_ppal = 'NN NOMBRE' (provincia) o NO CONSTA</t>
+          <t>prov_trabajo_ppal = 'NN NOMBRE' (provincia), 'MAR' o NO CONSTA</t>
         </is>
       </c>
       <c r="G425" s="2" t="inlineStr">
@@ -30302,7 +30306,11 @@
       </c>
       <c r="M425" s="2" t="inlineStr"/>
       <c r="N425" s="2" t="n"/>
-      <c r="O425" s="2" t="inlineStr"/>
+      <c r="O425" s="2" t="inlineStr">
+        <is>
+          <t>Regla ajustada 2026-09-24: 'MAR' es etiqueta valida sin codigo numerico.</t>
+        </is>
+      </c>
       <c r="P425" s="2" t="inlineStr">
         <is>
           <t>prov_trabajo_ppal IS NOT NULL AND prov_trabajo_ppal &lt;&gt; 'NO CONSTA' AND NOT regexp_matches(prov_trabajo_ppal, '^[0-9]{2} .+')</t>
@@ -39556,10 +39564,10 @@
         <v>338</v>
       </c>
       <c r="C4" t="n">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D4" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="5">
@@ -39572,10 +39580,10 @@
         <v>561</v>
       </c>
       <c r="C5" t="n">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="D5" t="n">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="6"/>
@@ -39627,10 +39635,10 @@
         <v>120</v>
       </c>
       <c r="C9" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D9" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10">
@@ -39679,7 +39687,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="15">
@@ -39689,7 +39697,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
ETL: codificacion comun de provincias (53 La Palma, 56 Mar, 66 y 98 Extranjero)
provincias_dict.csv pasa a servir todas las variables de provincia: 53 Isla de La
Palma (Prov_fiscal_actual, modelo 190), 56 Mar (CCC del Regimen del Mar), 66 Extranjero
(nacidos fuera, guia MCVL) y 98 Extranjero (residencia fiscal fuera). En el CCC el 53
tambien es del Mar y se pasa a 56 antes de decodificar (1 persona). Sustituye el
caso especial "MAR" del commit anterior.

Efecto verificado con Grupo H regenerado (1.359.056 x 72; solo cambian Prov_trabajo_ppal,
Prov_fiscal_actual y 05 PROV_NACIMIENTO): 503 en '56 MAR', 1.564 '53 ISLA DE LA PALMA',
1.020 '98 EXTRANJERO', 220.047 '66 EXTRANJERO'. Reglas: C-180 y C-338 ajustadas al
nuevo etiquetado; B-013/B-029/C-124 pasan.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/reglas_consistencia_resultados_sin_ipf.xlsx
+++ b/tests/reglas_consistencia_resultados_sin_ipf.xlsx
@@ -1352,17 +1352,17 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E16" s="2" t="n">
         <v>90084</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>6.628</v>
+        <v>6.6284</v>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>B-014, C-166, B-030, B-012, B-013, C-169, B-028, B-029</t>
+          <t>B-012, B-014, B-028, B-030, C-166, C-169</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1423,7 +1423,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>C-153: 2.615 con orfandad y más de 60 años; la pensión empieza a edad mediana 46 (95 %: 22 o más), 50/50 por sexo, 65 % Nunca_ha_cotizado; discapacidad no lo explica. C-124 CORREGIDO 2026-09-24: 503 con prov_trabajo_ppal NO CONSTA y tiempo; en 502 el código de provincia del CCC (dígitos 5-6 de CCC_2) es 56 (y 53 en 79 episodios), que no está en provincias_dict.csv: 100 % de esos episodios son Régimen del Mar (08xx), domicilio A Coruña (15) o Pontevedra (36). C-314: 278, pendiente de reformular (desfasada tras clave_subclave_ppal). Resuelto: el código 56/53 se etiqueta 'MAR' (solo en Prov_trabajo_ppal; en Prov_fiscal_actual el 53 es Isla de La Palma).</t>
+          <t>C-153: 2.615 con orfandad y más de 60 años; la pensión empieza a edad mediana 46 (95 %: 22 o más), 50/50 por sexo, 65 % Nunca_ha_cotizado; discapacidad no lo explica. C-124 CORREGIDO 2026-09-24: 503 con prov_trabajo_ppal NO CONSTA y tiempo; en 502 el código de provincia del CCC (dígitos 5-6 de CCC_2) es 56 (y 53 en 79 episodios), que no está en provincias_dict.csv: 100 % de esos episodios son Régimen del Mar (08xx), domicilio A Coruña (15) o Pontevedra (36). C-314: 278, pendiente de reformular (desfasada tras clave_subclave_ppal). Resuelto: el código 56/53 se etiqueta '56 MAR' (solo en Prov_trabajo_ppal; el 53 fiscal es Isla de La Palma (53) y el 98 Extranjero: codificación común de provincias, 66 Extranjero para nacidos fuera).</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -1467,14 +1467,14 @@
         <v>11</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>61377</v>
+        <v>61583</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>4.516</v>
+        <v>4.5313</v>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>C-338, C-312, C-311, C-313, C-309, C-302, C-310, C-300, C-301, C-306, C-299</t>
+          <t>C-299, C-300, C-301, C-302, C-306, C-309, C-310, C-311, C-312, C-313, C-338</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -10190,19 +10190,19 @@
       </c>
       <c r="I125" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J125" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Corregido</t>
         </is>
       </c>
       <c r="K125" s="2" t="n">
-        <v>169</v>
+        <v>0</v>
       </c>
       <c r="L125" s="2" t="n">
-        <v>0.0124</v>
+        <v>0</v>
       </c>
       <c r="M125" s="2" t="inlineStr">
         <is>
@@ -10210,7 +10210,11 @@
         </is>
       </c>
       <c r="N125" s="2" t="n"/>
-      <c r="O125" s="2" t="inlineStr"/>
+      <c r="O125" s="2" t="inlineStr">
+        <is>
+          <t>Corregido 2026-09-24: 169 ocupados sin provincia de trabajo eran del Regimen del Mar (codigo 56 del CCC), ahora '56 MAR'.</t>
+        </is>
+      </c>
       <c r="P125" s="2" t="inlineStr">
         <is>
           <t>situacion_paro_ocupacion = 'Ocupado' AND NOT (prov_trabajo_ppal IS NOT NULL AND prov_trabajo_ppal NOT IN ('NO CONSTA','No consta','0 NO CONSTA','00 No consta'))</t>
@@ -11282,19 +11286,19 @@
       </c>
       <c r="I141" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J141" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Corregido</t>
         </is>
       </c>
       <c r="K141" s="2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="L141" s="2" t="n">
-        <v>0.0005</v>
+        <v>0</v>
       </c>
       <c r="M141" s="2" t="inlineStr">
         <is>
@@ -11302,7 +11306,11 @@
         </is>
       </c>
       <c r="N141" s="2" t="n"/>
-      <c r="O141" s="2" t="inlineStr"/>
+      <c r="O141" s="2" t="inlineStr">
+        <is>
+          <t>Corregido 2026-09-24: 7 casos del Regimen del Mar (codigo 56 del CCC), ahora '56 MAR'.</t>
+        </is>
+      </c>
       <c r="P141" s="2" t="inlineStr">
         <is>
           <t>situacion_paro_ocupacion = 'Ocupado_y_pensionista' AND NOT (prov_trabajo_ppal IS NOT NULL AND prov_trabajo_ppal NOT IN ('NO CONSTA','No consta','0 NO CONSTA','00 No consta'))</t>
@@ -25218,7 +25226,7 @@
       <c r="N348" s="2" t="n"/>
       <c r="O348" s="2" t="inlineStr">
         <is>
-          <t>Corregido 2026-09-24 (G16): los codigos 53/56 del CCC (Regimen del Mar, A Coruña/Pontevedra) se etiquetan 'MAR' en Prov_trabajo_ppal en vez de NO CONSTA (503 personas).</t>
+          <t>Corregido 2026-09-24 (G16): codificacion comun de provincias; los codigos 53/56 del CCC (Regimen del Mar) se etiquetan '56 MAR' en Prov_trabajo_ppal (503 personas).</t>
         </is>
       </c>
       <c r="P348" s="2" t="inlineStr">
@@ -28037,10 +28045,10 @@
         </is>
       </c>
       <c r="K390" s="2" t="n">
-        <v>3030</v>
+        <v>446</v>
       </c>
       <c r="L390" s="2" t="n">
-        <v>0.2229</v>
+        <v>0.0328</v>
       </c>
       <c r="M390" s="2" t="inlineStr">
         <is>
@@ -28048,7 +28056,11 @@
         </is>
       </c>
       <c r="N390" s="2" t="n"/>
-      <c r="O390" s="2" t="inlineStr"/>
+      <c r="O390" s="2" t="inlineStr">
+        <is>
+          <t>Mejora 2026-09-24: la provincia fiscal 53 (Isla de La Palma) y 98 (Extranjero) ya se decodifican (codificacion comun).</t>
+        </is>
+      </c>
       <c r="P390" s="2" t="inlineStr">
         <is>
           <t>ingresos_bruto_total_2024 &gt; 0 AND NOT (prov_fiscal_actual IS NOT NULL AND prov_fiscal_actual NOT IN ('NO CONSTA','No consta','0 NO CONSTA','00 No consta'))</t>
@@ -28986,7 +28998,7 @@
       <c r="N404" s="2" t="n"/>
       <c r="O404" s="2" t="inlineStr">
         <is>
-          <t>Regla ajustada 2026-09-24 (G16): 'N99 No consta' también es país desconocido.</t>
+          <t>Regla ajustada 2026-09-24: '66 EXTRANJERO' (nacidos en el extranjero) no es provincia española.</t>
         </is>
       </c>
       <c r="P404" s="2" t="inlineStr">
@@ -30275,7 +30287,7 @@
       <c r="E425" s="2" t="inlineStr"/>
       <c r="F425" s="2" t="inlineStr">
         <is>
-          <t>prov_trabajo_ppal = 'NN NOMBRE' (provincia), 'MAR' o NO CONSTA</t>
+          <t>prov_trabajo_ppal = 'NN NOMBRE' (provincia) o NO CONSTA</t>
         </is>
       </c>
       <c r="G425" s="2" t="inlineStr">
@@ -30306,11 +30318,7 @@
       </c>
       <c r="M425" s="2" t="inlineStr"/>
       <c r="N425" s="2" t="n"/>
-      <c r="O425" s="2" t="inlineStr">
-        <is>
-          <t>Regla ajustada 2026-09-24: 'MAR' es etiqueta valida sin codigo numerico.</t>
-        </is>
-      </c>
+      <c r="O425" s="2" t="n"/>
       <c r="P425" s="2" t="inlineStr">
         <is>
           <t>prov_trabajo_ppal IS NOT NULL AND prov_trabajo_ppal &lt;&gt; 'NO CONSTA' AND NOT regexp_matches(prov_trabajo_ppal, '^[0-9]{2} .+')</t>
@@ -39457,10 +39465,10 @@
         </is>
       </c>
       <c r="K562" s="2" t="n">
-        <v>61377</v>
+        <v>61583</v>
       </c>
       <c r="L562" s="2" t="n">
-        <v>4.5161</v>
+        <v>4.5313</v>
       </c>
       <c r="M562" s="2" t="inlineStr">
         <is>
@@ -39470,7 +39478,7 @@
       <c r="N562" s="2" t="n"/>
       <c r="O562" s="2" t="inlineStr">
         <is>
-          <t>El domicilio fiscal es el del 31-12-2024; puede haber mudanzas</t>
+          <t>El domicilio fiscal es el del 31-12-2024; puede haber mudanzas | Regla ajustada 2026-09-24: el 53 fiscal (Isla de La Palma) es provincia 38 en el INE y el 98 (residencia fiscal en el extranjero) no es comparable.</t>
         </is>
       </c>
       <c r="P562" s="2" t="inlineStr">
@@ -39548,10 +39556,10 @@
         <v>112</v>
       </c>
       <c r="C3" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D3" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4">
@@ -39580,10 +39588,10 @@
         <v>561</v>
       </c>
       <c r="C5" t="n">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="D5" t="n">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="6"/>
@@ -39651,10 +39659,10 @@
         <v>60</v>
       </c>
       <c r="C10" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D10" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11"/>
@@ -39687,7 +39695,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="15">
@@ -39697,7 +39705,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
tests: reglas sobre el final regenerado sin numexpr (404 de 561 pasan)
Resultados sin IPF actualizados con el final del otro PC (H repetido sin numexpr). A y B
identicas; C se mueve 1-3 personas por el calculo no determinista de los tiempos por
categoria. C-062/C-068 (748.798) pasan a 0: eran del Parquet roto (%T_total_DESEMPLEO a 0).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/reglas_consistencia_resultados_sin_ipf.xlsx
+++ b/tests/reglas_consistencia_resultados_sin_ipf.xlsx
@@ -628,22 +628,18 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>748798</v>
+        <v>0</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>55.097</v>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>C-062, C-068</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2 personas con T_total_NO_EMPLEO negativo (C-010, C-025, C-067) y 1 con pct_t_total_empleo &gt; 100 (C-061).</t>
+          <t>2 personas con T_total_NO_EMPLEO negativo (C-010, C-025, C-067) y 1 con pct_t_total_empleo &gt; 100 (C-061). NOTA 2026-09-24: C-062 y C-068 (748.798) venian de un Parquet roto (%T_total_DESEMPLEO a 0 por fallo intermitente de numexpr, ya desactivado); con el Parquet bueno pasan.</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -687,14 +683,14 @@
         <v>7</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0</v>
+        <v>0.0002</v>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>C-044, C-042, C-043, C-041, C-045, C-049, C-050</t>
+          <t>C-041, C-042, C-043, C-044, C-045, C-049, C-050</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -746,11 +742,11 @@
         <v>37024</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>2.724</v>
+        <v>2.7242</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>C-107, C-079, C-105, C-058, C-168, C-054, C-056, C-051, C-053, C-106, C-083, C-052, C-055, A-093, C-114, C-115, C-057, C-239, B-073, B-070, C-096, C-251, B-043, B-040, B-054, C-097, B-084, C-085</t>
+          <t>A-093, B-040, B-043, B-054, B-070, B-073, B-084, C-051, C-052, C-053, C-054, C-055, C-056, C-057, C-058, C-079, C-083, C-085, C-096, C-097, C-105, C-106, C-107, C-114, C-115, C-168, C-239, C-251</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -1187,14 +1183,14 @@
         <v>11</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>8907</v>
+        <v>8906</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0.655</v>
+        <v>0.6553</v>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>C-230, C-232, C-231, C-234, C-236, C-235, C-233, C-240, C-238, C-237, C-241</t>
+          <t>C-230, C-231, C-232, C-233, C-234, C-235, C-236, C-237, C-238, C-240, C-241</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1578,11 +1574,11 @@
         <v>19912</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>1.465</v>
+        <v>1.4651</v>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>C-095, C-250, C-247, C-248, C-243, C-249, C-244, C-245, C-246</t>
+          <t>C-095, C-243, C-244, C-245, C-246, C-247, C-248, C-249, C-250</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -18736,23 +18732,27 @@
       </c>
       <c r="I252" s="6" t="inlineStr">
         <is>
-          <t>PASA</t>
+          <t>INCUMPLE</t>
         </is>
       </c>
       <c r="J252" s="6" t="inlineStr">
         <is>
-          <t>Pasan</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="K252" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L252" s="2" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="M252" s="2" t="inlineStr"/>
       <c r="N252" s="2" t="n"/>
-      <c r="O252" s="2" t="inlineStr"/>
+      <c r="O252" s="2" t="inlineStr">
+        <is>
+          <t>Cifra actualizada 2026-09-24: variación de unas pocas personas por el cálculo no determinista de los tiempos por categoría (374 personas difieren entre regeneraciones).</t>
+        </is>
+      </c>
       <c r="P252" s="2" t="inlineStr">
         <is>
           <t>t_tot_grupo_ppal &gt; edad_actual_fecha_corte + 1</t>
@@ -18882,9 +18882,13 @@
       <c r="L254" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="M254" s="2" t="inlineStr"/>
+      <c r="M254" s="2" t="n"/>
       <c r="N254" s="2" t="n"/>
-      <c r="O254" s="2" t="inlineStr"/>
+      <c r="O254" s="2" t="inlineStr">
+        <is>
+          <t>Cifra actualizada 2026-09-24: variación de unas pocas personas por el cálculo no determinista de los tiempos por categoría (374 personas difieren entre regeneraciones).</t>
+        </is>
+      </c>
       <c r="P254" s="2" t="inlineStr">
         <is>
           <t>t_tot_tipo_contrato_ppal &gt; edad_actual_fecha_corte + 1</t>
@@ -18948,9 +18952,13 @@
       <c r="L255" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="M255" s="2" t="inlineStr"/>
+      <c r="M255" s="2" t="n"/>
       <c r="N255" s="2" t="n"/>
-      <c r="O255" s="2" t="inlineStr"/>
+      <c r="O255" s="2" t="inlineStr">
+        <is>
+          <t>Cifra actualizada 2026-09-24: variación de unas pocas personas por el cálculo no determinista de los tiempos por categoría (374 personas difieren entre regeneraciones).</t>
+        </is>
+      </c>
       <c r="P255" s="2" t="inlineStr">
         <is>
           <t>t_tot_prov_ppal &gt; edad_actual_fecha_corte + 1</t>
@@ -19618,7 +19626,11 @@
         </is>
       </c>
       <c r="N265" s="2" t="n"/>
-      <c r="O265" s="2" t="inlineStr"/>
+      <c r="O265" s="2" t="inlineStr">
+        <is>
+          <t>Cifra actualizada 2026-09-24: variación de unas pocas personas por el cálculo no determinista de los tiempos por categoría (374 personas difieren entre regeneraciones).</t>
+        </is>
+      </c>
       <c r="P265" s="2" t="inlineStr">
         <is>
           <t>t_tot_reg_ppal &gt; tiempo_total_desde_inicio_vl + 1</t>
@@ -19688,7 +19700,11 @@
         </is>
       </c>
       <c r="N266" s="2" t="n"/>
-      <c r="O266" s="2" t="inlineStr"/>
+      <c r="O266" s="2" t="inlineStr">
+        <is>
+          <t>Cifra actualizada 2026-09-24: variación de unas pocas personas por el cálculo no determinista de los tiempos por categoría (374 personas difieren entre regeneraciones).</t>
+        </is>
+      </c>
       <c r="P266" s="2" t="inlineStr">
         <is>
           <t>t_tot_grupo_ppal &gt; tiempo_total_desde_inicio_vl + 1</t>
@@ -19747,7 +19763,7 @@
         </is>
       </c>
       <c r="K267" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L267" s="2" t="n">
         <v>0.0001</v>
@@ -19758,7 +19774,11 @@
         </is>
       </c>
       <c r="N267" s="2" t="n"/>
-      <c r="O267" s="2" t="inlineStr"/>
+      <c r="O267" s="2" t="inlineStr">
+        <is>
+          <t>Cifra actualizada 2026-09-24: variación de unas pocas personas por el cálculo no determinista de los tiempos por categoría (374 personas difieren entre regeneraciones).</t>
+        </is>
+      </c>
       <c r="P267" s="2" t="inlineStr">
         <is>
           <t>t_tot_tipo_contrato_ppal &gt; tiempo_total_desde_inicio_vl + 1</t>
@@ -19817,10 +19837,10 @@
         </is>
       </c>
       <c r="K268" s="2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L268" s="2" t="n">
-        <v>0.0004</v>
+        <v>0.0002</v>
       </c>
       <c r="M268" s="2" t="inlineStr">
         <is>
@@ -19828,7 +19848,11 @@
         </is>
       </c>
       <c r="N268" s="2" t="n"/>
-      <c r="O268" s="2" t="inlineStr"/>
+      <c r="O268" s="2" t="inlineStr">
+        <is>
+          <t>Cifra actualizada 2026-09-24: variación de unas pocas personas por el cálculo no determinista de los tiempos por categoría (374 personas difieren entre regeneraciones).</t>
+        </is>
+      </c>
       <c r="P268" s="2" t="inlineStr">
         <is>
           <t>t_tot_prov_ppal &gt; tiempo_total_desde_inicio_vl + 1</t>
@@ -19887,7 +19911,7 @@
         </is>
       </c>
       <c r="K269" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L269" s="2" t="n">
         <v>0.0001</v>
@@ -19898,7 +19922,11 @@
         </is>
       </c>
       <c r="N269" s="2" t="n"/>
-      <c r="O269" s="2" t="inlineStr"/>
+      <c r="O269" s="2" t="inlineStr">
+        <is>
+          <t>Cifra actualizada 2026-09-24: variación de unas pocas personas por el cálculo no determinista de los tiempos por categoría (374 personas difieren entre regeneraciones).</t>
+        </is>
+      </c>
       <c r="P269" s="2" t="inlineStr">
         <is>
           <t>t_tot_act_econ_ppal &gt; tiempo_total_desde_inicio_vl + 1</t>
@@ -20308,7 +20336,7 @@
       <c r="N275" s="2" t="n"/>
       <c r="O275" s="2" t="inlineStr">
         <is>
-          <t>16 años (decisión del usuario). Hasta 1980 la edad mínima legal era 14: pueden salir casos antiguos legítimos</t>
+          <t>16 años (decisión del usuario). Hasta 1980 la edad mínima legal era 14: pueden salir casos antiguos legítimos | Cifra actualizada 2026-09-24: variación de unas pocas personas por el cálculo no determinista de los tiempos por categoría (374 personas difieren entre regeneraciones).</t>
         </is>
       </c>
       <c r="P275" s="2" t="inlineStr">
@@ -20382,7 +20410,7 @@
       <c r="N276" s="2" t="n"/>
       <c r="O276" s="2" t="inlineStr">
         <is>
-          <t>16 años (decisión del usuario). Hasta 1980 la edad mínima legal era 14: pueden salir casos antiguos legítimos</t>
+          <t>16 años (decisión del usuario). Hasta 1980 la edad mínima legal era 14: pueden salir casos antiguos legítimos | Cifra actualizada 2026-09-24: variación de unas pocas personas por el cálculo no determinista de los tiempos por categoría (374 personas difieren entre regeneraciones).</t>
         </is>
       </c>
       <c r="P276" s="2" t="inlineStr">
@@ -20456,7 +20484,7 @@
       <c r="N277" s="2" t="n"/>
       <c r="O277" s="2" t="inlineStr">
         <is>
-          <t>16 años (decisión del usuario). Hasta 1980 la edad mínima legal era 14: pueden salir casos antiguos legítimos</t>
+          <t>16 años (decisión del usuario). Hasta 1980 la edad mínima legal era 14: pueden salir casos antiguos legítimos | Cifra actualizada 2026-09-24: variación de unas pocas personas por el cálculo no determinista de los tiempos por categoría (374 personas difieren entre regeneraciones).</t>
         </is>
       </c>
       <c r="P277" s="2" t="inlineStr">
@@ -20517,10 +20545,10 @@
         </is>
       </c>
       <c r="K278" s="2" t="n">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="L278" s="2" t="n">
-        <v>0.0304</v>
+        <v>0.0302</v>
       </c>
       <c r="M278" s="2" t="inlineStr">
         <is>
@@ -20530,7 +20558,7 @@
       <c r="N278" s="2" t="n"/>
       <c r="O278" s="2" t="inlineStr">
         <is>
-          <t>16 años (decisión del usuario). Hasta 1980 la edad mínima legal era 14: pueden salir casos antiguos legítimos</t>
+          <t>16 años (decisión del usuario). Hasta 1980 la edad mínima legal era 14: pueden salir casos antiguos legítimos | Cifra actualizada 2026-09-24: variación de unas pocas personas por el cálculo no determinista de los tiempos por categoría (374 personas difieren entre regeneraciones).</t>
         </is>
       </c>
       <c r="P278" s="2" t="inlineStr">
@@ -21072,27 +21100,27 @@
       </c>
       <c r="I286" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J286" s="4" t="inlineStr">
         <is>
-          <t>Baja calidad de los datos</t>
+          <t>Pasan</t>
         </is>
       </c>
       <c r="K286" s="2" t="n">
-        <v>748798</v>
+        <v>0</v>
       </c>
       <c r="L286" s="2" t="n">
-        <v>55.0969</v>
-      </c>
-      <c r="M286" s="2" t="inlineStr">
-        <is>
-          <t>G02</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M286" s="2" t="n"/>
       <c r="N286" s="2" t="n"/>
-      <c r="O286" s="2" t="inlineStr"/>
+      <c r="O286" s="2" t="inlineStr">
+        <is>
+          <t>Actualizado 2026-09-24: las 748.798 incumplidoras anteriores venian de un Parquet roto (%T_total_DESEMPLEO a 0 por fallo intermitente de numexpr); con el Parquet bueno la regla pasa.</t>
+        </is>
+      </c>
       <c r="P286" s="2" t="inlineStr">
         <is>
           <t>tiempo_total_desde_inicio_vl &gt; 0 AND ABS(pct_t_total_desempleo - 100 * t_total_desempleo / tiempo_total_desde_inicio_vl) &gt; 0.5</t>
@@ -21460,27 +21488,27 @@
       </c>
       <c r="I292" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J292" s="4" t="inlineStr">
         <is>
-          <t>Baja calidad de los datos</t>
+          <t>Pasan</t>
         </is>
       </c>
       <c r="K292" s="2" t="n">
-        <v>748798</v>
+        <v>0</v>
       </c>
       <c r="L292" s="2" t="n">
-        <v>55.0969</v>
-      </c>
-      <c r="M292" s="2" t="inlineStr">
-        <is>
-          <t>G02</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M292" s="2" t="n"/>
       <c r="N292" s="2" t="n"/>
-      <c r="O292" s="2" t="inlineStr"/>
+      <c r="O292" s="2" t="inlineStr">
+        <is>
+          <t>Actualizado 2026-09-24: las 748.798 incumplidoras anteriores venian de un Parquet roto (%T_total_DESEMPLEO a 0 por fallo intermitente de numexpr); con el Parquet bueno la regla pasa.</t>
+        </is>
+      </c>
       <c r="P292" s="2" t="inlineStr">
         <is>
           <t>ABS(pct_t_total_empleo + pct_t_total_desempleo + pct_t_total_mixto_empl_desempl + pct_t_total_no_empleo - 100) &gt; 0.5</t>
@@ -32113,10 +32141,10 @@
         </is>
       </c>
       <c r="K454" s="2" t="n">
-        <v>8907</v>
+        <v>8906</v>
       </c>
       <c r="L454" s="2" t="n">
-        <v>0.6554</v>
+        <v>0.6553</v>
       </c>
       <c r="M454" s="2" t="inlineStr">
         <is>
@@ -32126,7 +32154,7 @@
       <c r="N454" s="2" t="n"/>
       <c r="O454" s="2" t="inlineStr">
         <is>
-          <t>La actividad principal puede ser de otro periodo</t>
+          <t>La actividad principal puede ser de otro periodo | Cifra actualizada 2026-09-24 (variacion de 1 persona por el cálculo no determinista).</t>
         </is>
       </c>
       <c r="P454" s="2" t="inlineStr">
@@ -32338,7 +32366,11 @@
         </is>
       </c>
       <c r="N457" s="2" t="n"/>
-      <c r="O457" s="2" t="inlineStr"/>
+      <c r="O457" s="2" t="inlineStr">
+        <is>
+          <t>Cifra actualizada 2026-09-24: variación de unas pocas personas por el cálculo no determinista de los tiempos por categoría (374 personas difieren entre regeneraciones).</t>
+        </is>
+      </c>
       <c r="P457" s="2" t="inlineStr">
         <is>
           <t>reg_cotiz_ppal_agrupado LIKE '0138 %' AND (act_econ_ppal IS NOT NULL AND act_econ_ppal NOT IN ('NO CONSTA','No consta','0 NO CONSTA','00 No consta')) AND act_econ_ppal NOT LIKE '970%'</t>
@@ -32537,7 +32569,7 @@
         </is>
       </c>
       <c r="K460" s="2" t="n">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="L460" s="2" t="n">
         <v>0.0124</v>
@@ -32548,7 +32580,11 @@
         </is>
       </c>
       <c r="N460" s="2" t="n"/>
-      <c r="O460" s="2" t="inlineStr"/>
+      <c r="O460" s="2" t="inlineStr">
+        <is>
+          <t>Cifra actualizada 2026-09-24 (variacion de 1 persona por el cálculo no determinista).</t>
+        </is>
+      </c>
       <c r="P460" s="2" t="inlineStr">
         <is>
           <t>reg_cotiz_ppal_agrupado LIKE '05 %' AND grupo_cotiz_ppal NOT IN ('0 NO CONSTA','NO CONSTA')</t>
@@ -32677,10 +32713,10 @@
         </is>
       </c>
       <c r="K462" s="2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="L462" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0009</v>
       </c>
       <c r="M462" s="2" t="inlineStr">
         <is>
@@ -32688,7 +32724,11 @@
         </is>
       </c>
       <c r="N462" s="2" t="n"/>
-      <c r="O462" s="2" t="inlineStr"/>
+      <c r="O462" s="2" t="inlineStr">
+        <is>
+          <t>Cifra actualizada 2026-09-24 (variacion de 1 persona por el cálculo no determinista).</t>
+        </is>
+      </c>
       <c r="P462" s="2" t="inlineStr">
         <is>
           <t>reg_cotiz_ppal_agrupado LIKE '05 %' AND tipo_contr_ppal_agrupado NOT IN ('No consta')</t>
@@ -32828,7 +32868,11 @@
         </is>
       </c>
       <c r="N464" s="2" t="n"/>
-      <c r="O464" s="2" t="inlineStr"/>
+      <c r="O464" s="2" t="inlineStr">
+        <is>
+          <t>Cifra actualizada 2026-09-24: variación de unas pocas personas por el cálculo no determinista de los tiempos por categoría (374 personas difieren entre regeneraciones).</t>
+        </is>
+      </c>
       <c r="P464" s="2" t="inlineStr">
         <is>
           <t>reg_cotiz_ppal_agrupado LIKE '06 %' AND t_tot_reg_ppal &gt; 45.5</t>
@@ -32962,9 +33006,13 @@
       <c r="L466" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="M466" s="2" t="inlineStr"/>
+      <c r="M466" s="2" t="n"/>
       <c r="N466" s="2" t="n"/>
-      <c r="O466" s="2" t="inlineStr"/>
+      <c r="O466" s="2" t="inlineStr">
+        <is>
+          <t>Cifra actualizada 2026-09-24: variación de unas pocas personas por el cálculo no determinista de los tiempos por categoría (374 personas difieren entre regeneraciones).</t>
+        </is>
+      </c>
       <c r="P466" s="2" t="inlineStr">
         <is>
           <t>reg_cotiz_ppal_agrupado LIKE '0138 %' AND t_tot_reg_ppal &gt; 13.5</t>
@@ -33513,10 +33561,10 @@
         </is>
       </c>
       <c r="K474" s="2" t="n">
-        <v>17708</v>
+        <v>17707</v>
       </c>
       <c r="L474" s="2" t="n">
-        <v>1.303</v>
+        <v>1.3029</v>
       </c>
       <c r="M474" s="2" t="inlineStr">
         <is>
@@ -33524,7 +33572,11 @@
         </is>
       </c>
       <c r="N474" s="2" t="n"/>
-      <c r="O474" s="2" t="inlineStr"/>
+      <c r="O474" s="2" t="inlineStr">
+        <is>
+          <t>Cifra actualizada 2026-09-24 (variacion de 1 persona por el cálculo no determinista).</t>
+        </is>
+      </c>
       <c r="P474" s="2" t="inlineStr">
         <is>
           <t>grupo_cotiz_1er_empleo_signif LIKE '10 %' AND edad_primer_empleo_signif &lt; 17.9</t>
@@ -39572,10 +39624,10 @@
         <v>338</v>
       </c>
       <c r="C4" t="n">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D4" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="5">
@@ -39588,10 +39640,10 @@
         <v>561</v>
       </c>
       <c r="C5" t="n">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="D5" t="n">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="6"/>
@@ -39627,10 +39679,10 @@
         <v>381</v>
       </c>
       <c r="C8" t="n">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="D8" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9">
@@ -39685,7 +39737,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>400</v>
+        <v>401</v>
       </c>
     </row>
     <row r="14">
@@ -39705,7 +39757,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="16">
@@ -39715,7 +39767,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="17"/>

</xml_diff>

<commit_message>
reglas: reformula C-314 (clave fiscal NO CONSTA <=> ingresos nulos o 0)
Las 278 incumplidoras eran personas con fila fiscal con ingresos a 0 en todas las partes:
la clave sale de la percepcion con mas ingresos y con 0 no hay ninguna. Con la regla
nueva, 0 incumplimientos (tambien en el sentido clave real con ingresos 0).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/reglas_consistencia_resultados_sin_ipf.xlsx
+++ b/tests/reglas_consistencia_resultados_sin_ipf.xlsx
@@ -1395,7 +1395,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Orfandad en mayores, clave fiscal y provincia del Mar</t>
+          <t>Orfandad en mayores de 60</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -1404,7 +1404,7 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E17" s="2" t="n">
         <v>2615</v>
@@ -1414,12 +1414,12 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>C-153, C-314</t>
+          <t>C-153</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>C-153: 2.615 con orfandad y más de 60 años; la pensión empieza a edad mediana 46 (95 %: 22 o más), 50/50 por sexo, 65 % Nunca_ha_cotizado; discapacidad no lo explica. C-124 CORREGIDO 2026-09-24: 503 con prov_trabajo_ppal NO CONSTA y tiempo; en 502 el código de provincia del CCC (dígitos 5-6 de CCC_2) es 56 (y 53 en 79 episodios), que no está en provincias_dict.csv: 100 % de esos episodios son Régimen del Mar (08xx), domicilio A Coruña (15) o Pontevedra (36). C-314: 278, pendiente de reformular (desfasada tras clave_subclave_ppal). Resuelto: el código 56/53 se etiqueta '56 MAR' (solo en Prov_trabajo_ppal; el 53 fiscal es Isla de La Palma (53) y el 98 Extranjero: codificación común de provincias, 66 Extranjero para nacidos fuera).</t>
+          <t>C-153: 2.615 con orfandad y más de 60 años; la pensión empieza a edad mediana 46 (95 %: 22 o más), 50/50 por sexo, 65 % Nunca_ha_cotizado; discapacidad no lo explica. C-124 CORREGIDO 2026-09-24: 503 con prov_trabajo_ppal NO CONSTA y tiempo; en 502 el código de provincia del CCC (dígitos 5-6 de CCC_2) es 56 (y 53 en 79 episodios), que no está en provincias_dict.csv: 100 % de esos episodios son Régimen del Mar (08xx), domicilio A Coruña (15) o Pontevedra (36). C-314: 278, pendiente de reformular (desfasada tras clave_subclave_ppal). Resuelto: el código 56/53 se etiqueta '56 MAR' (solo en Prov_trabajo_ppal; el 53 fiscal es Isla de La Palma (53) y el 98 Extranjero: codificación común de provincias, 66 Extranjero para nacidos fuera). C-314 CORREGIDA 2026-09-24: regla reformulada (clave NO CONSTA ⇔ ingresos nulos o 0), 0 incumplimientos.</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>C-153: seguir hablando. C-314: reformular.</t>
+          <t>C-153: seguir hablando.</t>
         </is>
       </c>
     </row>
@@ -37925,7 +37925,7 @@
       </c>
       <c r="F538" s="2" t="inlineStr">
         <is>
-          <t>clave_subclave_ppal = NO CONSTA ⇔ no hay datos fiscales</t>
+          <t>clave_subclave_ppal = NO CONSTA ⇔ ingresos fiscales nulos o 0</t>
         </is>
       </c>
       <c r="G538" s="2" t="inlineStr">
@@ -37940,19 +37940,19 @@
       </c>
       <c r="I538" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J538" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Corregido</t>
         </is>
       </c>
       <c r="K538" s="2" t="n">
-        <v>278</v>
+        <v>0</v>
       </c>
       <c r="L538" s="2" t="n">
-        <v>0.0205</v>
+        <v>0</v>
       </c>
       <c r="M538" s="2" t="inlineStr">
         <is>
@@ -37960,10 +37960,14 @@
         </is>
       </c>
       <c r="N538" s="2" t="n"/>
-      <c r="O538" s="2" t="inlineStr"/>
+      <c r="O538" s="2" t="inlineStr">
+        <is>
+          <t>Regla reformulada 2026-09-24 (G16): la clave sale de la percepción con más ingresos; las 278 personas con fila fiscal a 0 no tienen ninguna que elegir. Con la regla nueva, 0 incumplimientos.</t>
+        </is>
+      </c>
       <c r="P538" s="2" t="inlineStr">
         <is>
-          <t>(clave_subclave_ppal = 'NO CONSTA') &lt;&gt; (ingresos_bruto_total_2024 IS NULL)</t>
+          <t>(clave_subclave_ppal = 'NO CONSTA') &lt;&gt; (COALESCE(ingresos_bruto_total_2024, 0) = 0)</t>
         </is>
       </c>
     </row>
@@ -39624,10 +39628,10 @@
         <v>338</v>
       </c>
       <c r="C4" t="n">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D4" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5">
@@ -39640,10 +39644,10 @@
         <v>561</v>
       </c>
       <c r="C5" t="n">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D5" t="n">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="6"/>
@@ -39679,10 +39683,10 @@
         <v>381</v>
       </c>
       <c r="C8" t="n">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="D8" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9">
@@ -39747,7 +39751,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="15">
@@ -39757,7 +39761,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
reglas: C-153 admite orfandad vitalicia (sin limite de edad); G16 cerrado
La orfandad no tiene tope de edad si el beneficiario tiene incapacidad permanente
(art. 224 LGSS; guia MCVL 4.030 prestacion vitalicia). 2.603 de las 2.615 incumplidoras
tenian orfandad vitalicia; quedan 12 (G22, baja calidad). Tabla auxiliar orfandad_vitalicia
en ejecutar_reglas.py, leida del Parquet de pensiones.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/reglas_consistencia_resultados_sin_ipf.xlsx
+++ b/tests/reglas_consistencia_resultados_sin_ipf.xlsx
@@ -1395,41 +1395,37 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Orfandad en mayores de 60</t>
+          <t>Orfandad en mayores de 60 (orfandad vitalicia por incapacidad)</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Corregido</t>
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>2615</v>
+        <v>0</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>0.1924</v>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>C-153</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="G17" s="2" t="inlineStr"/>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>C-153: 2.615 con orfandad y más de 60 años; la pensión empieza a edad mediana 46 (95 %: 22 o más), 50/50 por sexo, 65 % Nunca_ha_cotizado; discapacidad no lo explica. C-124 CORREGIDO 2026-09-24: 503 con prov_trabajo_ppal NO CONSTA y tiempo; en 502 el código de provincia del CCC (dígitos 5-6 de CCC_2) es 56 (y 53 en 79 episodios), que no está en provincias_dict.csv: 100 % de esos episodios son Régimen del Mar (08xx), domicilio A Coruña (15) o Pontevedra (36). C-314: 278, pendiente de reformular (desfasada tras clave_subclave_ppal). Resuelto: el código 56/53 se etiqueta '56 MAR' (solo en Prov_trabajo_ppal; el 53 fiscal es Isla de La Palma (53) y el 98 Extranjero: codificación común de provincias, 66 Extranjero para nacidos fuera). C-314 CORREGIDA 2026-09-24: regla reformulada (clave NO CONSTA ⇔ ingresos nulos o 0), 0 incumplimientos.</t>
+          <t>C-153: 2.615 con orfandad y más de 60 años; 2.603 (99,5 %) con orfandad vitalicia (incapacidad permanente reconocida, sin límite de edad: art. 224 LGSS, guía MCVL 4.030). Quedan 12 sin vitalicia (G22). C-124 y C-314 también resueltas (ver Resultados).</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>C-153: por decidir (¿huérfanos adultos incapacitados o régimen antiguo?). C-314: reformular.</t>
+          <t>La regla asumía un tope de edad que la normativa no impone a los incapacitados.</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>A decidir</t>
+          <t>Regla mal planteada</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1439,7 +1435,7 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>C-153: seguir hablando.</t>
+          <t>Ninguna acción sobre el ETL. Reglas C-124 (MAR), C-153 y C-314 ajustadas.</t>
         </is>
       </c>
     </row>
@@ -1736,7 +1732,7 @@
         </is>
       </c>
       <c r="D23" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E23" s="2" t="n">
         <v>1088</v>
@@ -1746,12 +1742,12 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>C-279, C-088, C-087, A-106, A-052, B-004, A-078, C-086, C-156, A-074, A-098</t>
+          <t>A-052, A-074, A-078, A-098, A-106, B-004, C-086, C-087, C-088, C-153, C-156, C-279</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>C-088 (1.088) y C-087 (24): racha sin empleo a menos de 360 días del primer empleo o antes (88 % subsidio/asimilado, mediana 184 días). A-106 (486): Nunca_ha_cotizado con incapacidad, sobre todo Incapacidad&gt;65, edad mediana 89. C-279 (8) tras excluir solo-prestaciones y empleo abierto. Resto (1-5 personas cada una): A-052, B-004, A-078, C-086, C-156, A-074, A-098.</t>
+          <t>C-088 (1.088) y C-087 (24): racha sin empleo a menos de 360 días del primer empleo o antes (88 % subsidio/asimilado, mediana 184 días). A-106 (486): Nunca_ha_cotizado con incapacidad, sobre todo Incapacidad&gt;65, edad mediana 89. C-279 (8) tras excluir solo-prestaciones y empleo abierto. Resto (1-5 personas cada una): A-052, B-004, A-078, C-086, C-156, A-074, A-098. C-153 (12): orfandad con más de 60 años sin orfandad vitalicia.</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -27183,7 +27179,7 @@
       </c>
       <c r="F377" s="2" t="inlineStr">
         <is>
-          <t>Orfandad ⇒ edad ≤ 60</t>
+          <t>Orfandad ⇒ edad ≤ 60, salvo orfandad vitalicia (incapacidad permanente reconocida, sin límite de edad)</t>
         </is>
       </c>
       <c r="G377" s="2" t="inlineStr">
@@ -27203,29 +27199,29 @@
       </c>
       <c r="J377" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K377" s="2" t="n">
-        <v>2615</v>
+        <v>12</v>
       </c>
       <c r="L377" s="2" t="n">
-        <v>0.1924</v>
+        <v>0.0009</v>
       </c>
       <c r="M377" s="2" t="inlineStr">
         <is>
-          <t>G16</t>
+          <t>G22</t>
         </is>
       </c>
       <c r="N377" s="2" t="n"/>
       <c r="O377" s="2" t="inlineStr">
         <is>
-          <t>Puede haber orfandad de discapacitados</t>
+          <t>Regla ajustada 2026-09-24 (G16): la orfandad no tiene límite de edad con incapacidad permanente (art. 224 LGSS; guía MCVL 4.030). De las 2.615 anteriores, 2.603 (99,5 %) tenían orfandad vitalicia; quedan 12 solo con orfandad temporal.</t>
         </is>
       </c>
       <c r="P377" s="2" t="inlineStr">
         <is>
-          <t>array_to_string(pension_actual, ',') LIKE '%Orfandad%' AND edad_actual_fecha_corte &gt; 60</t>
+          <t>array_to_string(pension_actual, ',') LIKE '%Orfandad%' AND edad_actual_fecha_corte &gt; 60 AND ipf NOT IN (SELECT ipf FROM orfandad_vitalicia)</t>
         </is>
       </c>
     </row>
@@ -39761,7 +39757,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="16">
@@ -39771,7 +39767,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="17"/>

</xml_diff>

<commit_message>
tests: G16 cerrado - clase 42 verificada como orfandad absoluta
La tabla de claves de la guia (4.004) trae las descripciones una fila por encima de su codigo;
los volumenes confirman 31 viudedad general, 41 orfandad simple, 42 orfandad absoluta.
El mapeo del ETL es correcto. Anotados los 12 casos residuales de C-153 en G22.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/reglas_consistencia_resultados_sin_ipf.xlsx
+++ b/tests/reglas_consistencia_resultados_sin_ipf.xlsx
@@ -1415,7 +1415,7 @@
       <c r="G17" s="2" t="inlineStr"/>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>C-153: 2.615 con orfandad y más de 60 años; 2.603 (99,5 %) con orfandad vitalicia (incapacidad permanente reconocida, sin límite de edad: art. 224 LGSS, guía MCVL 4.030). Quedan 12 sin vitalicia (G22). C-124 y C-314 también resueltas (ver Resultados).</t>
+          <t>C-153: 2.615 con orfandad y más de 60 años; 2.603 (99,5 %) con orfandad vitalicia (incapacidad permanente reconocida, sin límite de edad: art. 224 LGSS, guía MCVL 4.030). Quedan 12 sin vitalicia (G22). C-124 y C-314 también resueltas (ver Resultados). VERIFICADO 2026-09-24: la clase de pensión 42 es Orfandad absoluta (falta el segundo progenitor; encaja con inicio a mediana de 51 años y 100 % vitalicia), no 'a favor de familiares': en la tabla de claves de la guía (4.004) las descripciones aparecen una fila por encima de su código, y los volúmenes lo confirman (31 = viudedad en general, 1,34 M filas; 41 = orfandad simple; 42 = orfandad absoluta). El mapeo del ETL (30-32 viudedad, 40-42 orfandad, 51-54 familiares) es correcto.</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -1747,7 +1747,7 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>C-088 (1.088) y C-087 (24): racha sin empleo a menos de 360 días del primer empleo o antes (88 % subsidio/asimilado, mediana 184 días). A-106 (486): Nunca_ha_cotizado con incapacidad, sobre todo Incapacidad&gt;65, edad mediana 89. C-279 (8) tras excluir solo-prestaciones y empleo abierto. Resto (1-5 personas cada una): A-052, B-004, A-078, C-086, C-156, A-074, A-098. C-153 (12): orfandad con más de 60 años sin orfandad vitalicia.</t>
+          <t>C-088 (1.088) y C-087 (24): racha sin empleo a menos de 360 días del primer empleo o antes (88 % subsidio/asimilado, mediana 184 días). A-106 (486): Nunca_ha_cotizado con incapacidad, sobre todo Incapacidad&gt;65, edad mediana 89. C-279 (8) tras excluir solo-prestaciones y empleo abierto. Resto (1-5 personas cada una): A-052, B-004, A-078, C-086, C-156, A-074, A-098. C-153 (12): orfandad con más de 60 años sin orfandad vitalicia. Los 12 de C-153: todas mujeres nacidas 1946-1958, orfandad no vitalicia desde 1989-2015 iniciada a los 31-64 años; sin causa confirmada (¿régimen antiguo?), no hay indicio de error del ETL.</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -39646,7 +39646,6 @@
         <v>156</v>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
@@ -39717,7 +39716,6 @@
         <v>44</v>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -39770,7 +39768,6 @@
         <v>46</v>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
tests: los 12 casos de C-153 son prestaciones complementarias (regimenes 68/38)
Diez del regimen 68 (Fondo de la Mutualidad de Prevision) y dos del 38 (Mutualidad de
Funcionarios), marcados en la guia (4.010) como prestaciones complementarias, con reglas
propias. Se dejan como estan en Pension_actual (decision del usuario). Corregida la nota de
G16: el desplazamiento de la tabla 4.004 era del texto extraido, no de la guia original.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/reglas_consistencia_resultados_sin_ipf.xlsx
+++ b/tests/reglas_consistencia_resultados_sin_ipf.xlsx
@@ -1415,7 +1415,7 @@
       <c r="G17" s="2" t="inlineStr"/>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>C-153: 2.615 con orfandad y más de 60 años; 2.603 (99,5 %) con orfandad vitalicia (incapacidad permanente reconocida, sin límite de edad: art. 224 LGSS, guía MCVL 4.030). Quedan 12 sin vitalicia (G22). C-124 y C-314 también resueltas (ver Resultados). VERIFICADO 2026-09-24: la clase de pensión 42 es Orfandad absoluta (falta el segundo progenitor; encaja con inicio a mediana de 51 años y 100 % vitalicia), no 'a favor de familiares': en la tabla de claves de la guía (4.004) las descripciones aparecen una fila por encima de su código, y los volúmenes lo confirman (31 = viudedad en general, 1,34 M filas; 41 = orfandad simple; 42 = orfandad absoluta). El mapeo del ETL (30-32 viudedad, 40-42 orfandad, 51-54 familiares) es correcto.</t>
+          <t>C-153: 2.615 con orfandad y más de 60 años; 2.603 (99,5 %) con orfandad vitalicia (incapacidad permanente reconocida, sin límite de edad: art. 224 LGSS, guía MCVL 4.030). Quedan 12 sin vitalicia (G22). C-124 y C-314 también resueltas (ver Resultados). VERIFICADO 2026-09-24: la clase de pensión 42 es Orfandad absoluta (30 viudedad con resolución provisional, 31 viudedad general, 32 viudedad MUNPAL, 40 orfandad con resolución provisional, 41 orfandad simple, 42 orfandad absoluta; confirmado en la tabla 4.004 de la guía original y con los volúmenes de los datos). Encaja con inicio a mediana de 51 años y 100 % vitalicia (falta el segundo progenitor; incapacidad permanente). El mapeo del ETL (30-32 viudedad, 40-42 orfandad, 51-54 familiares) es correcto. Aviso: en el texto extraído .tmp/guia_mcvl.txt las descripciones de esa tabla salen una fila desplazada; la guía original está bien, no usar ese texto para esta tabla.</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -1747,12 +1747,12 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>C-088 (1.088) y C-087 (24): racha sin empleo a menos de 360 días del primer empleo o antes (88 % subsidio/asimilado, mediana 184 días). A-106 (486): Nunca_ha_cotizado con incapacidad, sobre todo Incapacidad&gt;65, edad mediana 89. C-279 (8) tras excluir solo-prestaciones y empleo abierto. Resto (1-5 personas cada una): A-052, B-004, A-078, C-086, C-156, A-074, A-098. C-153 (12): orfandad con más de 60 años sin orfandad vitalicia. Los 12 de C-153: todas mujeres nacidas 1946-1958, orfandad no vitalicia desde 1989-2015 iniciada a los 31-64 años; sin causa confirmada (¿régimen antiguo?), no hay indicio de error del ETL.</t>
+          <t>C-088 (1.088) y C-087 (24): racha sin empleo a menos de 360 días del primer empleo o antes (88 % subsidio/asimilado, mediana 184 días). A-106 (486): Nunca_ha_cotizado con incapacidad, sobre todo Incapacidad&gt;65, edad mediana 89. C-279 (8) tras excluir solo-prestaciones y empleo abierto. Resto (1-5 personas cada una): A-052, B-004, A-078, C-086, C-156, A-074, A-098. C-153 (12): orfandad con más de 60 años sin orfandad vitalicia. Los 12 de C-153 EXPLICADOS 2026-09-24: son prestaciones COMPLEMENTARIAS, no pensiones básicas de la Seguridad Social: 10 del régimen de pensión 68 (Fondo de la Mutualidad de Previsión) y 2 del 38 (Mutualidad de Funcionarios), que la guía (4.010) marca como 'Prest. complementarias'. Tienen sus propias condiciones (todas mujeres, no vitalicias, inicio a los 31-64 años, cobran también jubilación). El ETL las cuenta en Pension_actual/Tipo_pension sin distinguir régimen (decisión del usuario 2026-09-24: se dejan como están). Personas con pensión en regímenes complementarios en la edición 2024: 68 → 179 (65 con orfandad), 38 → 252 (19), 32 → 8, 39 → 2, 31 → 1.</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>Cotización previa fuera de la muestra (mismo motivo que G08) y errores puntuales del dato de origen.</t>
+          <t>Prestaciones complementarias de mutualidades (regímenes 38/68), con reglas propias distintas de la LGSS.</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
@@ -1767,7 +1767,7 @@
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>Ninguna acción sobre el ETL.</t>
+          <t>Ninguna acción: se dejan como están en Pension_actual (decisión del usuario).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
reglas: G04 - edad minima legal por cohorte (14 hasta 1965, 16 despues)
El Estatuto de los Trabajadores (Ley 8/1980) subio el minimo de 14 a 16; las reglas de inicio de
vida laboral asumian 16 para todos. 16 reglas (C-051..058, C-079, C-083, C-085, C-105..107,
B-043, B-073) usan CASE WHEN year(fecha_nacimiento) <= 1965 THEN 14 ELSE 16. C-079 baja de
28.841 a 1.636, C-105 de 27.871 a 389, C-107 de 37.024 a 2.117, C-058 de 18.746 a 1.421.
Las de edad actual < 16 no cambian. Las graficas de la app no se tocan (decision del usuario).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/reglas_consistencia_resultados_sin_ipf.xlsx
+++ b/tests/reglas_consistencia_resultados_sin_ipf.xlsx
@@ -727,7 +727,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Edad mínima legal 16 años</t>
+          <t>Edad mínima legal (14 hasta la cohorte 1965, 16 después)</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -739,10 +739,10 @@
         <v>28</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>37024</v>
+        <v>2117</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>2.7242</v>
+        <v>0.1558</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
@@ -751,17 +751,17 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>29.079 personas (2,1 %) empiezan a trabajar antes de los 16 (C-079); C-107 (edad − tiempo desde inicio &lt; 16): 37.262.</t>
+          <t>Con el mínimo de 16 para todos: 29.079 personas empezaban a trabajar antes de los 16 (C-079) y C-107 daba 37.262. CORREGIDO 2026-09-24 (decisión del usuario): mínimo por cohorte, 14 para nacidos hasta 1965 y 16 después. C-079 baja de 28.841 a 1.636, C-105 de 27.871 a 389, C-107 de 37.024 a 2.117 y C-058 de 18.746 a 1.421. El 94 % de C-079 empezó a los 14-15 años antes de 1981, legalmente. Residuo de C-079 (1.636): 169 nacidos hasta 1965 con primer empleo antes de los 14 (45 con menos de 12) y 1.467 nacidos desde 1966 (891 con menos de 12 años, 278 con 12-13 y 298 con 14-15). Los 287 menores de 16 actuales con afiliación son los mismos de A-093, C-114 y C-115. Las reglas de edad ACTUAL menor de 16 no cambian.</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Hasta 1980 la edad mínima legal era 14, no 16 - la regla asume el mínimo actual para toda la serie histórica.</t>
+          <t>El mínimo legal era 14 hasta la Ley 8/1980 (Estatuto de los Trabajadores, en vigor desde marzo de 1980) y 16 después. El corte por cohorte es aproximado. Residuo pendiente de revisar: ¿menores autorizados (espectáculos públicos, art. 6.4 ET) o errores de fecha?</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Regla demasiado estricta</t>
+          <t>Regla demasiado estricta (corregida) + residuo de datos</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -771,7 +771,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Acotar las reglas de edad mínima a cohortes posteriores a 1965 y mirar aparte los casos antiguos - sin decidir.</t>
+          <t>Revisar el residuo (menores de 14 nacidos hasta 1965 y menores de 16 nacidos desde 1966, sobre todo los de menos de 12 años). Pendiente aparte: las gráficas por edad de Trayectorias de colectivos cortan en 16 (app/routers/trayectorias.py) y omiten los 14-15 años legítimos de las cohortes antiguas; el usuario decidió dejarlo para más adelante.</t>
         </is>
       </c>
     </row>
@@ -12215,7 +12215,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>Parado_LD ⇒ tiempo sin empleo ≤ edad − 16 años</t>
+          <t>Parado_LD ⇒ tiempo sin empleo ≤ edad − mínimo legal (14 hasta la cohorte 1965, 16 después)</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -12252,12 +12252,12 @@
       <c r="N155" s="2" t="n"/>
       <c r="O155" s="2" t="inlineStr">
         <is>
-          <t>16 años (decisión del usuario); antes de 1980 la edad mínima legal era 14</t>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte, 14 años para nacidos hasta 1965 (el ET de 1980 lo subió a 16) y 16 para los posteriores. Antes: 16 para todos.</t>
         </is>
       </c>
       <c r="P155" s="2" t="inlineStr">
         <is>
-          <t>situacion_paro_ocupacion = 'Parado_LD' AND duracion_actual_sin_empleo / 365.25 &gt; edad_actual_fecha_corte - 16</t>
+          <t>situacion_paro_ocupacion = 'Parado_LD' AND duracion_actual_sin_empleo / 365.25 &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END)</t>
         </is>
       </c>
     </row>
@@ -14287,7 +14287,7 @@
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>Parado_NoLD ⇒ tiempo sin empleo ≤ edad − 16 años</t>
+          <t>Parado_NoLD ⇒ tiempo sin empleo ≤ edad − mínimo legal (14 hasta la cohorte 1965, 16 después)</t>
         </is>
       </c>
       <c r="G185" s="2" t="inlineStr">
@@ -14324,12 +14324,12 @@
       <c r="N185" s="2" t="n"/>
       <c r="O185" s="2" t="inlineStr">
         <is>
-          <t>16 años (decisión del usuario); antes de 1980 la edad mínima legal era 14</t>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte, 14 años para nacidos hasta 1965 (el ET de 1980 lo subió a 16) y 16 para los posteriores. Antes: 16 para todos.</t>
         </is>
       </c>
       <c r="P185" s="2" t="inlineStr">
         <is>
-          <t>situacion_paro_ocupacion = 'Parado_NoLD' AND duracion_actual_sin_empleo / 365.25 &gt; edad_actual_fecha_corte - 16</t>
+          <t>situacion_paro_ocupacion = 'Parado_NoLD' AND duracion_actual_sin_empleo / 365.25 &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END)</t>
         </is>
       </c>
     </row>
@@ -20295,7 +20295,7 @@
       </c>
       <c r="F275" s="2" t="inlineStr">
         <is>
-          <t>t_tot_reg_ppal no puede superar edad − 16 años (+1): no se trabaja antes de los 16</t>
+          <t>t_tot_reg_ppal no puede superar edad − mínimo legal (+1): no se trabaja antes de la edad mínima legal (14 hasta la cohorte 1965, 16 después)</t>
         </is>
       </c>
       <c r="G275" s="2" t="inlineStr">
@@ -20319,10 +20319,10 @@
         </is>
       </c>
       <c r="K275" s="2" t="n">
-        <v>384</v>
+        <v>288</v>
       </c>
       <c r="L275" s="2" t="n">
-        <v>0.0283</v>
+        <v>0.0212</v>
       </c>
       <c r="M275" s="2" t="inlineStr">
         <is>
@@ -20332,12 +20332,12 @@
       <c r="N275" s="2" t="n"/>
       <c r="O275" s="2" t="inlineStr">
         <is>
-          <t>16 años (decisión del usuario). Hasta 1980 la edad mínima legal era 14: pueden salir casos antiguos legítimos | Cifra actualizada 2026-09-24: variación de unas pocas personas por el cálculo no determinista de los tiempos por categoría (374 personas difieren entre regeneraciones).</t>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte, 14 años para nacidos hasta 1965 (el ET de 1980 lo subió a 16) y 16 para los posteriores. Antes: 16 para todos.</t>
         </is>
       </c>
       <c r="P275" s="2" t="inlineStr">
         <is>
-          <t>t_tot_reg_ppal &gt; edad_actual_fecha_corte - 16 + 1</t>
+          <t>t_tot_reg_ppal &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) + 1</t>
         </is>
       </c>
     </row>
@@ -20369,7 +20369,7 @@
       </c>
       <c r="F276" s="2" t="inlineStr">
         <is>
-          <t>t_tot_grupo_ppal no puede superar edad − 16 años (+1): no se trabaja antes de los 16</t>
+          <t>t_tot_grupo_ppal no puede superar edad − mínimo legal (+1): no se trabaja antes de la edad mínima legal (14 hasta la cohorte 1965, 16 después)</t>
         </is>
       </c>
       <c r="G276" s="2" t="inlineStr">
@@ -20393,10 +20393,10 @@
         </is>
       </c>
       <c r="K276" s="2" t="n">
-        <v>296</v>
+        <v>276</v>
       </c>
       <c r="L276" s="2" t="n">
-        <v>0.0218</v>
+        <v>0.0203</v>
       </c>
       <c r="M276" s="2" t="inlineStr">
         <is>
@@ -20406,12 +20406,12 @@
       <c r="N276" s="2" t="n"/>
       <c r="O276" s="2" t="inlineStr">
         <is>
-          <t>16 años (decisión del usuario). Hasta 1980 la edad mínima legal era 14: pueden salir casos antiguos legítimos | Cifra actualizada 2026-09-24: variación de unas pocas personas por el cálculo no determinista de los tiempos por categoría (374 personas difieren entre regeneraciones).</t>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte, 14 años para nacidos hasta 1965 (el ET de 1980 lo subió a 16) y 16 para los posteriores. Antes: 16 para todos.</t>
         </is>
       </c>
       <c r="P276" s="2" t="inlineStr">
         <is>
-          <t>t_tot_grupo_ppal &gt; edad_actual_fecha_corte - 16 + 1</t>
+          <t>t_tot_grupo_ppal &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) + 1</t>
         </is>
       </c>
     </row>
@@ -20443,7 +20443,7 @@
       </c>
       <c r="F277" s="2" t="inlineStr">
         <is>
-          <t>t_tot_tipo_contrato_ppal no puede superar edad − 16 años (+1): no se trabaja antes de los 16</t>
+          <t>t_tot_tipo_contrato_ppal no puede superar edad − mínimo legal (+1): no se trabaja antes de la edad mínima legal (14 hasta la cohorte 1965, 16 después)</t>
         </is>
       </c>
       <c r="G277" s="2" t="inlineStr">
@@ -20467,10 +20467,10 @@
         </is>
       </c>
       <c r="K277" s="2" t="n">
-        <v>314</v>
+        <v>277</v>
       </c>
       <c r="L277" s="2" t="n">
-        <v>0.0231</v>
+        <v>0.0204</v>
       </c>
       <c r="M277" s="2" t="inlineStr">
         <is>
@@ -20480,12 +20480,12 @@
       <c r="N277" s="2" t="n"/>
       <c r="O277" s="2" t="inlineStr">
         <is>
-          <t>16 años (decisión del usuario). Hasta 1980 la edad mínima legal era 14: pueden salir casos antiguos legítimos | Cifra actualizada 2026-09-24: variación de unas pocas personas por el cálculo no determinista de los tiempos por categoría (374 personas difieren entre regeneraciones).</t>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte, 14 años para nacidos hasta 1965 (el ET de 1980 lo subió a 16) y 16 para los posteriores. Antes: 16 para todos.</t>
         </is>
       </c>
       <c r="P277" s="2" t="inlineStr">
         <is>
-          <t>t_tot_tipo_contrato_ppal &gt; edad_actual_fecha_corte - 16 + 1</t>
+          <t>t_tot_tipo_contrato_ppal &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) + 1</t>
         </is>
       </c>
     </row>
@@ -20517,7 +20517,7 @@
       </c>
       <c r="F278" s="2" t="inlineStr">
         <is>
-          <t>t_tot_prov_ppal no puede superar edad − 16 años (+1): no se trabaja antes de los 16</t>
+          <t>t_tot_prov_ppal no puede superar edad − mínimo legal (+1): no se trabaja antes de la edad mínima legal (14 hasta la cohorte 1965, 16 después)</t>
         </is>
       </c>
       <c r="G278" s="2" t="inlineStr">
@@ -20541,10 +20541,10 @@
         </is>
       </c>
       <c r="K278" s="2" t="n">
-        <v>411</v>
+        <v>286</v>
       </c>
       <c r="L278" s="2" t="n">
-        <v>0.0302</v>
+        <v>0.021</v>
       </c>
       <c r="M278" s="2" t="inlineStr">
         <is>
@@ -20554,12 +20554,12 @@
       <c r="N278" s="2" t="n"/>
       <c r="O278" s="2" t="inlineStr">
         <is>
-          <t>16 años (decisión del usuario). Hasta 1980 la edad mínima legal era 14: pueden salir casos antiguos legítimos | Cifra actualizada 2026-09-24: variación de unas pocas personas por el cálculo no determinista de los tiempos por categoría (374 personas difieren entre regeneraciones).</t>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte, 14 años para nacidos hasta 1965 (el ET de 1980 lo subió a 16) y 16 para los posteriores. Antes: 16 para todos.</t>
         </is>
       </c>
       <c r="P278" s="2" t="inlineStr">
         <is>
-          <t>t_tot_prov_ppal &gt; edad_actual_fecha_corte - 16 + 1</t>
+          <t>t_tot_prov_ppal &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) + 1</t>
         </is>
       </c>
     </row>
@@ -20591,7 +20591,7 @@
       </c>
       <c r="F279" s="2" t="inlineStr">
         <is>
-          <t>t_tot_act_econ_ppal no puede superar edad − 16 años (+1): no se trabaja antes de los 16</t>
+          <t>t_tot_act_econ_ppal no puede superar edad − mínimo legal (+1): no se trabaja antes de la edad mínima legal (14 hasta la cohorte 1965, 16 después)</t>
         </is>
       </c>
       <c r="G279" s="2" t="inlineStr">
@@ -20615,10 +20615,10 @@
         </is>
       </c>
       <c r="K279" s="2" t="n">
-        <v>292</v>
+        <v>273</v>
       </c>
       <c r="L279" s="2" t="n">
-        <v>0.0215</v>
+        <v>0.0201</v>
       </c>
       <c r="M279" s="2" t="inlineStr">
         <is>
@@ -20628,12 +20628,12 @@
       <c r="N279" s="2" t="n"/>
       <c r="O279" s="2" t="inlineStr">
         <is>
-          <t>16 años (decisión del usuario). Hasta 1980 la edad mínima legal era 14: pueden salir casos antiguos legítimos</t>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte, 14 años para nacidos hasta 1965 (el ET de 1980 lo subió a 16) y 16 para los posteriores. Antes: 16 para todos.</t>
         </is>
       </c>
       <c r="P279" s="2" t="inlineStr">
         <is>
-          <t>t_tot_act_econ_ppal &gt; edad_actual_fecha_corte - 16 + 1</t>
+          <t>t_tot_act_econ_ppal &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) + 1</t>
         </is>
       </c>
     </row>
@@ -20665,7 +20665,7 @@
       </c>
       <c r="F280" s="2" t="inlineStr">
         <is>
-          <t>t_total_empleo no puede superar edad − 16 años (+1): no se trabaja antes de los 16</t>
+          <t>t_total_empleo no puede superar edad − mínimo legal (+1): no se trabaja antes de la edad mínima legal (14 hasta la cohorte 1965, 16 después)</t>
         </is>
       </c>
       <c r="G280" s="2" t="inlineStr">
@@ -20689,10 +20689,10 @@
         </is>
       </c>
       <c r="K280" s="2" t="n">
-        <v>406</v>
+        <v>294</v>
       </c>
       <c r="L280" s="2" t="n">
-        <v>0.0299</v>
+        <v>0.0216</v>
       </c>
       <c r="M280" s="2" t="inlineStr">
         <is>
@@ -20702,12 +20702,12 @@
       <c r="N280" s="2" t="n"/>
       <c r="O280" s="2" t="inlineStr">
         <is>
-          <t>16 años (decisión del usuario). Hasta 1980 la edad mínima legal era 14: pueden salir casos antiguos legítimos</t>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte, 14 años para nacidos hasta 1965 (el ET de 1980 lo subió a 16) y 16 para los posteriores. Antes: 16 para todos.</t>
         </is>
       </c>
       <c r="P280" s="2" t="inlineStr">
         <is>
-          <t>t_total_empleo &gt; edad_actual_fecha_corte - 16 + 1</t>
+          <t>t_total_empleo &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) + 1</t>
         </is>
       </c>
     </row>
@@ -20739,7 +20739,7 @@
       </c>
       <c r="F281" s="2" t="inlineStr">
         <is>
-          <t>t_contrato_mas_largo no puede superar edad − 16 años (+1): no se trabaja antes de los 16</t>
+          <t>t_contrato_mas_largo no puede superar edad − mínimo legal (+1): no se trabaja antes de la edad mínima legal (14 hasta la cohorte 1965, 16 después)</t>
         </is>
       </c>
       <c r="G281" s="2" t="inlineStr">
@@ -20763,10 +20763,10 @@
         </is>
       </c>
       <c r="K281" s="2" t="n">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="L281" s="2" t="n">
-        <v>0.0205</v>
+        <v>0.02</v>
       </c>
       <c r="M281" s="2" t="inlineStr">
         <is>
@@ -20776,12 +20776,12 @@
       <c r="N281" s="2" t="n"/>
       <c r="O281" s="2" t="inlineStr">
         <is>
-          <t>16 años (decisión del usuario). Hasta 1980 la edad mínima legal era 14: pueden salir casos antiguos legítimos</t>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte, 14 años para nacidos hasta 1965 (el ET de 1980 lo subió a 16) y 16 para los posteriores. Antes: 16 para todos.</t>
         </is>
       </c>
       <c r="P281" s="2" t="inlineStr">
         <is>
-          <t>t_contrato_mas_largo &gt; edad_actual_fecha_corte - 16 + 1</t>
+          <t>t_contrato_mas_largo &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) + 1</t>
         </is>
       </c>
     </row>
@@ -20813,7 +20813,7 @@
       </c>
       <c r="F282" s="2" t="inlineStr">
         <is>
-          <t>tiempo_total_desde_inicio_vl no puede superar edad − 16 años (+1): no se trabaja antes de los 16</t>
+          <t>tiempo_total_desde_inicio_vl no puede superar edad − mínimo legal (+1): no se trabaja antes de la edad mínima legal (14 hasta la cohorte 1965, 16 después)</t>
         </is>
       </c>
       <c r="G282" s="2" t="inlineStr">
@@ -20837,10 +20837,10 @@
         </is>
       </c>
       <c r="K282" s="2" t="n">
-        <v>18746</v>
+        <v>1421</v>
       </c>
       <c r="L282" s="2" t="n">
-        <v>1.3793</v>
+        <v>0.1046</v>
       </c>
       <c r="M282" s="2" t="inlineStr">
         <is>
@@ -20850,12 +20850,12 @@
       <c r="N282" s="2" t="n"/>
       <c r="O282" s="2" t="inlineStr">
         <is>
-          <t>16 años (decisión del usuario). Hasta 1980 la edad mínima legal era 14: pueden salir casos antiguos legítimos</t>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte, 14 años para nacidos hasta 1965 (el ET de 1980 lo subió a 16) y 16 para los posteriores. Antes: 16 para todos.</t>
         </is>
       </c>
       <c r="P282" s="2" t="inlineStr">
         <is>
-          <t>tiempo_total_desde_inicio_vl &gt; edad_actual_fecha_corte - 16 + 1</t>
+          <t>tiempo_total_desde_inicio_vl &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) + 1</t>
         </is>
       </c>
     </row>
@@ -22227,7 +22227,7 @@
       </c>
       <c r="F303" s="2" t="inlineStr">
         <is>
-          <t>Primer empleo a los 16 años o más</t>
+          <t>Primer empleo a la edad mínima legal o más (14 hasta la cohorte 1965, 16 después)</t>
         </is>
       </c>
       <c r="G303" s="2" t="inlineStr">
@@ -22251,10 +22251,10 @@
         </is>
       </c>
       <c r="K303" s="2" t="n">
-        <v>28841</v>
+        <v>1636</v>
       </c>
       <c r="L303" s="2" t="n">
-        <v>2.1221</v>
+        <v>0.1204</v>
       </c>
       <c r="M303" s="2" t="inlineStr">
         <is>
@@ -22262,10 +22262,14 @@
         </is>
       </c>
       <c r="N303" s="2" t="n"/>
-      <c r="O303" s="2" t="inlineStr"/>
+      <c r="O303" s="2" t="inlineStr">
+        <is>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte, 14 años para nacidos hasta 1965 (el ET de 1980 lo subió a 16) y 16 para los posteriores. Antes: 16 para todos.</t>
+        </is>
+      </c>
       <c r="P303" s="2" t="inlineStr">
         <is>
-          <t>date_diff('year', fecha_nacimiento, fecha_ini_primer_empleo) &lt; 16</t>
+          <t>date_diff('year', fecha_nacimiento, fecha_ini_primer_empleo) &lt; (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END)</t>
         </is>
       </c>
     </row>
@@ -22495,7 +22499,7 @@
       </c>
       <c r="F307" s="2" t="inlineStr">
         <is>
-          <t>Última baja a los 16 años o más</t>
+          <t>Última baja a la edad mínima legal o más (14 hasta la cohorte 1965, 16 después)</t>
         </is>
       </c>
       <c r="G307" s="2" t="inlineStr">
@@ -22519,10 +22523,10 @@
         </is>
       </c>
       <c r="K307" s="2" t="n">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="L307" s="2" t="n">
-        <v>0.0225</v>
+        <v>0.0224</v>
       </c>
       <c r="M307" s="2" t="inlineStr">
         <is>
@@ -22530,10 +22534,14 @@
         </is>
       </c>
       <c r="N307" s="2" t="n"/>
-      <c r="O307" s="2" t="inlineStr"/>
+      <c r="O307" s="2" t="inlineStr">
+        <is>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte, 14 años para nacidos hasta 1965 (el ET de 1980 lo subió a 16) y 16 para los posteriores. Antes: 16 para todos.</t>
+        </is>
+      </c>
       <c r="P307" s="2" t="inlineStr">
         <is>
-          <t>date_diff('year', fecha_nacimiento, fecha_ultima_baja) &lt; 16 AND (fecha_ultima_baja IS NULL OR year(fecha_ultima_baja) &lt;&gt; 2099)</t>
+          <t>date_diff('year', fecha_nacimiento, fecha_ultima_baja) &lt; (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) AND (fecha_ultima_baja IS NULL OR year(fecha_ultima_baja) &lt;&gt; 2099)</t>
         </is>
       </c>
     </row>
@@ -22627,7 +22635,7 @@
       </c>
       <c r="F309" s="2" t="inlineStr">
         <is>
-          <t>Inicio de racha sin empleo a los 16 años o más</t>
+          <t>Inicio de racha sin empleo a la edad mínima legal o más (14 hasta la cohorte 1965, 16 después)</t>
         </is>
       </c>
       <c r="G309" s="2" t="inlineStr">
@@ -22662,10 +22670,14 @@
         </is>
       </c>
       <c r="N309" s="2" t="n"/>
-      <c r="O309" s="2" t="inlineStr"/>
+      <c r="O309" s="2" t="inlineStr">
+        <is>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte, 14 años para nacidos hasta 1965 (el ET de 1980 lo subió a 16) y 16 para los posteriores. Antes: 16 para todos.</t>
+        </is>
+      </c>
       <c r="P309" s="2" t="inlineStr">
         <is>
-          <t>date_diff('year', fecha_nacimiento, fecha_inicio_ultima_racha_sin_empleo) &lt; 16</t>
+          <t>date_diff('year', fecha_nacimiento, fecha_inicio_ultima_racha_sin_empleo) &lt; (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END)</t>
         </is>
       </c>
     </row>
@@ -23947,7 +23959,7 @@
       <c r="E329" s="2" t="inlineStr"/>
       <c r="F329" s="2" t="inlineStr">
         <is>
-          <t>Primer empleo significativo a los 16 o más</t>
+          <t>Primer empleo significativo a la edad mínima legal o más (14 hasta la cohorte 1965, 16 después)</t>
         </is>
       </c>
       <c r="G329" s="2" t="inlineStr">
@@ -23971,10 +23983,10 @@
         </is>
       </c>
       <c r="K329" s="2" t="n">
-        <v>27871</v>
+        <v>389</v>
       </c>
       <c r="L329" s="2" t="n">
-        <v>2.0508</v>
+        <v>0.0286</v>
       </c>
       <c r="M329" s="2" t="inlineStr">
         <is>
@@ -23982,10 +23994,14 @@
         </is>
       </c>
       <c r="N329" s="2" t="n"/>
-      <c r="O329" s="2" t="inlineStr"/>
+      <c r="O329" s="2" t="inlineStr">
+        <is>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte, 14 años para nacidos hasta 1965 (el ET de 1980 lo subió a 16) y 16 para los posteriores. Antes: 16 para todos.</t>
+        </is>
+      </c>
       <c r="P329" s="2" t="inlineStr">
         <is>
-          <t>edad_primer_empleo_signif &lt; 16</t>
+          <t>edad_primer_empleo_signif &lt; (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END)</t>
         </is>
       </c>
     </row>
@@ -24013,7 +24029,7 @@
       <c r="E330" s="2" t="inlineStr"/>
       <c r="F330" s="2" t="inlineStr">
         <is>
-          <t>Edad al final del último empleo ≥ 16</t>
+          <t>Edad al final del último empleo ≥ mínimo legal (14 hasta la cohorte 1965, 16 después)</t>
         </is>
       </c>
       <c r="G330" s="2" t="inlineStr">
@@ -24037,10 +24053,10 @@
         </is>
       </c>
       <c r="K330" s="2" t="n">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="L330" s="2" t="n">
-        <v>0.0227</v>
+        <v>0.0224</v>
       </c>
       <c r="M330" s="2" t="inlineStr">
         <is>
@@ -24048,10 +24064,14 @@
         </is>
       </c>
       <c r="N330" s="2" t="n"/>
-      <c r="O330" s="2" t="inlineStr"/>
+      <c r="O330" s="2" t="inlineStr">
+        <is>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte, 14 años para nacidos hasta 1965 (el ET de 1980 lo subió a 16) y 16 para los posteriores. Antes: 16 para todos.</t>
+        </is>
+      </c>
       <c r="P330" s="2" t="inlineStr">
         <is>
-          <t>edad_ultimo_empleo &lt; 16</t>
+          <t>edad_ultimo_empleo &lt; (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END)</t>
         </is>
       </c>
     </row>
@@ -24083,7 +24103,7 @@
       </c>
       <c r="F331" s="2" t="inlineStr">
         <is>
-          <t>edad − tiempo desde inicio de vida laboral ≥ 16</t>
+          <t>edad − tiempo desde inicio de vida laboral ≥ mínimo legal (14 hasta la cohorte 1965, 16 después)</t>
         </is>
       </c>
       <c r="G331" s="2" t="inlineStr">
@@ -24107,10 +24127,10 @@
         </is>
       </c>
       <c r="K331" s="2" t="n">
-        <v>37024</v>
+        <v>2117</v>
       </c>
       <c r="L331" s="2" t="n">
-        <v>2.7242</v>
+        <v>0.1558</v>
       </c>
       <c r="M331" s="2" t="inlineStr">
         <is>
@@ -24118,10 +24138,14 @@
         </is>
       </c>
       <c r="N331" s="2" t="n"/>
-      <c r="O331" s="2" t="inlineStr"/>
+      <c r="O331" s="2" t="inlineStr">
+        <is>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte, 14 años para nacidos hasta 1965 (el ET de 1980 lo subió a 16) y 16 para los posteriores. Antes: 16 para todos.</t>
+        </is>
+      </c>
       <c r="P331" s="2" t="inlineStr">
         <is>
-          <t>edad_actual_fecha_corte - tiempo_total_desde_inicio_vl &lt; 16</t>
+          <t>edad_actual_fecha_corte - tiempo_total_desde_inicio_vl &lt; (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END)</t>
         </is>
       </c>
     </row>
@@ -39646,6 +39670,7 @@
         <v>156</v>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
@@ -39716,6 +39741,7 @@
         <v>44</v>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -39768,6 +39794,7 @@
         <v>46</v>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
reglas: G04 - excepcion de menores autorizados (artistas, espectaculos, publicidad, deporte)
Art. 6.4 ET permite menores de 16 en espectaculos publicos con autorizacion. Tabla auxiliar
menor_autorizado en ejecutar_reglas.py: episodio que empieza antes del minimo legal (14 hasta la
cohorte 1965, 16 despues) en regimen 0112 (Regimen General - Artistas) o CNAE 59, 60, 90, 93, 73,
781, 742, 855. Aplicada a las 16 reglas de edad minima: C-079 397 (antes 1.636), C-107 878
(2.117), C-058 232 (1.421), C-056 23 (294); B-043 y B-073 pasan a 0.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/reglas_consistencia_resultados_sin_ipf.xlsx
+++ b/tests/reglas_consistencia_resultados_sin_ipf.xlsx
@@ -736,22 +736,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>2117</v>
+        <v>1625</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0.1558</v>
+        <v>0.1196</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>A-093, B-040, B-043, B-054, B-070, B-073, B-084, C-051, C-052, C-053, C-054, C-055, C-056, C-057, C-058, C-079, C-083, C-085, C-096, C-097, C-105, C-106, C-107, C-114, C-115, C-168, C-239, C-251</t>
+          <t>A-093, B-040, B-054, B-070, B-084, C-051, C-052, C-053, C-054, C-055, C-056, C-057, C-058, C-079, C-083, C-085, C-096, C-097, C-105, C-106, C-107, C-114, C-115, C-168, C-239, C-251</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Con el mínimo de 16 para todos: 29.079 personas empezaban a trabajar antes de los 16 (C-079) y C-107 daba 37.262. CORREGIDO 2026-09-24 (decisión del usuario): mínimo por cohorte, 14 para nacidos hasta 1965 y 16 después. C-079 baja de 28.841 a 1.636, C-105 de 27.871 a 389, C-107 de 37.024 a 2.117 y C-058 de 18.746 a 1.421. El 94 % de C-079 empezó a los 14-15 años antes de 1981, legalmente. Residuo de C-079 (1.636): 169 nacidos hasta 1965 con primer empleo antes de los 14 (45 con menos de 12) y 1.467 nacidos desde 1966 (891 con menos de 12 años, 278 con 12-13 y 298 con 14-15). Los 287 menores de 16 actuales con afiliación son los mismos de A-093, C-114 y C-115. Las reglas de edad ACTUAL menor de 16 no cambian.</t>
+          <t>Con el mínimo de 16 para todos: 29.079 personas empezaban a trabajar antes de los 16 (C-079) y C-107 daba 37.262. CORREGIDO 2026-09-24 (decisión del usuario): mínimo por cohorte, 14 para nacidos hasta 1965 y 16 después. C-079 baja de 28.841 a 1.636, C-105 de 27.871 a 389, C-107 de 37.024 a 2.117 y C-058 de 18.746 a 1.421. El 94 % de C-079 empezó a los 14-15 años antes de 1981, legalmente. Residuo de C-079 (1.636): 169 nacidos hasta 1965 con primer empleo antes de los 14 (45 con menos de 12) y 1.467 nacidos desde 1966 (891 con menos de 12 años, 278 con 12-13 y 298 con 14-15). Los 287 menores de 16 actuales con afiliación son los mismos de A-093, C-114 y C-115. Las reglas de edad ACTUAL menor de 16 no cambian. EXCEPCIÓN DE MENORES AUTORIZADOS 2026-09-24 (decisión del usuario): en el residuo, el 61 % de los nacidos desde 1966 empezó en el régimen 0112 (Régimen General - Artistas) o en sectores de cine/TV, radio, artes y espectáculos, publicidad, deporte, casting, fotografía o educación cultural (art. 6.4 ET permite menores en espectáculos públicos con autorización). Las reglas de edad mínima excluyen a quien tiene un episodio que empieza antes del mínimo en esos regímenes/sectores. Resultado: C-079 397 (antes 1.636), C-107 878 (2.117), C-058 232 (1.421), C-105 383 (389), C-056 23 (294); B-043 y B-073 pasan a 0. CNAE desconocido (0) NO se considera plausible.</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -12230,19 +12230,19 @@
       </c>
       <c r="I155" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J155" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Corregido</t>
         </is>
       </c>
       <c r="K155" s="2" t="n">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="L155" s="2" t="n">
-        <v>0.0051</v>
+        <v>0</v>
       </c>
       <c r="M155" s="2" t="inlineStr">
         <is>
@@ -12252,12 +12252,12 @@
       <c r="N155" s="2" t="n"/>
       <c r="O155" s="2" t="inlineStr">
         <is>
-          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte, 14 años para nacidos hasta 1965 (el ET de 1980 lo subió a 16) y 16 para los posteriores. Antes: 16 para todos.</t>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte (14 hasta 1965, 16 después) y excepción de menores autorizados (régimen 0112 artistas y sectores de espectáculos, artes, publicidad, deporte y casting: art. 6.4 ET).</t>
         </is>
       </c>
       <c r="P155" s="2" t="inlineStr">
         <is>
-          <t>situacion_paro_ocupacion = 'Parado_LD' AND duracion_actual_sin_empleo / 365.25 &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END)</t>
+          <t>situacion_paro_ocupacion = 'Parado_LD' AND duracion_actual_sin_empleo / 365.25 &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
         </is>
       </c>
     </row>
@@ -14302,19 +14302,19 @@
       </c>
       <c r="I185" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J185" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Corregido</t>
         </is>
       </c>
       <c r="K185" s="2" t="n">
-        <v>217</v>
+        <v>0</v>
       </c>
       <c r="L185" s="2" t="n">
-        <v>0.016</v>
+        <v>0</v>
       </c>
       <c r="M185" s="2" t="inlineStr">
         <is>
@@ -14324,12 +14324,12 @@
       <c r="N185" s="2" t="n"/>
       <c r="O185" s="2" t="inlineStr">
         <is>
-          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte, 14 años para nacidos hasta 1965 (el ET de 1980 lo subió a 16) y 16 para los posteriores. Antes: 16 para todos.</t>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte (14 hasta 1965, 16 después) y excepción de menores autorizados (régimen 0112 artistas y sectores de espectáculos, artes, publicidad, deporte y casting: art. 6.4 ET).</t>
         </is>
       </c>
       <c r="P185" s="2" t="inlineStr">
         <is>
-          <t>situacion_paro_ocupacion = 'Parado_NoLD' AND duracion_actual_sin_empleo / 365.25 &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END)</t>
+          <t>situacion_paro_ocupacion = 'Parado_NoLD' AND duracion_actual_sin_empleo / 365.25 &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
         </is>
       </c>
     </row>
@@ -20319,10 +20319,10 @@
         </is>
       </c>
       <c r="K275" s="2" t="n">
-        <v>288</v>
+        <v>17</v>
       </c>
       <c r="L275" s="2" t="n">
-        <v>0.0212</v>
+        <v>0.0013</v>
       </c>
       <c r="M275" s="2" t="inlineStr">
         <is>
@@ -20332,12 +20332,12 @@
       <c r="N275" s="2" t="n"/>
       <c r="O275" s="2" t="inlineStr">
         <is>
-          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte, 14 años para nacidos hasta 1965 (el ET de 1980 lo subió a 16) y 16 para los posteriores. Antes: 16 para todos.</t>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte (14 hasta 1965, 16 después) y excepción de menores autorizados (régimen 0112 artistas y sectores de espectáculos, artes, publicidad, deporte y casting: art. 6.4 ET).</t>
         </is>
       </c>
       <c r="P275" s="2" t="inlineStr">
         <is>
-          <t>t_tot_reg_ppal &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) + 1</t>
+          <t>t_tot_reg_ppal &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) + 1 AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
         </is>
       </c>
     </row>
@@ -20393,10 +20393,10 @@
         </is>
       </c>
       <c r="K276" s="2" t="n">
-        <v>276</v>
+        <v>5</v>
       </c>
       <c r="L276" s="2" t="n">
-        <v>0.0203</v>
+        <v>0.0004</v>
       </c>
       <c r="M276" s="2" t="inlineStr">
         <is>
@@ -20406,12 +20406,12 @@
       <c r="N276" s="2" t="n"/>
       <c r="O276" s="2" t="inlineStr">
         <is>
-          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte, 14 años para nacidos hasta 1965 (el ET de 1980 lo subió a 16) y 16 para los posteriores. Antes: 16 para todos.</t>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte (14 hasta 1965, 16 después) y excepción de menores autorizados (régimen 0112 artistas y sectores de espectáculos, artes, publicidad, deporte y casting: art. 6.4 ET).</t>
         </is>
       </c>
       <c r="P276" s="2" t="inlineStr">
         <is>
-          <t>t_tot_grupo_ppal &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) + 1</t>
+          <t>t_tot_grupo_ppal &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) + 1 AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
         </is>
       </c>
     </row>
@@ -20467,10 +20467,10 @@
         </is>
       </c>
       <c r="K277" s="2" t="n">
-        <v>277</v>
+        <v>7</v>
       </c>
       <c r="L277" s="2" t="n">
-        <v>0.0204</v>
+        <v>0.0005</v>
       </c>
       <c r="M277" s="2" t="inlineStr">
         <is>
@@ -20480,12 +20480,12 @@
       <c r="N277" s="2" t="n"/>
       <c r="O277" s="2" t="inlineStr">
         <is>
-          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte, 14 años para nacidos hasta 1965 (el ET de 1980 lo subió a 16) y 16 para los posteriores. Antes: 16 para todos.</t>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte (14 hasta 1965, 16 después) y excepción de menores autorizados (régimen 0112 artistas y sectores de espectáculos, artes, publicidad, deporte y casting: art. 6.4 ET).</t>
         </is>
       </c>
       <c r="P277" s="2" t="inlineStr">
         <is>
-          <t>t_tot_tipo_contrato_ppal &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) + 1</t>
+          <t>t_tot_tipo_contrato_ppal &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) + 1 AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
         </is>
       </c>
     </row>
@@ -20541,10 +20541,10 @@
         </is>
       </c>
       <c r="K278" s="2" t="n">
-        <v>286</v>
+        <v>16</v>
       </c>
       <c r="L278" s="2" t="n">
-        <v>0.021</v>
+        <v>0.0012</v>
       </c>
       <c r="M278" s="2" t="inlineStr">
         <is>
@@ -20554,12 +20554,12 @@
       <c r="N278" s="2" t="n"/>
       <c r="O278" s="2" t="inlineStr">
         <is>
-          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte, 14 años para nacidos hasta 1965 (el ET de 1980 lo subió a 16) y 16 para los posteriores. Antes: 16 para todos.</t>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte (14 hasta 1965, 16 después) y excepción de menores autorizados (régimen 0112 artistas y sectores de espectáculos, artes, publicidad, deporte y casting: art. 6.4 ET).</t>
         </is>
       </c>
       <c r="P278" s="2" t="inlineStr">
         <is>
-          <t>t_tot_prov_ppal &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) + 1</t>
+          <t>t_tot_prov_ppal &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) + 1 AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
         </is>
       </c>
     </row>
@@ -20615,10 +20615,10 @@
         </is>
       </c>
       <c r="K279" s="2" t="n">
-        <v>273</v>
+        <v>3</v>
       </c>
       <c r="L279" s="2" t="n">
-        <v>0.0201</v>
+        <v>0.0002</v>
       </c>
       <c r="M279" s="2" t="inlineStr">
         <is>
@@ -20628,12 +20628,12 @@
       <c r="N279" s="2" t="n"/>
       <c r="O279" s="2" t="inlineStr">
         <is>
-          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte, 14 años para nacidos hasta 1965 (el ET de 1980 lo subió a 16) y 16 para los posteriores. Antes: 16 para todos.</t>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte (14 hasta 1965, 16 después) y excepción de menores autorizados (régimen 0112 artistas y sectores de espectáculos, artes, publicidad, deporte y casting: art. 6.4 ET).</t>
         </is>
       </c>
       <c r="P279" s="2" t="inlineStr">
         <is>
-          <t>t_tot_act_econ_ppal &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) + 1</t>
+          <t>t_tot_act_econ_ppal &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) + 1 AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
         </is>
       </c>
     </row>
@@ -20689,10 +20689,10 @@
         </is>
       </c>
       <c r="K280" s="2" t="n">
-        <v>294</v>
+        <v>23</v>
       </c>
       <c r="L280" s="2" t="n">
-        <v>0.0216</v>
+        <v>0.0017</v>
       </c>
       <c r="M280" s="2" t="inlineStr">
         <is>
@@ -20702,12 +20702,12 @@
       <c r="N280" s="2" t="n"/>
       <c r="O280" s="2" t="inlineStr">
         <is>
-          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte, 14 años para nacidos hasta 1965 (el ET de 1980 lo subió a 16) y 16 para los posteriores. Antes: 16 para todos.</t>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte (14 hasta 1965, 16 después) y excepción de menores autorizados (régimen 0112 artistas y sectores de espectáculos, artes, publicidad, deporte y casting: art. 6.4 ET).</t>
         </is>
       </c>
       <c r="P280" s="2" t="inlineStr">
         <is>
-          <t>t_total_empleo &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) + 1</t>
+          <t>t_total_empleo &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) + 1 AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
         </is>
       </c>
     </row>
@@ -20763,10 +20763,10 @@
         </is>
       </c>
       <c r="K281" s="2" t="n">
-        <v>272</v>
+        <v>3</v>
       </c>
       <c r="L281" s="2" t="n">
-        <v>0.02</v>
+        <v>0.0002</v>
       </c>
       <c r="M281" s="2" t="inlineStr">
         <is>
@@ -20776,12 +20776,12 @@
       <c r="N281" s="2" t="n"/>
       <c r="O281" s="2" t="inlineStr">
         <is>
-          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte, 14 años para nacidos hasta 1965 (el ET de 1980 lo subió a 16) y 16 para los posteriores. Antes: 16 para todos.</t>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte (14 hasta 1965, 16 después) y excepción de menores autorizados (régimen 0112 artistas y sectores de espectáculos, artes, publicidad, deporte y casting: art. 6.4 ET).</t>
         </is>
       </c>
       <c r="P281" s="2" t="inlineStr">
         <is>
-          <t>t_contrato_mas_largo &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) + 1</t>
+          <t>t_contrato_mas_largo &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) + 1 AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
         </is>
       </c>
     </row>
@@ -20837,10 +20837,10 @@
         </is>
       </c>
       <c r="K282" s="2" t="n">
-        <v>1421</v>
+        <v>232</v>
       </c>
       <c r="L282" s="2" t="n">
-        <v>0.1046</v>
+        <v>0.0171</v>
       </c>
       <c r="M282" s="2" t="inlineStr">
         <is>
@@ -20850,12 +20850,12 @@
       <c r="N282" s="2" t="n"/>
       <c r="O282" s="2" t="inlineStr">
         <is>
-          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte, 14 años para nacidos hasta 1965 (el ET de 1980 lo subió a 16) y 16 para los posteriores. Antes: 16 para todos.</t>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte (14 hasta 1965, 16 después) y excepción de menores autorizados (régimen 0112 artistas y sectores de espectáculos, artes, publicidad, deporte y casting: art. 6.4 ET).</t>
         </is>
       </c>
       <c r="P282" s="2" t="inlineStr">
         <is>
-          <t>tiempo_total_desde_inicio_vl &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) + 1</t>
+          <t>tiempo_total_desde_inicio_vl &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) + 1 AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
         </is>
       </c>
     </row>
@@ -22251,10 +22251,10 @@
         </is>
       </c>
       <c r="K303" s="2" t="n">
-        <v>1636</v>
+        <v>397</v>
       </c>
       <c r="L303" s="2" t="n">
-        <v>0.1204</v>
+        <v>0.0292</v>
       </c>
       <c r="M303" s="2" t="inlineStr">
         <is>
@@ -22264,12 +22264,12 @@
       <c r="N303" s="2" t="n"/>
       <c r="O303" s="2" t="inlineStr">
         <is>
-          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte, 14 años para nacidos hasta 1965 (el ET de 1980 lo subió a 16) y 16 para los posteriores. Antes: 16 para todos.</t>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte (14 hasta 1965, 16 después) y excepción de menores autorizados (régimen 0112 artistas y sectores de espectáculos, artes, publicidad, deporte y casting: art. 6.4 ET).</t>
         </is>
       </c>
       <c r="P303" s="2" t="inlineStr">
         <is>
-          <t>date_diff('year', fecha_nacimiento, fecha_ini_primer_empleo) &lt; (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END)</t>
+          <t>date_diff('year', fecha_nacimiento, fecha_ini_primer_empleo) &lt; (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
         </is>
       </c>
     </row>
@@ -22523,10 +22523,10 @@
         </is>
       </c>
       <c r="K307" s="2" t="n">
-        <v>304</v>
+        <v>5</v>
       </c>
       <c r="L307" s="2" t="n">
-        <v>0.0224</v>
+        <v>0.0004</v>
       </c>
       <c r="M307" s="2" t="inlineStr">
         <is>
@@ -22536,12 +22536,12 @@
       <c r="N307" s="2" t="n"/>
       <c r="O307" s="2" t="inlineStr">
         <is>
-          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte, 14 años para nacidos hasta 1965 (el ET de 1980 lo subió a 16) y 16 para los posteriores. Antes: 16 para todos.</t>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte (14 hasta 1965, 16 después) y excepción de menores autorizados (régimen 0112 artistas y sectores de espectáculos, artes, publicidad, deporte y casting: art. 6.4 ET).</t>
         </is>
       </c>
       <c r="P307" s="2" t="inlineStr">
         <is>
-          <t>date_diff('year', fecha_nacimiento, fecha_ultima_baja) &lt; (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) AND (fecha_ultima_baja IS NULL OR year(fecha_ultima_baja) &lt;&gt; 2099)</t>
+          <t>date_diff('year', fecha_nacimiento, fecha_ultima_baja) &lt; (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) AND (fecha_ultima_baja IS NULL OR year(fecha_ultima_baja) &lt;&gt; 2099) AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
         </is>
       </c>
     </row>
@@ -22672,12 +22672,12 @@
       <c r="N309" s="2" t="n"/>
       <c r="O309" s="2" t="inlineStr">
         <is>
-          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte, 14 años para nacidos hasta 1965 (el ET de 1980 lo subió a 16) y 16 para los posteriores. Antes: 16 para todos.</t>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte (14 hasta 1965, 16 después) y excepción de menores autorizados (régimen 0112 artistas y sectores de espectáculos, artes, publicidad, deporte y casting: art. 6.4 ET).</t>
         </is>
       </c>
       <c r="P309" s="2" t="inlineStr">
         <is>
-          <t>date_diff('year', fecha_nacimiento, fecha_inicio_ultima_racha_sin_empleo) &lt; (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END)</t>
+          <t>date_diff('year', fecha_nacimiento, fecha_inicio_ultima_racha_sin_empleo) &lt; (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
         </is>
       </c>
     </row>
@@ -23983,10 +23983,10 @@
         </is>
       </c>
       <c r="K329" s="2" t="n">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="L329" s="2" t="n">
-        <v>0.0286</v>
+        <v>0.0282</v>
       </c>
       <c r="M329" s="2" t="inlineStr">
         <is>
@@ -23996,12 +23996,12 @@
       <c r="N329" s="2" t="n"/>
       <c r="O329" s="2" t="inlineStr">
         <is>
-          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte, 14 años para nacidos hasta 1965 (el ET de 1980 lo subió a 16) y 16 para los posteriores. Antes: 16 para todos.</t>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte (14 hasta 1965, 16 después) y excepción de menores autorizados (régimen 0112 artistas y sectores de espectáculos, artes, publicidad, deporte y casting: art. 6.4 ET).</t>
         </is>
       </c>
       <c r="P329" s="2" t="inlineStr">
         <is>
-          <t>edad_primer_empleo_signif &lt; (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END)</t>
+          <t>edad_primer_empleo_signif &lt; (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
         </is>
       </c>
     </row>
@@ -24053,10 +24053,10 @@
         </is>
       </c>
       <c r="K330" s="2" t="n">
-        <v>304</v>
+        <v>4</v>
       </c>
       <c r="L330" s="2" t="n">
-        <v>0.0224</v>
+        <v>0.0003</v>
       </c>
       <c r="M330" s="2" t="inlineStr">
         <is>
@@ -24066,12 +24066,12 @@
       <c r="N330" s="2" t="n"/>
       <c r="O330" s="2" t="inlineStr">
         <is>
-          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte, 14 años para nacidos hasta 1965 (el ET de 1980 lo subió a 16) y 16 para los posteriores. Antes: 16 para todos.</t>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte (14 hasta 1965, 16 después) y excepción de menores autorizados (régimen 0112 artistas y sectores de espectáculos, artes, publicidad, deporte y casting: art. 6.4 ET).</t>
         </is>
       </c>
       <c r="P330" s="2" t="inlineStr">
         <is>
-          <t>edad_ultimo_empleo &lt; (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END)</t>
+          <t>edad_ultimo_empleo &lt; (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
         </is>
       </c>
     </row>
@@ -24127,10 +24127,10 @@
         </is>
       </c>
       <c r="K331" s="2" t="n">
-        <v>2117</v>
+        <v>878</v>
       </c>
       <c r="L331" s="2" t="n">
-        <v>0.1558</v>
+        <v>0.0646</v>
       </c>
       <c r="M331" s="2" t="inlineStr">
         <is>
@@ -24140,12 +24140,12 @@
       <c r="N331" s="2" t="n"/>
       <c r="O331" s="2" t="inlineStr">
         <is>
-          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte, 14 años para nacidos hasta 1965 (el ET de 1980 lo subió a 16) y 16 para los posteriores. Antes: 16 para todos.</t>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte (14 hasta 1965, 16 después) y excepción de menores autorizados (régimen 0112 artistas y sectores de espectáculos, artes, publicidad, deporte y casting: art. 6.4 ET).</t>
         </is>
       </c>
       <c r="P331" s="2" t="inlineStr">
         <is>
-          <t>edad_actual_fecha_corte - tiempo_total_desde_inicio_vl &lt; (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END)</t>
+          <t>edad_actual_fecha_corte - tiempo_total_desde_inicio_vl &lt; (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
         </is>
       </c>
     </row>
@@ -39632,10 +39632,10 @@
         <v>112</v>
       </c>
       <c r="C3" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D3" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4">
@@ -39664,10 +39664,10 @@
         <v>561</v>
       </c>
       <c r="C5" t="n">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="D5" t="n">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="6"/>
@@ -39719,10 +39719,10 @@
         <v>120</v>
       </c>
       <c r="C9" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D9" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="10">
@@ -39771,7 +39771,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15">
@@ -39781,7 +39781,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
tests: G04 cerrado - residuo de edad minima como baja calidad de los datos
Residuo tras el corte por cohorte y la excepcion de menores autorizados: C-079 397 (336 con CNAE
desconocido), C-107 878, C-058 232. Se descarta ampliar la excepcion a CNAE desconocido. Pendiente
aparte y sin tocar: el corte en 16 de las graficas por edad de Trayectorias de colectivos.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/reglas_consistencia_resultados_sin_ipf.xlsx
+++ b/tests/reglas_consistencia_resultados_sin_ipf.xlsx
@@ -732,7 +732,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
@@ -771,7 +771,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Revisar el residuo (menores de 14 nacidos hasta 1965 y menores de 16 nacidos desde 1966, sobre todo los de menos de 12 años). Pendiente aparte: las gráficas por edad de Trayectorias de colectivos cortan en 16 (app/routers/trayectorias.py) y omiten los 14-15 años legítimos de las cohortes antiguas; el usuario decidió dejarlo para más adelante.</t>
+          <t>CERRADO 2026-09-24 (decisión del usuario). Residuo como baja calidad de los datos: 397 en C-079 (336 con CNAE desconocido, 329 en régimen general; 150 con 12-13 años, 133 con 14-15 y 114 con menos de 12), 878 en C-107 y 232 en C-058: episodios sin sector conocido que pueden ser errores de fecha o menores autorizados sin CNAE. Se descarta ampliar la excepción a CNAE desconocido (dejaría pasar cualquier error de fecha). Pendiente aparte: las gráficas por edad de Trayectorias de colectivos cortan en 16 (app/routers/trayectorias.py) y omiten los 14-15 años legítimos de las cohortes antiguas; el usuario decidió dejarlo para más adelante.</t>
         </is>
       </c>
     </row>
@@ -8081,7 +8081,7 @@
       </c>
       <c r="J94" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K94" s="2" t="n">
@@ -12029,7 +12029,7 @@
       </c>
       <c r="J152" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K152" s="2" t="n">
@@ -12997,7 +12997,7 @@
       </c>
       <c r="J166" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K166" s="2" t="n">
@@ -14101,7 +14101,7 @@
       </c>
       <c r="J182" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K182" s="2" t="n">
@@ -15065,7 +15065,7 @@
       </c>
       <c r="J196" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K196" s="2" t="n">
@@ -20315,7 +20315,7 @@
       </c>
       <c r="J275" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K275" s="2" t="n">
@@ -20389,7 +20389,7 @@
       </c>
       <c r="J276" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K276" s="2" t="n">
@@ -20463,7 +20463,7 @@
       </c>
       <c r="J277" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K277" s="2" t="n">
@@ -20537,7 +20537,7 @@
       </c>
       <c r="J278" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K278" s="2" t="n">
@@ -20611,7 +20611,7 @@
       </c>
       <c r="J279" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K279" s="2" t="n">
@@ -20685,7 +20685,7 @@
       </c>
       <c r="J280" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K280" s="2" t="n">
@@ -20759,7 +20759,7 @@
       </c>
       <c r="J281" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K281" s="2" t="n">
@@ -20833,7 +20833,7 @@
       </c>
       <c r="J282" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K282" s="2" t="n">
@@ -22247,7 +22247,7 @@
       </c>
       <c r="J303" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K303" s="2" t="n">
@@ -22519,7 +22519,7 @@
       </c>
       <c r="J307" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K307" s="2" t="n">
@@ -22655,7 +22655,7 @@
       </c>
       <c r="J309" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K309" s="2" t="n">
@@ -23381,7 +23381,7 @@
       </c>
       <c r="J320" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K320" s="2" t="n">
@@ -23447,7 +23447,7 @@
       </c>
       <c r="J321" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K321" s="2" t="n">
@@ -23979,7 +23979,7 @@
       </c>
       <c r="J329" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K329" s="2" t="n">
@@ -24049,7 +24049,7 @@
       </c>
       <c r="J330" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K330" s="2" t="n">
@@ -24123,7 +24123,7 @@
       </c>
       <c r="J331" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K331" s="2" t="n">
@@ -24589,7 +24589,7 @@
       </c>
       <c r="J338" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K338" s="2" t="n">
@@ -24659,7 +24659,7 @@
       </c>
       <c r="J339" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K339" s="2" t="n">
@@ -28229,7 +28229,7 @@
       </c>
       <c r="J392" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K392" s="2" t="n">
@@ -32803,7 +32803,7 @@
       </c>
       <c r="J463" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K463" s="2" t="n">
@@ -33651,7 +33651,7 @@
       </c>
       <c r="J475" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K475" s="2" t="n">
@@ -39781,7 +39781,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>86</v>
+        <v>60</v>
       </c>
     </row>
     <row r="16">
@@ -39791,7 +39791,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>46</v>
+        <v>72</v>
       </c>
     </row>
     <row r="17"/>

</xml_diff>

<commit_message>
tests: G21 cerrado - tramos deterministas regenerados (411 de 561 pasan)
Reglas sobre el final/parcial/tramos regenerados con orden total en las ventanas: C-265 83 -> 1, C-264
176 -> 1, C-262 120 -> 0, C-266/C-267 -> 0, C-252 186 -> 112. B-046/B-076 reformuladas (suman
t_total_mixto_empl_desempl): 0. G21 corregido; G11 actualizado.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/reglas_consistencia_resultados_sin_ipf.xlsx
+++ b/tests/reglas_consistencia_resultados_sin_ipf.xlsx
@@ -683,10 +683,10 @@
         <v>7</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.0002</v>
+        <v>0.0001</v>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
@@ -798,11 +798,11 @@
         <v>7779</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.572</v>
+        <v>0.5724</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>C-254, C-253, C-252, A-057, B-016, C-020</t>
+          <t>A-057, B-016, C-020, C-252, C-253, C-254</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -851,14 +851,14 @@
         <v>10</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>16674</v>
+        <v>16660</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>1.227</v>
+        <v>1.2259</v>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>C-158, A-105, C-157, C-159, B-060, B-061, A-064, A-072, B-090, B-091</t>
+          <t>A-064, A-072, A-105, B-060, B-061, B-090, B-091, C-157, C-158, C-159</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -1124,22 +1124,22 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E12" s="2" t="n">
         <v>9196</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0.677</v>
+        <v>0.6766</v>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>C-260, C-069, C-070, C-268, C-072, C-264, C-073, C-262, C-074, C-075, C-076, C-267, C-266</t>
+          <t>C-069, C-070, C-072, C-073, C-074, C-075, C-076, C-260, C-264, C-268</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Con las bajas reales (2026-09-21), C-255 (bajas &gt; altas) pasa a 0 y C-257/C-258 (enteros) se corrigieron (factor 365 vs 365,25). Siguen: 9.198 con más causas distintas que altas + 1,5 (C-260), ~2.100 con más de 20 altas/bajas por año (C-069/C-070).</t>
+          <t>Con las bajas reales (2026-09-21), C-255 (bajas &gt; altas) pasa a 0 y C-257/C-258 (enteros) se corrigieron (factor 365 vs 365,25). Siguen: 9.198 con más causas distintas que altas + 1,5 (C-260), ~2.100 con más de 20 altas/bajas por año (C-069/C-070). ACTUALIZACIÓN 2026-09-24: C-262 (120), C-264 (176), C-266 y C-267 pasan a 0 o 1 tras corregir los tramos de afiliación (ver G21).</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1667,51 +1667,51 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Residuo tras G08 sin investigar</t>
+          <t>Tramos de afiliación no deterministas + regla que ignoraba el tiempo mixto</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Corregido</t>
         </is>
       </c>
       <c r="D22" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>83</v>
+        <v>1</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>0.0061</v>
+        <v>0.0001</v>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>B-046, B-076, C-265</t>
+          <t>C-265</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>B-046/B-076: 26 personas Parado_LD/Parado_NoLD sin empleo real que no son del colectivo solo-prestaciones (ninguna con episodio de duración nula). C-265: 83 con duración del primer empleo significativo mayor que el tiempo total de empleo.</t>
+          <t>C-265 (83): personas, casi todas agrarias con muchos episodios y episodios de empleo larguísimos (uno de 31,7 años) cuyo EMPLEO+MIXTO de tabla_afiliacion_tramos.parquet salía muy por debajo de sus propios episodios. B-046/B-076 (26+26): 52 personas Parado con t_total_empleo = 0 que sí trabajaron, siempre a la vez que cobraban prestación (tiempo en t_total_mixto_empl_desempl).</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Por investigar.</t>
+          <t>VERIFICADO 2026-09-24: la fusión de tramos (fase1b_tramos_fusionados_duckdb) y la de categoría ganadora (_sql_categoria_ppal_fusionada) ordenaban sus ventanas solo por fecha_alta: episodios de una misma persona y categoría que empiezan el mismo día quedaban en un orden no fijado, distinto entre las dos ventanas, y el resultado cambiaba entre ejecuciones idénticas (5.001 de 1.313.883 personas, hasta 44 años de diferencia; 159-254 personas con un episodio más largo que su EMPLEO+MIXTO). El fichero de tramos difería del cálculo correcto en 2.476 personas (2.020 con días de más y 244 con días de menos).</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>A investigar</t>
+          <t>Bug del ETL, corregido</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>Investigar cuando haya tiempo; volumen muy pequeño.</t>
+          <t>ARREGLADO: ORDER BY fecha_alta, fecha_baja, rn (file_row_number) en las dos ventanas de ambas funciones (commit 3ec2fe5); acción 'tramos' en ejecutar_paso.py (f00acb7); etl/verificar_tramos.py comprueba determinismo y violaciones. Verificado a escala completa en el PC corporativo: 0 diferencias entre ejecuciones y 0 violaciones. Tramos, parcial y final regenerados. Resultado: C-265 83 -&gt; 1, C-264 176 -&gt; 1, C-262 120 -&gt; 0, C-266/C-267 -&gt; 0, C-252 186 -&gt; 112. B-046/B-076 reformuladas (suman t_total_mixto_empl_desempl): 0.</t>
         </is>
       </c>
     </row>
@@ -5331,10 +5331,10 @@
         </is>
       </c>
       <c r="K53" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L53" s="2" t="n">
-        <v>0.0004</v>
+        <v>0.0003</v>
       </c>
       <c r="M53" s="2" t="inlineStr">
         <is>
@@ -5342,7 +5342,11 @@
         </is>
       </c>
       <c r="N53" s="2" t="n"/>
-      <c r="O53" s="2" t="inlineStr"/>
+      <c r="O53" s="2" t="inlineStr">
+        <is>
+          <t>Cifra actualizada 2026-09-24 (variación de 1 a 14 personas).</t>
+        </is>
+      </c>
       <c r="P53" s="2" t="inlineStr">
         <is>
           <t>situacion_actual_afiliacion = 'Alta_ocupado' AND COALESCE(t_total_empleo, 0) = 0</t>
@@ -9577,10 +9581,10 @@
         </is>
       </c>
       <c r="K116" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L116" s="2" t="n">
-        <v>0.0004</v>
+        <v>0.0003</v>
       </c>
       <c r="M116" s="2" t="inlineStr">
         <is>
@@ -9588,7 +9592,11 @@
         </is>
       </c>
       <c r="N116" s="2" t="n"/>
-      <c r="O116" s="2" t="inlineStr"/>
+      <c r="O116" s="2" t="inlineStr">
+        <is>
+          <t>Cifra actualizada 2026-09-24 (variación de 1 a 14 personas).</t>
+        </is>
+      </c>
       <c r="P116" s="2" t="inlineStr">
         <is>
           <t>situacion_paro_ocupacion = 'Ocupado' AND COALESCE(t_total_empleo, 0) = 0</t>
@@ -12425,7 +12433,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>Parado_LD ⇒ ha trabajado alguna vez (t_total_empleo &gt; 0)</t>
+          <t>Parado_LD ⇒ ha trabajado alguna vez (t_total_empleo + t_total_mixto_empl_desempl &gt; 0)</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -12440,19 +12448,19 @@
       </c>
       <c r="I158" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J158" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Corregido</t>
         </is>
       </c>
       <c r="K158" s="2" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="L158" s="2" t="n">
-        <v>0.0019</v>
+        <v>0</v>
       </c>
       <c r="M158" s="2" t="inlineStr">
         <is>
@@ -12462,12 +12470,12 @@
       <c r="N158" s="2" t="n"/>
       <c r="O158" s="2" t="inlineStr">
         <is>
-          <t>Alguien puede haber tenido solo prestaciones | Regla ajustada 2026-09-24 (G08): excluye a quien solo tiene episodios TRL 7xx/400 (dato de origen, p. ej. agrarios con trabajo temporal mal registrado).</t>
+          <t>Regla reformulada 2026-09-24 (G21): suma también t_total_mixto_empl_desempl; los 52 casos (26+26) trabajaron siempre a la vez que cobraban prestación y tenían t_total_empleo = 0.</t>
         </is>
       </c>
       <c r="P158" s="2" t="inlineStr">
         <is>
-          <t>situacion_paro_ocupacion = 'Parado_LD' AND COALESCE(t_total_empleo, 0) = 0</t>
+          <t>situacion_paro_ocupacion = 'Parado_LD' AND COALESCE(t_total_empleo, 0) + COALESCE(t_total_mixto_empl_desempl, 0) = 0 AND ipf NOT IN (SELECT ipf FROM solo_prestaciones)</t>
         </is>
       </c>
     </row>
@@ -14493,7 +14501,7 @@
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>Parado_NoLD ⇒ ha trabajado alguna vez (t_total_empleo &gt; 0)</t>
+          <t>Parado_NoLD ⇒ ha trabajado alguna vez (t_total_empleo + t_total_mixto_empl_desempl &gt; 0)</t>
         </is>
       </c>
       <c r="G188" s="2" t="inlineStr">
@@ -14508,19 +14516,19 @@
       </c>
       <c r="I188" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J188" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Corregido</t>
         </is>
       </c>
       <c r="K188" s="2" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="L188" s="2" t="n">
-        <v>0.0019</v>
+        <v>0</v>
       </c>
       <c r="M188" s="2" t="inlineStr">
         <is>
@@ -14530,12 +14538,12 @@
       <c r="N188" s="2" t="n"/>
       <c r="O188" s="2" t="inlineStr">
         <is>
-          <t>Alguien puede haber tenido solo prestaciones | Regla ajustada 2026-09-24 (G08): excluye a quien solo tiene episodios TRL 7xx/400 (dato de origen, p. ej. agrarios con trabajo temporal mal registrado).</t>
+          <t>Regla reformulada 2026-09-24 (G21): suma también t_total_mixto_empl_desempl; los 52 casos (26+26) trabajaron siempre a la vez que cobraban prestación y tenían t_total_empleo = 0.</t>
         </is>
       </c>
       <c r="P188" s="2" t="inlineStr">
         <is>
-          <t>situacion_paro_ocupacion = 'Parado_NoLD' AND COALESCE(t_total_empleo, 0) = 0</t>
+          <t>situacion_paro_ocupacion = 'Parado_NoLD' AND COALESCE(t_total_empleo, 0) + COALESCE(t_total_mixto_empl_desempl, 0) = 0 AND ipf NOT IN (SELECT ipf FROM solo_prestaciones)</t>
         </is>
       </c>
     </row>
@@ -18728,25 +18736,25 @@
       </c>
       <c r="I252" s="6" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J252" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pasan</t>
         </is>
       </c>
       <c r="K252" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L252" s="2" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
       <c r="M252" s="2" t="inlineStr"/>
       <c r="N252" s="2" t="n"/>
       <c r="O252" s="2" t="inlineStr">
         <is>
-          <t>Cifra actualizada 2026-09-24: variación de unas pocas personas por el cálculo no determinista de los tiempos por categoría (374 personas difieren entre regeneraciones).</t>
+          <t>Cifra actualizada 2026-09-24: variación de unas pocas personas por el cálculo no determinista de los tiempos por categoría (374 personas difieren entre regeneraciones). | Actualizado 2026-09-24: tramos de afiliación regenerados con orden total en las ventanas (la fusión anterior no era determinista: 2.476 personas cambian).</t>
         </is>
       </c>
       <c r="P252" s="2" t="inlineStr">
@@ -19685,7 +19693,7 @@
         </is>
       </c>
       <c r="K266" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L266" s="2" t="n">
         <v>0.0001</v>
@@ -19698,7 +19706,7 @@
       <c r="N266" s="2" t="n"/>
       <c r="O266" s="2" t="inlineStr">
         <is>
-          <t>Cifra actualizada 2026-09-24: variación de unas pocas personas por el cálculo no determinista de los tiempos por categoría (374 personas difieren entre regeneraciones).</t>
+          <t>Cifra actualizada 2026-09-24: variación de unas pocas personas por el cálculo no determinista de los tiempos por categoría (374 personas difieren entre regeneraciones). | Actualizado 2026-09-24: tramos de afiliación regenerados con orden total en las ventanas (la fusión anterior no era determinista: 2.476 personas cambian).</t>
         </is>
       </c>
       <c r="P266" s="2" t="inlineStr">
@@ -19833,10 +19841,10 @@
         </is>
       </c>
       <c r="K268" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L268" s="2" t="n">
-        <v>0.0002</v>
+        <v>0.0001</v>
       </c>
       <c r="M268" s="2" t="inlineStr">
         <is>
@@ -19846,7 +19854,7 @@
       <c r="N268" s="2" t="n"/>
       <c r="O268" s="2" t="inlineStr">
         <is>
-          <t>Cifra actualizada 2026-09-24: variación de unas pocas personas por el cálculo no determinista de los tiempos por categoría (374 personas difieren entre regeneraciones).</t>
+          <t>Cifra actualizada 2026-09-24: variación de unas pocas personas por el cálculo no determinista de los tiempos por categoría (374 personas difieren entre regeneraciones). | Actualizado 2026-09-24: tramos de afiliación regenerados con orden total en las ventanas (la fusión anterior no era determinista: 2.476 personas cambian).</t>
         </is>
       </c>
       <c r="P268" s="2" t="inlineStr">
@@ -19907,7 +19915,7 @@
         </is>
       </c>
       <c r="K269" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L269" s="2" t="n">
         <v>0.0001</v>
@@ -19920,7 +19928,7 @@
       <c r="N269" s="2" t="n"/>
       <c r="O269" s="2" t="inlineStr">
         <is>
-          <t>Cifra actualizada 2026-09-24: variación de unas pocas personas por el cálculo no determinista de los tiempos por categoría (374 personas difieren entre regeneraciones).</t>
+          <t>Cifra actualizada 2026-09-24: variación de unas pocas personas por el cálculo no determinista de los tiempos por categoría (374 personas difieren entre regeneraciones). | Actualizado 2026-09-24: tramos de afiliación regenerados con orden total en las ventanas (la fusión anterior no era determinista: 2.476 personas cambian).</t>
         </is>
       </c>
       <c r="P269" s="2" t="inlineStr">
@@ -20393,10 +20401,10 @@
         </is>
       </c>
       <c r="K276" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L276" s="2" t="n">
-        <v>0.0004</v>
+        <v>0.0003</v>
       </c>
       <c r="M276" s="2" t="inlineStr">
         <is>
@@ -20406,7 +20414,7 @@
       <c r="N276" s="2" t="n"/>
       <c r="O276" s="2" t="inlineStr">
         <is>
-          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte (14 hasta 1965, 16 después) y excepción de menores autorizados (régimen 0112 artistas y sectores de espectáculos, artes, publicidad, deporte y casting: art. 6.4 ET).</t>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte (14 hasta 1965, 16 después) y excepción de menores autorizados (régimen 0112 artistas y sectores de espectáculos, artes, publicidad, deporte y casting: art. 6.4 ET). | Actualizado 2026-09-24: tramos de afiliación regenerados con orden total en las ventanas (la fusión anterior no era determinista: 2.476 personas cambian).</t>
         </is>
       </c>
       <c r="P276" s="2" t="inlineStr">
@@ -27573,10 +27581,10 @@
         </is>
       </c>
       <c r="K382" s="2" t="n">
-        <v>16674</v>
+        <v>16660</v>
       </c>
       <c r="L382" s="2" t="n">
-        <v>1.2269</v>
+        <v>1.2259</v>
       </c>
       <c r="M382" s="2" t="inlineStr">
         <is>
@@ -27586,7 +27594,7 @@
       <c r="N382" s="2" t="n"/>
       <c r="O382" s="2" t="inlineStr">
         <is>
-          <t>Faltan datos anteriores a 1967</t>
+          <t>Faltan datos anteriores a 1967 | Cifra actualizada 2026-09-24 (variación de 1 a 14 personas).</t>
         </is>
       </c>
       <c r="P382" s="2" t="inlineStr">
@@ -33581,10 +33589,10 @@
         </is>
       </c>
       <c r="K474" s="2" t="n">
-        <v>17707</v>
+        <v>17708</v>
       </c>
       <c r="L474" s="2" t="n">
-        <v>1.3029</v>
+        <v>1.303</v>
       </c>
       <c r="M474" s="2" t="inlineStr">
         <is>
@@ -33594,7 +33602,7 @@
       <c r="N474" s="2" t="n"/>
       <c r="O474" s="2" t="inlineStr">
         <is>
-          <t>Cifra actualizada 2026-09-24 (variacion de 1 persona por el cálculo no determinista).</t>
+          <t>Cifra actualizada 2026-09-24 (variacion de 1 persona por el cálculo no determinista). | Cifra actualizada 2026-09-24 (variación de 1 a 14 personas).</t>
         </is>
       </c>
       <c r="P474" s="2" t="inlineStr">
@@ -33721,10 +33729,10 @@
         </is>
       </c>
       <c r="K476" s="2" t="n">
-        <v>186</v>
+        <v>112</v>
       </c>
       <c r="L476" s="2" t="n">
-        <v>0.0137</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="M476" s="2" t="inlineStr">
         <is>
@@ -33734,7 +33742,7 @@
       <c r="N476" s="2" t="n"/>
       <c r="O476" s="2" t="inlineStr">
         <is>
-          <t>Unidad: euros por año cotizado (confirmado por el usuario); el pluriempleo puede sumar bases</t>
+          <t>Unidad: euros por año cotizado (confirmado por el usuario); el pluriempleo puede sumar bases | Actualizado 2026-09-24: tramos de afiliación regenerados con orden total en las ventanas (la fusión anterior no era determinista: 2.476 personas cambian).</t>
         </is>
       </c>
       <c r="P476" s="2" t="inlineStr">
@@ -34404,19 +34412,19 @@
       </c>
       <c r="I486" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J486" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Corregido</t>
         </is>
       </c>
       <c r="K486" s="2" t="n">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="L486" s="2" t="n">
-        <v>0.008800000000000001</v>
+        <v>0</v>
       </c>
       <c r="M486" s="2" t="inlineStr">
         <is>
@@ -34426,7 +34434,7 @@
       <c r="N486" s="2" t="n"/>
       <c r="O486" s="2" t="inlineStr">
         <is>
-          <t>El tiempo 'mixto' (empleo y desempleo a la vez) también es empleo; regla corregida tras la 1ª ejecución con las tablas v2.2</t>
+          <t>El tiempo 'mixto' (empleo y desempleo a la vez) también es empleo; regla corregida tras la 1ª ejecución con las tablas v2.2 | Actualizado 2026-09-24: tramos de afiliación regenerados con orden total en las ventanas (la fusión anterior no era determinista: 2.476 personas cambian).</t>
         </is>
       </c>
       <c r="P486" s="2" t="inlineStr">
@@ -34553,10 +34561,10 @@
         </is>
       </c>
       <c r="K488" s="2" t="n">
-        <v>176</v>
+        <v>1</v>
       </c>
       <c r="L488" s="2" t="n">
-        <v>0.013</v>
+        <v>0.0001</v>
       </c>
       <c r="M488" s="2" t="inlineStr">
         <is>
@@ -34564,7 +34572,11 @@
         </is>
       </c>
       <c r="N488" s="2" t="n"/>
-      <c r="O488" s="2" t="inlineStr"/>
+      <c r="O488" s="2" t="inlineStr">
+        <is>
+          <t>Actualizado 2026-09-24: tramos de afiliación regenerados con orden total en las ventanas (la fusión anterior no era determinista: 2.476 personas cambian).</t>
+        </is>
+      </c>
       <c r="P488" s="2" t="inlineStr">
         <is>
           <t>t_contrato_mas_largo &gt; COALESCE(t_total_empleo,0) + COALESCE(t_total_mixto_empl_desempl,0) + 1</t>
@@ -34623,10 +34635,10 @@
         </is>
       </c>
       <c r="K489" s="2" t="n">
-        <v>83</v>
+        <v>1</v>
       </c>
       <c r="L489" s="2" t="n">
-        <v>0.0061</v>
+        <v>0.0001</v>
       </c>
       <c r="M489" s="2" t="inlineStr">
         <is>
@@ -34636,7 +34648,7 @@
       <c r="N489" s="2" t="n"/>
       <c r="O489" s="2" t="inlineStr">
         <is>
-          <t>Regla ajustada 2026-09-24 (G08): excluye a quien solo tiene episodios TRL 7xx/400 (dato de origen, p. ej. agrarios con trabajo temporal mal registrado).</t>
+          <t>Regla ajustada 2026-09-24 (G08): excluye a quien solo tiene episodios TRL 7xx/400 (dato de origen, p. ej. agrarios con trabajo temporal mal registrado). | Actualizado 2026-09-24: tramos de afiliación regenerados con orden total en las ventanas (la fusión anterior no era determinista: 2.476 personas cambian).</t>
         </is>
       </c>
       <c r="P489" s="2" t="inlineStr">
@@ -34688,19 +34700,19 @@
       </c>
       <c r="I490" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J490" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Corregido</t>
         </is>
       </c>
       <c r="K490" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L490" s="2" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
       <c r="M490" s="2" t="inlineStr">
         <is>
@@ -34710,7 +34722,7 @@
       <c r="N490" s="2" t="n"/>
       <c r="O490" s="2" t="inlineStr">
         <is>
-          <t>La categoría 'principal' es la de más tiempo</t>
+          <t>La categoría 'principal' es la de más tiempo | Actualizado 2026-09-24: tramos de afiliación regenerados con orden total en las ventanas (la fusión anterior no era determinista: 2.476 personas cambian).</t>
         </is>
       </c>
       <c r="P490" s="2" t="inlineStr">
@@ -34762,19 +34774,19 @@
       </c>
       <c r="I491" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J491" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Corregido</t>
         </is>
       </c>
       <c r="K491" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L491" s="2" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
       <c r="M491" s="2" t="inlineStr">
         <is>
@@ -34784,7 +34796,7 @@
       <c r="N491" s="2" t="n"/>
       <c r="O491" s="2" t="inlineStr">
         <is>
-          <t>La categoría 'principal' es la de más tiempo</t>
+          <t>La categoría 'principal' es la de más tiempo | Actualizado 2026-09-24: tramos de afiliación regenerados con orden total en las ventanas (la fusión anterior no era determinista: 2.476 personas cambian).</t>
         </is>
       </c>
       <c r="P491" s="2" t="inlineStr">
@@ -39632,10 +39644,10 @@
         <v>112</v>
       </c>
       <c r="C3" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D3" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4">
@@ -39648,10 +39660,10 @@
         <v>338</v>
       </c>
       <c r="C4" t="n">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="D4" t="n">
-        <v>97</v>
+        <v>93</v>
       </c>
     </row>
     <row r="5">
@@ -39664,10 +39676,10 @@
         <v>561</v>
       </c>
       <c r="C5" t="n">
-        <v>407</v>
+        <v>413</v>
       </c>
       <c r="D5" t="n">
-        <v>154</v>
+        <v>148</v>
       </c>
     </row>
     <row r="6"/>
@@ -39703,10 +39715,10 @@
         <v>381</v>
       </c>
       <c r="C8" t="n">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="D8" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9">
@@ -39719,10 +39731,10 @@
         <v>120</v>
       </c>
       <c r="C9" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D9" t="n">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10">
@@ -39735,10 +39747,10 @@
         <v>60</v>
       </c>
       <c r="C10" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D10" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11"/>
@@ -39761,7 +39773,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>401</v>
+        <v>402</v>
       </c>
     </row>
     <row r="14">
@@ -39771,7 +39783,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
     </row>
     <row r="15">
@@ -39781,7 +39793,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
ETL: toda clave de grupo de cotizacion fuera de 00-12 se asimila al 00 NO CONSTA
Generaliza el cambio anterior (solo 21 y 23): 13, 14, 19, 20, 21, 23, 31, 63 y cualquier clave futura fuera de
00-12 cuentan como 00 en Grupo_cotiz_ppal/t_tot_grupo_ppal (la guia: valores fuera de la tabla = el dato no
consta; las otras variables de grupo ya las decodifican asi). NULL sigue excluido. Sobre las 335 personas de
C-268: 335 -> 0; sobre una muestra de 29.004 personas solo cambia el grupo principal de 38 (0,13 %), todas a 00.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/reglas_consistencia_resultados_sin_ipf.xlsx
+++ b/tests/reglas_consistencia_resultados_sin_ipf.xlsx
@@ -1139,7 +1139,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Con las bajas reales (2026-09-21), C-255 (bajas &gt; altas) pasa a 0 y C-257/C-258 (enteros) se corrigieron (factor 365 vs 365,25). Siguen: 9.198 con más causas distintas que altas + 1,5 (C-260), ~2.100 con más de 20 altas/bajas por año (C-069/C-070). ACTUALIZACIÓN 2026-09-24: C-262 (120), C-264 (176), C-266 y C-267 pasan a 0 o 1 tras corregir los tramos de afiliación (ver G21). CERRADO 2026-09-25 (decisión del usuario): la variable causas_baja_distintas se ELIMINA (ETL, app y sus 11 reglas: A-018, A-044, C-026, C-077, C-139, C-140, C-144, C-145, C-259, C-260, C-261) porque contaba causas de todos los episodios y no era comparable con las altas de empleo; los umbrales de valores extremos C-069, C-070 (más de 20 altas o bajas por año: perfil real de contratación muy fragmentada, mediana 222 altas) y C-072 a C-076 se QUITAN por ser casos reales, no errores. C-268 (335): los grupos de cotización 21 y 23 son del R.E. Agrario Cuenta Propia (0721) y la guía dice que valores fuera de 00-12 = 'no consta'; el ETL los asimila ahora al 00 NO CONSTA (335 -&gt; 7).</t>
+          <t>Con las bajas reales (2026-09-21), C-255 (bajas &gt; altas) pasa a 0 y C-257/C-258 (enteros) se corrigieron (factor 365 vs 365,25). Siguen: 9.198 con más causas distintas que altas + 1,5 (C-260), ~2.100 con más de 20 altas/bajas por año (C-069/C-070). ACTUALIZACIÓN 2026-09-24: C-262 (120), C-264 (176), C-266 y C-267 pasan a 0 o 1 tras corregir los tramos de afiliación (ver G21). CERRADO 2026-09-25 (decisión del usuario): la variable causas_baja_distintas se ELIMINA (ETL, app y sus 11 reglas: A-018, A-044, C-026, C-077, C-139, C-140, C-144, C-145, C-259, C-260, C-261) porque contaba causas de todos los episodios y no era comparable con las altas de empleo; los umbrales de valores extremos C-069, C-070 (más de 20 altas o bajas por año: perfil real de contratación muy fragmentada, mediana 222 altas) y C-072 a C-076 se QUITAN por ser casos reales, no errores. C-268 (335): los grupos de cotización 21 y 23 son del R.E. Agrario Cuenta Propia (0721) y la guía dice que valores fuera de 00-12 = 'no consta'; el ETL asimila ahora TODA clave fuera de 00-12 (13, 14, 19, 20, 21, 23, 31, 63) al 00 NO CONSTA (335 -&gt; 0 en la prueba; en una muestra de 29.004 personas solo cambia el grupo principal de 38, el 0,13 %).</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Regenerar tramos/Personas/Fase 3 con el ETL nuevo (grupos 21 y 23 -&gt; 00 y sin causas_baja_distintas) y volver a pasar las reglas: C-268 debe bajar de 335 a unos 7. C-264 (1 persona) sin acción.</t>
+          <t>Regenerar tramos/Personas/Fase 3 con el ETL nuevo (claves fuera de 00-12 -&gt; 00 y sin causas_baja_distintas) y volver a pasar las reglas: C-268 debe bajar de 335 a 0 o casi. C-264 (1 persona) sin acción.</t>
         </is>
       </c>
     </row>
@@ -33658,7 +33658,7 @@
       <c r="N474" s="2" t="n"/>
       <c r="O474" s="2" t="inlineStr">
         <is>
-          <t>ETL cambiado 2026-09-25 (decisión del usuario): los grupos de cotización 21 y 23 (R.E. Agrario Cuenta Propia, 0721) se asimilan al 00 NO CONSTA en Grupo_cotiz_ppal/t_tot_grupo_ppal, como indica la guía. Probado sobre las 335 personas: 335 -&gt; 7. Pendiente de regenerar los Parquet.</t>
+          <t>ETL cambiado 2026-09-25 (decisión del usuario): cualquier clave de grupo de cotización fuera de 00-12 (13, 14, 19, 20, 21, 23, 31, 63) se asimila al 00 NO CONSTA en Grupo_cotiz_ppal/t_tot_grupo_ppal, como indica la guía (las 335 personas tenían sus años de empleo en los grupos 21/23 del R.E. Agrario Cuenta Propia). Probado sobre las 335: 335 -&gt; 0. Pendiente de regenerar los Parquet.</t>
         </is>
       </c>
       <c r="P474" s="2" t="inlineStr">

</xml_diff>

<commit_message>
reglas: G09 - "no fallecido antes de 2025" pasa a "antes de 2024"; C-270 baja calidad
Las 3.115 incumplidoras fallecieron todas en 2024, cuando aun cobraban prestacion o pension (edicion
2024). A-055, A-108, B-007, B-023, B-048, B-062, B-078 y B-092 pasan a 0. C-270 (7 personas, baja por
fallecimiento sin fecha en Personas) queda como dato de origen.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/reglas_consistencia_resultados_sin_ipf.xlsx
+++ b/tests/reglas_consistencia_resultados_sin_ipf.xlsx
@@ -1016,22 +1016,22 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>2160</v>
+        <v>1177</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0.159</v>
+        <v>0.0866</v>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>B-062, B-108, B-078, B-048, B-110, C-071, B-092, A-054, B-022, A-108, B-006, C-270, A-055, B-007, B-109, B-023</t>
+          <t>A-054, B-006, B-022, B-108, B-109, B-110, C-071, C-270</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>4.319 Parado_LD_pension_no_jubilacion fallecidos antes de 2025 (B-062; pudieron cobrar pensión en 2024); 1.046 Pensionistas con más de 100 años (B-108); 501 Parado_NoLD y 385 Parado_LD fallecidos antes de 2025.</t>
+          <t>4.319 Parado_LD_pension_no_jubilacion fallecidos antes de 2025 (B-062; pudieron cobrar pensión en 2024); 1.046 Pensionistas con más de 100 años (B-108); 501 Parado_NoLD y 385 Parado_LD fallecidos antes de 2025. VERIFICADO 2026-09-25: las 3.115 personas de las reglas 'no fallecido antes de 2025' fallecieron TODAS en 2024 (ninguna antes). Reglas ajustadas a 'antes de 2024' (&lt;= 202312): A-055, A-108, B-007, B-023, B-048, B-062, B-078, B-092 pasan a 0. C-270 (7): dato de origen. Edades altas: 1.276 personas con más de 100 años, de ellas 528 fallecidas cuya edad se calcula a la fecha de corte (no al fallecimiento): pendiente decidir si Edad_Actual_Fecha_Corte debe usar la fecha de fallecimiento.</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -1041,7 +1041,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Regla demasiado estricta / dato de origen</t>
+          <t>Regla mal planteada (corregida) + edades altas pendientes</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -5385,7 +5385,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Alta_ocupado ⇒ no fallecido antes de 2025</t>
+          <t>Alta_ocupado ⇒ no fallecido antes de 2024</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -5400,19 +5400,19 @@
       </c>
       <c r="I54" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J54" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Corregido</t>
         </is>
       </c>
       <c r="K54" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L54" s="2" t="n">
-        <v>0.0004</v>
+        <v>0</v>
       </c>
       <c r="M54" s="2" t="inlineStr">
         <is>
@@ -5422,12 +5422,12 @@
       <c r="N54" s="2" t="n"/>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>La guía admite retrasos al registrar fallecimientos, pero no al revés</t>
+          <t>Regla ajustada 2026-09-25 (G09, decisión del usuario): 'antes de 2024' (&lt;= 202312). En la edición 2024, quien murió durante 2024 aún cobraba prestación o pensión ese año; las 3.115 incumplidoras anteriores fallecieron todas en 2024.</t>
         </is>
       </c>
       <c r="P54" s="2" t="inlineStr">
         <is>
-          <t>situacion_actual_afiliacion = 'Alta_ocupado' AND fecha_fallecimiento BETWEEN 1 AND 202412</t>
+          <t>situacion_actual_afiliacion = 'Alta_ocupado' AND fecha_fallecimiento BETWEEN 1 AND 202312</t>
         </is>
       </c>
     </row>
@@ -8959,7 +8959,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>Asimilado_otros ⇒ no fallecido antes de 2025</t>
+          <t>Asimilado_otros ⇒ no fallecido antes de 2024</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -8974,19 +8974,19 @@
       </c>
       <c r="I107" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J107" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Corregido</t>
         </is>
       </c>
       <c r="K107" s="2" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="L107" s="2" t="n">
-        <v>0.0011</v>
+        <v>0</v>
       </c>
       <c r="M107" s="2" t="inlineStr">
         <is>
@@ -8994,10 +8994,14 @@
         </is>
       </c>
       <c r="N107" s="2" t="n"/>
-      <c r="O107" s="2" t="inlineStr"/>
+      <c r="O107" s="2" t="inlineStr">
+        <is>
+          <t>Regla ajustada 2026-09-25 (G09, decisión del usuario): 'antes de 2024' (&lt;= 202312). En la edición 2024, quien murió durante 2024 aún cobraba prestación o pensión ese año; las 3.115 incumplidoras anteriores fallecieron todas en 2024.</t>
+        </is>
+      </c>
       <c r="P107" s="2" t="inlineStr">
         <is>
-          <t>situacion_actual_afiliacion = 'Asimilado_otros' AND fecha_fallecimiento BETWEEN 1 AND 202412</t>
+          <t>situacion_actual_afiliacion = 'Asimilado_otros' AND fecha_fallecimiento BETWEEN 1 AND 202312</t>
         </is>
       </c>
     </row>
@@ -9635,7 +9639,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>Ocupado ⇒ no fallecido antes de 2025</t>
+          <t>Ocupado ⇒ no fallecido antes de 2024</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -9650,19 +9654,19 @@
       </c>
       <c r="I117" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J117" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Corregido</t>
         </is>
       </c>
       <c r="K117" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="L117" s="2" t="n">
-        <v>0.0003</v>
+        <v>0</v>
       </c>
       <c r="M117" s="2" t="inlineStr">
         <is>
@@ -9670,10 +9674,14 @@
         </is>
       </c>
       <c r="N117" s="2" t="n"/>
-      <c r="O117" s="2" t="inlineStr"/>
+      <c r="O117" s="2" t="inlineStr">
+        <is>
+          <t>Regla ajustada 2026-09-25 (G09, decisión del usuario): 'antes de 2024' (&lt;= 202312). En la edición 2024, quien murió durante 2024 aún cobraba prestación o pensión ese año; las 3.115 incumplidoras anteriores fallecieron todas en 2024.</t>
+        </is>
+      </c>
       <c r="P117" s="2" t="inlineStr">
         <is>
-          <t>situacion_paro_ocupacion = 'Ocupado' AND fecha_fallecimiento BETWEEN 1 AND 202412</t>
+          <t>situacion_paro_ocupacion = 'Ocupado' AND fecha_fallecimiento BETWEEN 1 AND 202312</t>
         </is>
       </c>
     </row>
@@ -10731,7 +10739,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>Ocupado_y_pensionista ⇒ no fallecido antes de 2025</t>
+          <t>Ocupado_y_pensionista ⇒ no fallecido antes de 2024</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -10746,19 +10754,19 @@
       </c>
       <c r="I133" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J133" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Corregido</t>
         </is>
       </c>
       <c r="K133" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L133" s="2" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
       <c r="M133" s="2" t="inlineStr">
         <is>
@@ -10766,10 +10774,14 @@
         </is>
       </c>
       <c r="N133" s="2" t="n"/>
-      <c r="O133" s="2" t="inlineStr"/>
+      <c r="O133" s="2" t="inlineStr">
+        <is>
+          <t>Regla ajustada 2026-09-25 (G09, decisión del usuario): 'antes de 2024' (&lt;= 202312). En la edición 2024, quien murió durante 2024 aún cobraba prestación o pensión ese año; las 3.115 incumplidoras anteriores fallecieron todas en 2024.</t>
+        </is>
+      </c>
       <c r="P133" s="2" t="inlineStr">
         <is>
-          <t>situacion_paro_ocupacion = 'Ocupado_y_pensionista' AND fecha_fallecimiento BETWEEN 1 AND 202412</t>
+          <t>situacion_paro_ocupacion = 'Ocupado_y_pensionista' AND fecha_fallecimiento BETWEEN 1 AND 202312</t>
         </is>
       </c>
     </row>
@@ -12445,7 +12457,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>Parado_LD ⇒ no fallecido antes de 2025</t>
+          <t>Parado_LD ⇒ no fallecido antes de 2024</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -12460,19 +12472,19 @@
       </c>
       <c r="I158" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J158" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Corregido</t>
         </is>
       </c>
       <c r="K158" s="2" t="n">
-        <v>387</v>
+        <v>0</v>
       </c>
       <c r="L158" s="2" t="n">
-        <v>0.0285</v>
+        <v>0</v>
       </c>
       <c r="M158" s="2" t="inlineStr">
         <is>
@@ -12480,10 +12492,14 @@
         </is>
       </c>
       <c r="N158" s="2" t="n"/>
-      <c r="O158" s="2" t="inlineStr"/>
+      <c r="O158" s="2" t="inlineStr">
+        <is>
+          <t>Regla ajustada 2026-09-25 (G09, decisión del usuario): 'antes de 2024' (&lt;= 202312). En la edición 2024, quien murió durante 2024 aún cobraba prestación o pensión ese año; las 3.115 incumplidoras anteriores fallecieron todas en 2024.</t>
+        </is>
+      </c>
       <c r="P158" s="2" t="inlineStr">
         <is>
-          <t>situacion_paro_ocupacion = 'Parado_LD' AND fecha_fallecimiento BETWEEN 1 AND 202412</t>
+          <t>situacion_paro_ocupacion = 'Parado_LD' AND fecha_fallecimiento BETWEEN 1 AND 202312</t>
         </is>
       </c>
     </row>
@@ -13413,7 +13429,7 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>Parado_LD_pension_no_jubilacion ⇒ no fallecido antes de 2025</t>
+          <t>Parado_LD_pension_no_jubilacion ⇒ no fallecido antes de 2024</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
@@ -13428,19 +13444,19 @@
       </c>
       <c r="I172" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J172" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Corregido</t>
         </is>
       </c>
       <c r="K172" s="2" t="n">
-        <v>2160</v>
+        <v>0</v>
       </c>
       <c r="L172" s="2" t="n">
-        <v>0.1589</v>
+        <v>0</v>
       </c>
       <c r="M172" s="2" t="inlineStr">
         <is>
@@ -13448,10 +13464,14 @@
         </is>
       </c>
       <c r="N172" s="2" t="n"/>
-      <c r="O172" s="2" t="inlineStr"/>
+      <c r="O172" s="2" t="inlineStr">
+        <is>
+          <t>Regla ajustada 2026-09-25 (G09, decisión del usuario): 'antes de 2024' (&lt;= 202312). En la edición 2024, quien murió durante 2024 aún cobraba prestación o pensión ese año; las 3.115 incumplidoras anteriores fallecieron todas en 2024.</t>
+        </is>
+      </c>
       <c r="P172" s="2" t="inlineStr">
         <is>
-          <t>situacion_paro_ocupacion = 'Parado_LD_pension_no_jubilacion' AND fecha_fallecimiento BETWEEN 1 AND 202412</t>
+          <t>situacion_paro_ocupacion = 'Parado_LD_pension_no_jubilacion' AND fecha_fallecimiento BETWEEN 1 AND 202312</t>
         </is>
       </c>
     </row>
@@ -14513,7 +14533,7 @@
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>Parado_NoLD ⇒ no fallecido antes de 2025</t>
+          <t>Parado_NoLD ⇒ no fallecido antes de 2024</t>
         </is>
       </c>
       <c r="G188" s="2" t="inlineStr">
@@ -14528,19 +14548,19 @@
       </c>
       <c r="I188" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J188" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Corregido</t>
         </is>
       </c>
       <c r="K188" s="2" t="n">
-        <v>499</v>
+        <v>0</v>
       </c>
       <c r="L188" s="2" t="n">
-        <v>0.0367</v>
+        <v>0</v>
       </c>
       <c r="M188" s="2" t="inlineStr">
         <is>
@@ -14548,10 +14568,14 @@
         </is>
       </c>
       <c r="N188" s="2" t="n"/>
-      <c r="O188" s="2" t="inlineStr"/>
+      <c r="O188" s="2" t="inlineStr">
+        <is>
+          <t>Regla ajustada 2026-09-25 (G09, decisión del usuario): 'antes de 2024' (&lt;= 202312). En la edición 2024, quien murió durante 2024 aún cobraba prestación o pensión ese año; las 3.115 incumplidoras anteriores fallecieron todas en 2024.</t>
+        </is>
+      </c>
       <c r="P188" s="2" t="inlineStr">
         <is>
-          <t>situacion_paro_ocupacion = 'Parado_NoLD' AND fecha_fallecimiento BETWEEN 1 AND 202412</t>
+          <t>situacion_paro_ocupacion = 'Parado_NoLD' AND fecha_fallecimiento BETWEEN 1 AND 202312</t>
         </is>
       </c>
     </row>
@@ -15477,7 +15501,7 @@
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>Parado_NoLD_pension_no_jubilacion ⇒ no fallecido antes de 2025</t>
+          <t>Parado_NoLD_pension_no_jubilacion ⇒ no fallecido antes de 2024</t>
         </is>
       </c>
       <c r="G202" s="2" t="inlineStr">
@@ -15492,19 +15516,19 @@
       </c>
       <c r="I202" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J202" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Corregido</t>
         </is>
       </c>
       <c r="K202" s="2" t="n">
-        <v>53</v>
+        <v>0</v>
       </c>
       <c r="L202" s="2" t="n">
-        <v>0.0039</v>
+        <v>0</v>
       </c>
       <c r="M202" s="2" t="inlineStr">
         <is>
@@ -15512,10 +15536,14 @@
         </is>
       </c>
       <c r="N202" s="2" t="n"/>
-      <c r="O202" s="2" t="inlineStr"/>
+      <c r="O202" s="2" t="inlineStr">
+        <is>
+          <t>Regla ajustada 2026-09-25 (G09, decisión del usuario): 'antes de 2024' (&lt;= 202312). En la edición 2024, quien murió durante 2024 aún cobraba prestación o pensión ese año; las 3.115 incumplidoras anteriores fallecieron todas en 2024.</t>
+        </is>
+      </c>
       <c r="P202" s="2" t="inlineStr">
         <is>
-          <t>situacion_paro_ocupacion = 'Parado_NoLD_pension_no_jubilacion' AND fecha_fallecimiento BETWEEN 1 AND 202412</t>
+          <t>situacion_paro_ocupacion = 'Parado_NoLD_pension_no_jubilacion' AND fecha_fallecimiento BETWEEN 1 AND 202312</t>
         </is>
       </c>
     </row>
@@ -33785,7 +33813,7 @@
       </c>
       <c r="J476" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K476" s="2" t="n">
@@ -33800,7 +33828,11 @@
         </is>
       </c>
       <c r="N476" s="2" t="n"/>
-      <c r="O476" s="2" t="inlineStr"/>
+      <c r="O476" s="2" t="inlineStr">
+        <is>
+          <t>Dato de origen (decisión del usuario 2026-09-25): baja por fallecimiento (causa 56) en Afiliación sin fecha de fallecimiento en Personas; la guía admite retrasos en registrarlo.</t>
+        </is>
+      </c>
       <c r="P476" s="2" t="inlineStr">
         <is>
           <t>causa_ult_baja LIKE '56 %' AND fecha_fallecimiento = 0</t>
@@ -38416,10 +38448,10 @@
         <v>109</v>
       </c>
       <c r="C2" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D2" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3">
@@ -38432,10 +38464,10 @@
         <v>112</v>
       </c>
       <c r="C3" t="n">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="D3" t="n">
-        <v>37</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4">
@@ -38464,12 +38496,13 @@
         <v>543</v>
       </c>
       <c r="C5" t="n">
-        <v>403</v>
+        <v>411</v>
       </c>
       <c r="D5" t="n">
-        <v>140</v>
-      </c>
-    </row>
+        <v>132</v>
+      </c>
+    </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
@@ -38518,10 +38551,10 @@
         <v>120</v>
       </c>
       <c r="C9" t="n">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="D9" t="n">
-        <v>66</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10">
@@ -38540,6 +38573,7 @@
         <v>34</v>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -38569,7 +38603,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>33</v>
+        <v>41</v>
       </c>
     </row>
     <row r="15">
@@ -38579,7 +38613,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>46</v>
+        <v>37</v>
       </c>
     </row>
     <row r="16">
@@ -38589,9 +38623,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>72</v>
-      </c>
-    </row>
+        <v>73</v>
+      </c>
+    </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
tests: reglas sobre los Parquet regenerados (edad de fallecidos, grupos fuera de 00-12, sin causas_baja_distintas)
C-268 335 -> 0 (G11 cerrado); B-108 1.177 -> 1.048, B-110 97 -> 83, C-071 80 -> 67 (fallecidos por edad al
fallecer); C-334 y C-102 reformuladas pasan. Efecto colateral: 14 fallecidos con episodio de empleo abierto
al morir tienen Edad_Ultimo_Empleo mayor que su edad al fallecer (C-039, B-015, C-108, C-113).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/reglas_consistencia_resultados_sin_ipf.xlsx
+++ b/tests/reglas_consistencia_resultados_sin_ipf.xlsx
@@ -739,7 +739,7 @@
         <v>26</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>1625</v>
+        <v>1626</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>0.1196</v>
@@ -1019,10 +1019,10 @@
         <v>8</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>1177</v>
+        <v>1048</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0.0866</v>
+        <v>0.0771</v>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
@@ -1031,7 +1031,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>4.319 Parado_LD_pension_no_jubilacion fallecidos antes de 2025 (B-062; pudieron cobrar pensión en 2024); 1.046 Pensionistas con más de 100 años (B-108); 501 Parado_NoLD y 385 Parado_LD fallecidos antes de 2025. VERIFICADO 2026-09-25: las 3.115 personas de las reglas 'no fallecido antes de 2025' fallecieron TODAS en 2024 (ninguna antes). Reglas ajustadas a 'antes de 2024' (&lt;= 202312): A-055, A-108, B-007, B-023, B-048, B-062, B-078, B-092 pasan a 0. C-270 (7): dato de origen. Edades altas: 1.276 personas con más de 100 años, de ellas 528 fallecidas cuya edad se calcula a la fecha de corte (no al fallecimiento): pendiente decidir si Edad_Actual_Fecha_Corte debe usar la fecha de fallecimiento.</t>
+          <t>4.319 Parado_LD_pension_no_jubilacion fallecidos antes de 2025 (B-062; pudieron cobrar pensión en 2024); 1.046 Pensionistas con más de 100 años (B-108); 501 Parado_NoLD y 385 Parado_LD fallecidos antes de 2025. VERIFICADO 2026-09-25: las 3.115 personas de las reglas 'no fallecido antes de 2025' fallecieron TODAS en 2024 (ninguna antes). Reglas ajustadas a 'antes de 2024' (&lt;= 202312): A-055, A-108, B-007, B-023, B-048, B-062, B-078, B-092 pasan a 0. C-270 (7): dato de origen. Edades altas: 1.276 personas con más de 100 años, de ellas 528 fallecidas cuya edad se calcula a la fecha de corte (no al fallecimiento): pendiente decidir si Edad_Actual_Fecha_Corte debe usar la fecha de fallecimiento. TRAS REGENERAR (2026-09-25): Edad_Actual_Fecha_Corte de los 18.801 fallecidos = edad_fallecimiento; los fallecidos de más de 100 años pasan de 528 a 385; B-108 1.177 -&gt; 1.048, B-110 97 -&gt; 83, C-071 80 -&gt; 67. Efecto colateral: 14 fallecidos con episodio de empleo aún abierto al morir tienen Edad_Ultimo_Empleo mayor que su edad al fallecer (C-039, B-015, C-108, C-113).</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -1115,26 +1115,26 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Tasas y recuentos (casi resuelto; falta regenerar para C-268)</t>
+          <t>Tasas y recuentos (resuelto)</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Corregido</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>335</v>
+        <v>1</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>0.0246</v>
+        <v>0.0001</v>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>C-264, C-268</t>
+          <t>C-264</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Regenerar tramos/Personas/Fase 3 con el ETL nuevo (claves fuera de 00-12 -&gt; 00 y sin causas_baja_distintas) y volver a pasar las reglas: C-268 debe bajar de 335 a 0 o casi. C-264 (1 persona) sin acción.</t>
+          <t>Regenerado 2026-09-25: C-268 pasa de 335 a 0 (claves de grupo fuera de 00-12 al 00). Queda C-264 (1 persona), sin acción.</t>
         </is>
       </c>
     </row>
@@ -1242,11 +1242,11 @@
         <v>24</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0.002</v>
+        <v>0.0018</v>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>B-058, B-057, B-087, B-044</t>
+          <t>B-044, B-057, B-058, B-087</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1295,10 +1295,10 @@
         <v>4</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>2948</v>
+        <v>2944</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>0.217</v>
+        <v>0.2166</v>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
@@ -10214,25 +10214,25 @@
       </c>
       <c r="I125" s="6" t="inlineStr">
         <is>
-          <t>PASA</t>
+          <t>INCUMPLE</t>
         </is>
       </c>
       <c r="J125" s="6" t="inlineStr">
         <is>
-          <t>Pasan</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="K125" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L125" s="2" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="M125" s="2" t="inlineStr"/>
       <c r="N125" s="2" t="n"/>
       <c r="O125" s="2" t="inlineStr">
         <is>
-          <t>edad_ultimo_empleo = edad al FINAL del último empleo (confirmado por el usuario)</t>
+          <t>edad_ultimo_empleo = edad al FINAL del último empleo (confirmado por el usuario) | Actualizado 2026-09-25 tras regenerar con: Edad_Actual_Fecha_Corte de fallecidos a su fecha de fallecimiento, claves de grupo fuera de 00-12 al 00 y sin causas_baja_distintas.</t>
         </is>
       </c>
       <c r="P125" s="2" t="inlineStr">
@@ -12555,10 +12555,10 @@
         </is>
       </c>
       <c r="K159" s="2" t="n">
-        <v>2948</v>
+        <v>2944</v>
       </c>
       <c r="L159" s="2" t="n">
-        <v>0.2169</v>
+        <v>0.2166</v>
       </c>
       <c r="M159" s="2" t="inlineStr">
         <is>
@@ -12568,7 +12568,7 @@
       <c r="N159" s="2" t="n"/>
       <c r="O159" s="2" t="inlineStr">
         <is>
-          <t>El tiempo actual sin empleo se cuenta desde que terminó el último empleo</t>
+          <t>El tiempo actual sin empleo se cuenta desde que terminó el último empleo | Actualizado 2026-09-25 tras regenerar con: Edad_Actual_Fecha_Corte de fallecidos a su fecha de fallecimiento, claves de grupo fuera de 00-12 al 00 y sin causas_baja_distintas.</t>
         </is>
       </c>
       <c r="P159" s="2" t="inlineStr">
@@ -13099,7 +13099,7 @@
         </is>
       </c>
       <c r="K167" s="2" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L167" s="2" t="n">
         <v>0.0015</v>
@@ -13112,7 +13112,7 @@
       <c r="N167" s="2" t="n"/>
       <c r="O167" s="2" t="inlineStr">
         <is>
-          <t>16 años (decisión del usuario); antes de 1980 la edad mínima legal era 14</t>
+          <t>16 años (decisión del usuario); antes de 1980 la edad mínima legal era 14 | Actualizado 2026-09-25 tras regenerar con: Edad_Actual_Fecha_Corte de fallecidos a su fecha de fallecimiento, claves de grupo fuera de 00-12 al 00 y sin causas_baja_distintas.</t>
         </is>
       </c>
       <c r="P167" s="2" t="inlineStr">
@@ -13527,10 +13527,10 @@
         </is>
       </c>
       <c r="K173" s="2" t="n">
-        <v>1405</v>
+        <v>1403</v>
       </c>
       <c r="L173" s="2" t="n">
-        <v>0.1034</v>
+        <v>0.1032</v>
       </c>
       <c r="M173" s="2" t="inlineStr">
         <is>
@@ -13540,7 +13540,7 @@
       <c r="N173" s="2" t="n"/>
       <c r="O173" s="2" t="inlineStr">
         <is>
-          <t>El tiempo actual sin empleo se cuenta desde que terminó el último empleo</t>
+          <t>El tiempo actual sin empleo se cuenta desde que terminó el último empleo | Actualizado 2026-09-25 tras regenerar con: Edad_Actual_Fecha_Corte de fallecidos a su fecha de fallecimiento, claves de grupo fuera de 00-12 al 00 y sin causas_baja_distintas.</t>
         </is>
       </c>
       <c r="P173" s="2" t="inlineStr">
@@ -16617,10 +16617,10 @@
         </is>
       </c>
       <c r="K218" s="2" t="n">
-        <v>1177</v>
+        <v>1048</v>
       </c>
       <c r="L218" s="2" t="n">
-        <v>0.0866</v>
+        <v>0.0771</v>
       </c>
       <c r="M218" s="2" t="inlineStr">
         <is>
@@ -16628,7 +16628,11 @@
         </is>
       </c>
       <c r="N218" s="2" t="n"/>
-      <c r="O218" s="2" t="inlineStr"/>
+      <c r="O218" s="2" t="inlineStr">
+        <is>
+          <t>Actualizado 2026-09-25 tras regenerar con: Edad_Actual_Fecha_Corte de fallecidos a su fecha de fallecimiento, claves de grupo fuera de 00-12 al 00 y sin causas_baja_distintas.</t>
+        </is>
+      </c>
       <c r="P218" s="2" t="inlineStr">
         <is>
           <t>situacion_paro_ocupacion = 'Pensionista' AND edad_actual_fecha_corte &gt; 100</t>
@@ -16757,10 +16761,10 @@
         </is>
       </c>
       <c r="K220" s="2" t="n">
-        <v>97</v>
+        <v>83</v>
       </c>
       <c r="L220" s="2" t="n">
-        <v>0.0071</v>
+        <v>0.0061</v>
       </c>
       <c r="M220" s="2" t="inlineStr">
         <is>
@@ -16768,7 +16772,11 @@
         </is>
       </c>
       <c r="N220" s="2" t="n"/>
-      <c r="O220" s="2" t="inlineStr"/>
+      <c r="O220" s="2" t="inlineStr">
+        <is>
+          <t>Actualizado 2026-09-25 tras regenerar con: Edad_Actual_Fecha_Corte de fallecidos a su fecha de fallecimiento, claves de grupo fuera de 00-12 al 00 y sin causas_baja_distintas.</t>
+        </is>
+      </c>
       <c r="P220" s="2" t="inlineStr">
         <is>
           <t>situacion_paro_ocupacion = 'Parado_LD_pension_no_jubilacion' AND edad_actual_fecha_corte &gt; 100</t>
@@ -19308,23 +19316,27 @@
       </c>
       <c r="I260" s="6" t="inlineStr">
         <is>
-          <t>PASA</t>
+          <t>INCUMPLE</t>
         </is>
       </c>
       <c r="J260" s="6" t="inlineStr">
         <is>
-          <t>Pasan</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="K260" s="2" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="L260" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="M260" s="2" t="inlineStr"/>
       <c r="N260" s="2" t="n"/>
-      <c r="O260" s="2" t="inlineStr"/>
+      <c r="O260" s="2" t="inlineStr">
+        <is>
+          <t>Actualizado 2026-09-25 tras regenerar con: Edad_Actual_Fecha_Corte de fallecidos a su fecha de fallecimiento, claves de grupo fuera de 00-12 al 00 y sin causas_baja_distintas.</t>
+        </is>
+      </c>
       <c r="P260" s="2" t="inlineStr">
         <is>
           <t>edad_ultimo_empleo &gt; edad_actual_fecha_corte + 0.05</t>
@@ -20679,10 +20691,10 @@
         </is>
       </c>
       <c r="K279" s="2" t="n">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="L279" s="2" t="n">
-        <v>0.0171</v>
+        <v>0.0173</v>
       </c>
       <c r="M279" s="2" t="inlineStr">
         <is>
@@ -20692,7 +20704,7 @@
       <c r="N279" s="2" t="n"/>
       <c r="O279" s="2" t="inlineStr">
         <is>
-          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte (14 hasta 1965, 16 después) y excepción de menores autorizados (régimen 0112 artistas y sectores de espectáculos, artes, publicidad, deporte y casting: art. 6.4 ET).</t>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte (14 hasta 1965, 16 después) y excepción de menores autorizados (régimen 0112 artistas y sectores de espectáculos, artes, publicidad, deporte y casting: art. 6.4 ET). | Actualizado 2026-09-25 tras regenerar con: Edad_Actual_Fecha_Corte de fallecidos a su fecha de fallecimiento, claves de grupo fuera de 00-12 al 00 y sin causas_baja_distintas.</t>
         </is>
       </c>
       <c r="P279" s="2" t="inlineStr">
@@ -21401,10 +21413,10 @@
         </is>
       </c>
       <c r="K290" s="2" t="n">
-        <v>80</v>
+        <v>67</v>
       </c>
       <c r="L290" s="2" t="n">
-        <v>0.0059</v>
+        <v>0.0049</v>
       </c>
       <c r="M290" s="2" t="inlineStr">
         <is>
@@ -21414,7 +21426,7 @@
       <c r="N290" s="2" t="n"/>
       <c r="O290" s="2" t="inlineStr">
         <is>
-          <t>Detección de outliers/errores</t>
+          <t>Detección de outliers/errores | Actualizado 2026-09-25 tras regenerar con: Edad_Actual_Fecha_Corte de fallecidos a su fecha de fallecimiento, claves de grupo fuera de 00-12 al 00 y sin causas_baja_distintas.</t>
         </is>
       </c>
       <c r="P290" s="2" t="inlineStr">
@@ -23055,7 +23067,7 @@
       </c>
       <c r="F315" s="2" t="inlineStr">
         <is>
-          <t>edad_actual = (1-5-2025 − nacimiento)/365,25 (±0,02)</t>
+          <t>Para no fallecidos: edad_actual = (1-5-2025 − nacimiento)/365,25 (±0,02)</t>
         </is>
       </c>
       <c r="G315" s="2" t="inlineStr">
@@ -23089,7 +23101,7 @@
       <c r="O315" s="2" t="inlineStr"/>
       <c r="P315" s="2" t="inlineStr">
         <is>
-          <t>ABS(edad_actual_fecha_corte - date_diff('day', fecha_nacimiento, DATE '2025-05-01') / 365.25) &gt; 0.02</t>
+          <t>ha_fallecido = 'NO' AND ABS(edad_actual_fecha_corte - date_diff('day', fecha_nacimiento, DATE '2025-05-01') / 365.25) &gt; 0.02</t>
         </is>
       </c>
     </row>
@@ -23417,10 +23429,10 @@
         </is>
       </c>
       <c r="K320" s="2" t="n">
-        <v>878</v>
+        <v>915</v>
       </c>
       <c r="L320" s="2" t="n">
-        <v>0.0646</v>
+        <v>0.0673</v>
       </c>
       <c r="M320" s="2" t="inlineStr">
         <is>
@@ -23430,7 +23442,7 @@
       <c r="N320" s="2" t="n"/>
       <c r="O320" s="2" t="inlineStr">
         <is>
-          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte (14 hasta 1965, 16 después) y excepción de menores autorizados (régimen 0112 artistas y sectores de espectáculos, artes, publicidad, deporte y casting: art. 6.4 ET).</t>
+          <t>Regla ajustada 2026-09-24 (G04, decisión del usuario): mínimo legal por cohorte (14 hasta 1965, 16 después) y excepción de menores autorizados (régimen 0112 artistas y sectores de espectáculos, artes, publicidad, deporte y casting: art. 6.4 ET). | Actualizado 2026-09-25 tras regenerar con: Edad_Actual_Fecha_Corte de fallecidos a su fecha de fallecimiento, claves de grupo fuera de 00-12 al 00 y sin causas_baja_distintas.</t>
         </is>
       </c>
       <c r="P320" s="2" t="inlineStr">
@@ -23482,23 +23494,27 @@
       </c>
       <c r="I321" s="6" t="inlineStr">
         <is>
-          <t>PASA</t>
+          <t>INCUMPLE</t>
         </is>
       </c>
       <c r="J321" s="6" t="inlineStr">
         <is>
-          <t>Pasan</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="K321" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L321" s="2" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="M321" s="2" t="inlineStr"/>
       <c r="N321" s="2" t="n"/>
-      <c r="O321" s="2" t="inlineStr"/>
+      <c r="O321" s="2" t="inlineStr">
+        <is>
+          <t>Actualizado 2026-09-25 tras regenerar con: Edad_Actual_Fecha_Corte de fallecidos a su fecha de fallecimiento, claves de grupo fuera de 00-12 al 00 y sin causas_baja_distintas.</t>
+        </is>
+      </c>
       <c r="P321" s="2" t="inlineStr">
         <is>
           <t>edad_primer_empleo_signif + duracion_1er_empleo_signif &gt; edad_actual_fecha_corte + 1</t>
@@ -23808,23 +23824,27 @@
       </c>
       <c r="I326" s="6" t="inlineStr">
         <is>
-          <t>PASA</t>
+          <t>INCUMPLE</t>
         </is>
       </c>
       <c r="J326" s="6" t="inlineStr">
         <is>
-          <t>Pasan</t>
+          <t>Pendiente</t>
         </is>
       </c>
       <c r="K326" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L326" s="2" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="M326" s="2" t="inlineStr"/>
       <c r="N326" s="2" t="n"/>
-      <c r="O326" s="2" t="inlineStr"/>
+      <c r="O326" s="2" t="inlineStr">
+        <is>
+          <t>Actualizado 2026-09-25 tras regenerar con: Edad_Actual_Fecha_Corte de fallecidos a su fecha de fallecimiento, claves de grupo fuera de 00-12 al 00 y sin causas_baja_distintas.</t>
+        </is>
+      </c>
       <c r="P326" s="2" t="inlineStr">
         <is>
           <t>situacion_actual_afiliacion = 'Alta_ocupado' AND ABS(edad_ultimo_empleo - edad_actual_fecha_corte) &gt; 1</t>
@@ -27259,7 +27279,7 @@
         </is>
       </c>
       <c r="K377" s="2" t="n">
-        <v>1625</v>
+        <v>1626</v>
       </c>
       <c r="L377" s="2" t="n">
         <v>0.1196</v>
@@ -27272,7 +27292,7 @@
       <c r="N377" s="2" t="n"/>
       <c r="O377" s="2" t="inlineStr">
         <is>
-          <t>Las pensiones de orfandad también constan como ingresos</t>
+          <t>Las pensiones de orfandad también constan como ingresos | Actualizado 2026-09-25 tras regenerar con: Edad_Actual_Fecha_Corte de fallecidos a su fecha de fallecimiento, claves de grupo fuera de 00-12 al 00 y sin causas_baja_distintas.</t>
         </is>
       </c>
       <c r="P377" s="2" t="inlineStr">
@@ -31615,10 +31635,10 @@
         </is>
       </c>
       <c r="K445" s="2" t="n">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="L445" s="2" t="n">
-        <v>0.0124</v>
+        <v>0.0119</v>
       </c>
       <c r="M445" s="2" t="inlineStr">
         <is>
@@ -31628,7 +31648,7 @@
       <c r="N445" s="2" t="n"/>
       <c r="O445" s="2" t="inlineStr">
         <is>
-          <t>Cifra actualizada 2026-09-24 (variacion de 1 persona por el cálculo no determinista).</t>
+          <t>Cifra actualizada 2026-09-24 (variacion de 1 persona por el cálculo no determinista). | Actualizado 2026-09-25 tras regenerar con: Edad_Actual_Fecha_Corte de fallecidos a su fecha de fallecimiento, claves de grupo fuera de 00-12 al 00 y sin causas_baja_distintas.</t>
         </is>
       </c>
       <c r="P445" s="2" t="inlineStr">
@@ -32117,10 +32137,10 @@
         </is>
       </c>
       <c r="K452" s="2" t="n">
-        <v>1391</v>
+        <v>1369</v>
       </c>
       <c r="L452" s="2" t="n">
-        <v>0.1024</v>
+        <v>0.1007</v>
       </c>
       <c r="M452" s="2" t="inlineStr">
         <is>
@@ -32128,7 +32148,11 @@
         </is>
       </c>
       <c r="N452" s="2" t="n"/>
-      <c r="O452" s="2" t="inlineStr"/>
+      <c r="O452" s="2" t="inlineStr">
+        <is>
+          <t>Actualizado 2026-09-25 tras regenerar con: Edad_Actual_Fecha_Corte de fallecidos a su fecha de fallecimiento, claves de grupo fuera de 00-12 al 00 y sin causas_baja_distintas.</t>
+        </is>
+      </c>
       <c r="P452" s="2" t="inlineStr">
         <is>
           <t>grupo_cotiz_ppal LIKE '11 %' AND t_tot_grupo_ppal &gt; 2.1</t>
@@ -32187,10 +32211,10 @@
         </is>
       </c>
       <c r="K453" s="2" t="n">
-        <v>694</v>
+        <v>673</v>
       </c>
       <c r="L453" s="2" t="n">
-        <v>0.0511</v>
+        <v>0.0495</v>
       </c>
       <c r="M453" s="2" t="inlineStr">
         <is>
@@ -32198,7 +32222,11 @@
         </is>
       </c>
       <c r="N453" s="2" t="n"/>
-      <c r="O453" s="2" t="inlineStr"/>
+      <c r="O453" s="2" t="inlineStr">
+        <is>
+          <t>Actualizado 2026-09-25 tras regenerar con: Edad_Actual_Fecha_Corte de fallecidos a su fecha de fallecimiento, claves de grupo fuera de 00-12 al 00 y sin causas_baja_distintas.</t>
+        </is>
+      </c>
       <c r="P453" s="2" t="inlineStr">
         <is>
           <t>grupo_cotiz_ppal LIKE '12 %' AND t_tot_grupo_ppal &gt; 1.1</t>
@@ -33664,19 +33692,19 @@
       </c>
       <c r="I474" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J474" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Corregido</t>
         </is>
       </c>
       <c r="K474" s="2" t="n">
-        <v>335</v>
+        <v>0</v>
       </c>
       <c r="L474" s="2" t="n">
-        <v>0.0246</v>
+        <v>0</v>
       </c>
       <c r="M474" s="2" t="inlineStr">
         <is>
@@ -33686,7 +33714,7 @@
       <c r="N474" s="2" t="n"/>
       <c r="O474" s="2" t="inlineStr">
         <is>
-          <t>ETL cambiado 2026-09-25 (decisión del usuario): cualquier clave de grupo de cotización fuera de 00-12 (13, 14, 19, 20, 21, 23, 31, 63) se asimila al 00 NO CONSTA en Grupo_cotiz_ppal/t_tot_grupo_ppal, como indica la guía (las 335 personas tenían sus años de empleo en los grupos 21/23 del R.E. Agrario Cuenta Propia). Probado sobre las 335: 335 -&gt; 0. Pendiente de regenerar los Parquet.</t>
+          <t>ETL cambiado 2026-09-25 (decisión del usuario): cualquier clave de grupo de cotización fuera de 00-12 (13, 14, 19, 20, 21, 23, 31, 63) se asimila al 00 NO CONSTA en Grupo_cotiz_ppal/t_tot_grupo_ppal, como indica la guía (las 335 personas tenían sus años de empleo en los grupos 21/23 del R.E. Agrario Cuenta Propia). Probado sobre las 335: 335 -&gt; 0. Pendiente de regenerar los Parquet. | Actualizado 2026-09-25 tras regenerar con: Edad_Actual_Fecha_Corte de fallecidos a su fecha de fallecimiento, claves de grupo fuera de 00-12 al 00 y sin causas_baja_distintas.</t>
         </is>
       </c>
       <c r="P474" s="2" t="inlineStr">
@@ -38081,7 +38109,7 @@
       </c>
       <c r="F540" s="2" t="inlineStr">
         <is>
-          <t>La edad al fallecer es anterior a la edad a fecha de corte</t>
+          <t>Fallecidos: edad_actual_fecha_corte = edad_fallecimiento (la edad se calcula a la fecha de fallecimiento)</t>
         </is>
       </c>
       <c r="G540" s="2" t="inlineStr">
@@ -38119,7 +38147,7 @@
       </c>
       <c r="P540" s="2" t="inlineStr">
         <is>
-          <t>ha_fallecido = 'SI' AND edad_fallecimiento &gt;= edad_actual_fecha_corte</t>
+          <t>ha_fallecido = 'SI' AND ABS(edad_actual_fecha_corte - edad_fallecimiento) &gt; 0.01</t>
         </is>
       </c>
     </row>
@@ -38464,10 +38492,10 @@
         <v>112</v>
       </c>
       <c r="C3" t="n">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D3" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4">
@@ -38480,10 +38508,10 @@
         <v>322</v>
       </c>
       <c r="C4" t="n">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="D4" t="n">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="5">
@@ -38496,10 +38524,10 @@
         <v>543</v>
       </c>
       <c r="C5" t="n">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="D5" t="n">
-        <v>132</v>
+        <v>135</v>
       </c>
     </row>
     <row r="6"/>
@@ -38535,10 +38563,10 @@
         <v>372</v>
       </c>
       <c r="C8" t="n">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="D8" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9">
@@ -38567,10 +38595,10 @@
         <v>51</v>
       </c>
       <c r="C10" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D10" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11"/>
@@ -38593,7 +38621,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>392</v>
+        <v>388</v>
       </c>
     </row>
     <row r="14">
@@ -38603,7 +38631,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="15">
@@ -38613,7 +38641,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
tests: reglas tras limitar el ultimo empleo de los fallecidos a su fallecimiento (411 de 543 pasan)
C-039 14 -> 0, B-015 y C-113 1 -> 0. Queda C-108 con 1 persona.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/reglas_consistencia_resultados_sin_ipf.xlsx
+++ b/tests/reglas_consistencia_resultados_sin_ipf.xlsx
@@ -1031,7 +1031,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>4.319 Parado_LD_pension_no_jubilacion fallecidos antes de 2025 (B-062; pudieron cobrar pensión en 2024); 1.046 Pensionistas con más de 100 años (B-108); 501 Parado_NoLD y 385 Parado_LD fallecidos antes de 2025. VERIFICADO 2026-09-25: las 3.115 personas de las reglas 'no fallecido antes de 2025' fallecieron TODAS en 2024 (ninguna antes). Reglas ajustadas a 'antes de 2024' (&lt;= 202312): A-055, A-108, B-007, B-023, B-048, B-062, B-078, B-092 pasan a 0. C-270 (7): dato de origen. Edades altas: 1.276 personas con más de 100 años, de ellas 528 fallecidas cuya edad se calcula a la fecha de corte (no al fallecimiento): pendiente decidir si Edad_Actual_Fecha_Corte debe usar la fecha de fallecimiento. TRAS REGENERAR (2026-09-25): Edad_Actual_Fecha_Corte de los 18.801 fallecidos = edad_fallecimiento; los fallecidos de más de 100 años pasan de 528 a 385; B-108 1.177 -&gt; 1.048, B-110 97 -&gt; 83, C-071 80 -&gt; 67. Efecto colateral: 14 fallecidos con episodio de empleo aún abierto al morir tienen Edad_Ultimo_Empleo mayor que su edad al fallecer (C-039, B-015, C-108, C-113).</t>
+          <t>4.319 Parado_LD_pension_no_jubilacion fallecidos antes de 2025 (B-062; pudieron cobrar pensión en 2024); 1.046 Pensionistas con más de 100 años (B-108); 501 Parado_NoLD y 385 Parado_LD fallecidos antes de 2025. VERIFICADO 2026-09-25: las 3.115 personas de las reglas 'no fallecido antes de 2025' fallecieron TODAS en 2024 (ninguna antes). Reglas ajustadas a 'antes de 2024' (&lt;= 202312): A-055, A-108, B-007, B-023, B-048, B-062, B-078, B-092 pasan a 0. C-270 (7): dato de origen. Edades altas: 1.276 personas con más de 100 años, de ellas 528 fallecidas cuya edad se calcula a la fecha de corte (no al fallecimiento): pendiente decidir si Edad_Actual_Fecha_Corte debe usar la fecha de fallecimiento. TRAS REGENERAR (2026-09-25): Edad_Actual_Fecha_Corte de los 18.801 fallecidos = edad_fallecimiento; los fallecidos de más de 100 años pasan de 528 a 385; B-108 1.177 -&gt; 1.048, B-110 97 -&gt; 83, C-071 80 -&gt; 67. Efecto colateral RESUELTO el mismo día: 14 fallecidos con episodio de empleo aún abierto al morir tenían Edad_Ultimo_Empleo mayor que su edad al fallecer; Fecha_final_Ultimo_Empleo se limita ahora a su fecha de fallecimiento (C-039 14 -&gt; 0, B-015 y C-113 1 -&gt; 0; queda C-108 con 1).</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -10214,25 +10214,25 @@
       </c>
       <c r="I125" s="6" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J125" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pasan</t>
         </is>
       </c>
       <c r="K125" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L125" s="2" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
       <c r="M125" s="2" t="inlineStr"/>
       <c r="N125" s="2" t="n"/>
       <c r="O125" s="2" t="inlineStr">
         <is>
-          <t>edad_ultimo_empleo = edad al FINAL del último empleo (confirmado por el usuario) | Actualizado 2026-09-25 tras regenerar con: Edad_Actual_Fecha_Corte de fallecidos a su fecha de fallecimiento, claves de grupo fuera de 00-12 al 00 y sin causas_baja_distintas.</t>
+          <t>edad_ultimo_empleo = edad al FINAL del último empleo (confirmado por el usuario) | Actualizado 2026-09-25 tras regenerar con: Edad_Actual_Fecha_Corte de fallecidos a su fecha de fallecimiento, claves de grupo fuera de 00-12 al 00 y sin causas_baja_distintas. | Actualizado 2026-09-25: Fecha_final_Ultimo_Empleo de los fallecidos limitada a su fecha de fallecimiento (Edad_Ultimo_Empleo cambia en 14 personas).</t>
         </is>
       </c>
       <c r="P125" s="2" t="inlineStr">
@@ -19316,25 +19316,25 @@
       </c>
       <c r="I260" s="6" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J260" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pasan</t>
         </is>
       </c>
       <c r="K260" s="2" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="L260" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="M260" s="2" t="inlineStr"/>
       <c r="N260" s="2" t="n"/>
       <c r="O260" s="2" t="inlineStr">
         <is>
-          <t>Actualizado 2026-09-25 tras regenerar con: Edad_Actual_Fecha_Corte de fallecidos a su fecha de fallecimiento, claves de grupo fuera de 00-12 al 00 y sin causas_baja_distintas.</t>
+          <t>Actualizado 2026-09-25 tras regenerar con: Edad_Actual_Fecha_Corte de fallecidos a su fecha de fallecimiento, claves de grupo fuera de 00-12 al 00 y sin causas_baja_distintas. | Actualizado 2026-09-25: Fecha_final_Ultimo_Empleo de los fallecidos limitada a su fecha de fallecimiento (Edad_Ultimo_Empleo cambia en 14 personas).</t>
         </is>
       </c>
       <c r="P260" s="2" t="inlineStr">
@@ -23824,25 +23824,25 @@
       </c>
       <c r="I326" s="6" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J326" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Pasan</t>
         </is>
       </c>
       <c r="K326" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L326" s="2" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
       <c r="M326" s="2" t="inlineStr"/>
       <c r="N326" s="2" t="n"/>
       <c r="O326" s="2" t="inlineStr">
         <is>
-          <t>Actualizado 2026-09-25 tras regenerar con: Edad_Actual_Fecha_Corte de fallecidos a su fecha de fallecimiento, claves de grupo fuera de 00-12 al 00 y sin causas_baja_distintas.</t>
+          <t>Actualizado 2026-09-25 tras regenerar con: Edad_Actual_Fecha_Corte de fallecidos a su fecha de fallecimiento, claves de grupo fuera de 00-12 al 00 y sin causas_baja_distintas. | Actualizado 2026-09-25: Fecha_final_Ultimo_Empleo de los fallecidos limitada a su fecha de fallecimiento (Edad_Ultimo_Empleo cambia en 14 personas).</t>
         </is>
       </c>
       <c r="P326" s="2" t="inlineStr">
@@ -38492,10 +38492,10 @@
         <v>112</v>
       </c>
       <c r="C3" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D3" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4">
@@ -38508,10 +38508,10 @@
         <v>322</v>
       </c>
       <c r="C4" t="n">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="D4" t="n">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5">
@@ -38524,10 +38524,10 @@
         <v>543</v>
       </c>
       <c r="C5" t="n">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="D5" t="n">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6"/>
@@ -38563,10 +38563,10 @@
         <v>372</v>
       </c>
       <c r="C8" t="n">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="D8" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9">
@@ -38621,7 +38621,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>388</v>
+        <v>391</v>
       </c>
     </row>
     <row r="14">
@@ -38641,7 +38641,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
reglas: G17 - quita C-312 y los umbrales C-299/C-300/C-301; C-302 y C-306 excluyen menores autorizados
C-312 (premisa incorrecta: la clave B incluye bajas por enfermedad) y los tres umbrales de valores extremos se quitan. C-302 262 -> 13 y C-306 11 -> 5 con la excepcion de menores autorizados. Variable renombrada en las reglas restantes. G17 queda como baja calidad de los datos. Quedan 539 reglas.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/reglas_consistencia_resultados_sin_ipf.xlsx
+++ b/tests/reglas_consistencia_resultados_sin_ipf.xlsx
@@ -1452,11 +1452,11 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="D18" s="2" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>61583</v>
@@ -1466,12 +1466,12 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>C-299, C-300, C-301, C-302, C-306, C-309, C-310, C-311, C-312, C-313, C-338</t>
+          <t>C-302, C-306, C-309, C-310, C-311, C-313, C-338</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>De las 54 reglas nuevas, la mayoria pasan (identidades de ingresos por tipo, clave_subclave, fallecimiento y domicilio). Siguen sin decidir: 61.392 con provincia de residencia distinta de la fiscal (C-338/339, confianza baja), 48.782 con pensión en fiscal sin pensión en la tabla de pensiones (C-312/313), 3.876 con sueldo en 2024 y última baja anterior a 2024 (C-311).</t>
+          <t>De las 54 reglas nuevas, la mayoria pasan (identidades de ingresos por tipo, clave_subclave, fallecimiento y domicilio). Siguen sin decidir: 61.392 con provincia de residencia distinta de la fiscal (C-338/339, confianza baja), 48.782 con pensión en fiscal sin pensión en la tabla de pensiones (C-312/313), 3.876 con sueldo en 2024 y última baja anterior a 2024 (C-311). CERRADO 2026-09-25 (decisión del usuario). C-312 (48.780) se QUITA: la clave B del modelo 190 incluye, además de pensiones y haberes pasivos, las bajas por incapacidad temporal pagadas por la Seguridad Social o la mutua (B01) y las prestaciones de mutualidades de funcionarios (B03); solo 1.809 de las 48.780 tienen 65 años o más. La variable ingresos_pension_2024 se RENOMBRA a ingresos_pension_y_bajas_2024. Los umbrales C-299, C-300 y C-301 (retenciones y sueldos/actividad extremos) se quitan por ser casos reales. C-302 y C-306 excluyen a los menores autorizados (262 -&gt; 13, 11 -&gt; 5). C-311 (sueldo mediano 328 €, 2.926 en Baja_para_pension), C-309, C-310, C-313 y C-338 (mudanzas y domicilios fiscales antiguos): dato de origen.</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>A investigar / reglas de confianza baja</t>
+          <t>Dato de origen / reglas de confianza baja</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>Las 278 personas con importe fiscal 0 (C-317/320/321) SI se corrigieron: clave_subclave_ppal pasa a NO CONSTA en vez de un tipo arbitrario (decision del usuario, 2026-09-22). El resto de este grupo sigue sin decidir.</t>
+          <t>Ninguna acción sobre el ETL más allá del renombrado. Renombrado en el ETL y la app (compatible con un Parquet antiguo); el Parquet actual lo lleva con el nombre antiguo hasta regenerar el Grupo H.</t>
         </is>
       </c>
     </row>
@@ -1782,7 +1782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P544"/>
+  <dimension ref="A1:P540"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4397,7 +4397,7 @@
       </c>
       <c r="P39" s="2" t="inlineStr">
         <is>
-          <t>situacion_actual_afiliacion &lt;&gt; 'Nunca_ha_cotizado' AND fecha_ini_primer_empleo IS NULL</t>
+          <t>situacion_actual_afiliacion &lt;&gt; 'Nunca_ha_cotizado' AND fecha_ini_primer_empleo IS NULL AND ipf NOT IN (SELECT ipf FROM solo_prestaciones)</t>
         </is>
       </c>
     </row>
@@ -4603,7 +4603,7 @@
       </c>
       <c r="P42" s="2" t="inlineStr">
         <is>
-          <t>situacion_actual_afiliacion &lt;&gt; 'Nunca_ha_cotizado' AND t_total_empleo IS NULL</t>
+          <t>situacion_actual_afiliacion &lt;&gt; 'Nunca_ha_cotizado' AND t_total_empleo IS NULL AND ipf NOT IN (SELECT ipf FROM solo_prestaciones)</t>
         </is>
       </c>
     </row>
@@ -4677,7 +4677,7 @@
       </c>
       <c r="P43" s="2" t="inlineStr">
         <is>
-          <t>situacion_actual_afiliacion &lt;&gt; 'Nunca_ha_cotizado' AND num_altas_anual_promedio IS NULL</t>
+          <t>situacion_actual_afiliacion &lt;&gt; 'Nunca_ha_cotizado' AND num_altas_anual_promedio IS NULL AND ipf NOT IN (SELECT ipf FROM solo_prestaciones)</t>
         </is>
       </c>
     </row>
@@ -4813,7 +4813,7 @@
       </c>
       <c r="P45" s="2" t="inlineStr">
         <is>
-          <t>situacion_actual_afiliacion &lt;&gt; 'Nunca_ha_cotizado' AND edad_ultimo_empleo IS NULL</t>
+          <t>situacion_actual_afiliacion &lt;&gt; 'Nunca_ha_cotizado' AND edad_ultimo_empleo IS NULL AND ipf NOT IN (SELECT ipf FROM solo_prestaciones)</t>
         </is>
       </c>
     </row>
@@ -12425,7 +12425,7 @@
       </c>
       <c r="P157" s="2" t="inlineStr">
         <is>
-          <t>situacion_paro_ocupacion = 'Parado_LD' AND fecha_ini_primer_empleo IS NULL</t>
+          <t>situacion_paro_ocupacion = 'Parado_LD' AND fecha_ini_primer_empleo IS NULL AND ipf NOT IN (SELECT ipf FROM solo_prestaciones)</t>
         </is>
       </c>
     </row>
@@ -14501,7 +14501,7 @@
       </c>
       <c r="P187" s="2" t="inlineStr">
         <is>
-          <t>situacion_paro_ocupacion = 'Parado_NoLD' AND fecha_ini_primer_empleo IS NULL</t>
+          <t>situacion_paro_ocupacion = 'Parado_NoLD' AND fecha_ini_primer_empleo IS NULL AND ipf NOT IN (SELECT ipf FROM solo_prestaciones)</t>
         </is>
       </c>
     </row>
@@ -16936,7 +16936,7 @@
           <t>t_tot_reg_ppal</t>
         </is>
       </c>
-      <c r="E223" s="2" t="inlineStr"/>
+      <c r="E223" s="2" t="n"/>
       <c r="F223" s="2" t="inlineStr">
         <is>
           <t>t_tot_reg_ppal no puede ser negativa</t>
@@ -16998,7 +16998,7 @@
           <t>t_tot_grupo_ppal</t>
         </is>
       </c>
-      <c r="E224" s="2" t="inlineStr"/>
+      <c r="E224" s="2" t="n"/>
       <c r="F224" s="2" t="inlineStr">
         <is>
           <t>t_tot_grupo_ppal no puede ser negativa</t>
@@ -17060,7 +17060,7 @@
           <t>t_contrato_mas_largo</t>
         </is>
       </c>
-      <c r="E225" s="2" t="inlineStr"/>
+      <c r="E225" s="2" t="n"/>
       <c r="F225" s="2" t="inlineStr">
         <is>
           <t>t_contrato_mas_largo no puede ser negativa</t>
@@ -17122,7 +17122,7 @@
           <t>t_tot_tipo_contrato_ppal</t>
         </is>
       </c>
-      <c r="E226" s="2" t="inlineStr"/>
+      <c r="E226" s="2" t="n"/>
       <c r="F226" s="2" t="inlineStr">
         <is>
           <t>t_tot_tipo_contrato_ppal no puede ser negativa</t>
@@ -17184,7 +17184,7 @@
           <t>duracion_1er_empleo_signif</t>
         </is>
       </c>
-      <c r="E227" s="2" t="inlineStr"/>
+      <c r="E227" s="2" t="n"/>
       <c r="F227" s="2" t="inlineStr">
         <is>
           <t>duracion_1er_empleo_signif no puede ser negativa</t>
@@ -17246,7 +17246,7 @@
           <t>duracion_promedio_empleo</t>
         </is>
       </c>
-      <c r="E228" s="2" t="inlineStr"/>
+      <c r="E228" s="2" t="n"/>
       <c r="F228" s="2" t="inlineStr">
         <is>
           <t>duracion_promedio_empleo no puede ser negativa</t>
@@ -17308,7 +17308,7 @@
           <t>t_total_empleo</t>
         </is>
       </c>
-      <c r="E229" s="2" t="inlineStr"/>
+      <c r="E229" s="2" t="n"/>
       <c r="F229" s="2" t="inlineStr">
         <is>
           <t>t_total_empleo no puede ser negativa</t>
@@ -17370,7 +17370,7 @@
           <t>t_total_desempleo</t>
         </is>
       </c>
-      <c r="E230" s="2" t="inlineStr"/>
+      <c r="E230" s="2" t="n"/>
       <c r="F230" s="2" t="inlineStr">
         <is>
           <t>t_total_desempleo no puede ser negativa</t>
@@ -17432,7 +17432,7 @@
           <t>t_total_mixto_empl_desempl</t>
         </is>
       </c>
-      <c r="E231" s="2" t="inlineStr"/>
+      <c r="E231" s="2" t="n"/>
       <c r="F231" s="2" t="inlineStr">
         <is>
           <t>t_total_mixto_empl_desempl no puede ser negativa</t>
@@ -17494,7 +17494,7 @@
           <t>t_total_no_empleo</t>
         </is>
       </c>
-      <c r="E232" s="2" t="inlineStr"/>
+      <c r="E232" s="2" t="n"/>
       <c r="F232" s="2" t="inlineStr">
         <is>
           <t>t_total_no_empleo no puede ser negativa</t>
@@ -17556,7 +17556,7 @@
           <t>t_tot_prov_ppal</t>
         </is>
       </c>
-      <c r="E233" s="2" t="inlineStr"/>
+      <c r="E233" s="2" t="n"/>
       <c r="F233" s="2" t="inlineStr">
         <is>
           <t>t_tot_prov_ppal no puede ser negativa</t>
@@ -17618,7 +17618,7 @@
           <t>t_tot_act_econ_ppal</t>
         </is>
       </c>
-      <c r="E234" s="2" t="inlineStr"/>
+      <c r="E234" s="2" t="n"/>
       <c r="F234" s="2" t="inlineStr">
         <is>
           <t>t_tot_act_econ_ppal no puede ser negativa</t>
@@ -17680,7 +17680,7 @@
           <t>ingresos_bruto_total_2024</t>
         </is>
       </c>
-      <c r="E235" s="2" t="inlineStr"/>
+      <c r="E235" s="2" t="n"/>
       <c r="F235" s="2" t="inlineStr">
         <is>
           <t>ingresos_bruto_total_2024 no puede ser negativa</t>
@@ -17742,7 +17742,7 @@
           <t>edad_ultimo_empleo</t>
         </is>
       </c>
-      <c r="E236" s="2" t="inlineStr"/>
+      <c r="E236" s="2" t="n"/>
       <c r="F236" s="2" t="inlineStr">
         <is>
           <t>edad_ultimo_empleo no puede ser negativa</t>
@@ -17804,7 +17804,7 @@
           <t>tiempo_total_desde_inicio_vl</t>
         </is>
       </c>
-      <c r="E237" s="2" t="inlineStr"/>
+      <c r="E237" s="2" t="n"/>
       <c r="F237" s="2" t="inlineStr">
         <is>
           <t>tiempo_total_desde_inicio_vl no puede ser negativa</t>
@@ -17866,7 +17866,7 @@
           <t>edad_actual_fecha_corte</t>
         </is>
       </c>
-      <c r="E238" s="2" t="inlineStr"/>
+      <c r="E238" s="2" t="n"/>
       <c r="F238" s="2" t="inlineStr">
         <is>
           <t>edad_actual_fecha_corte no puede ser negativa</t>
@@ -17928,7 +17928,7 @@
           <t>edad_primer_empleo_signif</t>
         </is>
       </c>
-      <c r="E239" s="2" t="inlineStr"/>
+      <c r="E239" s="2" t="n"/>
       <c r="F239" s="2" t="inlineStr">
         <is>
           <t>edad_primer_empleo_signif no puede ser negativa</t>
@@ -17990,7 +17990,7 @@
           <t>num_altas_anual_promedio</t>
         </is>
       </c>
-      <c r="E240" s="2" t="inlineStr"/>
+      <c r="E240" s="2" t="n"/>
       <c r="F240" s="2" t="inlineStr">
         <is>
           <t>num_altas_anual_promedio no puede ser negativa</t>
@@ -18052,7 +18052,7 @@
           <t>num_bajas_anual_promedio</t>
         </is>
       </c>
-      <c r="E241" s="2" t="inlineStr"/>
+      <c r="E241" s="2" t="n"/>
       <c r="F241" s="2" t="inlineStr">
         <is>
           <t>num_bajas_anual_promedio no puede ser negativa</t>
@@ -18114,7 +18114,7 @@
           <t>cotizado_anual_promedio</t>
         </is>
       </c>
-      <c r="E242" s="2" t="inlineStr"/>
+      <c r="E242" s="2" t="n"/>
       <c r="F242" s="2" t="inlineStr">
         <is>
           <t>cotizado_anual_promedio no puede ser negativa</t>
@@ -18180,7 +18180,7 @@
           <t>duracion_actual_sin_empleo</t>
         </is>
       </c>
-      <c r="E243" s="2" t="inlineStr"/>
+      <c r="E243" s="2" t="n"/>
       <c r="F243" s="2" t="inlineStr">
         <is>
           <t>duracion_actual_sin_empleo no puede ser negativa</t>
@@ -18242,7 +18242,7 @@
           <t>pct_t_total_empleo</t>
         </is>
       </c>
-      <c r="E244" s="2" t="inlineStr"/>
+      <c r="E244" s="2" t="n"/>
       <c r="F244" s="2" t="inlineStr">
         <is>
           <t>pct_t_total_empleo no puede ser negativa</t>
@@ -18304,7 +18304,7 @@
           <t>pct_t_total_desempleo</t>
         </is>
       </c>
-      <c r="E245" s="2" t="inlineStr"/>
+      <c r="E245" s="2" t="n"/>
       <c r="F245" s="2" t="inlineStr">
         <is>
           <t>pct_t_total_desempleo no puede ser negativa</t>
@@ -18366,7 +18366,7 @@
           <t>pct_t_total_mixto_empl_desempl</t>
         </is>
       </c>
-      <c r="E246" s="2" t="inlineStr"/>
+      <c r="E246" s="2" t="n"/>
       <c r="F246" s="2" t="inlineStr">
         <is>
           <t>pct_t_total_mixto_empl_desempl no puede ser negativa</t>
@@ -18428,7 +18428,7 @@
           <t>pct_t_total_no_empleo</t>
         </is>
       </c>
-      <c r="E247" s="2" t="inlineStr"/>
+      <c r="E247" s="2" t="n"/>
       <c r="F247" s="2" t="inlineStr">
         <is>
           <t>pct_t_total_no_empleo no puede ser negativa</t>
@@ -20866,7 +20866,7 @@
           <t>pct_t_total_empleo</t>
         </is>
       </c>
-      <c r="E282" s="2" t="inlineStr"/>
+      <c r="E282" s="2" t="n"/>
       <c r="F282" s="2" t="inlineStr">
         <is>
           <t>pct_t_total_empleo está entre 0 y 100</t>
@@ -20998,7 +20998,7 @@
           <t>pct_t_total_desempleo</t>
         </is>
       </c>
-      <c r="E284" s="2" t="inlineStr"/>
+      <c r="E284" s="2" t="n"/>
       <c r="F284" s="2" t="inlineStr">
         <is>
           <t>pct_t_total_desempleo está entre 0 y 100</t>
@@ -21126,7 +21126,7 @@
           <t>pct_t_total_mixto_empl_desempl</t>
         </is>
       </c>
-      <c r="E286" s="2" t="inlineStr"/>
+      <c r="E286" s="2" t="n"/>
       <c r="F286" s="2" t="inlineStr">
         <is>
           <t>pct_t_total_mixto_empl_desempl está entre 0 y 100</t>
@@ -21254,7 +21254,7 @@
           <t>pct_t_total_no_empleo</t>
         </is>
       </c>
-      <c r="E288" s="2" t="inlineStr"/>
+      <c r="E288" s="2" t="n"/>
       <c r="F288" s="2" t="inlineStr">
         <is>
           <t>pct_t_total_no_empleo está entre 0 y 100</t>
@@ -21386,7 +21386,7 @@
           <t>edad_actual_fecha_corte</t>
         </is>
       </c>
-      <c r="E290" s="2" t="inlineStr"/>
+      <c r="E290" s="2" t="n"/>
       <c r="F290" s="2" t="inlineStr">
         <is>
           <t>edad_actual_fecha_corte no debería superar 105</t>
@@ -21645,7 +21645,7 @@
       </c>
       <c r="P293" s="2" t="inlineStr">
         <is>
-          <t>fecha_ultima_baja &lt; fecha_ini_primer_empleo</t>
+          <t>fecha_ultima_baja &lt; fecha_ini_primer_empleo AND ipf NOT IN (SELECT ipf FROM solo_prestaciones)</t>
         </is>
       </c>
     </row>
@@ -21670,7 +21670,7 @@
           <t>fecha_ini_primer_empleo</t>
         </is>
       </c>
-      <c r="E294" s="2" t="inlineStr"/>
+      <c r="E294" s="2" t="n"/>
       <c r="F294" s="2" t="inlineStr">
         <is>
           <t>Primer empleo no posterior al 31-12-2024 (última alta real de la MCVL)</t>
@@ -21732,7 +21732,7 @@
           <t>fecha_ultima_baja</t>
         </is>
       </c>
-      <c r="E295" s="2" t="inlineStr"/>
+      <c r="E295" s="2" t="n"/>
       <c r="F295" s="2" t="inlineStr">
         <is>
           <t>Última baja no posterior al 30-04-2025 (última baja real; 2099 = vigente)</t>
@@ -21868,7 +21868,7 @@
           <t>fecha_inicio_ultima_racha_sin_empleo</t>
         </is>
       </c>
-      <c r="E297" s="2" t="inlineStr"/>
+      <c r="E297" s="2" t="n"/>
       <c r="F297" s="2" t="inlineStr">
         <is>
           <t>Inicio de la última racha sin empleo no posterior al 31-12-2024 (última alta real)</t>
@@ -22214,7 +22214,7 @@
           <t>fecha_fallecimiento</t>
         </is>
       </c>
-      <c r="E302" s="2" t="inlineStr"/>
+      <c r="E302" s="2" t="n"/>
       <c r="F302" s="2" t="inlineStr">
         <is>
           <t>fecha_fallecimiento tiene formato aaaamm con mes 1-12 (guía 1.008)</t>
@@ -22276,7 +22276,7 @@
           <t>fecha_fallecimiento</t>
         </is>
       </c>
-      <c r="E303" s="2" t="inlineStr"/>
+      <c r="E303" s="2" t="n"/>
       <c r="F303" s="2" t="inlineStr">
         <is>
           <t>fecha_fallecimiento no es posterior a abril de 2025 (último fallecimiento registrado)</t>
@@ -22470,7 +22470,7 @@
           <t>fecha_nacimiento</t>
         </is>
       </c>
-      <c r="E306" s="2" t="inlineStr"/>
+      <c r="E306" s="2" t="n"/>
       <c r="F306" s="2" t="inlineStr">
         <is>
           <t>Nacimiento no posterior al corte</t>
@@ -22532,7 +22532,7 @@
           <t>fecha_nacimiento</t>
         </is>
       </c>
-      <c r="E307" s="2" t="inlineStr"/>
+      <c r="E307" s="2" t="n"/>
       <c r="F307" s="2" t="inlineStr">
         <is>
           <t>Nacimiento no anterior a 1900</t>
@@ -22594,7 +22594,7 @@
           <t>fecha_ini_primer_empleo</t>
         </is>
       </c>
-      <c r="E308" s="2" t="inlineStr"/>
+      <c r="E308" s="2" t="n"/>
       <c r="F308" s="2" t="inlineStr">
         <is>
           <t>Primer empleo no anterior a 1967 (la guía dice que hay datos desde 1967)</t>
@@ -22660,7 +22660,7 @@
           <t>fecha_ultima_baja</t>
         </is>
       </c>
-      <c r="E309" s="2" t="inlineStr"/>
+      <c r="E309" s="2" t="n"/>
       <c r="F309" s="2" t="inlineStr">
         <is>
           <t>Última baja no anterior a 1967 (datos desde 1967, guía 2.008)</t>
@@ -22726,7 +22726,7 @@
           <t>fecha_inicio_ultima_racha_sin_empleo</t>
         </is>
       </c>
-      <c r="E310" s="2" t="inlineStr"/>
+      <c r="E310" s="2" t="n"/>
       <c r="F310" s="2" t="inlineStr">
         <is>
           <t>Inicio de racha no anterior a 1967</t>
@@ -23258,7 +23258,7 @@
           <t>edad_primer_empleo_signif</t>
         </is>
       </c>
-      <c r="E318" s="2" t="inlineStr"/>
+      <c r="E318" s="2" t="n"/>
       <c r="F318" s="2" t="inlineStr">
         <is>
           <t>Primer empleo significativo a la edad mínima legal o más (14 hasta la cohorte 1965, 16 después)</t>
@@ -23328,7 +23328,7 @@
           <t>edad_ultimo_empleo</t>
         </is>
       </c>
-      <c r="E319" s="2" t="inlineStr"/>
+      <c r="E319" s="2" t="n"/>
       <c r="F319" s="2" t="inlineStr">
         <is>
           <t>Edad al final del último empleo ≥ mínimo legal (14 hasta la cohorte 1965, 16 después)</t>
@@ -24857,7 +24857,7 @@
       </c>
       <c r="P341" s="2" t="inlineStr">
         <is>
-          <t>fecha_ini_primer_empleo IS NULL AND tiempo_total_desde_inicio_vl IS NOT NULL</t>
+          <t>fecha_ini_primer_empleo IS NULL AND tiempo_total_desde_inicio_vl IS NOT NULL AND ipf NOT IN (SELECT ipf FROM solo_prestaciones)</t>
         </is>
       </c>
     </row>
@@ -24997,7 +24997,7 @@
       </c>
       <c r="P343" s="2" t="inlineStr">
         <is>
-          <t>t_total_empleo IS NULL AND tiempo_total_desde_inicio_vl IS NOT NULL</t>
+          <t>t_total_empleo IS NULL AND tiempo_total_desde_inicio_vl IS NOT NULL AND ipf NOT IN (SELECT ipf FROM solo_prestaciones)</t>
         </is>
       </c>
     </row>
@@ -25137,7 +25137,7 @@
       </c>
       <c r="P345" s="2" t="inlineStr">
         <is>
-          <t>num_altas_anual_promedio IS NULL AND tiempo_total_desde_inicio_vl IS NOT NULL</t>
+          <t>num_altas_anual_promedio IS NULL AND tiempo_total_desde_inicio_vl IS NOT NULL AND ipf NOT IN (SELECT ipf FROM solo_prestaciones)</t>
         </is>
       </c>
     </row>
@@ -25405,7 +25405,7 @@
       </c>
       <c r="P349" s="2" t="inlineStr">
         <is>
-          <t>edad_ultimo_empleo IS NULL AND tiempo_total_desde_inicio_vl IS NOT NULL</t>
+          <t>edad_ultimo_empleo IS NULL AND tiempo_total_desde_inicio_vl IS NOT NULL AND ipf NOT IN (SELECT ipf FROM solo_prestaciones)</t>
         </is>
       </c>
     </row>
@@ -25545,7 +25545,7 @@
       </c>
       <c r="P351" s="2" t="inlineStr">
         <is>
-          <t>t_total_desempleo IS NULL AND tiempo_total_desde_inicio_vl IS NOT NULL</t>
+          <t>t_total_desempleo IS NULL AND tiempo_total_desde_inicio_vl IS NOT NULL AND ipf NOT IN (SELECT ipf FROM solo_prestaciones)</t>
         </is>
       </c>
     </row>
@@ -26732,7 +26732,7 @@
           <t>pension_actual</t>
         </is>
       </c>
-      <c r="E369" s="2" t="inlineStr"/>
+      <c r="E369" s="2" t="n"/>
       <c r="F369" s="2" t="inlineStr">
         <is>
           <t>pension_actual solo contiene los 6 tipos conocidos</t>
@@ -26794,7 +26794,7 @@
           <t>pension_todas_cobradas</t>
         </is>
       </c>
-      <c r="E370" s="2" t="inlineStr"/>
+      <c r="E370" s="2" t="n"/>
       <c r="F370" s="2" t="inlineStr">
         <is>
           <t>pension_todas_cobradas solo contiene los 6 tipos conocidos</t>
@@ -26856,7 +26856,7 @@
           <t>pension_todas_cobradas</t>
         </is>
       </c>
-      <c r="E371" s="2" t="inlineStr"/>
+      <c r="E371" s="2" t="n"/>
       <c r="F371" s="2" t="inlineStr">
         <is>
           <t>pension_todas_cobradas no repite tipos (es 'tipos distintos')</t>
@@ -26918,7 +26918,7 @@
           <t>pension_actual</t>
         </is>
       </c>
-      <c r="E372" s="2" t="inlineStr"/>
+      <c r="E372" s="2" t="n"/>
       <c r="F372" s="2" t="inlineStr">
         <is>
           <t>pension_actual no repite tipos (es 'tipos distintos')</t>
@@ -26984,7 +26984,7 @@
           <t>pension_actual</t>
         </is>
       </c>
-      <c r="E373" s="2" t="inlineStr"/>
+      <c r="E373" s="2" t="n"/>
       <c r="F373" s="2" t="inlineStr">
         <is>
           <t>Sin pensión ⇒ NULL, no lista vacía</t>
@@ -27046,7 +27046,7 @@
           <t>pension_todas_cobradas</t>
         </is>
       </c>
-      <c r="E374" s="2" t="inlineStr"/>
+      <c r="E374" s="2" t="n"/>
       <c r="F374" s="2" t="inlineStr">
         <is>
           <t>Sin pensiones ⇒ NULL, no lista vacía</t>
@@ -27322,7 +27322,7 @@
           <t>ingresos_bruto_total_2024</t>
         </is>
       </c>
-      <c r="E378" s="2" t="inlineStr"/>
+      <c r="E378" s="2" t="n"/>
       <c r="F378" s="2" t="inlineStr">
         <is>
           <t>Ingresos brutos anuales ≤ 1.000.000 €</t>
@@ -28097,7 +28097,7 @@
       </c>
       <c r="P389" s="2" t="inlineStr">
         <is>
-          <t>(prov_nacimiento IS NOT NULL AND prov_nacimiento NOT IN ('NO CONSTA','No consta','0 NO CONSTA','00 No consta')) AND pais_nacimiento NOT LIKE 'N00%' AND pais_nacimiento &lt;&gt; 'NO CONSTA'</t>
+          <t>(prov_nacimiento IS NOT NULL AND prov_nacimiento NOT IN ('NO CONSTA','No consta','0 NO CONSTA','00 No consta')) AND pais_nacimiento NOT LIKE 'N00%' AND pais_nacimiento &lt;&gt; 'NO CONSTA' AND pais_nacimiento NOT LIKE 'N99%' AND prov_nacimiento &lt;&gt; '66 EXTRANJERO'</t>
         </is>
       </c>
     </row>
@@ -28122,7 +28122,7 @@
           <t>sexo</t>
         </is>
       </c>
-      <c r="E390" s="2" t="inlineStr"/>
+      <c r="E390" s="2" t="n"/>
       <c r="F390" s="2" t="inlineStr">
         <is>
           <t>sexo ∈ {Hombre, Mujer, NO CONSTA}</t>
@@ -28184,7 +28184,7 @@
           <t>domic_resid_habitual</t>
         </is>
       </c>
-      <c r="E391" s="2" t="inlineStr"/>
+      <c r="E391" s="2" t="n"/>
       <c r="F391" s="2" t="inlineStr">
         <is>
           <t>El domicilio (INE) es NO CONSTA o 5 dígitos con provincia 01-52 (guía 1.007)</t>
@@ -28510,7 +28510,7 @@
           <t>grupo_cotiz_ppal</t>
         </is>
       </c>
-      <c r="E396" s="2" t="inlineStr"/>
+      <c r="E396" s="2" t="n"/>
       <c r="F396" s="2" t="inlineStr">
         <is>
           <t>Cada código de grupo de cotización tiene una única etiqueta en grupo_cotiz_ppal</t>
@@ -28572,7 +28572,7 @@
           <t>grupo_ultimo_empleo</t>
         </is>
       </c>
-      <c r="E397" s="2" t="inlineStr"/>
+      <c r="E397" s="2" t="n"/>
       <c r="F397" s="2" t="inlineStr">
         <is>
           <t>Cada código de grupo de cotización tiene una única etiqueta en grupo_ultimo_empleo</t>
@@ -28634,7 +28634,7 @@
           <t>grupo_cotiz_1er_empleo_signif</t>
         </is>
       </c>
-      <c r="E398" s="2" t="inlineStr"/>
+      <c r="E398" s="2" t="n"/>
       <c r="F398" s="2" t="inlineStr">
         <is>
           <t>Cada código de grupo de cotización tiene una única etiqueta en grupo_cotiz_1er_empleo_signif</t>
@@ -28696,7 +28696,7 @@
           <t>grupo_cotiz_ppal</t>
         </is>
       </c>
-      <c r="E399" s="2" t="inlineStr"/>
+      <c r="E399" s="2" t="n"/>
       <c r="F399" s="2" t="inlineStr">
         <is>
           <t>grupo_cotiz_ppal solo toma valores de la tabla de grupos de cotización (0-12) o NO CONSTA (guía 2.003)</t>
@@ -28758,7 +28758,7 @@
           <t>grupo_ultimo_empleo</t>
         </is>
       </c>
-      <c r="E400" s="2" t="inlineStr"/>
+      <c r="E400" s="2" t="n"/>
       <c r="F400" s="2" t="inlineStr">
         <is>
           <t>grupo_ultimo_empleo solo toma valores de la tabla de grupos de cotización (0-12) o NO CONSTA (guía 2.003)</t>
@@ -28820,7 +28820,7 @@
           <t>grupo_cotiz_1er_empleo_signif</t>
         </is>
       </c>
-      <c r="E401" s="2" t="inlineStr"/>
+      <c r="E401" s="2" t="n"/>
       <c r="F401" s="2" t="inlineStr">
         <is>
           <t>grupo_cotiz_1er_empleo_signif solo toma valores de la tabla de grupos de cotización (0-12) o NO CONSTA (guía 2.003)</t>
@@ -28882,7 +28882,7 @@
           <t>reg_cotiz_ppal_agrupado</t>
         </is>
       </c>
-      <c r="E402" s="2" t="inlineStr"/>
+      <c r="E402" s="2" t="n"/>
       <c r="F402" s="2" t="inlineStr">
         <is>
           <t>reg_cotiz_ppal_agrupado solo toma los regímenes 01, 0138, 05, 06, 07, 08, 09, 12</t>
@@ -28944,7 +28944,7 @@
           <t>tipo_contr_ppal_agrupado</t>
         </is>
       </c>
-      <c r="E403" s="2" t="inlineStr"/>
+      <c r="E403" s="2" t="n"/>
       <c r="F403" s="2" t="inlineStr">
         <is>
           <t>tipo_contr_ppal_agrupado solo toma las 7 categorías de tipo de contrato</t>
@@ -29006,7 +29006,7 @@
           <t>tipo_contr_ult_baja</t>
         </is>
       </c>
-      <c r="E404" s="2" t="inlineStr"/>
+      <c r="E404" s="2" t="n"/>
       <c r="F404" s="2" t="inlineStr">
         <is>
           <t>tipo_contr_ult_baja solo toma las 7 categorías de tipo de contrato</t>
@@ -29068,7 +29068,7 @@
           <t>causa_ult_baja</t>
         </is>
       </c>
-      <c r="E405" s="2" t="inlineStr"/>
+      <c r="E405" s="2" t="n"/>
       <c r="F405" s="2" t="inlineStr">
         <is>
           <t>causa_ult_baja solo toma claves de causa de baja de la guía 2.008 o NO CONSTA</t>
@@ -29130,7 +29130,7 @@
           <t>causa_baja_trab_ppal</t>
         </is>
       </c>
-      <c r="E406" s="2" t="inlineStr"/>
+      <c r="E406" s="2" t="n"/>
       <c r="F406" s="2" t="inlineStr">
         <is>
           <t>causa_baja_trab_ppal solo toma claves de causa de baja de la guía 2.008 o NO CONSTA</t>
@@ -29192,7 +29192,7 @@
           <t>causa_baja_mas_comun</t>
         </is>
       </c>
-      <c r="E407" s="2" t="inlineStr"/>
+      <c r="E407" s="2" t="n"/>
       <c r="F407" s="2" t="inlineStr">
         <is>
           <t>causa_baja_mas_comun solo toma claves de causa de baja de la guía 2.008 o NO CONSTA</t>
@@ -29254,7 +29254,7 @@
           <t>act_econ_ppal</t>
         </is>
       </c>
-      <c r="E408" s="2" t="inlineStr"/>
+      <c r="E408" s="2" t="n"/>
       <c r="F408" s="2" t="inlineStr">
         <is>
           <t>act_econ_ppal = 'NNN texto' (CNAE 3 dígitos) o NO CONSTA</t>
@@ -29316,7 +29316,7 @@
           <t>act_econ_ult_baja</t>
         </is>
       </c>
-      <c r="E409" s="2" t="inlineStr"/>
+      <c r="E409" s="2" t="n"/>
       <c r="F409" s="2" t="inlineStr">
         <is>
           <t>act_econ_ult_baja = 'NNN texto' (CNAE 3 dígitos) o NO CONSTA</t>
@@ -29378,7 +29378,7 @@
           <t>prov_trabajo_ppal</t>
         </is>
       </c>
-      <c r="E410" s="2" t="inlineStr"/>
+      <c r="E410" s="2" t="n"/>
       <c r="F410" s="2" t="inlineStr">
         <is>
           <t>prov_trabajo_ppal = 'NN NOMBRE' (provincia) o NO CONSTA</t>
@@ -29440,7 +29440,7 @@
           <t>prov_fiscal_actual</t>
         </is>
       </c>
-      <c r="E411" s="2" t="inlineStr"/>
+      <c r="E411" s="2" t="n"/>
       <c r="F411" s="2" t="inlineStr">
         <is>
           <t>prov_fiscal_actual = 'NN NOMBRE' (provincia) o NO CONSTA</t>
@@ -29502,7 +29502,7 @@
           <t>prov_nacimiento</t>
         </is>
       </c>
-      <c r="E412" s="2" t="inlineStr"/>
+      <c r="E412" s="2" t="n"/>
       <c r="F412" s="2" t="inlineStr">
         <is>
           <t>prov_nacimiento = 'NN NOMBRE' (provincia) o NO CONSTA</t>
@@ -29564,7 +29564,7 @@
           <t>prov_1a_afiliacion</t>
         </is>
       </c>
-      <c r="E413" s="2" t="inlineStr"/>
+      <c r="E413" s="2" t="n"/>
       <c r="F413" s="2" t="inlineStr">
         <is>
           <t>prov_1a_afiliacion = 'NN NOMBRE' (provincia) o NO CONSTA</t>
@@ -29626,7 +29626,7 @@
           <t>prov_resid_habitual</t>
         </is>
       </c>
-      <c r="E414" s="2" t="inlineStr"/>
+      <c r="E414" s="2" t="n"/>
       <c r="F414" s="2" t="inlineStr">
         <is>
           <t>prov_resid_habitual = 'NN NOMBRE' (provincia) o NO CONSTA</t>
@@ -29688,7 +29688,7 @@
           <t>nacionalidad_agrupado</t>
         </is>
       </c>
-      <c r="E415" s="2" t="inlineStr"/>
+      <c r="E415" s="2" t="n"/>
       <c r="F415" s="2" t="inlineStr">
         <is>
           <t>nacionalidad_agrupado ∈ 5 grupos conocidos</t>
@@ -29750,7 +29750,7 @@
           <t>pais_nacim_agrupado</t>
         </is>
       </c>
-      <c r="E416" s="2" t="inlineStr"/>
+      <c r="E416" s="2" t="n"/>
       <c r="F416" s="2" t="inlineStr">
         <is>
           <t>pais_nacim_agrupado ∈ 5 grupos conocidos</t>
@@ -29812,7 +29812,7 @@
           <t>cobra_pension_2024_5</t>
         </is>
       </c>
-      <c r="E417" s="2" t="inlineStr"/>
+      <c r="E417" s="2" t="n"/>
       <c r="F417" s="2" t="inlineStr">
         <is>
           <t>cobra_pension_2024_5 ∈ {SI, NO}</t>
@@ -29874,7 +29874,7 @@
           <t>ha_fallecido</t>
         </is>
       </c>
-      <c r="E418" s="2" t="inlineStr"/>
+      <c r="E418" s="2" t="n"/>
       <c r="F418" s="2" t="inlineStr">
         <is>
           <t>ha_fallecido ∈ {SI, NO}</t>
@@ -29936,7 +29936,7 @@
           <t>situacion_actual_afiliacion</t>
         </is>
       </c>
-      <c r="E419" s="2" t="inlineStr"/>
+      <c r="E419" s="2" t="n"/>
       <c r="F419" s="2" t="inlineStr">
         <is>
           <t>situacion_actual_afiliacion ∈ 9 categorías conocidas</t>
@@ -29998,7 +29998,7 @@
           <t>situacion_paro_ocupacion</t>
         </is>
       </c>
-      <c r="E420" s="2" t="inlineStr"/>
+      <c r="E420" s="2" t="n"/>
       <c r="F420" s="2" t="inlineStr">
         <is>
           <t>situacion_paro_ocupacion ∈ 7 categorías conocidas</t>
@@ -30060,7 +30060,7 @@
           <t>ipf</t>
         </is>
       </c>
-      <c r="E421" s="2" t="inlineStr"/>
+      <c r="E421" s="2" t="n"/>
       <c r="F421" s="2" t="inlineStr">
         <is>
           <t>ipf no puede ser nulo</t>
@@ -30122,7 +30122,7 @@
           <t>fecha_nacimiento</t>
         </is>
       </c>
-      <c r="E422" s="2" t="inlineStr"/>
+      <c r="E422" s="2" t="n"/>
       <c r="F422" s="2" t="inlineStr">
         <is>
           <t>fecha_nacimiento no puede ser nulo</t>
@@ -30184,7 +30184,7 @@
           <t>sexo</t>
         </is>
       </c>
-      <c r="E423" s="2" t="inlineStr"/>
+      <c r="E423" s="2" t="n"/>
       <c r="F423" s="2" t="inlineStr">
         <is>
           <t>sexo no puede ser nulo</t>
@@ -30246,7 +30246,7 @@
           <t>edad_actual_fecha_corte</t>
         </is>
       </c>
-      <c r="E424" s="2" t="inlineStr"/>
+      <c r="E424" s="2" t="n"/>
       <c r="F424" s="2" t="inlineStr">
         <is>
           <t>edad_actual_fecha_corte no puede ser nulo</t>
@@ -30308,7 +30308,7 @@
           <t>situacion_actual_afiliacion</t>
         </is>
       </c>
-      <c r="E425" s="2" t="inlineStr"/>
+      <c r="E425" s="2" t="n"/>
       <c r="F425" s="2" t="inlineStr">
         <is>
           <t>situacion_actual_afiliacion no puede ser nulo</t>
@@ -30370,7 +30370,7 @@
           <t>situacion_paro_ocupacion</t>
         </is>
       </c>
-      <c r="E426" s="2" t="inlineStr"/>
+      <c r="E426" s="2" t="n"/>
       <c r="F426" s="2" t="inlineStr">
         <is>
           <t>situacion_paro_ocupacion no puede ser nulo</t>
@@ -30432,7 +30432,7 @@
           <t>nacionalidad</t>
         </is>
       </c>
-      <c r="E427" s="2" t="inlineStr"/>
+      <c r="E427" s="2" t="n"/>
       <c r="F427" s="2" t="inlineStr">
         <is>
           <t>nacionalidad no puede ser nulo</t>
@@ -30494,7 +30494,7 @@
           <t>pais_nacimiento</t>
         </is>
       </c>
-      <c r="E428" s="2" t="inlineStr"/>
+      <c r="E428" s="2" t="n"/>
       <c r="F428" s="2" t="inlineStr">
         <is>
           <t>pais_nacimiento no puede ser nulo</t>
@@ -30556,7 +30556,7 @@
           <t>prov_nacimiento</t>
         </is>
       </c>
-      <c r="E429" s="2" t="inlineStr"/>
+      <c r="E429" s="2" t="n"/>
       <c r="F429" s="2" t="inlineStr">
         <is>
           <t>prov_nacimiento no puede ser nulo</t>
@@ -30618,7 +30618,7 @@
           <t>cobra_pension_2024_5</t>
         </is>
       </c>
-      <c r="E430" s="2" t="inlineStr"/>
+      <c r="E430" s="2" t="n"/>
       <c r="F430" s="2" t="inlineStr">
         <is>
           <t>cobra_pension_2024_5 no puede ser nulo</t>
@@ -30680,7 +30680,7 @@
           <t>discap_afiliacion</t>
         </is>
       </c>
-      <c r="E431" s="2" t="inlineStr"/>
+      <c r="E431" s="2" t="n"/>
       <c r="F431" s="2" t="inlineStr">
         <is>
           <t>discap_afiliacion no puede ser nulo</t>
@@ -30742,7 +30742,7 @@
           <t>discap_pension</t>
         </is>
       </c>
-      <c r="E432" s="2" t="inlineStr"/>
+      <c r="E432" s="2" t="n"/>
       <c r="F432" s="2" t="inlineStr">
         <is>
           <t>discap_pension no puede ser nulo</t>
@@ -30804,7 +30804,7 @@
           <t>discap_fiscal</t>
         </is>
       </c>
-      <c r="E433" s="2" t="inlineStr"/>
+      <c r="E433" s="2" t="n"/>
       <c r="F433" s="2" t="inlineStr">
         <is>
           <t>discap_fiscal no puede ser nulo</t>
@@ -30866,7 +30866,7 @@
           <t>domic_resid_habitual</t>
         </is>
       </c>
-      <c r="E434" s="2" t="inlineStr"/>
+      <c r="E434" s="2" t="n"/>
       <c r="F434" s="2" t="inlineStr">
         <is>
           <t>domic_resid_habitual no puede ser nulo</t>
@@ -30928,7 +30928,7 @@
           <t>prov_resid_habitual</t>
         </is>
       </c>
-      <c r="E435" s="2" t="inlineStr"/>
+      <c r="E435" s="2" t="n"/>
       <c r="F435" s="2" t="inlineStr">
         <is>
           <t>prov_resid_habitual no puede ser nulo</t>
@@ -30990,7 +30990,7 @@
           <t>ha_fallecido</t>
         </is>
       </c>
-      <c r="E436" s="2" t="inlineStr"/>
+      <c r="E436" s="2" t="n"/>
       <c r="F436" s="2" t="inlineStr">
         <is>
           <t>ha_fallecido no puede ser nulo</t>
@@ -31052,7 +31052,7 @@
           <t>clave_subclave_ppal</t>
         </is>
       </c>
-      <c r="E437" s="2" t="inlineStr"/>
+      <c r="E437" s="2" t="n"/>
       <c r="F437" s="2" t="inlineStr">
         <is>
           <t>clave_subclave_ppal no puede ser nulo</t>
@@ -31114,7 +31114,7 @@
           <t>ipf</t>
         </is>
       </c>
-      <c r="E438" s="2" t="inlineStr"/>
+      <c r="E438" s="2" t="n"/>
       <c r="F438" s="2" t="inlineStr">
         <is>
           <t>ipf es único (una fila por persona)</t>
@@ -32748,7 +32748,7 @@
           <t>cotizado_anual_promedio</t>
         </is>
       </c>
-      <c r="E461" s="2" t="inlineStr"/>
+      <c r="E461" s="2" t="n"/>
       <c r="F461" s="2" t="inlineStr">
         <is>
           <t>Cotizado anual promedio ≤ 100.000 €/año (la base máxima ronda 57.000 €/año)</t>
@@ -32818,7 +32818,7 @@
           <t>cotizado_anual_promedio</t>
         </is>
       </c>
-      <c r="E462" s="2" t="inlineStr"/>
+      <c r="E462" s="2" t="n"/>
       <c r="F462" s="2" t="inlineStr">
         <is>
           <t>Si es positivo, no es inferior a 100 €/año</t>
@@ -33497,7 +33497,7 @@
       </c>
       <c r="P471" s="2" t="inlineStr">
         <is>
-          <t>duracion_1er_empleo_signif &gt; COALESCE(t_total_empleo,0) + COALESCE(t_total_mixto_empl_desempl,0) + 1</t>
+          <t>duracion_1er_empleo_signif &gt; COALESCE(t_total_empleo,0) + COALESCE(t_total_mixto_empl_desempl,0) + 1 AND ipf NOT IN (SELECT ipf FROM solo_prestaciones)</t>
         </is>
       </c>
     </row>
@@ -34469,7 +34469,7 @@
       </c>
       <c r="P485" s="2" t="inlineStr">
         <is>
-          <t>t_total_desempleo &gt; 0 AND num_bajas_anual_promedio IS NULL</t>
+          <t>t_total_desempleo &gt; 0 AND num_bajas_anual_promedio IS NULL AND ipf NOT IN (SELECT ipf FROM solo_prestaciones) AND situacion_actual_afiliacion &lt;&gt; 'Alta_ocupado'</t>
         </is>
       </c>
     </row>
@@ -34539,7 +34539,7 @@
       </c>
       <c r="P486" s="2" t="inlineStr">
         <is>
-          <t>situacion_actual_afiliacion &lt;&gt; 'Nunca_ha_cotizado' AND fecha_ini_primer_empleo IS NULL</t>
+          <t>situacion_actual_afiliacion &lt;&gt; 'Nunca_ha_cotizado' AND fecha_ini_primer_empleo IS NULL AND ipf NOT IN (SELECT ipf FROM solo_prestaciones)</t>
         </is>
       </c>
     </row>
@@ -34770,7 +34770,7 @@
           <t>duracion_actual_sin_empleo</t>
         </is>
       </c>
-      <c r="E490" s="2" t="inlineStr"/>
+      <c r="E490" s="2" t="n"/>
       <c r="F490" s="2" t="inlineStr">
         <is>
           <t>duracion_actual_sin_empleo es un número entero de días</t>
@@ -34900,12 +34900,12 @@
       </c>
       <c r="E492" s="2" t="inlineStr">
         <is>
-          <t>ingresos_pension_2024</t>
+          <t>ingresos_pension_y_bajas_2024</t>
         </is>
       </c>
       <c r="F492" s="2" t="inlineStr">
         <is>
-          <t>ingresos_pension_2024 informado solo si hay datos fiscales (y al revés)</t>
+          <t>ingresos_pension_y_bajas_2024 informado solo si hay datos fiscales (y al revés)</t>
         </is>
       </c>
       <c r="G492" s="2" t="inlineStr">
@@ -34939,7 +34939,7 @@
       <c r="O492" s="2" t="inlineStr"/>
       <c r="P492" s="2" t="inlineStr">
         <is>
-          <t>(ingresos_bruto_total_2024 IS NULL) &lt;&gt; (ingresos_pension_2024 IS NULL)</t>
+          <t>(ingresos_bruto_total_2024 IS NULL) &lt;&gt; (ingresos_pension_y_bajas_2024 IS NULL)</t>
         </is>
       </c>
     </row>
@@ -35228,7 +35228,7 @@
           <t>ingresos_bruto_total_2024</t>
         </is>
       </c>
-      <c r="E497" s="2" t="inlineStr"/>
+      <c r="E497" s="2" t="n"/>
       <c r="F497" s="2" t="inlineStr">
         <is>
           <t>Las 5 partes suman el total de ingresos (±0,01 €)</t>
@@ -35265,7 +35265,7 @@
       <c r="O497" s="2" t="inlineStr"/>
       <c r="P497" s="2" t="inlineStr">
         <is>
-          <t>ingresos_bruto_total_2024 IS NOT NULL AND ABS(ingresos_bruto_total_2024 - (ingresos_sueldo_2024 + ingresos_pension_2024 + ingresos_prestacion_2024 + ingresos_actividad_2024 + ingresos_otras_exentas_2024)) &gt; 0.01</t>
+          <t>ingresos_bruto_total_2024 IS NOT NULL AND ABS(ingresos_bruto_total_2024 - (ingresos_sueldo_2024 + ingresos_pension_y_bajas_2024 + ingresos_prestacion_2024 + ingresos_actividad_2024 + ingresos_otras_exentas_2024)) &gt; 0.01</t>
         </is>
       </c>
     </row>
@@ -35290,7 +35290,7 @@
           <t>ingresos_sueldo_2024</t>
         </is>
       </c>
-      <c r="E498" s="2" t="inlineStr"/>
+      <c r="E498" s="2" t="n"/>
       <c r="F498" s="2" t="inlineStr">
         <is>
           <t>ingresos_sueldo_2024 ≥ 0</t>
@@ -35353,13 +35353,13 @@
       </c>
       <c r="D499" s="2" t="inlineStr">
         <is>
-          <t>ingresos_pension_2024</t>
-        </is>
-      </c>
-      <c r="E499" s="2" t="inlineStr"/>
+          <t>ingresos_pension_y_bajas_2024</t>
+        </is>
+      </c>
+      <c r="E499" s="2" t="n"/>
       <c r="F499" s="2" t="inlineStr">
         <is>
-          <t>ingresos_pension_2024 ≥ 0</t>
+          <t>ingresos_pension_y_bajas_2024 ≥ 0</t>
         </is>
       </c>
       <c r="G499" s="2" t="inlineStr">
@@ -35397,7 +35397,7 @@
       </c>
       <c r="P499" s="2" t="inlineStr">
         <is>
-          <t>ingresos_pension_2024 &lt; 0</t>
+          <t>ingresos_pension_y_bajas_2024 &lt; 0</t>
         </is>
       </c>
     </row>
@@ -35422,7 +35422,7 @@
           <t>ingresos_prestacion_2024</t>
         </is>
       </c>
-      <c r="E500" s="2" t="inlineStr"/>
+      <c r="E500" s="2" t="n"/>
       <c r="F500" s="2" t="inlineStr">
         <is>
           <t>ingresos_prestacion_2024 ≥ 0</t>
@@ -35488,7 +35488,7 @@
           <t>ingresos_actividad_2024</t>
         </is>
       </c>
-      <c r="E501" s="2" t="inlineStr"/>
+      <c r="E501" s="2" t="n"/>
       <c r="F501" s="2" t="inlineStr">
         <is>
           <t>ingresos_actividad_2024 ≥ 0</t>
@@ -35554,7 +35554,7 @@
           <t>ingresos_otras_exentas_2024</t>
         </is>
       </c>
-      <c r="E502" s="2" t="inlineStr"/>
+      <c r="E502" s="2" t="n"/>
       <c r="F502" s="2" t="inlineStr">
         <is>
           <t>ingresos_otras_exentas_2024 ≥ 0</t>
@@ -35620,7 +35620,7 @@
           <t>retenciones_irpf_2024</t>
         </is>
       </c>
-      <c r="E503" s="2" t="inlineStr"/>
+      <c r="E503" s="2" t="n"/>
       <c r="F503" s="2" t="inlineStr">
         <is>
           <t>Las retenciones de IRPF no son negativas</t>
@@ -35730,7 +35730,7 @@
     <row r="505">
       <c r="A505" s="2" t="inlineStr">
         <is>
-          <t>C-299</t>
+          <t>C-302</t>
         </is>
       </c>
       <c r="B505" s="2" t="inlineStr">
@@ -35745,17 +35745,17 @@
       </c>
       <c r="D505" s="2" t="inlineStr">
         <is>
-          <t>retenciones_irpf_2024</t>
+          <t>ingresos_sueldo_2024</t>
         </is>
       </c>
       <c r="E505" s="2" t="inlineStr">
         <is>
-          <t>ingresos_bruto_total_2024</t>
+          <t>edad_actual_fecha_corte</t>
         </is>
       </c>
       <c r="F505" s="2" t="inlineStr">
         <is>
-          <t>Retenciones ≤ 50 % del total (tipo máximo de IRPF ≈ 47 %)</t>
+          <t>Con ingresos de sueldo ⇒ edad ≥ 16</t>
         </is>
       </c>
       <c r="G505" s="2" t="inlineStr">
@@ -35765,7 +35765,7 @@
       </c>
       <c r="H505" s="2" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I505" s="7" t="inlineStr">
@@ -35775,14 +35775,14 @@
       </c>
       <c r="J505" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K505" s="2" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="L505" s="2" t="n">
-        <v>0.0001</v>
+        <v>0.001</v>
       </c>
       <c r="M505" s="2" t="inlineStr">
         <is>
@@ -35790,17 +35790,21 @@
         </is>
       </c>
       <c r="N505" s="2" t="n"/>
-      <c r="O505" s="2" t="inlineStr"/>
+      <c r="O505" s="2" t="inlineStr">
+        <is>
+          <t>Excluye a los menores autorizados (art. 6.4 ET; decisión del usuario 2026-09-25): 262 -&gt; 13 y 11 -&gt; 5. El resto, dato de origen.</t>
+        </is>
+      </c>
       <c r="P505" s="2" t="inlineStr">
         <is>
-          <t>ingresos_bruto_total_2024 &gt; 0 AND retenciones_irpf_2024 &gt; 0.5 * ingresos_bruto_total_2024</t>
+          <t>ingresos_sueldo_2024 &gt; 0 AND edad_actual_fecha_corte &lt; 16 AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
         </is>
       </c>
     </row>
     <row r="506">
       <c r="A506" s="2" t="inlineStr">
         <is>
-          <t>C-300</t>
+          <t>C-303</t>
         </is>
       </c>
       <c r="B506" s="2" t="inlineStr">
@@ -35818,59 +35822,55 @@
           <t>ingresos_sueldo_2024</t>
         </is>
       </c>
-      <c r="E506" s="2" t="inlineStr"/>
+      <c r="E506" s="2" t="inlineStr">
+        <is>
+          <t>fecha_fallecimiento</t>
+        </is>
+      </c>
       <c r="F506" s="2" t="inlineStr">
         <is>
-          <t>Sueldo anual ≤ 1.000.000 €</t>
+          <t>Con ingresos de sueldo 2024 ⇒ no fallecido antes de 2024</t>
         </is>
       </c>
       <c r="G506" s="2" t="inlineStr">
         <is>
-          <t>Dominio (Seg. Social / lógica)</t>
+          <t>Guía MCVL</t>
         </is>
       </c>
       <c r="H506" s="2" t="inlineStr">
         <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I506" s="7" t="inlineStr">
-        <is>
-          <t>INCUMPLE</t>
-        </is>
-      </c>
-      <c r="J506" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I506" s="6" t="inlineStr">
+        <is>
+          <t>PASA</t>
+        </is>
+      </c>
+      <c r="J506" s="6" t="inlineStr">
+        <is>
+          <t>Pasan</t>
         </is>
       </c>
       <c r="K506" s="2" t="n">
-        <v>53</v>
+        <v>0</v>
       </c>
       <c r="L506" s="2" t="n">
-        <v>0.0039</v>
-      </c>
-      <c r="M506" s="2" t="inlineStr">
-        <is>
-          <t>G17</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M506" s="2" t="inlineStr"/>
       <c r="N506" s="2" t="n"/>
-      <c r="O506" s="2" t="inlineStr">
-        <is>
-          <t>Outliers (directivos)</t>
-        </is>
-      </c>
+      <c r="O506" s="2" t="inlineStr"/>
       <c r="P506" s="2" t="inlineStr">
         <is>
-          <t>ingresos_sueldo_2024 &gt; 1000000</t>
+          <t>ingresos_sueldo_2024 &gt; 0 AND fecha_fallecimiento BETWEEN 1 AND 202312</t>
         </is>
       </c>
     </row>
     <row r="507">
       <c r="A507" s="2" t="inlineStr">
         <is>
-          <t>C-301</t>
+          <t>C-304</t>
         </is>
       </c>
       <c r="B507" s="2" t="inlineStr">
@@ -35885,13 +35885,17 @@
       </c>
       <c r="D507" s="2" t="inlineStr">
         <is>
-          <t>ingresos_actividad_2024</t>
-        </is>
-      </c>
-      <c r="E507" s="2" t="inlineStr"/>
+          <t>ingresos_prestacion_2024</t>
+        </is>
+      </c>
+      <c r="E507" s="2" t="inlineStr">
+        <is>
+          <t>edad_actual_fecha_corte</t>
+        </is>
+      </c>
       <c r="F507" s="2" t="inlineStr">
         <is>
-          <t>Ingresos de actividad anual ≤ 1.000.000 €</t>
+          <t>Con ingresos de prestación ⇒ edad ≥ 16</t>
         </is>
       </c>
       <c r="G507" s="2" t="inlineStr">
@@ -35901,46 +35905,38 @@
       </c>
       <c r="H507" s="2" t="inlineStr">
         <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I507" s="7" t="inlineStr">
-        <is>
-          <t>INCUMPLE</t>
-        </is>
-      </c>
-      <c r="J507" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I507" s="6" t="inlineStr">
+        <is>
+          <t>PASA</t>
+        </is>
+      </c>
+      <c r="J507" s="6" t="inlineStr">
+        <is>
+          <t>Pasan</t>
         </is>
       </c>
       <c r="K507" s="2" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="L507" s="2" t="n">
-        <v>0.0026</v>
-      </c>
-      <c r="M507" s="2" t="inlineStr">
-        <is>
-          <t>G17</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M507" s="2" t="inlineStr"/>
       <c r="N507" s="2" t="n"/>
-      <c r="O507" s="2" t="inlineStr">
-        <is>
-          <t>Outliers</t>
-        </is>
-      </c>
+      <c r="O507" s="2" t="inlineStr"/>
       <c r="P507" s="2" t="inlineStr">
         <is>
-          <t>ingresos_actividad_2024 &gt; 1000000</t>
+          <t>ingresos_prestacion_2024 &gt; 0 AND edad_actual_fecha_corte &lt; 16</t>
         </is>
       </c>
     </row>
     <row r="508">
       <c r="A508" s="2" t="inlineStr">
         <is>
-          <t>C-302</t>
+          <t>C-305</t>
         </is>
       </c>
       <c r="B508" s="2" t="inlineStr">
@@ -35955,62 +35951,58 @@
       </c>
       <c r="D508" s="2" t="inlineStr">
         <is>
-          <t>ingresos_sueldo_2024</t>
+          <t>ingresos_prestacion_2024</t>
         </is>
       </c>
       <c r="E508" s="2" t="inlineStr">
         <is>
-          <t>edad_actual_fecha_corte</t>
+          <t>fecha_fallecimiento</t>
         </is>
       </c>
       <c r="F508" s="2" t="inlineStr">
         <is>
-          <t>Con ingresos de sueldo ⇒ edad ≥ 16</t>
+          <t>Con ingresos de prestación 2024 ⇒ no fallecido antes de 2024</t>
         </is>
       </c>
       <c r="G508" s="2" t="inlineStr">
         <is>
-          <t>Dominio (Seg. Social / lógica)</t>
+          <t>Guía MCVL</t>
         </is>
       </c>
       <c r="H508" s="2" t="inlineStr">
         <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="I508" s="7" t="inlineStr">
-        <is>
-          <t>INCUMPLE</t>
-        </is>
-      </c>
-      <c r="J508" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I508" s="6" t="inlineStr">
+        <is>
+          <t>PASA</t>
+        </is>
+      </c>
+      <c r="J508" s="6" t="inlineStr">
+        <is>
+          <t>Pasan</t>
         </is>
       </c>
       <c r="K508" s="2" t="n">
-        <v>262</v>
+        <v>0</v>
       </c>
       <c r="L508" s="2" t="n">
-        <v>0.0193</v>
-      </c>
-      <c r="M508" s="2" t="inlineStr">
-        <is>
-          <t>G17</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M508" s="2" t="inlineStr"/>
       <c r="N508" s="2" t="n"/>
       <c r="O508" s="2" t="inlineStr"/>
       <c r="P508" s="2" t="inlineStr">
         <is>
-          <t>ingresos_sueldo_2024 &gt; 0 AND edad_actual_fecha_corte &lt; 16</t>
+          <t>ingresos_prestacion_2024 &gt; 0 AND fecha_fallecimiento BETWEEN 1 AND 202312</t>
         </is>
       </c>
     </row>
     <row r="509">
       <c r="A509" s="2" t="inlineStr">
         <is>
-          <t>C-303</t>
+          <t>C-306</t>
         </is>
       </c>
       <c r="B509" s="2" t="inlineStr">
@@ -36025,58 +36017,66 @@
       </c>
       <c r="D509" s="2" t="inlineStr">
         <is>
-          <t>ingresos_sueldo_2024</t>
+          <t>ingresos_actividad_2024</t>
         </is>
       </c>
       <c r="E509" s="2" t="inlineStr">
         <is>
-          <t>fecha_fallecimiento</t>
+          <t>edad_actual_fecha_corte</t>
         </is>
       </c>
       <c r="F509" s="2" t="inlineStr">
         <is>
-          <t>Con ingresos de sueldo 2024 ⇒ no fallecido antes de 2024</t>
+          <t>Con ingresos de actividad ⇒ edad ≥ 16</t>
         </is>
       </c>
       <c r="G509" s="2" t="inlineStr">
         <is>
-          <t>Guía MCVL</t>
+          <t>Dominio (Seg. Social / lógica)</t>
         </is>
       </c>
       <c r="H509" s="2" t="inlineStr">
         <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="I509" s="6" t="inlineStr">
-        <is>
-          <t>PASA</t>
-        </is>
-      </c>
-      <c r="J509" s="6" t="inlineStr">
-        <is>
-          <t>Pasan</t>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I509" s="7" t="inlineStr">
+        <is>
+          <t>INCUMPLE</t>
+        </is>
+      </c>
+      <c r="J509" s="5" t="inlineStr">
+        <is>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K509" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L509" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M509" s="2" t="inlineStr"/>
+        <v>0.0004</v>
+      </c>
+      <c r="M509" s="2" t="inlineStr">
+        <is>
+          <t>G17</t>
+        </is>
+      </c>
       <c r="N509" s="2" t="n"/>
-      <c r="O509" s="2" t="inlineStr"/>
+      <c r="O509" s="2" t="inlineStr">
+        <is>
+          <t>Excluye a los menores autorizados (art. 6.4 ET; decisión del usuario 2026-09-25): 262 -&gt; 13 y 11 -&gt; 5. El resto, dato de origen.</t>
+        </is>
+      </c>
       <c r="P509" s="2" t="inlineStr">
         <is>
-          <t>ingresos_sueldo_2024 &gt; 0 AND fecha_fallecimiento BETWEEN 1 AND 202312</t>
+          <t>ingresos_actividad_2024 &gt; 0 AND edad_actual_fecha_corte &lt; 16 AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
         </is>
       </c>
     </row>
     <row r="510">
       <c r="A510" s="2" t="inlineStr">
         <is>
-          <t>C-304</t>
+          <t>C-307</t>
         </is>
       </c>
       <c r="B510" s="2" t="inlineStr">
@@ -36091,27 +36091,27 @@
       </c>
       <c r="D510" s="2" t="inlineStr">
         <is>
-          <t>ingresos_prestacion_2024</t>
+          <t>ingresos_actividad_2024</t>
         </is>
       </c>
       <c r="E510" s="2" t="inlineStr">
         <is>
-          <t>edad_actual_fecha_corte</t>
+          <t>fecha_fallecimiento</t>
         </is>
       </c>
       <c r="F510" s="2" t="inlineStr">
         <is>
-          <t>Con ingresos de prestación ⇒ edad ≥ 16</t>
+          <t>Con ingresos de actividad 2024 ⇒ no fallecido antes de 2024</t>
         </is>
       </c>
       <c r="G510" s="2" t="inlineStr">
         <is>
-          <t>Dominio (Seg. Social / lógica)</t>
+          <t>Guía MCVL</t>
         </is>
       </c>
       <c r="H510" s="2" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="I510" s="6" t="inlineStr">
@@ -36135,14 +36135,14 @@
       <c r="O510" s="2" t="inlineStr"/>
       <c r="P510" s="2" t="inlineStr">
         <is>
-          <t>ingresos_prestacion_2024 &gt; 0 AND edad_actual_fecha_corte &lt; 16</t>
+          <t>ingresos_actividad_2024 &gt; 0 AND fecha_fallecimiento BETWEEN 1 AND 202312</t>
         </is>
       </c>
     </row>
     <row r="511">
       <c r="A511" s="2" t="inlineStr">
         <is>
-          <t>C-305</t>
+          <t>C-308</t>
         </is>
       </c>
       <c r="B511" s="2" t="inlineStr">
@@ -36157,7 +36157,7 @@
       </c>
       <c r="D511" s="2" t="inlineStr">
         <is>
-          <t>ingresos_prestacion_2024</t>
+          <t>ingresos_pension_y_bajas_2024</t>
         </is>
       </c>
       <c r="E511" s="2" t="inlineStr">
@@ -36167,7 +36167,7 @@
       </c>
       <c r="F511" s="2" t="inlineStr">
         <is>
-          <t>Con ingresos de prestación 2024 ⇒ no fallecido antes de 2024</t>
+          <t>Con pensiones cobradas en 2024 ⇒ no fallecido antes de 2024</t>
         </is>
       </c>
       <c r="G511" s="2" t="inlineStr">
@@ -36201,14 +36201,14 @@
       <c r="O511" s="2" t="inlineStr"/>
       <c r="P511" s="2" t="inlineStr">
         <is>
-          <t>ingresos_prestacion_2024 &gt; 0 AND fecha_fallecimiento BETWEEN 1 AND 202312</t>
+          <t>ingresos_pension_y_bajas_2024 &gt; 0 AND fecha_fallecimiento BETWEEN 1 AND 202312</t>
         </is>
       </c>
     </row>
     <row r="512">
       <c r="A512" s="2" t="inlineStr">
         <is>
-          <t>C-306</t>
+          <t>C-309</t>
         </is>
       </c>
       <c r="B512" s="2" t="inlineStr">
@@ -36223,17 +36223,17 @@
       </c>
       <c r="D512" s="2" t="inlineStr">
         <is>
-          <t>ingresos_actividad_2024</t>
+          <t>ingresos_prestacion_2024</t>
         </is>
       </c>
       <c r="E512" s="2" t="inlineStr">
         <is>
-          <t>edad_actual_fecha_corte</t>
+          <t>t_total_desempleo</t>
         </is>
       </c>
       <c r="F512" s="2" t="inlineStr">
         <is>
-          <t>Con ingresos de actividad ⇒ edad ≥ 16</t>
+          <t>Con prestación por desempleo en 2024 ⇒ ha tenido tiempo de desempleo</t>
         </is>
       </c>
       <c r="G512" s="2" t="inlineStr">
@@ -36253,14 +36253,14 @@
       </c>
       <c r="J512" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K512" s="2" t="n">
-        <v>11</v>
+        <v>383</v>
       </c>
       <c r="L512" s="2" t="n">
-        <v>0.0008</v>
+        <v>0.0282</v>
       </c>
       <c r="M512" s="2" t="inlineStr">
         <is>
@@ -36268,17 +36268,21 @@
         </is>
       </c>
       <c r="N512" s="2" t="n"/>
-      <c r="O512" s="2" t="inlineStr"/>
+      <c r="O512" s="2" t="inlineStr">
+        <is>
+          <t>Los subsidios pueden no figurar como desempleo en afiliación</t>
+        </is>
+      </c>
       <c r="P512" s="2" t="inlineStr">
         <is>
-          <t>ingresos_actividad_2024 &gt; 0 AND edad_actual_fecha_corte &lt; 16</t>
+          <t>ingresos_prestacion_2024 &gt; 0 AND COALESCE(t_total_desempleo, 0) + COALESCE(t_total_mixto_empl_desempl, 0) = 0</t>
         </is>
       </c>
     </row>
     <row r="513">
       <c r="A513" s="2" t="inlineStr">
         <is>
-          <t>C-307</t>
+          <t>C-310</t>
         </is>
       </c>
       <c r="B513" s="2" t="inlineStr">
@@ -36293,58 +36297,66 @@
       </c>
       <c r="D513" s="2" t="inlineStr">
         <is>
-          <t>ingresos_actividad_2024</t>
+          <t>ingresos_sueldo_2024</t>
         </is>
       </c>
       <c r="E513" s="2" t="inlineStr">
         <is>
-          <t>fecha_fallecimiento</t>
+          <t>fecha_ini_primer_empleo</t>
         </is>
       </c>
       <c r="F513" s="2" t="inlineStr">
         <is>
-          <t>Con ingresos de actividad 2024 ⇒ no fallecido antes de 2024</t>
+          <t>Con sueldo en 2024 ⇒ tiene primer empleo en afiliación</t>
         </is>
       </c>
       <c r="G513" s="2" t="inlineStr">
         <is>
-          <t>Guía MCVL</t>
+          <t>Significado del nombre</t>
         </is>
       </c>
       <c r="H513" s="2" t="inlineStr">
         <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="I513" s="6" t="inlineStr">
-        <is>
-          <t>PASA</t>
-        </is>
-      </c>
-      <c r="J513" s="6" t="inlineStr">
-        <is>
-          <t>Pasan</t>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I513" s="7" t="inlineStr">
+        <is>
+          <t>INCUMPLE</t>
+        </is>
+      </c>
+      <c r="J513" s="5" t="inlineStr">
+        <is>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K513" s="2" t="n">
-        <v>0</v>
+        <v>211</v>
       </c>
       <c r="L513" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M513" s="2" t="inlineStr"/>
+        <v>0.0155</v>
+      </c>
+      <c r="M513" s="2" t="inlineStr">
+        <is>
+          <t>G17</t>
+        </is>
+      </c>
       <c r="N513" s="2" t="n"/>
-      <c r="O513" s="2" t="inlineStr"/>
+      <c r="O513" s="2" t="inlineStr">
+        <is>
+          <t>Los funcionarios de MUFACE no cotizan en el sistema de la MCVL</t>
+        </is>
+      </c>
       <c r="P513" s="2" t="inlineStr">
         <is>
-          <t>ingresos_actividad_2024 &gt; 0 AND fecha_fallecimiento BETWEEN 1 AND 202312</t>
+          <t>ingresos_sueldo_2024 &gt; 0 AND fecha_ini_primer_empleo IS NULL</t>
         </is>
       </c>
     </row>
     <row r="514">
       <c r="A514" s="2" t="inlineStr">
         <is>
-          <t>C-308</t>
+          <t>C-311</t>
         </is>
       </c>
       <c r="B514" s="2" t="inlineStr">
@@ -36359,58 +36371,66 @@
       </c>
       <c r="D514" s="2" t="inlineStr">
         <is>
-          <t>ingresos_pension_2024</t>
+          <t>ingresos_sueldo_2024</t>
         </is>
       </c>
       <c r="E514" s="2" t="inlineStr">
         <is>
-          <t>fecha_fallecimiento</t>
+          <t>fecha_ultima_baja</t>
         </is>
       </c>
       <c r="F514" s="2" t="inlineStr">
         <is>
-          <t>Con pensiones cobradas en 2024 ⇒ no fallecido antes de 2024</t>
+          <t>Con sueldo en 2024 ⇒ la última baja no es anterior a 2024</t>
         </is>
       </c>
       <c r="G514" s="2" t="inlineStr">
         <is>
-          <t>Guía MCVL</t>
+          <t>Dominio (Seg. Social / lógica)</t>
         </is>
       </c>
       <c r="H514" s="2" t="inlineStr">
         <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="I514" s="6" t="inlineStr">
-        <is>
-          <t>PASA</t>
-        </is>
-      </c>
-      <c r="J514" s="6" t="inlineStr">
-        <is>
-          <t>Pasan</t>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="I514" s="7" t="inlineStr">
+        <is>
+          <t>INCUMPLE</t>
+        </is>
+      </c>
+      <c r="J514" s="5" t="inlineStr">
+        <is>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K514" s="2" t="n">
-        <v>0</v>
+        <v>3867</v>
       </c>
       <c r="L514" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M514" s="2" t="inlineStr"/>
+        <v>0.2845</v>
+      </c>
+      <c r="M514" s="2" t="inlineStr">
+        <is>
+          <t>G17</t>
+        </is>
+      </c>
       <c r="N514" s="2" t="n"/>
-      <c r="O514" s="2" t="inlineStr"/>
+      <c r="O514" s="2" t="inlineStr">
+        <is>
+          <t>Pagos atrasados o indemnizaciones podrían dar sueldo sin alta en 2024</t>
+        </is>
+      </c>
       <c r="P514" s="2" t="inlineStr">
         <is>
-          <t>ingresos_pension_2024 &gt; 0 AND fecha_fallecimiento BETWEEN 1 AND 202312</t>
+          <t>ingresos_sueldo_2024 &gt; 0 AND fecha_ultima_baja IS NOT NULL AND year(fecha_ultima_baja) &lt; 2024</t>
         </is>
       </c>
     </row>
     <row r="515">
       <c r="A515" s="2" t="inlineStr">
         <is>
-          <t>C-309</t>
+          <t>C-313</t>
         </is>
       </c>
       <c r="B515" s="2" t="inlineStr">
@@ -36425,17 +36445,17 @@
       </c>
       <c r="D515" s="2" t="inlineStr">
         <is>
-          <t>ingresos_prestacion_2024</t>
+          <t>cobra_pension_2024_5</t>
         </is>
       </c>
       <c r="E515" s="2" t="inlineStr">
         <is>
-          <t>t_total_desempleo</t>
+          <t>ingresos_pension_y_bajas_2024</t>
         </is>
       </c>
       <c r="F515" s="2" t="inlineStr">
         <is>
-          <t>Con prestación por desempleo en 2024 ⇒ ha tenido tiempo de desempleo</t>
+          <t>Cobra pensión en la tabla de pensiones ⇒ tiene pensión en fiscal (si consta en fiscal)</t>
         </is>
       </c>
       <c r="G515" s="2" t="inlineStr">
@@ -36445,7 +36465,7 @@
       </c>
       <c r="H515" s="2" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="I515" s="7" t="inlineStr">
@@ -36455,14 +36475,14 @@
       </c>
       <c r="J515" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K515" s="2" t="n">
-        <v>383</v>
+        <v>2030</v>
       </c>
       <c r="L515" s="2" t="n">
-        <v>0.0282</v>
+        <v>0.1494</v>
       </c>
       <c r="M515" s="2" t="inlineStr">
         <is>
@@ -36472,19 +36492,19 @@
       <c r="N515" s="2" t="n"/>
       <c r="O515" s="2" t="inlineStr">
         <is>
-          <t>Los subsidios pueden no figurar como desempleo en afiliación</t>
+          <t>Puede haber empezado a cobrar en 2025</t>
         </is>
       </c>
       <c r="P515" s="2" t="inlineStr">
         <is>
-          <t>ingresos_prestacion_2024 &gt; 0 AND COALESCE(t_total_desempleo, 0) + COALESCE(t_total_mixto_empl_desempl, 0) = 0</t>
+          <t>cobra_pension_2024_5 = 'SI' AND ingresos_bruto_total_2024 IS NOT NULL AND ingresos_pension_y_bajas_2024 = 0</t>
         </is>
       </c>
     </row>
     <row r="516">
       <c r="A516" s="2" t="inlineStr">
         <is>
-          <t>C-310</t>
+          <t>C-314</t>
         </is>
       </c>
       <c r="B516" s="2" t="inlineStr">
@@ -36494,22 +36514,22 @@
       </c>
       <c r="C516" s="2" t="inlineStr">
         <is>
-          <t>Ingresos por tipo (v2.2)</t>
+          <t>Clave y subclave de percepción (v2.2)</t>
         </is>
       </c>
       <c r="D516" s="2" t="inlineStr">
         <is>
-          <t>ingresos_sueldo_2024</t>
+          <t>clave_subclave_ppal</t>
         </is>
       </c>
       <c r="E516" s="2" t="inlineStr">
         <is>
-          <t>fecha_ini_primer_empleo</t>
+          <t>ingresos_bruto_total_2024</t>
         </is>
       </c>
       <c r="F516" s="2" t="inlineStr">
         <is>
-          <t>Con sueldo en 2024 ⇒ tiene primer empleo en afiliación</t>
+          <t>clave_subclave_ppal = NO CONSTA ⇔ ingresos fiscales nulos o 0</t>
         </is>
       </c>
       <c r="G516" s="2" t="inlineStr">
@@ -36519,46 +36539,46 @@
       </c>
       <c r="H516" s="2" t="inlineStr">
         <is>
-          <t>Baja</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="I516" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J516" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Corregido</t>
         </is>
       </c>
       <c r="K516" s="2" t="n">
-        <v>211</v>
+        <v>0</v>
       </c>
       <c r="L516" s="2" t="n">
-        <v>0.0155</v>
+        <v>0</v>
       </c>
       <c r="M516" s="2" t="inlineStr">
         <is>
-          <t>G17</t>
+          <t>G16</t>
         </is>
       </c>
       <c r="N516" s="2" t="n"/>
       <c r="O516" s="2" t="inlineStr">
         <is>
-          <t>Los funcionarios de MUFACE no cotizan en el sistema de la MCVL</t>
+          <t>Regla reformulada 2026-09-24 (G16): la clave sale de la percepción con más ingresos; las 278 personas con fila fiscal a 0 no tienen ninguna que elegir. Con la regla nueva, 0 incumplimientos.</t>
         </is>
       </c>
       <c r="P516" s="2" t="inlineStr">
         <is>
-          <t>ingresos_sueldo_2024 &gt; 0 AND fecha_ini_primer_empleo IS NULL</t>
+          <t>(clave_subclave_ppal = 'NO CONSTA') &lt;&gt; (COALESCE(ingresos_bruto_total_2024, 0) = 0)</t>
         </is>
       </c>
     </row>
     <row r="517">
       <c r="A517" s="2" t="inlineStr">
         <is>
-          <t>C-311</t>
+          <t>C-315</t>
         </is>
       </c>
       <c r="B517" s="2" t="inlineStr">
@@ -36568,71 +36588,63 @@
       </c>
       <c r="C517" s="2" t="inlineStr">
         <is>
-          <t>Ingresos por tipo (v2.2)</t>
+          <t>Clave y subclave de percepción (v2.2)</t>
         </is>
       </c>
       <c r="D517" s="2" t="inlineStr">
         <is>
-          <t>ingresos_sueldo_2024</t>
-        </is>
-      </c>
-      <c r="E517" s="2" t="inlineStr">
-        <is>
-          <t>fecha_ultima_baja</t>
-        </is>
-      </c>
+          <t>clave_subclave_ppal</t>
+        </is>
+      </c>
+      <c r="E517" s="2" t="n"/>
       <c r="F517" s="2" t="inlineStr">
         <is>
-          <t>Con sueldo en 2024 ⇒ la última baja no es anterior a 2024</t>
+          <t>clave_subclave_ppal = 'letra + 2 (dígito/X)' con etiqueta, o NO CONSTA</t>
         </is>
       </c>
       <c r="G517" s="2" t="inlineStr">
         <is>
-          <t>Dominio (Seg. Social / lógica)</t>
+          <t>Guía MCVL</t>
         </is>
       </c>
       <c r="H517" s="2" t="inlineStr">
         <is>
-          <t>Media</t>
-        </is>
-      </c>
-      <c r="I517" s="7" t="inlineStr">
-        <is>
-          <t>INCUMPLE</t>
-        </is>
-      </c>
-      <c r="J517" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I517" s="6" t="inlineStr">
+        <is>
+          <t>PASA</t>
+        </is>
+      </c>
+      <c r="J517" s="6" t="inlineStr">
+        <is>
+          <t>Pasan</t>
         </is>
       </c>
       <c r="K517" s="2" t="n">
-        <v>3867</v>
+        <v>0</v>
       </c>
       <c r="L517" s="2" t="n">
-        <v>0.2845</v>
-      </c>
-      <c r="M517" s="2" t="inlineStr">
-        <is>
-          <t>G17</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M517" s="2" t="inlineStr"/>
       <c r="N517" s="2" t="n"/>
       <c r="O517" s="2" t="inlineStr">
         <is>
-          <t>Pagos atrasados o indemnizaciones podrían dar sueldo sin alta en 2024</t>
+          <t>Claves del modelo 190 presentes en la MCVL: A, B, C, F, G, H, L</t>
         </is>
       </c>
       <c r="P517" s="2" t="inlineStr">
         <is>
-          <t>ingresos_sueldo_2024 &gt; 0 AND fecha_ultima_baja IS NOT NULL AND year(fecha_ultima_baja) &lt; 2024</t>
+          <t>clave_subclave_ppal &lt;&gt; 'NO CONSTA' AND NOT regexp_matches(clave_subclave_ppal, '^[ABCFGHL][0-9X]{2}( .+)?$')</t>
         </is>
       </c>
     </row>
     <row r="518">
       <c r="A518" s="2" t="inlineStr">
         <is>
-          <t>C-312</t>
+          <t>C-316</t>
         </is>
       </c>
       <c r="B518" s="2" t="inlineStr">
@@ -36642,71 +36654,59 @@
       </c>
       <c r="C518" s="2" t="inlineStr">
         <is>
-          <t>Ingresos por tipo (v2.2)</t>
+          <t>Clave y subclave de percepción (v2.2)</t>
         </is>
       </c>
       <c r="D518" s="2" t="inlineStr">
         <is>
-          <t>ingresos_pension_2024</t>
-        </is>
-      </c>
-      <c r="E518" s="2" t="inlineStr">
-        <is>
-          <t>cobra_pension_2024_5</t>
-        </is>
-      </c>
+          <t>clave_subclave_ppal</t>
+        </is>
+      </c>
+      <c r="E518" s="2" t="n"/>
       <c r="F518" s="2" t="inlineStr">
         <is>
-          <t>Con pensión en fiscal ⇒ cobra pensión en la tabla de pensiones</t>
+          <t>Cada código de clave+subclave tiene una única etiqueta</t>
         </is>
       </c>
       <c r="G518" s="2" t="inlineStr">
         <is>
-          <t>Dominio (Seg. Social / lógica)</t>
+          <t>Significado del nombre</t>
         </is>
       </c>
       <c r="H518" s="2" t="inlineStr">
         <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I518" s="7" t="inlineStr">
-        <is>
-          <t>INCUMPLE</t>
-        </is>
-      </c>
-      <c r="J518" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I518" s="6" t="inlineStr">
+        <is>
+          <t>PASA</t>
+        </is>
+      </c>
+      <c r="J518" s="6" t="inlineStr">
+        <is>
+          <t>Pasan</t>
         </is>
       </c>
       <c r="K518" s="2" t="n">
-        <v>48780</v>
+        <v>0</v>
       </c>
       <c r="L518" s="2" t="n">
-        <v>3.5893</v>
-      </c>
-      <c r="M518" s="2" t="inlineStr">
-        <is>
-          <t>G17</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M518" s="2" t="inlineStr"/>
       <c r="N518" s="2" t="n"/>
-      <c r="O518" s="2" t="inlineStr">
-        <is>
-          <t>Mutualidades y Clases Pasivas pueden no estar en la tabla de pensiones de la MCVL</t>
-        </is>
-      </c>
+      <c r="O518" s="2" t="inlineStr"/>
       <c r="P518" s="2" t="inlineStr">
         <is>
-          <t>ingresos_pension_2024 &gt; 0 AND cobra_pension_2024_5 = 'NO'</t>
+          <t>split_part(clave_subclave_ppal, ' ', 1) IN (SELECT split_part(clave_subclave_ppal, ' ', 1) FROM personas WHERE clave_subclave_ppal &lt;&gt; 'NO CONSTA' GROUP BY 1 HAVING COUNT(DISTINCT clave_subclave_ppal) &gt; 1)</t>
         </is>
       </c>
     </row>
     <row r="519">
       <c r="A519" s="2" t="inlineStr">
         <is>
-          <t>C-313</t>
+          <t>C-317</t>
         </is>
       </c>
       <c r="B519" s="2" t="inlineStr">
@@ -36716,71 +36716,63 @@
       </c>
       <c r="C519" s="2" t="inlineStr">
         <is>
-          <t>Ingresos por tipo (v2.2)</t>
+          <t>Clave y subclave de percepción (v2.2)</t>
         </is>
       </c>
       <c r="D519" s="2" t="inlineStr">
         <is>
-          <t>cobra_pension_2024_5</t>
+          <t>clave_subclave_ppal</t>
         </is>
       </c>
       <c r="E519" s="2" t="inlineStr">
         <is>
-          <t>ingresos_pension_2024</t>
+          <t>ingresos_sueldo_2024</t>
         </is>
       </c>
       <c r="F519" s="2" t="inlineStr">
         <is>
-          <t>Cobra pensión en la tabla de pensiones ⇒ tiene pensión en fiscal (si consta en fiscal)</t>
+          <t>Tipo principal de sueldo (A) ⇒ ese importe es positivo</t>
         </is>
       </c>
       <c r="G519" s="2" t="inlineStr">
         <is>
-          <t>Dominio (Seg. Social / lógica)</t>
+          <t>Significado del nombre</t>
         </is>
       </c>
       <c r="H519" s="2" t="inlineStr">
         <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I519" s="7" t="inlineStr">
-        <is>
-          <t>INCUMPLE</t>
-        </is>
-      </c>
-      <c r="J519" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="I519" s="6" t="inlineStr">
+        <is>
+          <t>PASA</t>
+        </is>
+      </c>
+      <c r="J519" s="6" t="inlineStr">
+        <is>
+          <t>Pasan</t>
         </is>
       </c>
       <c r="K519" s="2" t="n">
-        <v>2030</v>
+        <v>0</v>
       </c>
       <c r="L519" s="2" t="n">
-        <v>0.1494</v>
-      </c>
-      <c r="M519" s="2" t="inlineStr">
-        <is>
-          <t>G17</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="M519" s="2" t="inlineStr"/>
       <c r="N519" s="2" t="n"/>
-      <c r="O519" s="2" t="inlineStr">
-        <is>
-          <t>Puede haber empezado a cobrar en 2025</t>
-        </is>
-      </c>
+      <c r="O519" s="2" t="inlineStr"/>
       <c r="P519" s="2" t="inlineStr">
         <is>
-          <t>cobra_pension_2024_5 = 'SI' AND ingresos_bruto_total_2024 IS NOT NULL AND ingresos_pension_2024 = 0</t>
+          <t>clave_subclave_ppal &lt;&gt; 'NO CONSTA' AND split_part(clave_subclave_ppal, ' ', 1) LIKE 'A%' AND COALESCE(ingresos_sueldo_2024, 0) &lt;= 0</t>
         </is>
       </c>
     </row>
     <row r="520">
       <c r="A520" s="2" t="inlineStr">
         <is>
-          <t>C-314</t>
+          <t>C-318</t>
         </is>
       </c>
       <c r="B520" s="2" t="inlineStr">
@@ -36800,12 +36792,12 @@
       </c>
       <c r="E520" s="2" t="inlineStr">
         <is>
-          <t>ingresos_bruto_total_2024</t>
+          <t>ingresos_pension_y_bajas_2024</t>
         </is>
       </c>
       <c r="F520" s="2" t="inlineStr">
         <is>
-          <t>clave_subclave_ppal = NO CONSTA ⇔ ingresos fiscales nulos o 0</t>
+          <t>Tipo principal de pensión (B, L06, L07, L08) ⇒ ese importe es positivo</t>
         </is>
       </c>
       <c r="G520" s="2" t="inlineStr">
@@ -36818,14 +36810,14 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="I520" s="7" t="inlineStr">
-        <is>
-          <t>PASA</t>
-        </is>
-      </c>
-      <c r="J520" s="5" t="inlineStr">
-        <is>
-          <t>Corregido</t>
+      <c r="I520" s="6" t="inlineStr">
+        <is>
+          <t>PASA</t>
+        </is>
+      </c>
+      <c r="J520" s="6" t="inlineStr">
+        <is>
+          <t>Pasan</t>
         </is>
       </c>
       <c r="K520" s="2" t="n">
@@ -36834,27 +36826,19 @@
       <c r="L520" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="M520" s="2" t="inlineStr">
-        <is>
-          <t>G16</t>
-        </is>
-      </c>
+      <c r="M520" s="2" t="inlineStr"/>
       <c r="N520" s="2" t="n"/>
-      <c r="O520" s="2" t="inlineStr">
-        <is>
-          <t>Regla reformulada 2026-09-24 (G16): la clave sale de la percepción con más ingresos; las 278 personas con fila fiscal a 0 no tienen ninguna que elegir. Con la regla nueva, 0 incumplimientos.</t>
-        </is>
-      </c>
+      <c r="O520" s="2" t="inlineStr"/>
       <c r="P520" s="2" t="inlineStr">
         <is>
-          <t>(clave_subclave_ppal = 'NO CONSTA') &lt;&gt; (COALESCE(ingresos_bruto_total_2024, 0) = 0)</t>
+          <t>clave_subclave_ppal &lt;&gt; 'NO CONSTA' AND (split_part(clave_subclave_ppal, ' ', 1) LIKE 'B%' OR split_part(clave_subclave_ppal, ' ', 1) IN ('L06','L07','L08')) AND COALESCE(ingresos_pension_y_bajas_2024, 0) &lt;= 0</t>
         </is>
       </c>
     </row>
     <row r="521">
       <c r="A521" s="2" t="inlineStr">
         <is>
-          <t>C-315</t>
+          <t>C-319</t>
         </is>
       </c>
       <c r="B521" s="2" t="inlineStr">
@@ -36872,15 +36856,19 @@
           <t>clave_subclave_ppal</t>
         </is>
       </c>
-      <c r="E521" s="2" t="inlineStr"/>
+      <c r="E521" s="2" t="inlineStr">
+        <is>
+          <t>ingresos_prestacion_2024</t>
+        </is>
+      </c>
       <c r="F521" s="2" t="inlineStr">
         <is>
-          <t>clave_subclave_ppal = 'letra + 2 (dígito/X)' con etiqueta, o NO CONSTA</t>
+          <t>Tipo principal de prestación (C) ⇒ ese importe es positivo</t>
         </is>
       </c>
       <c r="G521" s="2" t="inlineStr">
         <is>
-          <t>Guía MCVL</t>
+          <t>Significado del nombre</t>
         </is>
       </c>
       <c r="H521" s="2" t="inlineStr">
@@ -36906,21 +36894,17 @@
       </c>
       <c r="M521" s="2" t="inlineStr"/>
       <c r="N521" s="2" t="n"/>
-      <c r="O521" s="2" t="inlineStr">
-        <is>
-          <t>Claves del modelo 190 presentes en la MCVL: A, B, C, F, G, H, L</t>
-        </is>
-      </c>
+      <c r="O521" s="2" t="inlineStr"/>
       <c r="P521" s="2" t="inlineStr">
         <is>
-          <t>clave_subclave_ppal &lt;&gt; 'NO CONSTA' AND NOT regexp_matches(clave_subclave_ppal, '^[ABCFGHL][0-9X]{2}( .+)?$')</t>
+          <t>clave_subclave_ppal &lt;&gt; 'NO CONSTA' AND split_part(clave_subclave_ppal, ' ', 1) LIKE 'C%' AND COALESCE(ingresos_prestacion_2024, 0) &lt;= 0</t>
         </is>
       </c>
     </row>
     <row r="522">
       <c r="A522" s="2" t="inlineStr">
         <is>
-          <t>C-316</t>
+          <t>C-320</t>
         </is>
       </c>
       <c r="B522" s="2" t="inlineStr">
@@ -36938,10 +36922,14 @@
           <t>clave_subclave_ppal</t>
         </is>
       </c>
-      <c r="E522" s="2" t="inlineStr"/>
+      <c r="E522" s="2" t="inlineStr">
+        <is>
+          <t>ingresos_actividad_2024</t>
+        </is>
+      </c>
       <c r="F522" s="2" t="inlineStr">
         <is>
-          <t>Cada código de clave+subclave tiene una única etiqueta</t>
+          <t>Tipo principal de actividad (F, G, H) ⇒ ese importe es positivo</t>
         </is>
       </c>
       <c r="G522" s="2" t="inlineStr">
@@ -36975,14 +36963,14 @@
       <c r="O522" s="2" t="inlineStr"/>
       <c r="P522" s="2" t="inlineStr">
         <is>
-          <t>split_part(clave_subclave_ppal, ' ', 1) IN (SELECT split_part(clave_subclave_ppal, ' ', 1) FROM personas WHERE clave_subclave_ppal &lt;&gt; 'NO CONSTA' GROUP BY 1 HAVING COUNT(DISTINCT clave_subclave_ppal) &gt; 1)</t>
+          <t>clave_subclave_ppal &lt;&gt; 'NO CONSTA' AND (split_part(clave_subclave_ppal, ' ', 1) LIKE 'F%' OR split_part(clave_subclave_ppal, ' ', 1) LIKE 'G%' OR split_part(clave_subclave_ppal, ' ', 1) LIKE 'H%') AND COALESCE(ingresos_actividad_2024, 0) &lt;= 0</t>
         </is>
       </c>
     </row>
     <row r="523">
       <c r="A523" s="2" t="inlineStr">
         <is>
-          <t>C-317</t>
+          <t>C-321</t>
         </is>
       </c>
       <c r="B523" s="2" t="inlineStr">
@@ -37002,12 +36990,12 @@
       </c>
       <c r="E523" s="2" t="inlineStr">
         <is>
-          <t>ingresos_sueldo_2024</t>
+          <t>ingresos_otras_exentas_2024</t>
         </is>
       </c>
       <c r="F523" s="2" t="inlineStr">
         <is>
-          <t>Tipo principal de sueldo (A) ⇒ ese importe es positivo</t>
+          <t>Tipo principal de otras exentas (resto de L) ⇒ ese importe es positivo</t>
         </is>
       </c>
       <c r="G523" s="2" t="inlineStr">
@@ -37041,14 +37029,14 @@
       <c r="O523" s="2" t="inlineStr"/>
       <c r="P523" s="2" t="inlineStr">
         <is>
-          <t>clave_subclave_ppal &lt;&gt; 'NO CONSTA' AND split_part(clave_subclave_ppal, ' ', 1) LIKE 'A%' AND COALESCE(ingresos_sueldo_2024, 0) &lt;= 0</t>
+          <t>clave_subclave_ppal &lt;&gt; 'NO CONSTA' AND (split_part(clave_subclave_ppal, ' ', 1) LIKE 'L%' AND split_part(clave_subclave_ppal, ' ', 1) NOT IN ('L06','L07','L08')) AND COALESCE(ingresos_otras_exentas_2024, 0) &lt;= 0</t>
         </is>
       </c>
     </row>
     <row r="524">
       <c r="A524" s="2" t="inlineStr">
         <is>
-          <t>C-318</t>
+          <t>C-322</t>
         </is>
       </c>
       <c r="B524" s="2" t="inlineStr">
@@ -37063,17 +37051,17 @@
       </c>
       <c r="D524" s="2" t="inlineStr">
         <is>
-          <t>clave_subclave_ppal</t>
+          <t>clave_subclave_todas_cobradas</t>
         </is>
       </c>
       <c r="E524" s="2" t="inlineStr">
         <is>
-          <t>ingresos_pension_2024</t>
+          <t>ingresos_bruto_total_2024</t>
         </is>
       </c>
       <c r="F524" s="2" t="inlineStr">
         <is>
-          <t>Tipo principal de pensión (B, L06, L07, L08) ⇒ ese importe es positivo</t>
+          <t>Con lista de tipos cobrados ⇒ total de ingresos &gt; 0</t>
         </is>
       </c>
       <c r="G524" s="2" t="inlineStr">
@@ -37107,14 +37095,14 @@
       <c r="O524" s="2" t="inlineStr"/>
       <c r="P524" s="2" t="inlineStr">
         <is>
-          <t>clave_subclave_ppal &lt;&gt; 'NO CONSTA' AND (split_part(clave_subclave_ppal, ' ', 1) LIKE 'B%' OR split_part(clave_subclave_ppal, ' ', 1) IN ('L06','L07','L08')) AND COALESCE(ingresos_pension_2024, 0) &lt;= 0</t>
+          <t>clave_subclave_todas_cobradas IS NOT NULL AND COALESCE(ingresos_bruto_total_2024, 0) &lt;= 0</t>
         </is>
       </c>
     </row>
     <row r="525">
       <c r="A525" s="2" t="inlineStr">
         <is>
-          <t>C-319</t>
+          <t>C-323</t>
         </is>
       </c>
       <c r="B525" s="2" t="inlineStr">
@@ -37129,17 +37117,17 @@
       </c>
       <c r="D525" s="2" t="inlineStr">
         <is>
-          <t>clave_subclave_ppal</t>
+          <t>clave_subclave_todas_cobradas</t>
         </is>
       </c>
       <c r="E525" s="2" t="inlineStr">
         <is>
-          <t>ingresos_prestacion_2024</t>
+          <t>ingresos_bruto_total_2024</t>
         </is>
       </c>
       <c r="F525" s="2" t="inlineStr">
         <is>
-          <t>Tipo principal de prestación (C) ⇒ ese importe es positivo</t>
+          <t>Total de ingresos &gt; 0 ⇒ hay lista de tipos cobrados</t>
         </is>
       </c>
       <c r="G525" s="2" t="inlineStr">
@@ -37173,14 +37161,14 @@
       <c r="O525" s="2" t="inlineStr"/>
       <c r="P525" s="2" t="inlineStr">
         <is>
-          <t>clave_subclave_ppal &lt;&gt; 'NO CONSTA' AND split_part(clave_subclave_ppal, ' ', 1) LIKE 'C%' AND COALESCE(ingresos_prestacion_2024, 0) &lt;= 0</t>
+          <t>ingresos_bruto_total_2024 &gt; 0 AND clave_subclave_todas_cobradas IS NULL</t>
         </is>
       </c>
     </row>
     <row r="526">
       <c r="A526" s="2" t="inlineStr">
         <is>
-          <t>C-320</t>
+          <t>C-324</t>
         </is>
       </c>
       <c r="B526" s="2" t="inlineStr">
@@ -37195,17 +37183,17 @@
       </c>
       <c r="D526" s="2" t="inlineStr">
         <is>
+          <t>clave_subclave_todas_cobradas</t>
+        </is>
+      </c>
+      <c r="E526" s="2" t="inlineStr">
+        <is>
           <t>clave_subclave_ppal</t>
         </is>
       </c>
-      <c r="E526" s="2" t="inlineStr">
-        <is>
-          <t>ingresos_actividad_2024</t>
-        </is>
-      </c>
       <c r="F526" s="2" t="inlineStr">
         <is>
-          <t>Tipo principal de actividad (F, G, H) ⇒ ese importe es positivo</t>
+          <t>El primer tipo cobrado es el tipo principal</t>
         </is>
       </c>
       <c r="G526" s="2" t="inlineStr">
@@ -37239,14 +37227,14 @@
       <c r="O526" s="2" t="inlineStr"/>
       <c r="P526" s="2" t="inlineStr">
         <is>
-          <t>clave_subclave_ppal &lt;&gt; 'NO CONSTA' AND (split_part(clave_subclave_ppal, ' ', 1) LIKE 'F%' OR split_part(clave_subclave_ppal, ' ', 1) LIKE 'G%' OR split_part(clave_subclave_ppal, ' ', 1) LIKE 'H%') AND COALESCE(ingresos_actividad_2024, 0) &lt;= 0</t>
+          <t>clave_subclave_todas_cobradas IS NOT NULL AND clave_subclave_todas_cobradas[1] &lt;&gt; split_part(clave_subclave_ppal, ' ', 1)</t>
         </is>
       </c>
     </row>
     <row r="527">
       <c r="A527" s="2" t="inlineStr">
         <is>
-          <t>C-321</t>
+          <t>C-325</t>
         </is>
       </c>
       <c r="B527" s="2" t="inlineStr">
@@ -37261,17 +37249,13 @@
       </c>
       <c r="D527" s="2" t="inlineStr">
         <is>
-          <t>clave_subclave_ppal</t>
-        </is>
-      </c>
-      <c r="E527" s="2" t="inlineStr">
-        <is>
-          <t>ingresos_otras_exentas_2024</t>
-        </is>
-      </c>
+          <t>clave_subclave_todas_cobradas</t>
+        </is>
+      </c>
+      <c r="E527" s="2" t="n"/>
       <c r="F527" s="2" t="inlineStr">
         <is>
-          <t>Tipo principal de otras exentas (resto de L) ⇒ ese importe es positivo</t>
+          <t>La lista de tipos cobrados no repite códigos</t>
         </is>
       </c>
       <c r="G527" s="2" t="inlineStr">
@@ -37305,14 +37289,14 @@
       <c r="O527" s="2" t="inlineStr"/>
       <c r="P527" s="2" t="inlineStr">
         <is>
-          <t>clave_subclave_ppal &lt;&gt; 'NO CONSTA' AND (split_part(clave_subclave_ppal, ' ', 1) LIKE 'L%' AND split_part(clave_subclave_ppal, ' ', 1) NOT IN ('L06','L07','L08')) AND COALESCE(ingresos_otras_exentas_2024, 0) &lt;= 0</t>
+          <t>clave_subclave_todas_cobradas IS NOT NULL AND len(clave_subclave_todas_cobradas) &lt;&gt; len(list_distinct(clave_subclave_todas_cobradas))</t>
         </is>
       </c>
     </row>
     <row r="528">
       <c r="A528" s="2" t="inlineStr">
         <is>
-          <t>C-322</t>
+          <t>C-326</t>
         </is>
       </c>
       <c r="B528" s="2" t="inlineStr">
@@ -37330,19 +37314,15 @@
           <t>clave_subclave_todas_cobradas</t>
         </is>
       </c>
-      <c r="E528" s="2" t="inlineStr">
-        <is>
-          <t>ingresos_bruto_total_2024</t>
-        </is>
-      </c>
+      <c r="E528" s="2" t="n"/>
       <c r="F528" s="2" t="inlineStr">
         <is>
-          <t>Con lista de tipos cobrados ⇒ total de ingresos &gt; 0</t>
+          <t>Los códigos de la lista tienen formato letra + 2 (dígito/X)</t>
         </is>
       </c>
       <c r="G528" s="2" t="inlineStr">
         <is>
-          <t>Significado del nombre</t>
+          <t>Guía MCVL</t>
         </is>
       </c>
       <c r="H528" s="2" t="inlineStr">
@@ -37371,14 +37351,14 @@
       <c r="O528" s="2" t="inlineStr"/>
       <c r="P528" s="2" t="inlineStr">
         <is>
-          <t>clave_subclave_todas_cobradas IS NOT NULL AND COALESCE(ingresos_bruto_total_2024, 0) &lt;= 0</t>
+          <t>clave_subclave_todas_cobradas IS NOT NULL AND len(list_filter(clave_subclave_todas_cobradas, x -&gt; NOT regexp_matches(x, '^[ABCFGHL][0-9X]{2}$'))) &gt; 0</t>
         </is>
       </c>
     </row>
     <row r="529">
       <c r="A529" s="2" t="inlineStr">
         <is>
-          <t>C-323</t>
+          <t>C-327</t>
         </is>
       </c>
       <c r="B529" s="2" t="inlineStr">
@@ -37396,14 +37376,10 @@
           <t>clave_subclave_todas_cobradas</t>
         </is>
       </c>
-      <c r="E529" s="2" t="inlineStr">
-        <is>
-          <t>ingresos_bruto_total_2024</t>
-        </is>
-      </c>
+      <c r="E529" s="2" t="n"/>
       <c r="F529" s="2" t="inlineStr">
         <is>
-          <t>Total de ingresos &gt; 0 ⇒ hay lista de tipos cobrados</t>
+          <t>Sin tipos cobrados ⇒ NULL, no lista vacía</t>
         </is>
       </c>
       <c r="G529" s="2" t="inlineStr">
@@ -37413,7 +37389,7 @@
       </c>
       <c r="H529" s="2" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I529" s="6" t="inlineStr">
@@ -37437,14 +37413,14 @@
       <c r="O529" s="2" t="inlineStr"/>
       <c r="P529" s="2" t="inlineStr">
         <is>
-          <t>ingresos_bruto_total_2024 &gt; 0 AND clave_subclave_todas_cobradas IS NULL</t>
+          <t>clave_subclave_todas_cobradas IS NOT NULL AND len(clave_subclave_todas_cobradas) = 0</t>
         </is>
       </c>
     </row>
     <row r="530">
       <c r="A530" s="2" t="inlineStr">
         <is>
-          <t>C-324</t>
+          <t>C-328</t>
         </is>
       </c>
       <c r="B530" s="2" t="inlineStr">
@@ -37464,12 +37440,12 @@
       </c>
       <c r="E530" s="2" t="inlineStr">
         <is>
-          <t>clave_subclave_ppal</t>
+          <t>ingresos_sueldo_2024</t>
         </is>
       </c>
       <c r="F530" s="2" t="inlineStr">
         <is>
-          <t>El primer tipo cobrado es el tipo principal</t>
+          <t>A00 en la lista ⇔ sueldo positivo</t>
         </is>
       </c>
       <c r="G530" s="2" t="inlineStr">
@@ -37503,14 +37479,14 @@
       <c r="O530" s="2" t="inlineStr"/>
       <c r="P530" s="2" t="inlineStr">
         <is>
-          <t>clave_subclave_todas_cobradas IS NOT NULL AND clave_subclave_todas_cobradas[1] &lt;&gt; split_part(clave_subclave_ppal, ' ', 1)</t>
+          <t>COALESCE(list_contains(clave_subclave_todas_cobradas, 'A00'), false) &lt;&gt; (COALESCE(ingresos_sueldo_2024, 0) &gt; 0)</t>
         </is>
       </c>
     </row>
     <row r="531">
       <c r="A531" s="2" t="inlineStr">
         <is>
-          <t>C-325</t>
+          <t>C-329</t>
         </is>
       </c>
       <c r="B531" s="2" t="inlineStr">
@@ -37528,10 +37504,14 @@
           <t>clave_subclave_todas_cobradas</t>
         </is>
       </c>
-      <c r="E531" s="2" t="inlineStr"/>
+      <c r="E531" s="2" t="inlineStr">
+        <is>
+          <t>ingresos_prestacion_2024</t>
+        </is>
+      </c>
       <c r="F531" s="2" t="inlineStr">
         <is>
-          <t>La lista de tipos cobrados no repite códigos</t>
+          <t>C00 en la lista ⇔ prestación positiva</t>
         </is>
       </c>
       <c r="G531" s="2" t="inlineStr">
@@ -37565,14 +37545,14 @@
       <c r="O531" s="2" t="inlineStr"/>
       <c r="P531" s="2" t="inlineStr">
         <is>
-          <t>clave_subclave_todas_cobradas IS NOT NULL AND len(clave_subclave_todas_cobradas) &lt;&gt; len(list_distinct(clave_subclave_todas_cobradas))</t>
+          <t>COALESCE(list_contains(clave_subclave_todas_cobradas, 'C00'), false) &lt;&gt; (COALESCE(ingresos_prestacion_2024, 0) &gt; 0)</t>
         </is>
       </c>
     </row>
     <row r="532">
       <c r="A532" s="2" t="inlineStr">
         <is>
-          <t>C-326</t>
+          <t>C-330</t>
         </is>
       </c>
       <c r="B532" s="2" t="inlineStr">
@@ -37582,18 +37562,22 @@
       </c>
       <c r="C532" s="2" t="inlineStr">
         <is>
-          <t>Clave y subclave de percepción (v2.2)</t>
+          <t>Fallecimiento (v2.2)</t>
         </is>
       </c>
       <c r="D532" s="2" t="inlineStr">
         <is>
-          <t>clave_subclave_todas_cobradas</t>
-        </is>
-      </c>
-      <c r="E532" s="2" t="inlineStr"/>
+          <t>ha_fallecido</t>
+        </is>
+      </c>
+      <c r="E532" s="2" t="inlineStr">
+        <is>
+          <t>fecha_fallecimiento</t>
+        </is>
+      </c>
       <c r="F532" s="2" t="inlineStr">
         <is>
-          <t>Los códigos de la lista tienen formato letra + 2 (dígito/X)</t>
+          <t>ha_fallecido = SI ⇔ fecha_fallecimiento informada</t>
         </is>
       </c>
       <c r="G532" s="2" t="inlineStr">
@@ -37627,14 +37611,14 @@
       <c r="O532" s="2" t="inlineStr"/>
       <c r="P532" s="2" t="inlineStr">
         <is>
-          <t>clave_subclave_todas_cobradas IS NOT NULL AND len(list_filter(clave_subclave_todas_cobradas, x -&gt; NOT regexp_matches(x, '^[ABCFGHL][0-9X]{2}$'))) &gt; 0</t>
+          <t>(ha_fallecido = 'SI') &lt;&gt; (COALESCE(fecha_fallecimiento, 0) &lt;&gt; 0)</t>
         </is>
       </c>
     </row>
     <row r="533">
       <c r="A533" s="2" t="inlineStr">
         <is>
-          <t>C-327</t>
+          <t>C-331</t>
         </is>
       </c>
       <c r="B533" s="2" t="inlineStr">
@@ -37644,18 +37628,22 @@
       </c>
       <c r="C533" s="2" t="inlineStr">
         <is>
-          <t>Clave y subclave de percepción (v2.2)</t>
+          <t>Fallecimiento (v2.2)</t>
         </is>
       </c>
       <c r="D533" s="2" t="inlineStr">
         <is>
-          <t>clave_subclave_todas_cobradas</t>
-        </is>
-      </c>
-      <c r="E533" s="2" t="inlineStr"/>
+          <t>ha_fallecido</t>
+        </is>
+      </c>
+      <c r="E533" s="2" t="inlineStr">
+        <is>
+          <t>edad_fallecimiento</t>
+        </is>
+      </c>
       <c r="F533" s="2" t="inlineStr">
         <is>
-          <t>Sin tipos cobrados ⇒ NULL, no lista vacía</t>
+          <t>ha_fallecido = SI ⇔ edad_fallecimiento informada</t>
         </is>
       </c>
       <c r="G533" s="2" t="inlineStr">
@@ -37665,7 +37653,7 @@
       </c>
       <c r="H533" s="2" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="I533" s="6" t="inlineStr">
@@ -37689,14 +37677,14 @@
       <c r="O533" s="2" t="inlineStr"/>
       <c r="P533" s="2" t="inlineStr">
         <is>
-          <t>clave_subclave_todas_cobradas IS NOT NULL AND len(clave_subclave_todas_cobradas) = 0</t>
+          <t>(ha_fallecido = 'SI') &lt;&gt; (edad_fallecimiento IS NOT NULL)</t>
         </is>
       </c>
     </row>
     <row r="534">
       <c r="A534" s="2" t="inlineStr">
         <is>
-          <t>C-328</t>
+          <t>C-332</t>
         </is>
       </c>
       <c r="B534" s="2" t="inlineStr">
@@ -37706,22 +37694,18 @@
       </c>
       <c r="C534" s="2" t="inlineStr">
         <is>
-          <t>Clave y subclave de percepción (v2.2)</t>
+          <t>Fallecimiento (v2.2)</t>
         </is>
       </c>
       <c r="D534" s="2" t="inlineStr">
         <is>
-          <t>clave_subclave_todas_cobradas</t>
-        </is>
-      </c>
-      <c r="E534" s="2" t="inlineStr">
-        <is>
-          <t>ingresos_sueldo_2024</t>
-        </is>
-      </c>
+          <t>edad_fallecimiento</t>
+        </is>
+      </c>
+      <c r="E534" s="2" t="n"/>
       <c r="F534" s="2" t="inlineStr">
         <is>
-          <t>A00 en la lista ⇔ sueldo positivo</t>
+          <t>edad_fallecimiento ≥ 0 (no se muere antes de nacer)</t>
         </is>
       </c>
       <c r="G534" s="2" t="inlineStr">
@@ -37755,14 +37739,14 @@
       <c r="O534" s="2" t="inlineStr"/>
       <c r="P534" s="2" t="inlineStr">
         <is>
-          <t>COALESCE(list_contains(clave_subclave_todas_cobradas, 'A00'), false) &lt;&gt; (COALESCE(ingresos_sueldo_2024, 0) &gt; 0)</t>
+          <t>edad_fallecimiento &lt; 0</t>
         </is>
       </c>
     </row>
     <row r="535">
       <c r="A535" s="2" t="inlineStr">
         <is>
-          <t>C-329</t>
+          <t>C-333</t>
         </is>
       </c>
       <c r="B535" s="2" t="inlineStr">
@@ -37772,32 +37756,28 @@
       </c>
       <c r="C535" s="2" t="inlineStr">
         <is>
-          <t>Clave y subclave de percepción (v2.2)</t>
+          <t>Fallecimiento (v2.2)</t>
         </is>
       </c>
       <c r="D535" s="2" t="inlineStr">
         <is>
-          <t>clave_subclave_todas_cobradas</t>
-        </is>
-      </c>
-      <c r="E535" s="2" t="inlineStr">
-        <is>
-          <t>ingresos_prestacion_2024</t>
-        </is>
-      </c>
+          <t>edad_fallecimiento</t>
+        </is>
+      </c>
+      <c r="E535" s="2" t="n"/>
       <c r="F535" s="2" t="inlineStr">
         <is>
-          <t>C00 en la lista ⇔ prestación positiva</t>
+          <t>edad_fallecimiento ≤ 115</t>
         </is>
       </c>
       <c r="G535" s="2" t="inlineStr">
         <is>
-          <t>Significado del nombre</t>
+          <t>Dominio (Seg. Social / lógica)</t>
         </is>
       </c>
       <c r="H535" s="2" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="I535" s="6" t="inlineStr">
@@ -37821,14 +37801,14 @@
       <c r="O535" s="2" t="inlineStr"/>
       <c r="P535" s="2" t="inlineStr">
         <is>
-          <t>COALESCE(list_contains(clave_subclave_todas_cobradas, 'C00'), false) &lt;&gt; (COALESCE(ingresos_prestacion_2024, 0) &gt; 0)</t>
+          <t>edad_fallecimiento &gt; 115</t>
         </is>
       </c>
     </row>
     <row r="536">
       <c r="A536" s="2" t="inlineStr">
         <is>
-          <t>C-330</t>
+          <t>C-334</t>
         </is>
       </c>
       <c r="B536" s="2" t="inlineStr">
@@ -37843,22 +37823,22 @@
       </c>
       <c r="D536" s="2" t="inlineStr">
         <is>
-          <t>ha_fallecido</t>
+          <t>edad_fallecimiento</t>
         </is>
       </c>
       <c r="E536" s="2" t="inlineStr">
         <is>
-          <t>fecha_fallecimiento</t>
+          <t>edad_actual_fecha_corte</t>
         </is>
       </c>
       <c r="F536" s="2" t="inlineStr">
         <is>
-          <t>ha_fallecido = SI ⇔ fecha_fallecimiento informada</t>
+          <t>Fallecidos: edad_actual_fecha_corte = edad_fallecimiento (la edad se calcula a la fecha de fallecimiento)</t>
         </is>
       </c>
       <c r="G536" s="2" t="inlineStr">
         <is>
-          <t>Guía MCVL</t>
+          <t>Significado del nombre</t>
         </is>
       </c>
       <c r="H536" s="2" t="inlineStr">
@@ -37884,17 +37864,21 @@
       </c>
       <c r="M536" s="2" t="inlineStr"/>
       <c r="N536" s="2" t="n"/>
-      <c r="O536" s="2" t="inlineStr"/>
+      <c r="O536" s="2" t="inlineStr">
+        <is>
+          <t>Comprobación pedida por el usuario 2026-09-21</t>
+        </is>
+      </c>
       <c r="P536" s="2" t="inlineStr">
         <is>
-          <t>(ha_fallecido = 'SI') &lt;&gt; (COALESCE(fecha_fallecimiento, 0) &lt;&gt; 0)</t>
+          <t>ha_fallecido = 'SI' AND ABS(edad_actual_fecha_corte - edad_fallecimiento) &gt; 0.01</t>
         </is>
       </c>
     </row>
     <row r="537">
       <c r="A537" s="2" t="inlineStr">
         <is>
-          <t>C-331</t>
+          <t>C-335</t>
         </is>
       </c>
       <c r="B537" s="2" t="inlineStr">
@@ -37909,17 +37893,17 @@
       </c>
       <c r="D537" s="2" t="inlineStr">
         <is>
-          <t>ha_fallecido</t>
+          <t>edad_fallecimiento</t>
         </is>
       </c>
       <c r="E537" s="2" t="inlineStr">
         <is>
-          <t>edad_fallecimiento</t>
+          <t>fecha_fallecimiento</t>
         </is>
       </c>
       <c r="F537" s="2" t="inlineStr">
         <is>
-          <t>ha_fallecido = SI ⇔ edad_fallecimiento informada</t>
+          <t>edad_fallecimiento = meses entre nacimiento y fallecimiento / 12 (±0,001)</t>
         </is>
       </c>
       <c r="G537" s="2" t="inlineStr">
@@ -37953,14 +37937,14 @@
       <c r="O537" s="2" t="inlineStr"/>
       <c r="P537" s="2" t="inlineStr">
         <is>
-          <t>(ha_fallecido = 'SI') &lt;&gt; (edad_fallecimiento IS NOT NULL)</t>
+          <t>ha_fallecido = 'SI' AND ABS(edad_fallecimiento - (((fecha_fallecimiento // 100 - year(fecha_nacimiento)) * 12 + (fecha_fallecimiento % 100 - month(fecha_nacimiento))) / 12.0)) &gt; 0.001</t>
         </is>
       </c>
     </row>
     <row r="538">
       <c r="A538" s="2" t="inlineStr">
         <is>
-          <t>C-332</t>
+          <t>C-336</t>
         </is>
       </c>
       <c r="B538" s="2" t="inlineStr">
@@ -37970,18 +37954,22 @@
       </c>
       <c r="C538" s="2" t="inlineStr">
         <is>
-          <t>Fallecimiento (v2.2)</t>
+          <t>Residencia (v2.2)</t>
         </is>
       </c>
       <c r="D538" s="2" t="inlineStr">
         <is>
-          <t>edad_fallecimiento</t>
-        </is>
-      </c>
-      <c r="E538" s="2" t="inlineStr"/>
+          <t>domic_resid_habitual</t>
+        </is>
+      </c>
+      <c r="E538" s="2" t="inlineStr">
+        <is>
+          <t>prov_resid_habitual</t>
+        </is>
+      </c>
       <c r="F538" s="2" t="inlineStr">
         <is>
-          <t>edad_fallecimiento ≥ 0 (no se muere antes de nacer)</t>
+          <t>domicilio NO CONSTA ⇔ provincia de residencia NO CONSTA</t>
         </is>
       </c>
       <c r="G538" s="2" t="inlineStr">
@@ -38015,14 +38003,14 @@
       <c r="O538" s="2" t="inlineStr"/>
       <c r="P538" s="2" t="inlineStr">
         <is>
-          <t>edad_fallecimiento &lt; 0</t>
+          <t>(domic_resid_habitual = 'NO CONSTA') &lt;&gt; (prov_resid_habitual = 'NO CONSTA')</t>
         </is>
       </c>
     </row>
     <row r="539">
       <c r="A539" s="2" t="inlineStr">
         <is>
-          <t>C-333</t>
+          <t>C-337</t>
         </is>
       </c>
       <c r="B539" s="2" t="inlineStr">
@@ -38032,28 +38020,32 @@
       </c>
       <c r="C539" s="2" t="inlineStr">
         <is>
-          <t>Fallecimiento (v2.2)</t>
+          <t>Residencia (v2.2)</t>
         </is>
       </c>
       <c r="D539" s="2" t="inlineStr">
         <is>
-          <t>edad_fallecimiento</t>
-        </is>
-      </c>
-      <c r="E539" s="2" t="inlineStr"/>
+          <t>domic_resid_habitual</t>
+        </is>
+      </c>
+      <c r="E539" s="2" t="inlineStr">
+        <is>
+          <t>prov_resid_habitual</t>
+        </is>
+      </c>
       <c r="F539" s="2" t="inlineStr">
         <is>
-          <t>edad_fallecimiento ≤ 115</t>
+          <t>El código de provincia del domicilio coincide con prov_resid_habitual</t>
         </is>
       </c>
       <c r="G539" s="2" t="inlineStr">
         <is>
-          <t>Dominio (Seg. Social / lógica)</t>
+          <t>Significado del nombre</t>
         </is>
       </c>
       <c r="H539" s="2" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="I539" s="6" t="inlineStr">
@@ -38077,14 +38069,14 @@
       <c r="O539" s="2" t="inlineStr"/>
       <c r="P539" s="2" t="inlineStr">
         <is>
-          <t>edad_fallecimiento &gt; 115</t>
+          <t>domic_resid_habitual &lt;&gt; 'NO CONSTA' AND split_part(prov_resid_habitual, ' ', 1) &lt;&gt; left(domic_resid_habitual, 2)</t>
         </is>
       </c>
     </row>
     <row r="540">
       <c r="A540" s="2" t="inlineStr">
         <is>
-          <t>C-334</t>
+          <t>C-338</t>
         </is>
       </c>
       <c r="B540" s="2" t="inlineStr">
@@ -38094,332 +38086,64 @@
       </c>
       <c r="C540" s="2" t="inlineStr">
         <is>
-          <t>Fallecimiento (v2.2)</t>
+          <t>Residencia (v2.2)</t>
         </is>
       </c>
       <c r="D540" s="2" t="inlineStr">
         <is>
-          <t>edad_fallecimiento</t>
+          <t>domic_resid_habitual</t>
         </is>
       </c>
       <c r="E540" s="2" t="inlineStr">
         <is>
-          <t>edad_actual_fecha_corte</t>
+          <t>prov_fiscal_actual</t>
         </is>
       </c>
       <c r="F540" s="2" t="inlineStr">
         <is>
-          <t>Fallecidos: edad_actual_fecha_corte = edad_fallecimiento (la edad se calcula a la fecha de fallecimiento)</t>
+          <t>La provincia de residencia coincide con la provincia fiscal</t>
         </is>
       </c>
       <c r="G540" s="2" t="inlineStr">
         <is>
-          <t>Significado del nombre</t>
+          <t>Dominio (Seg. Social / lógica)</t>
         </is>
       </c>
       <c r="H540" s="2" t="inlineStr">
         <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="I540" s="6" t="inlineStr">
-        <is>
-          <t>PASA</t>
-        </is>
-      </c>
-      <c r="J540" s="6" t="inlineStr">
-        <is>
-          <t>Pasan</t>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="I540" s="7" t="inlineStr">
+        <is>
+          <t>INCUMPLE</t>
+        </is>
+      </c>
+      <c r="J540" s="5" t="inlineStr">
+        <is>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K540" s="2" t="n">
-        <v>0</v>
+        <v>61583</v>
       </c>
       <c r="L540" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M540" s="2" t="inlineStr"/>
+        <v>4.5313</v>
+      </c>
+      <c r="M540" s="2" t="inlineStr">
+        <is>
+          <t>G17</t>
+        </is>
+      </c>
       <c r="N540" s="2" t="n"/>
       <c r="O540" s="2" t="inlineStr">
         <is>
-          <t>Comprobación pedida por el usuario 2026-09-21</t>
+          <t>El domicilio fiscal es el del 31-12-2024; puede haber mudanzas | Regla ajustada 2026-09-24: el 53 fiscal (Isla de La Palma) es provincia 38 en el INE y el 98 (residencia fiscal en el extranjero) no es comparable.</t>
         </is>
       </c>
       <c r="P540" s="2" t="inlineStr">
         <is>
-          <t>ha_fallecido = 'SI' AND ABS(edad_actual_fecha_corte - edad_fallecimiento) &gt; 0.01</t>
-        </is>
-      </c>
-    </row>
-    <row r="541">
-      <c r="A541" s="2" t="inlineStr">
-        <is>
-          <t>C-335</t>
-        </is>
-      </c>
-      <c r="B541" s="2" t="inlineStr">
-        <is>
-          <t>C · otras columnas</t>
-        </is>
-      </c>
-      <c r="C541" s="2" t="inlineStr">
-        <is>
-          <t>Fallecimiento (v2.2)</t>
-        </is>
-      </c>
-      <c r="D541" s="2" t="inlineStr">
-        <is>
-          <t>edad_fallecimiento</t>
-        </is>
-      </c>
-      <c r="E541" s="2" t="inlineStr">
-        <is>
-          <t>fecha_fallecimiento</t>
-        </is>
-      </c>
-      <c r="F541" s="2" t="inlineStr">
-        <is>
-          <t>edad_fallecimiento = meses entre nacimiento y fallecimiento / 12 (±0,001)</t>
-        </is>
-      </c>
-      <c r="G541" s="2" t="inlineStr">
-        <is>
-          <t>Significado del nombre</t>
-        </is>
-      </c>
-      <c r="H541" s="2" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="I541" s="6" t="inlineStr">
-        <is>
-          <t>PASA</t>
-        </is>
-      </c>
-      <c r="J541" s="6" t="inlineStr">
-        <is>
-          <t>Pasan</t>
-        </is>
-      </c>
-      <c r="K541" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L541" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M541" s="2" t="inlineStr"/>
-      <c r="N541" s="2" t="n"/>
-      <c r="O541" s="2" t="inlineStr"/>
-      <c r="P541" s="2" t="inlineStr">
-        <is>
-          <t>ha_fallecido = 'SI' AND ABS(edad_fallecimiento - (((fecha_fallecimiento // 100 - year(fecha_nacimiento)) * 12 + (fecha_fallecimiento % 100 - month(fecha_nacimiento))) / 12.0)) &gt; 0.001</t>
-        </is>
-      </c>
-    </row>
-    <row r="542">
-      <c r="A542" s="2" t="inlineStr">
-        <is>
-          <t>C-336</t>
-        </is>
-      </c>
-      <c r="B542" s="2" t="inlineStr">
-        <is>
-          <t>C · otras columnas</t>
-        </is>
-      </c>
-      <c r="C542" s="2" t="inlineStr">
-        <is>
-          <t>Residencia (v2.2)</t>
-        </is>
-      </c>
-      <c r="D542" s="2" t="inlineStr">
-        <is>
-          <t>domic_resid_habitual</t>
-        </is>
-      </c>
-      <c r="E542" s="2" t="inlineStr">
-        <is>
-          <t>prov_resid_habitual</t>
-        </is>
-      </c>
-      <c r="F542" s="2" t="inlineStr">
-        <is>
-          <t>domicilio NO CONSTA ⇔ provincia de residencia NO CONSTA</t>
-        </is>
-      </c>
-      <c r="G542" s="2" t="inlineStr">
-        <is>
-          <t>Significado del nombre</t>
-        </is>
-      </c>
-      <c r="H542" s="2" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="I542" s="6" t="inlineStr">
-        <is>
-          <t>PASA</t>
-        </is>
-      </c>
-      <c r="J542" s="6" t="inlineStr">
-        <is>
-          <t>Pasan</t>
-        </is>
-      </c>
-      <c r="K542" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L542" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M542" s="2" t="inlineStr"/>
-      <c r="N542" s="2" t="n"/>
-      <c r="O542" s="2" t="inlineStr"/>
-      <c r="P542" s="2" t="inlineStr">
-        <is>
-          <t>(domic_resid_habitual = 'NO CONSTA') &lt;&gt; (prov_resid_habitual = 'NO CONSTA')</t>
-        </is>
-      </c>
-    </row>
-    <row r="543">
-      <c r="A543" s="2" t="inlineStr">
-        <is>
-          <t>C-337</t>
-        </is>
-      </c>
-      <c r="B543" s="2" t="inlineStr">
-        <is>
-          <t>C · otras columnas</t>
-        </is>
-      </c>
-      <c r="C543" s="2" t="inlineStr">
-        <is>
-          <t>Residencia (v2.2)</t>
-        </is>
-      </c>
-      <c r="D543" s="2" t="inlineStr">
-        <is>
-          <t>domic_resid_habitual</t>
-        </is>
-      </c>
-      <c r="E543" s="2" t="inlineStr">
-        <is>
-          <t>prov_resid_habitual</t>
-        </is>
-      </c>
-      <c r="F543" s="2" t="inlineStr">
-        <is>
-          <t>El código de provincia del domicilio coincide con prov_resid_habitual</t>
-        </is>
-      </c>
-      <c r="G543" s="2" t="inlineStr">
-        <is>
-          <t>Significado del nombre</t>
-        </is>
-      </c>
-      <c r="H543" s="2" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="I543" s="6" t="inlineStr">
-        <is>
-          <t>PASA</t>
-        </is>
-      </c>
-      <c r="J543" s="6" t="inlineStr">
-        <is>
-          <t>Pasan</t>
-        </is>
-      </c>
-      <c r="K543" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L543" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M543" s="2" t="inlineStr"/>
-      <c r="N543" s="2" t="n"/>
-      <c r="O543" s="2" t="inlineStr"/>
-      <c r="P543" s="2" t="inlineStr">
-        <is>
-          <t>domic_resid_habitual &lt;&gt; 'NO CONSTA' AND split_part(prov_resid_habitual, ' ', 1) &lt;&gt; left(domic_resid_habitual, 2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="544">
-      <c r="A544" s="2" t="inlineStr">
-        <is>
-          <t>C-338</t>
-        </is>
-      </c>
-      <c r="B544" s="2" t="inlineStr">
-        <is>
-          <t>C · otras columnas</t>
-        </is>
-      </c>
-      <c r="C544" s="2" t="inlineStr">
-        <is>
-          <t>Residencia (v2.2)</t>
-        </is>
-      </c>
-      <c r="D544" s="2" t="inlineStr">
-        <is>
-          <t>domic_resid_habitual</t>
-        </is>
-      </c>
-      <c r="E544" s="2" t="inlineStr">
-        <is>
-          <t>prov_fiscal_actual</t>
-        </is>
-      </c>
-      <c r="F544" s="2" t="inlineStr">
-        <is>
-          <t>La provincia de residencia coincide con la provincia fiscal</t>
-        </is>
-      </c>
-      <c r="G544" s="2" t="inlineStr">
-        <is>
-          <t>Dominio (Seg. Social / lógica)</t>
-        </is>
-      </c>
-      <c r="H544" s="2" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="I544" s="7" t="inlineStr">
-        <is>
-          <t>INCUMPLE</t>
-        </is>
-      </c>
-      <c r="J544" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="K544" s="2" t="n">
-        <v>61583</v>
-      </c>
-      <c r="L544" s="2" t="n">
-        <v>4.5313</v>
-      </c>
-      <c r="M544" s="2" t="inlineStr">
-        <is>
-          <t>G17</t>
-        </is>
-      </c>
-      <c r="N544" s="2" t="n"/>
-      <c r="O544" s="2" t="inlineStr">
-        <is>
-          <t>El domicilio fiscal es el del 31-12-2024; puede haber mudanzas | Regla ajustada 2026-09-24: el 53 fiscal (Isla de La Palma) es provincia 38 en el INE y el 98 (residencia fiscal en el extranjero) no es comparable.</t>
-        </is>
-      </c>
-      <c r="P544" s="2" t="inlineStr">
-        <is>
-          <t>(domic_resid_habitual IS NOT NULL AND domic_resid_habitual NOT IN ('NO CONSTA','No consta','0 NO CONSTA','00 No consta')) AND (prov_fiscal_actual IS NOT NULL AND prov_fiscal_actual NOT IN ('NO CONSTA','No consta','0 NO CONSTA','00 No consta')) AND split_part(prov_fiscal_actual, ' ', 1) &lt;&gt; left(domic_resid_habitual, 2)</t>
+          <t>(domic_resid_habitual IS NOT NULL AND domic_resid_habitual NOT IN ('NO CONSTA','No consta','0 NO CONSTA','00 No consta')) AND (prov_fiscal_actual IS NOT NULL AND prov_fiscal_actual NOT IN ('NO CONSTA','No consta','0 NO CONSTA','00 No consta')) AND CASE WHEN split_part(prov_fiscal_actual, ' ', 1) = '53' THEN '38' ELSE split_part(prov_fiscal_actual, ' ', 1) END &lt;&gt; left(domic_resid_habitual, 2) AND split_part(prov_fiscal_actual, ' ', 1) &lt;&gt; '98'</t>
         </is>
       </c>
     </row>
@@ -38505,13 +38229,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="C4" t="n">
         <v>237</v>
       </c>
       <c r="D4" t="n">
-        <v>85</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5">
@@ -38521,13 +38245,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>543</v>
+        <v>539</v>
       </c>
       <c r="C5" t="n">
         <v>411</v>
       </c>
       <c r="D5" t="n">
-        <v>132</v>
+        <v>128</v>
       </c>
     </row>
     <row r="6"/>
@@ -38592,13 +38316,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C10" t="n">
         <v>18</v>
       </c>
       <c r="D10" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="11"/>
@@ -38641,7 +38365,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>37</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16">
@@ -38651,7 +38375,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>73</v>
+        <v>80</v>
       </c>
     </row>
     <row r="17"/>

</xml_diff>

<commit_message>
reglas: G06 - B-060/B-061/B-090/B-091 reformuladas; jubilados con poco empleo afiliado como baja calidad
B-060/B-061/B-090/B-091 suman el tiempo mixto y excluyen a quien solo tiene prestaciones o subsidios (G08): 560/544/1/1 -> 8/0/0/0 (las 8 con episodios de 1979-1984 con baja anterior al alta). A-105, C-158, C-159, C-157, A-064 y A-072 quedan como baja calidad de los datos (SOVI y carreras anteriores a 1967: 5.479 de 6.773 en A-105 y 7.607 de 16.660 en C-158 con pension SOVI). G06 cerrado.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/reglas_consistencia_resultados_sin_ipf.xlsx
+++ b/tests/reglas_consistencia_resultados_sin_ipf.xlsx
@@ -844,11 +844,11 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>16660</v>
@@ -858,12 +858,12 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>A-064, A-072, A-105, B-060, B-061, B-090, B-091, C-157, C-158, C-159</t>
+          <t>A-064, A-072, A-105, B-060, C-157, C-158, C-159</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>19.392 en baja de prestación/subsidio y Parado con jubilación (A-107); 6.773 Nunca_ha_cotizado con jubilación (A-105); 1.108 cobran jubilación e incapacidad a la vez (C-158); 16.669 jubilados con menos de 10 años de empleo (C-159). La parte de B-066/B-096 (Parado_LD/NoLD_y_pensionista con jubilación) SI se corrigió, ver más abajo.</t>
+          <t>19.392 en baja de prestación/subsidio y Parado con jubilación (A-107); 6.773 Nunca_ha_cotizado con jubilación (A-105); 1.108 cobran jubilación e incapacidad a la vez (C-158); 16.669 jubilados con menos de 10 años de empleo (C-159). La parte de B-066/B-096 (Parado_LD/NoLD_y_pensionista con jubilación) SI se corrigió, ver más abajo. CERRADO 2026-09-25 (decisión del usuario). A-105 (6.773), C-158 (16.660) y C-159 (613): jubilados con poco o ningún empleo afiliado, nacidos sobre todo entre 1920 y 1950 (edad mediana 82,7 años, 73 % mujeres); tienen pensión SOVI 5.479 de las 6.773 de A-105 y 7.607 de las 16.660 de C-158 (SOVI: cotizaciones anteriores a 1967, que no están en Afiliación); el resto, carreras en parte anteriores a 1967 o en regímenes sin registro en la MCVL. Clasificadas como baja calidad (no se quitan). C-157 (1.108): jubilación e incapacidad a la vez, solo 6 con SOVI; puede ser pluripensión (distintos regímenes). A-064 y A-072 (23 y 20): asimilados al alta con jubilación, de 79 y 73,5 años, episodios antiguos abiertos. Baja calidad. B-060, B-061, B-090 y B-091 (560, 544, 1 y 1) reformuladas como B-046/B-076: suman el tiempo mixto y excluyen a quien solo tiene prestaciones o subsidios (G08); quedan 8/0/0/0; las 8 tienen episodios de 1979-1984 con la baja anterior al alta (como G20).</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Decisión de diseño (parcialmente resuelta)</t>
+          <t>Dato de origen (carreras anteriores a 1967, SOVI) + reglas reformuladas</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -883,7 +883,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>CORREGIDO 2026-09-23 (decisión explícita del usuario) para B-066/B-096: Parado_LD/Parado_NoLD + jubilación pasa a 'Pensionista' directamente (ya no es 'en paro'); Ocupado_y_pensionista con jubilación NO se toca (jubilación activa es una situación real). Verificado con datos reales completos: 54.568 personas cambian (53.571+997), nadie más se mueve, se conserva el total exacto. El resto de este grupo (A-107, A-105, C-158, C-159) sigue sin decidir.</t>
+          <t>Ninguna acción sobre el ETL.</t>
         </is>
       </c>
     </row>
@@ -6011,7 +6011,7 @@
       </c>
       <c r="J63" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K63" s="2" t="n">
@@ -6543,7 +6543,7 @@
       </c>
       <c r="J71" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K71" s="2" t="n">
@@ -8765,7 +8765,7 @@
       </c>
       <c r="J104" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K104" s="2" t="n">
@@ -8782,7 +8782,7 @@
       <c r="N104" s="2" t="n"/>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>Faltan registros de afiliación anteriores a 1967</t>
+          <t>Faltan registros de afiliación anteriores a 1967 | Clasificada como baja calidad 2026-09-25 (decisión del usuario): jubilados con poco o ningún empleo afiliado. SOVI (NORMA_SOVI = 1): 5.479 de las 6.773 de A-105 y 7.607 de las 16.660 de C-158; el resto, carreras anteriores a 1967 o en regímenes sin registro en la MCVL.</t>
         </is>
       </c>
       <c r="P104" s="2" t="inlineStr">
@@ -13285,7 +13285,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>Parado_LD_pension_no_jubilacion ⇒ ha trabajado alguna vez (t_total_empleo &gt; 0)</t>
+          <t>Parado_LD_pension_no_jubilacion ⇒ ha trabajado alguna vez (t_total_empleo + t_total_mixto_empl_desempl &gt; 0)</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -13305,14 +13305,14 @@
       </c>
       <c r="J170" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K170" s="2" t="n">
-        <v>560</v>
+        <v>8</v>
       </c>
       <c r="L170" s="2" t="n">
-        <v>0.0412</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="M170" s="2" t="inlineStr">
         <is>
@@ -13322,12 +13322,12 @@
       <c r="N170" s="2" t="n"/>
       <c r="O170" s="2" t="inlineStr">
         <is>
-          <t>Alguien puede haber tenido solo prestaciones</t>
+          <t>Reformulada 2026-09-25 (G06, decisión del usuario, como B-046/B-076): suma el tiempo mixto y excluye a quien solo tiene episodios de prestación o subsidio TRL 7xx/400 (G08). Antes 560/544/1/1; quedan 8/0/0/0. Las 8 restantes tienen episodios de 1979-1984 con la baja anterior al alta (duración nula): dato de origen, igual que G20.</t>
         </is>
       </c>
       <c r="P170" s="2" t="inlineStr">
         <is>
-          <t>situacion_paro_ocupacion = 'Parado_LD_pension_no_jubilacion' AND COALESCE(t_total_empleo, 0) = 0</t>
+          <t>situacion_paro_ocupacion = 'Parado_LD_pension_no_jubilacion' AND COALESCE(t_total_empleo, 0) + COALESCE(t_total_mixto_empl_desempl, 0) = 0 AND ipf NOT IN (SELECT ipf FROM solo_prestaciones)</t>
         </is>
       </c>
     </row>
@@ -13374,19 +13374,19 @@
       </c>
       <c r="I171" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J171" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Corregido</t>
         </is>
       </c>
       <c r="K171" s="2" t="n">
-        <v>544</v>
+        <v>0</v>
       </c>
       <c r="L171" s="2" t="n">
-        <v>0.04</v>
+        <v>0</v>
       </c>
       <c r="M171" s="2" t="inlineStr">
         <is>
@@ -13394,10 +13394,14 @@
         </is>
       </c>
       <c r="N171" s="2" t="n"/>
-      <c r="O171" s="2" t="inlineStr"/>
+      <c r="O171" s="2" t="inlineStr">
+        <is>
+          <t>Reformulada 2026-09-25 (G06, decisión del usuario, como B-046/B-076): suma el tiempo mixto y excluye a quien solo tiene episodios de prestación o subsidio TRL 7xx/400 (G08). Antes 560/544/1/1; quedan 8/0/0/0.</t>
+        </is>
+      </c>
       <c r="P171" s="2" t="inlineStr">
         <is>
-          <t>situacion_paro_ocupacion = 'Parado_LD_pension_no_jubilacion' AND fecha_ini_primer_empleo IS NULL</t>
+          <t>situacion_paro_ocupacion = 'Parado_LD_pension_no_jubilacion' AND fecha_ini_primer_empleo IS NULL AND ipf NOT IN (SELECT ipf FROM solo_prestaciones)</t>
         </is>
       </c>
     </row>
@@ -15357,7 +15361,7 @@
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>Parado_NoLD_pension_no_jubilacion ⇒ ha trabajado alguna vez (t_total_empleo &gt; 0)</t>
+          <t>Parado_NoLD_pension_no_jubilacion ⇒ ha trabajado alguna vez (t_total_empleo + t_total_mixto_empl_desempl &gt; 0)</t>
         </is>
       </c>
       <c r="G200" s="2" t="inlineStr">
@@ -15372,19 +15376,19 @@
       </c>
       <c r="I200" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J200" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Corregido</t>
         </is>
       </c>
       <c r="K200" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L200" s="2" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
       <c r="M200" s="2" t="inlineStr">
         <is>
@@ -15394,12 +15398,12 @@
       <c r="N200" s="2" t="n"/>
       <c r="O200" s="2" t="inlineStr">
         <is>
-          <t>Alguien puede haber tenido solo prestaciones</t>
+          <t>Reformulada 2026-09-25 (G06, decisión del usuario, como B-046/B-076): suma el tiempo mixto y excluye a quien solo tiene episodios de prestación o subsidio TRL 7xx/400 (G08). Antes 560/544/1/1; quedan 8/0/0/0.</t>
         </is>
       </c>
       <c r="P200" s="2" t="inlineStr">
         <is>
-          <t>situacion_paro_ocupacion = 'Parado_NoLD_pension_no_jubilacion' AND COALESCE(t_total_empleo, 0) = 0</t>
+          <t>situacion_paro_ocupacion = 'Parado_NoLD_pension_no_jubilacion' AND COALESCE(t_total_empleo, 0) + COALESCE(t_total_mixto_empl_desempl, 0) = 0 AND ipf NOT IN (SELECT ipf FROM solo_prestaciones)</t>
         </is>
       </c>
     </row>
@@ -15446,19 +15450,19 @@
       </c>
       <c r="I201" s="7" t="inlineStr">
         <is>
-          <t>INCUMPLE</t>
+          <t>PASA</t>
         </is>
       </c>
       <c r="J201" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Corregido</t>
         </is>
       </c>
       <c r="K201" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L201" s="2" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
       <c r="M201" s="2" t="inlineStr">
         <is>
@@ -15466,10 +15470,14 @@
         </is>
       </c>
       <c r="N201" s="2" t="n"/>
-      <c r="O201" s="2" t="inlineStr"/>
+      <c r="O201" s="2" t="inlineStr">
+        <is>
+          <t>Reformulada 2026-09-25 (G06, decisión del usuario, como B-046/B-076): suma el tiempo mixto y excluye a quien solo tiene episodios de prestación o subsidio TRL 7xx/400 (G08). Antes 560/544/1/1; quedan 8/0/0/0.</t>
+        </is>
+      </c>
       <c r="P201" s="2" t="inlineStr">
         <is>
-          <t>situacion_paro_ocupacion = 'Parado_NoLD_pension_no_jubilacion' AND fecha_ini_primer_empleo IS NULL</t>
+          <t>situacion_paro_ocupacion = 'Parado_NoLD_pension_no_jubilacion' AND fecha_ini_primer_empleo IS NULL AND ipf NOT IN (SELECT ipf FROM solo_prestaciones)</t>
         </is>
       </c>
     </row>
@@ -26545,7 +26553,7 @@
       </c>
       <c r="J366" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K366" s="2" t="n">
@@ -26615,7 +26623,7 @@
       </c>
       <c r="J367" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K367" s="2" t="n">
@@ -26632,7 +26640,7 @@
       <c r="N367" s="2" t="n"/>
       <c r="O367" s="2" t="inlineStr">
         <is>
-          <t>Faltan datos anteriores a 1967 | Cifra actualizada 2026-09-24 (variación de 1 a 14 personas).</t>
+          <t>Faltan datos anteriores a 1967 | Cifra actualizada 2026-09-24 (variación de 1 a 14 personas). | Clasificada como baja calidad 2026-09-25 (decisión del usuario): jubilados con poco o ningún empleo afiliado. SOVI (NORMA_SOVI = 1): 5.479 de las 6.773 de A-105 y 7.607 de las 16.660 de C-158; el resto, carreras anteriores a 1967 o en regímenes sin registro en la MCVL.</t>
         </is>
       </c>
       <c r="P367" s="2" t="inlineStr">
@@ -26689,7 +26697,7 @@
       </c>
       <c r="J368" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K368" s="2" t="n">
@@ -26704,7 +26712,11 @@
         </is>
       </c>
       <c r="N368" s="2" t="n"/>
-      <c r="O368" s="2" t="inlineStr"/>
+      <c r="O368" s="2" t="inlineStr">
+        <is>
+          <t>Clasificada como baja calidad 2026-09-25 (decisión del usuario): jubilados con poco o ningún empleo afiliado. SOVI (NORMA_SOVI = 1): 5.479 de las 6.773 de A-105 y 7.607 de las 16.660 de C-158; el resto, carreras anteriores a 1967 o en regímenes sin registro en la MCVL.</t>
+        </is>
+      </c>
       <c r="P368" s="2" t="inlineStr">
         <is>
           <t>array_to_string(pension_actual, ',') LIKE '%Jubilaci%' AND edad_ultimo_empleo &lt; 30</t>
@@ -38216,10 +38228,10 @@
         <v>112</v>
       </c>
       <c r="C3" t="n">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D3" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4">
@@ -38248,10 +38260,10 @@
         <v>539</v>
       </c>
       <c r="C5" t="n">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="D5" t="n">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6"/>
@@ -38303,10 +38315,10 @@
         <v>120</v>
       </c>
       <c r="C9" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="D9" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10">
@@ -38355,7 +38367,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="15">
@@ -38365,7 +38377,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>26</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16">
@@ -38375,7 +38387,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>80</v>
+        <v>87</v>
       </c>
     </row>
     <row r="17"/>

</xml_diff>

<commit_message>
reglas: G09 - nueva categoria 'Casos raros (reales)'; edades altas clasificadas
B-108, B-110, C-071, A-054, B-006 y B-022 pasan a Casos raros (reales) con su explicacion; B-109 a baja calidad. La hoja Resumen incluye la categoria nueva.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/reglas_consistencia_resultados_sin_ipf.xlsx
+++ b/tests/reglas_consistencia_resultados_sin_ipf.xlsx
@@ -1012,7 +1012,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Casos raros (reales)</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
@@ -1031,7 +1031,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>4.319 Parado_LD_pension_no_jubilacion fallecidos antes de 2025 (B-062; pudieron cobrar pensión en 2024); 1.046 Pensionistas con más de 100 años (B-108); 501 Parado_NoLD y 385 Parado_LD fallecidos antes de 2025. VERIFICADO 2026-09-25: las 3.115 personas de las reglas 'no fallecido antes de 2025' fallecieron TODAS en 2024 (ninguna antes). Reglas ajustadas a 'antes de 2024' (&lt;= 202312): A-055, A-108, B-007, B-023, B-048, B-062, B-078, B-092 pasan a 0. C-270 (7): dato de origen. Edades altas: 1.276 personas con más de 100 años, de ellas 528 fallecidas cuya edad se calcula a la fecha de corte (no al fallecimiento): pendiente decidir si Edad_Actual_Fecha_Corte debe usar la fecha de fallecimiento. TRAS REGENERAR (2026-09-25): Edad_Actual_Fecha_Corte de los 18.801 fallecidos = edad_fallecimiento; los fallecidos de más de 100 años pasan de 528 a 385; B-108 1.177 -&gt; 1.048, B-110 97 -&gt; 83, C-071 80 -&gt; 67. Efecto colateral RESUELTO el mismo día: 14 fallecidos con episodio de empleo aún abierto al morir tenían Edad_Ultimo_Empleo mayor que su edad al fallecer; Fecha_final_Ultimo_Empleo se limita ahora a su fecha de fallecimiento (C-039 14 -&gt; 0, B-015 y C-113 1 -&gt; 0; queda C-108 con 1).</t>
+          <t>4.319 Parado_LD_pension_no_jubilacion fallecidos antes de 2025 (B-062; pudieron cobrar pensión en 2024); 1.046 Pensionistas con más de 100 años (B-108); 501 Parado_NoLD y 385 Parado_LD fallecidos antes de 2025. VERIFICADO 2026-09-25: las 3.115 personas de las reglas 'no fallecido antes de 2025' fallecieron TODAS en 2024 (ninguna antes). Reglas ajustadas a 'antes de 2024' (&lt;= 202312): A-055, A-108, B-007, B-023, B-048, B-062, B-078, B-092 pasan a 0. C-270 (7): dato de origen. Edades altas: 1.276 personas con más de 100 años, de ellas 528 fallecidas cuya edad se calcula a la fecha de corte (no al fallecimiento): pendiente decidir si Edad_Actual_Fecha_Corte debe usar la fecha de fallecimiento. TRAS REGENERAR (2026-09-25): Edad_Actual_Fecha_Corte de los 18.801 fallecidos = edad_fallecimiento; los fallecidos de más de 100 años pasan de 528 a 385; B-108 1.177 -&gt; 1.048, B-110 97 -&gt; 83, C-071 80 -&gt; 67. Efecto colateral RESUELTO el mismo día: 14 fallecidos con episodio de empleo aún abierto al morir tenían Edad_Ultimo_Empleo mayor que su edad al fallecer; Fecha_final_Ultimo_Empleo se limita ahora a su fecha de fallecimiento (C-039 14 -&gt; 0, B-015 y C-113 1 -&gt; 0; queda C-108 con 1). CLASIFICADO 2026-09-25 (decisión del usuario), con categoría nueva 'Casos raros (reales)': B-108 (1.048 pensionistas de más de 100 años: 366 fallecidos y 682 vivos con pensión, plausible), B-110 (83, la etiqueta 'parado' no mira la edad), C-071 (67 de más de 105 años; más de lo esperable, algunos serán errores), A-054, B-006 y B-022 (los mismos 29 autónomos de más de 90 años que siguen trabajando; B-006 y B-022 son A-054 dividido por tener o no pensión). B-109 (2 parados de más de 100 años sin pensión) y C-270 (7) como baja calidad de los datos.</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -1041,7 +1041,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Regla mal planteada (corregida) + edades altas pendientes</t>
+          <t>Casos raros reales + baja calidad</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1051,7 +1051,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Cambiar la regla a 'antes de 2024' y revisar los &gt; 100 años - sin decidir. (Nota: la pregunta de edades BAJAS con pension se investigo aparte el 2026-09-23 y son casos de orfandad, no jubilación - no forma parte de este grupo, que es sobre edades altas.)</t>
+          <t>Ninguna acción. Mejora futura opcional del ETL: que a edades muy avanzadas con pensión no jubilación la situación sea 'Pensionista' en vez de 'Parado_*_pension_no_jubilacion' (87 personas de más de 100 años y 13.859 entre 80 y 99).</t>
         </is>
       </c>
     </row>
@@ -5335,7 +5335,7 @@
       </c>
       <c r="J53" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Casos raros (reales)</t>
         </is>
       </c>
       <c r="K53" s="2" t="n">
@@ -5350,7 +5350,11 @@
         </is>
       </c>
       <c r="N53" s="2" t="n"/>
-      <c r="O53" s="2" t="inlineStr"/>
+      <c r="O53" s="2" t="inlineStr">
+        <is>
+          <t>CASOS RAROS REALES (decisión del usuario 2026-09-25). 29 ocupados de más de 90 años (mediana 92,3, máximo 97,4): 26 son autónomos (régimen 521) con episodios abiertos desde hace décadas (1970, 1978, 1994...), y 24 tienen ingresos fiscales en 2024 (mediana 32.832 €): siguen con actividad económica. Son las mismas 29 personas de B-006 (10, sin pensión) y B-022 (19, con pensión).</t>
+        </is>
+      </c>
       <c r="P53" s="2" t="inlineStr">
         <is>
           <t>situacion_actual_afiliacion = 'Alta_ocupado' AND edad_actual_fecha_corte &gt; 90</t>
@@ -9589,7 +9593,7 @@
       </c>
       <c r="J116" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Casos raros (reales)</t>
         </is>
       </c>
       <c r="K116" s="2" t="n">
@@ -9604,7 +9608,11 @@
         </is>
       </c>
       <c r="N116" s="2" t="n"/>
-      <c r="O116" s="2" t="inlineStr"/>
+      <c r="O116" s="2" t="inlineStr">
+        <is>
+          <t>CASOS RAROS REALES (decisión del usuario 2026-09-25). Mismas personas que A-054 (autónomos de más de 90 años que siguen trabajando), las 10 sin pensión. B-006 + B-022 = las 29 de A-054 vistas por la situación de paro/ocupación.</t>
+        </is>
+      </c>
       <c r="P116" s="2" t="inlineStr">
         <is>
           <t>situacion_paro_ocupacion = 'Ocupado' AND edad_actual_fecha_corte &gt; 90</t>
@@ -10689,7 +10697,7 @@
       </c>
       <c r="J132" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Casos raros (reales)</t>
         </is>
       </c>
       <c r="K132" s="2" t="n">
@@ -10704,7 +10712,11 @@
         </is>
       </c>
       <c r="N132" s="2" t="n"/>
-      <c r="O132" s="2" t="inlineStr"/>
+      <c r="O132" s="2" t="inlineStr">
+        <is>
+          <t>CASOS RAROS REALES (decisión del usuario 2026-09-25). Mismas personas que A-054 (autónomos de más de 90 años que siguen trabajando), las 19 que además cobran pensión (jubilación activa). B-006 + B-022 = las 29 de A-054.</t>
+        </is>
+      </c>
       <c r="P132" s="2" t="inlineStr">
         <is>
           <t>situacion_paro_ocupacion = 'Ocupado_y_pensionista' AND edad_actual_fecha_corte &gt; 90</t>
@@ -16621,7 +16633,7 @@
       </c>
       <c r="J218" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Casos raros (reales)</t>
         </is>
       </c>
       <c r="K218" s="2" t="n">
@@ -16638,7 +16650,7 @@
       <c r="N218" s="2" t="n"/>
       <c r="O218" s="2" t="inlineStr">
         <is>
-          <t>Actualizado 2026-09-25 tras regenerar con: Edad_Actual_Fecha_Corte de fallecidos a su fecha de fallecimiento, claves de grupo fuera de 00-12 al 00 y sin causas_baja_distintas.</t>
+          <t>CASOS RAROS REALES (decisión del usuario 2026-09-25). 1.048 pensionistas de más de 100 años: 366 fallecidos que murieron con más de 100 y 682 vivos con pensión en 2024 (cifra plausible: unos 560 esperables en una muestra del 4 %). 527 tienen jubilación y el resto viudedad o incapacidad de mayores de 65. Con el corte el 1-5-2025, quien nació entre enero y abril de 1925 tiene 100,0-100,3 años: parte es un efecto del umbral.</t>
         </is>
       </c>
       <c r="P218" s="2" t="inlineStr">
@@ -16695,7 +16707,7 @@
       </c>
       <c r="J219" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K219" s="2" t="n">
@@ -16710,7 +16722,11 @@
         </is>
       </c>
       <c r="N219" s="2" t="n"/>
-      <c r="O219" s="2" t="inlineStr"/>
+      <c r="O219" s="2" t="inlineStr">
+        <is>
+          <t>BAJA CALIDAD (decisión del usuario 2026-09-25). 2 personas de más de 100 años en Parado_LD y sin pensión: un desempleado de esa edad no es plausible (fecha de nacimiento errónea o registro sin cerrar).</t>
+        </is>
+      </c>
       <c r="P219" s="2" t="inlineStr">
         <is>
           <t>situacion_paro_ocupacion = 'Parado_LD' AND edad_actual_fecha_corte &gt; 100</t>
@@ -16765,7 +16781,7 @@
       </c>
       <c r="J220" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Casos raros (reales)</t>
         </is>
       </c>
       <c r="K220" s="2" t="n">
@@ -16782,7 +16798,7 @@
       <c r="N220" s="2" t="n"/>
       <c r="O220" s="2" t="inlineStr">
         <is>
-          <t>Actualizado 2026-09-25 tras regenerar con: Edad_Actual_Fecha_Corte de fallecidos a su fecha de fallecimiento, claves de grupo fuera de 00-12 al 00 y sin causas_baja_distintas.</t>
+          <t>CASOS RAROS REALES (decisión del usuario 2026-09-25). 83 personas de más de 100 años en Parado_LD_pension_no_jubilacion (19 fallecidas, 64 vivas): cobran viudedad o incapacidad, sin jubilación. La etiqueta 'parado' no mira la edad: 76 de los 83 dejaron de trabajar hace una mediana de 40,2 años. Las personas existen; lo raro es la etiqueta. Posible mejora futura del ETL: que a edades muy avanzadas con pensión no jubilación sean 'Pensionista'.</t>
         </is>
       </c>
       <c r="P220" s="2" t="inlineStr">
@@ -21417,7 +21433,7 @@
       </c>
       <c r="J290" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Casos raros (reales)</t>
         </is>
       </c>
       <c r="K290" s="2" t="n">
@@ -21434,7 +21450,7 @@
       <c r="N290" s="2" t="n"/>
       <c r="O290" s="2" t="inlineStr">
         <is>
-          <t>Detección de outliers/errores | Actualizado 2026-09-25 tras regenerar con: Edad_Actual_Fecha_Corte de fallecidos a su fecha de fallecimiento, claves de grupo fuera de 00-12 al 00 y sin causas_baja_distintas.</t>
+          <t>CASOS RAROS (decisión del usuario 2026-09-25). 67 personas de más de 105 años (23 fallecidas con esa edad al morir y 44 vivas con pensión), nacidas entre 1913 y 1920. Es más de lo esperable (unos 15 en una muestra del 4 %): algunas serán reales y otras, errores de fecha de nacimiento o fallecimientos no comunicados.</t>
         </is>
       </c>
       <c r="P290" s="2" t="inlineStr">
@@ -38101,7 +38117,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -38307,7 +38323,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16">
@@ -38317,10 +38333,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="17"/>
+        <v>93</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Casos raros (reales)</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>6</v>
+      </c>
+    </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
@@ -38328,6 +38353,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
reglas: reclasifica 25 reglas a Casos raros (reales) y anade la columna de explicaciones
25 reglas de baja calidad pasan a Casos raros (reales): G12 (C-230..C-235), G17 (C-338, C-311, C-313, C-309, C-310), G22 (C-088, C-087, C-153, C-156, A-074, A-098), G06 (C-157, A-064, A-072), G04 (C-168, C-239, C-251) y G15 (B-014, B-030). La hoja Resultados incluye una columna nueva con la explicacion de cada regla de Casos raros o Baja calidad (99 reglas). Resumen y Hallazgos actualizados: 31 casos raros, 68 baja calidad, 3 pendientes.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/reglas_consistencia_resultados_sin_ipf.xlsx
+++ b/tests/reglas_consistencia_resultados_sin_ipf.xlsx
@@ -732,7 +732,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Baja calidad de los datos</t>
+          <t>Casos raros y baja calidad</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
@@ -771,7 +771,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>CERRADO 2026-09-24 (decisión del usuario). Residuo como baja calidad de los datos: 397 en C-079 (336 con CNAE desconocido, 329 en régimen general; 150 con 12-13 años, 133 con 14-15 y 114 con menos de 12), 878 en C-107 y 232 en C-058: episodios sin sector conocido que pueden ser errores de fecha o menores autorizados sin CNAE. Se descarta ampliar la excepción a CNAE desconocido (dejaría pasar cualquier error de fecha). Pendiente aparte: las gráficas por edad de Trayectorias de colectivos cortan en 16 (app/routers/trayectorias.py) y omiten los 14-15 años legítimos de las cohortes antiguas; el usuario decidió dejarlo para más adelante.</t>
+          <t>CERRADO 2026-09-24 (decisión del usuario). Residuo como baja calidad de los datos: 397 en C-079 (336 con CNAE desconocido, 329 en régimen general; 150 con 12-13 años, 133 con 14-15 y 114 con menos de 12), 878 en C-107 y 232 en C-058: episodios sin sector conocido que pueden ser errores de fecha o menores autorizados sin CNAE. Se descarta ampliar la excepción a CNAE desconocido (dejaría pasar cualquier error de fecha). Pendiente aparte: las gráficas por edad de Trayectorias de colectivos cortan en 16 (app/routers/trayectorias.py) y omiten los 14-15 años legítimos de las cohortes antiguas; el usuario decidió dejarlo para más adelante. CLASIFICACIÓN 2026-09-25 (decisión del usuario): casos raros reales: C-168, C-239, C-251; baja calidad de los datos: A-093, B-040, B-054, B-070, B-084, C-051, C-052, C-053, C-054, C-055, C-056, C-057, C-058, C-079, C-083, C-085, C-096, C-097, C-105, C-106, C-107, C-114, C-115. Explicación por regla en la última columna de la hoja Resultados.</t>
         </is>
       </c>
     </row>
@@ -844,7 +844,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Baja calidad de los datos</t>
+          <t>Casos raros y baja calidad</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
@@ -883,7 +883,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Ninguna acción sobre el ETL.</t>
+          <t>Ninguna acción sobre el ETL. CLASIFICACIÓN 2026-09-25 (decisión del usuario): casos raros reales: A-064, A-072, C-157; baja calidad de los datos: A-105, B-060, C-158, C-159. Explicación por regla en la última columna de la hoja Resultados.</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Ninguna acción sobre el ETL ni sobre la regla. Se deja como detección informativa de baja confianza.</t>
+          <t>Ninguna acción sobre el ETL ni sobre la regla. Se deja como detección informativa de baja confianza. CLASIFICACIÓN 2026-09-25 (decisión del usuario): casos raros reales: ninguno; baja calidad de los datos: A-096, A-097, B-099, B-100, B-103, B-105, C-150. Explicación por regla en la última columna de la hoja Resultados.</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Ninguna acción. Mejora futura opcional del ETL: que a edades muy avanzadas con pensión no jubilación la situación sea 'Pensionista' en vez de 'Parado_*_pension_no_jubilacion' (87 personas de más de 100 años y 13.859 entre 80 y 99).</t>
+          <t>Ninguna acción. Mejora futura opcional del ETL: que a edades muy avanzadas con pensión no jubilación la situación sea 'Pensionista' en vez de 'Parado_*_pension_no_jubilacion' (87 personas de más de 100 años y 13.859 entre 80 y 99). CLASIFICACIÓN 2026-09-25 (decisión del usuario): casos raros reales: A-054, B-006, B-022, B-108, B-110, C-071; baja calidad de los datos: B-109, C-270. Explicación por regla en la última columna de la hoja Resultados.</t>
         </is>
       </c>
     </row>
@@ -1176,7 +1176,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Baja calidad de los datos</t>
+          <t>Casos raros y baja calidad</t>
         </is>
       </c>
       <c r="D13" s="2" t="n">
@@ -1215,7 +1215,7 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Ninguna acción sobre el ETL. Confianza baja/media, se deja como detección informativa.</t>
+          <t>Ninguna acción sobre el ETL. Confianza baja/media, se deja como detección informativa. CLASIFICACIÓN 2026-09-25 (decisión del usuario): casos raros reales: C-230, C-231, C-232, C-233, C-234, C-235; baja calidad de los datos: C-236, C-237, C-238, C-240, C-241. Explicación por regla en la última columna de la hoja Resultados.</t>
         </is>
       </c>
     </row>
@@ -1344,7 +1344,7 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Baja calidad de los datos</t>
+          <t>Casos raros y baja calidad</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>CERRADO 2026-09-25 (decisión del usuario): B-014/B-030 reformuladas (90.084 -&gt; 4.054 y 1.245 -&gt; 7); B-012, B-028, B-014, B-030 y C-166 como baja calidad de los datos; C-169 quitada. Ninguna acción sobre el ETL.</t>
+          <t>CERRADO 2026-09-25 (decisión del usuario): B-014/B-030 reformuladas (90.084 -&gt; 4.054 y 1.245 -&gt; 7); B-012, B-028, B-014, B-030 y C-166 como baja calidad de los datos; C-169 quitada. Ninguna acción sobre el ETL. CLASIFICACIÓN 2026-09-25 (decisión del usuario): casos raros reales: B-014, B-030; baja calidad de los datos: B-012, B-028, C-166. Explicación por regla en la última columna de la hoja Resultados.</t>
         </is>
       </c>
     </row>
@@ -1452,7 +1452,7 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Baja calidad de los datos</t>
+          <t>Casos raros y baja calidad</t>
         </is>
       </c>
       <c r="D18" s="2" t="n">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>Ninguna acción sobre el ETL más allá del renombrado. Renombrado en el ETL y la app (compatible con un Parquet antiguo); el Parquet actual lo lleva con el nombre antiguo hasta regenerar el Grupo H.</t>
+          <t>Ninguna acción sobre el ETL más allá del renombrado. Renombrado en el ETL y la app (compatible con un Parquet antiguo); el Parquet actual lo lleva con el nombre antiguo hasta regenerar el Grupo H. CLASIFICACIÓN 2026-09-25 (decisión del usuario): casos raros reales: C-309, C-310, C-311, C-313, C-338; baja calidad de los datos: C-302, C-306. Explicación por regla en la última columna de la hoja Resultados.</t>
         </is>
       </c>
     </row>
@@ -1599,7 +1599,7 @@
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>Ninguna acción sobre el ETL. Dejar las reglas como detección informativa de baja confianza, sin tratarlas como error pendiente de resolver.</t>
+          <t>Ninguna acción sobre el ETL. Dejar las reglas como detección informativa de baja confianza, sin tratarlas como error pendiente de resolver. CLASIFICACIÓN 2026-09-25 (decisión del usuario): casos raros reales: ninguno; baja calidad de los datos: C-095, C-243, C-244, C-245, C-246, C-247, C-248, C-249, C-250. Explicación por regla en la última columna de la hoja Resultados.</t>
         </is>
       </c>
     </row>
@@ -1655,7 +1655,7 @@
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>Ninguna acción sobre el ETL; volumen insignificante.</t>
+          <t>Ninguna acción sobre el ETL; volumen insignificante. CLASIFICACIÓN 2026-09-25 (decisión del usuario): casos raros reales: ninguno; baja calidad de los datos: A-042, A-043, A-092, C-080, C-130, C-132, C-138. Explicación por regla en la última columna de la hoja Resultados.</t>
         </is>
       </c>
     </row>
@@ -1728,7 +1728,7 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Baja calidad de los datos</t>
+          <t>Casos raros y baja calidad</t>
         </is>
       </c>
       <c r="D23" s="2" t="n">
@@ -1767,7 +1767,7 @@
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>Ninguna acción: se dejan como están en Pension_actual (decisión del usuario).</t>
+          <t>Ninguna acción: se dejan como están en Pension_actual (decisión del usuario). CLASIFICACIÓN 2026-09-25 (decisión del usuario): casos raros reales: A-074, A-098, C-087, C-088, C-153, C-156; baja calidad de los datos: A-052, A-078, A-106, B-004, C-086, C-279. Explicación por regla en la última columna de la hoja Resultados.</t>
         </is>
       </c>
     </row>
@@ -1782,7 +1782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P539"/>
+  <dimension ref="A1:Q539"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1801,6 +1801,7 @@
     <col width="40" customWidth="1" min="14" max="14"/>
     <col width="40" customWidth="1" min="15" max="15"/>
     <col width="80" customWidth="1" min="16" max="16"/>
+    <col width="110" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1884,6 +1885,11 @@
           <t>Condición de violación (SQL)</t>
         </is>
       </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Explicación (casos raros / baja calidad)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -4606,6 +4612,11 @@
           <t>situacion_actual_afiliacion &lt;&gt; 'Nunca_ha_cotizado' AND t_total_empleo IS NULL AND ipf NOT IN (SELECT ipf FROM solo_prestaciones)</t>
         </is>
       </c>
+      <c r="Q42" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Episodios de 1979-1984 con la fecha de baja anterior a la de alta: la duración de empleo sale nula y arrastra t_total_empleo, el número de altas y el tiempo total. Afecta a 6-9 personas; dato de origen. </t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -4678,6 +4689,11 @@
       <c r="P43" s="2" t="inlineStr">
         <is>
           <t>situacion_actual_afiliacion &lt;&gt; 'Nunca_ha_cotizado' AND num_altas_anual_promedio IS NULL AND ipf NOT IN (SELECT ipf FROM solo_prestaciones)</t>
+        </is>
+      </c>
+      <c r="Q43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Episodios de 1979-1984 con la fecha de baja anterior a la de alta: la duración de empleo sale nula y arrastra t_total_empleo, el número de altas y el tiempo total. Afecta a 6-9 personas; dato de origen. </t>
         </is>
       </c>
     </row>
@@ -5220,6 +5236,11 @@
           <t>situacion_actual_afiliacion = 'Alta_ocupado' AND COALESCE(t_total_empleo, 0) = 0</t>
         </is>
       </c>
+      <c r="Q51" s="2" t="inlineStr">
+        <is>
+          <t>4 personas Alta_ocupado sin tiempo de empleo: episodios de 1979-1984 con la baja anterior al alta (duración nula), como G20. Dato de origen.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -5360,6 +5381,11 @@
           <t>situacion_actual_afiliacion = 'Alta_ocupado' AND edad_actual_fecha_corte &gt; 90</t>
         </is>
       </c>
+      <c r="Q53" s="2" t="inlineStr">
+        <is>
+          <t>CASO RARO REAL. 29 ocupados de más de 90 años (mediana 92,3, máximo 97,4): 26 autónomos (régimen 521) con episodios abiertos desde hace décadas, y 24 con ingresos fiscales en 2024 (mediana 32.832 €): siguen con actividad económica. Son las mismas 29 personas de B-006 (10, sin pensión) y B-022 (19, con pensión).</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -6015,7 +6041,7 @@
       </c>
       <c r="J63" s="5" t="inlineStr">
         <is>
-          <t>Baja calidad de los datos</t>
+          <t>Casos raros (reales)</t>
         </is>
       </c>
       <c r="K63" s="2" t="n">
@@ -6034,6 +6060,11 @@
       <c r="P63" s="2" t="inlineStr">
         <is>
           <t>situacion_actual_afiliacion = 'Asimilado_al_alta_prest_subs' AND array_to_string(pension_actual, ',') LIKE '%Jubilaci%'</t>
+        </is>
+      </c>
+      <c r="Q63" s="2" t="inlineStr">
+        <is>
+          <t>CASO RARO. 23 asimilados al alta por prestación o subsidio con jubilación (edad media 79 años): probables episodios antiguos aún abiertos o compatibilidad de jubilación con subsidio. Volumen pequeño.</t>
         </is>
       </c>
     </row>
@@ -6547,7 +6578,7 @@
       </c>
       <c r="J71" s="5" t="inlineStr">
         <is>
-          <t>Baja calidad de los datos</t>
+          <t>Casos raros (reales)</t>
         </is>
       </c>
       <c r="K71" s="2" t="n">
@@ -6566,6 +6597,11 @@
       <c r="P71" s="2" t="inlineStr">
         <is>
           <t>situacion_actual_afiliacion = 'Asimilado_al_alta_subs52' AND array_to_string(pension_actual, ',') LIKE '%Jubilaci%'</t>
+        </is>
+      </c>
+      <c r="Q71" s="2" t="inlineStr">
+        <is>
+          <t>CASO RARO. 20 asimilados al alta por subsidio de mayores con jubilación (edad media 73,5 años): probables episodios antiguos aún abiertos o compatibilidad. Volumen pequeño.</t>
         </is>
       </c>
     </row>
@@ -6683,7 +6719,7 @@
       </c>
       <c r="J73" s="5" t="inlineStr">
         <is>
-          <t>Baja calidad de los datos</t>
+          <t>Casos raros (reales)</t>
         </is>
       </c>
       <c r="K73" s="2" t="n">
@@ -6706,6 +6742,11 @@
       <c r="P73" s="2" t="inlineStr">
         <is>
           <t>situacion_actual_afiliacion = 'Asimilado_al_alta_subs52' AND edad_actual_fecha_corte &lt; 45</t>
+        </is>
+      </c>
+      <c r="Q73" s="2" t="inlineStr">
+        <is>
+          <t>CASO RARO. 1 persona menor de 45 años con subsidio de mayores: los fijos discontinuos pueden ser más jóvenes (guía TRL 753/754).</t>
         </is>
       </c>
     </row>
@@ -6976,6 +7017,11 @@
           <t>situacion_actual_afiliacion = 'Baja_de_prestacion' AND fecha_inicio_ultima_racha_sin_empleo &gt; fecha_ultima_baja</t>
         </is>
       </c>
+      <c r="Q77" s="2" t="inlineStr">
+        <is>
+          <t>4 personas en Baja_de_prestacion con el inicio de la racha posterior a la última baja: fechas de racha incoherentes con la última baja por episodios solapados; volumen insignificante.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -7908,6 +7954,11 @@
           <t>situacion_actual_afiliacion = 'Baja_de_actividad' AND fecha_ultima_baja &lt; fecha_ini_primer_empleo</t>
         </is>
       </c>
+      <c r="Q91" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Episodios de 1979-1984 con la fecha de baja anterior a la de alta: la duración de empleo sale nula y arrastra t_total_empleo, el número de altas y el tiempo total. Afecta a 6-9 personas; dato de origen. </t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -7976,6 +8027,11 @@
       <c r="P92" s="2" t="inlineStr">
         <is>
           <t>situacion_actual_afiliacion = 'Baja_de_actividad' AND edad_actual_fecha_corte &lt; 16</t>
+        </is>
+      </c>
+      <c r="Q92" s="2" t="inlineStr">
+        <is>
+          <t>Menores de 16 años actuales con afiliación (287, los mismos en A-093, B-040, B-054, B-070, B-084, C-114 y C-115), nacidos sobre todo desde 2010. De los 262 que además tienen sueldo en 2024, 249 son menores autorizados en espectáculos (art. 6.4 ET); el resto son errores de fecha o afiliaciones de niños sin causa conocida.</t>
         </is>
       </c>
     </row>
@@ -8184,6 +8240,11 @@
           <t>situacion_actual_afiliacion = 'Baja_para_pension' AND cobra_pension_2024_5 &lt;&gt; 'SI'</t>
         </is>
       </c>
+      <c r="Q95" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Desfase temporal entre Afiliación y Pensiones: el 99,8 % de las 2.346 tiene Baja_para_pension con causa 58 (paso a pensionista) y la última baja muy reciente (1.926 en 2025, 415 en 2024), pero la tabla de Pensiones de esta edición aún no recoge esa pensión. Cada columna está bien calculada desde su tabla de origen. </t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -8254,6 +8315,11 @@
           <t>situacion_actual_afiliacion = 'Baja_para_pension' AND pension_todas_cobradas IS NULL</t>
         </is>
       </c>
+      <c r="Q96" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Desfase temporal entre Afiliación y Pensiones: el 99,8 % de las 2.346 tiene Baja_para_pension con causa 58 (paso a pensionista) y la última baja muy reciente (1.926 en 2025, 415 en 2024), pero la tabla de Pensiones de esta edición aún no recoge esa pensión. Cada columna está bien calculada desde su tabla de origen. </t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -8303,7 +8369,7 @@
       </c>
       <c r="J97" s="5" t="inlineStr">
         <is>
-          <t>Baja calidad de los datos</t>
+          <t>Casos raros (reales)</t>
         </is>
       </c>
       <c r="K97" s="2" t="n">
@@ -8322,6 +8388,11 @@
       <c r="P97" s="2" t="inlineStr">
         <is>
           <t>situacion_actual_afiliacion = 'Baja_para_pension' AND edad_actual_fecha_corte &lt; 20</t>
+        </is>
+      </c>
+      <c r="Q97" s="2" t="inlineStr">
+        <is>
+          <t>CASO RARO REAL. 1 persona de 18,8 años en Baja_para_pension: joven con pensión (posible orfandad); caso aislado.</t>
         </is>
       </c>
     </row>
@@ -8794,6 +8865,11 @@
           <t>situacion_actual_afiliacion = 'Nunca_ha_cotizado' AND array_to_string(pension_actual, ',') LIKE '%Jubilaci%'</t>
         </is>
       </c>
+      <c r="Q104" s="2" t="inlineStr">
+        <is>
+          <t>Jubilados sin ningún episodio de cotización en Afiliación (6.773), edad mediana 85,8 años: 5.479 tienen pensión SOVI (cotizaciones anteriores a 1967, no recogidas en Afiliación). Cobertura incompleta de origen.</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -8862,6 +8938,11 @@
       <c r="P105" s="2" t="inlineStr">
         <is>
           <t>situacion_actual_afiliacion = 'Nunca_ha_cotizado' AND array_to_string(pension_actual, ',') LIKE '%Incapacidad%'</t>
+        </is>
+      </c>
+      <c r="Q105" s="2" t="inlineStr">
+        <is>
+          <t>Nunca_ha_cotizado con pensión de incapacidad (486), sobre todo 'Incapacidad&gt;65', edad mediana 89 años: su trabajo es anterior a 1967 o está fuera de la MCVL. Cobertura incompleta de origen.</t>
         </is>
       </c>
     </row>
@@ -9478,6 +9559,11 @@
           <t>situacion_paro_ocupacion = 'Ocupado' AND COALESCE(t_total_empleo, 0) = 0</t>
         </is>
       </c>
+      <c r="Q114" s="2" t="inlineStr">
+        <is>
+          <t>4 personas Ocupado sin tiempo de empleo: episodios de 1979-1984 con la baja anterior al alta (duración nula), como G20. Dato de origen.</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -9618,6 +9704,11 @@
           <t>situacion_paro_ocupacion = 'Ocupado' AND edad_actual_fecha_corte &gt; 90</t>
         </is>
       </c>
+      <c r="Q116" s="2" t="inlineStr">
+        <is>
+          <t>CASO RARO REAL. Mismas personas que A-054 (autónomos de más de 90 años que siguen trabajando): las 10 sin pensión. B-006 + B-022 = las 29 de A-054.</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -10030,6 +10121,11 @@
           <t>situacion_paro_ocupacion = 'Ocupado' AND NOT (act_econ_ppal IS NOT NULL AND act_econ_ppal NOT IN ('NO CONSTA','No consta','0 NO CONSTA','00 No consta'))</t>
         </is>
       </c>
+      <c r="Q122" s="2" t="inlineStr">
+        <is>
+          <t>548 ocupados sin actividad económica principal: en su mayoría (521 de 570 entre B-012 y B-028) del régimen general, donde falta el CNAE de la cuenta de cotización; 28 autónomos y 13 empleados de hogar. Dato de origen.</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -10153,7 +10249,7 @@
       </c>
       <c r="J124" s="5" t="inlineStr">
         <is>
-          <t>Baja calidad de los datos</t>
+          <t>Casos raros (reales)</t>
         </is>
       </c>
       <c r="K124" s="2" t="n">
@@ -10176,6 +10272,11 @@
       <c r="P124" s="2" t="inlineStr">
         <is>
           <t>situacion_paro_ocupacion = 'Ocupado' AND ingresos_bruto_total_2024 IS NULL AND prov_trabajo_ppal NOT IN ('01 ÁLAVA','20 GIPUZKOA','48 BIZKAIA','31 NAVARRA') AND ipf NOT IN (SELECT ipf FROM sin_190_esperable)</t>
+        </is>
+      </c>
+      <c r="Q124" s="2" t="inlineStr">
+        <is>
+          <t>CASO RARO REAL. 4.054 ocupados sin ingresos fiscales en 2024 tras excluir territorios forales (la AEAT no tiene sus datos), autónomos, empleados de hogar y empleadores persona física. Residuo: 3.896 con empleador con NIF/CIF, 2.092 empleadores distintos sin concentración; perfil: 44,2 % extranjeros (24 % UE o Reino Unido) frente al 10,5 %, edad mediana 37,3 frente a 45,1 años y 67 % con el episodio abierto desde 2023 frente al 42 %. Hipótesis sin comprobar: extranjeros recientes que tributan como no residentes o desplazados (modelos 296 o 151, no el 190). Ninguno está en la tabla fiscal cruda: no es un fallo del ETL.</t>
         </is>
       </c>
     </row>
@@ -10722,6 +10823,11 @@
           <t>situacion_paro_ocupacion = 'Ocupado_y_pensionista' AND edad_actual_fecha_corte &gt; 90</t>
         </is>
       </c>
+      <c r="Q132" s="2" t="inlineStr">
+        <is>
+          <t>CASO RARO REAL. Mismas personas que A-054 (autónomos de más de 90 años que siguen trabajando): las 19 que además cobran pensión (jubilación activa). B-006 + B-022 = las 29 de A-054.</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -11134,6 +11240,11 @@
           <t>situacion_paro_ocupacion = 'Ocupado_y_pensionista' AND NOT (act_econ_ppal IS NOT NULL AND act_econ_ppal NOT IN ('NO CONSTA','No consta','0 NO CONSTA','00 No consta'))</t>
         </is>
       </c>
+      <c r="Q138" s="2" t="inlineStr">
+        <is>
+          <t>22 ocupados y pensionistas sin actividad económica principal: CNAE de la cuenta de cotización sin informar (ver B-012). Dato de origen.</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -11257,7 +11368,7 @@
       </c>
       <c r="J140" s="5" t="inlineStr">
         <is>
-          <t>Baja calidad de los datos</t>
+          <t>Casos raros (reales)</t>
         </is>
       </c>
       <c r="K140" s="2" t="n">
@@ -11280,6 +11391,11 @@
       <c r="P140" s="2" t="inlineStr">
         <is>
           <t>situacion_paro_ocupacion = 'Ocupado_y_pensionista' AND ingresos_bruto_total_2024 IS NULL AND prov_trabajo_ppal NOT IN ('01 ÁLAVA','20 GIPUZKOA','48 BIZKAIA','31 NAVARRA') AND ipf NOT IN (SELECT ipf FROM sin_190_esperable)</t>
+        </is>
+      </c>
+      <c r="Q140" s="2" t="inlineStr">
+        <is>
+          <t>CASO RARO REAL. Igual que B-014 (ver su explicación) para Ocupado_y_pensionista: de 1.245 a 7 tras excluir territorios forales, autónomos, empleados de hogar y empleador persona física.</t>
         </is>
       </c>
     </row>
@@ -11950,6 +12066,11 @@
           <t>situacion_paro_ocupacion = 'Parado_LD' AND edad_actual_fecha_corte &lt; 16</t>
         </is>
       </c>
+      <c r="Q150" s="2" t="inlineStr">
+        <is>
+          <t>Menores de 16 años actuales con afiliación (287, los mismos en A-093, B-040, B-054, B-070, B-084, C-114 y C-115), nacidos sobre todo desde 2010. De los 262 que además tienen sueldo en 2024, 249 son menores autorizados en espectáculos (art. 6.4 ET); el resto son errores de fecha o afiliaciones de niños sin causa conocida.</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -12922,6 +13043,11 @@
           <t>situacion_paro_ocupacion = 'Parado_LD_pension_no_jubilacion' AND edad_actual_fecha_corte &lt; 16</t>
         </is>
       </c>
+      <c r="Q164" s="2" t="inlineStr">
+        <is>
+          <t>Menores de 16 años actuales con afiliación (287, los mismos en A-093, B-040, B-054, B-070, B-084, C-114 y C-115), nacidos sobre todo desde 2010. De los 262 que además tienen sueldo en 2024, 249 son menores autorizados en espectáculos (art. 6.4 ET); el resto son errores de fecha o afiliaciones de niños sin causa conocida.</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -13342,6 +13468,11 @@
           <t>situacion_paro_ocupacion = 'Parado_LD_pension_no_jubilacion' AND COALESCE(t_total_empleo, 0) + COALESCE(t_total_mixto_empl_desempl, 0) = 0 AND ipf NOT IN (SELECT ipf FROM solo_prestaciones)</t>
         </is>
       </c>
+      <c r="Q170" s="2" t="inlineStr">
+        <is>
+          <t>8 personas Parado_LD con pensión no jubilación sin tiempo de empleo (tras excluir a quien solo tiene prestaciones y sumar el tiempo mixto): todas tienen episodios de 1979-1984 con la baja anterior al alta (duración nula), como G20. Dato de origen.</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -14034,6 +14165,11 @@
           <t>situacion_paro_ocupacion = 'Parado_NoLD' AND edad_actual_fecha_corte &lt; 16</t>
         </is>
       </c>
+      <c r="Q180" s="2" t="inlineStr">
+        <is>
+          <t>Menores de 16 años actuales con afiliación (287, los mismos en A-093, B-040, B-054, B-070, B-084, C-114 y C-115), nacidos sobre todo desde 2010. De los 262 que además tienen sueldo en 2024, 249 son menores autorizados en espectáculos (art. 6.4 ET); el resto son errores de fecha o afiliaciones de niños sin causa conocida.</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
@@ -15002,6 +15138,11 @@
           <t>situacion_paro_ocupacion = 'Parado_NoLD_pension_no_jubilacion' AND edad_actual_fecha_corte &lt; 16</t>
         </is>
       </c>
+      <c r="Q194" s="2" t="inlineStr">
+        <is>
+          <t>Menores de 16 años actuales con afiliación (287, los mismos en A-093, B-040, B-054, B-070, B-084, C-114 y C-115), nacidos sobre todo desde 2010. De los 262 que además tienen sueldo en 2024, 249 son menores autorizados en espectáculos (art. 6.4 ET); el resto son errores de fecha o afiliaciones de niños sin causa conocida.</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
@@ -16044,6 +16185,11 @@
           <t>situacion_paro_ocupacion = 'Pensionista' AND cobra_pension_2024_5 &lt;&gt; 'SI'</t>
         </is>
       </c>
+      <c r="Q209" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Desfase temporal entre Afiliación y Pensiones: el 99,8 % de las 2.346 tiene Baja_para_pension con causa 58 (paso a pensionista) y la última baja muy reciente (1.926 en 2025, 415 en 2024), pero la tabla de Pensiones de esta edición aún no recoge esa pensión. Cada columna está bien calculada desde su tabla de origen. </t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
@@ -16112,6 +16258,11 @@
       <c r="P210" s="2" t="inlineStr">
         <is>
           <t>situacion_paro_ocupacion = 'Pensionista' AND pension_actual IS NULL</t>
+        </is>
+      </c>
+      <c r="Q210" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Desfase temporal entre Afiliación y Pensiones: el 99,8 % de las 2.346 tiene Baja_para_pension con causa 58 (paso a pensionista) y la última baja muy reciente (1.926 en 2025, 415 en 2024), pero la tabla de Pensiones de esta edición aún no recoge esa pensión. Cada columna está bien calculada desde su tabla de origen. </t>
         </is>
       </c>
     </row>
@@ -16316,6 +16467,11 @@
           <t>situacion_paro_ocupacion = 'Pensionista' AND year(fecha_ultima_baja) = 2099</t>
         </is>
       </c>
+      <c r="Q213" s="2" t="inlineStr">
+        <is>
+          <t>53 pensionistas con un episodio de afiliación aún abierto (fecha_ultima_baja 2099): pensión reciente con el episodio sin cerrar; mismo origen temporal que el resto de G07 (probable, no comprobado).</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
@@ -16452,6 +16608,11 @@
           <t>situacion_paro_ocupacion IN ('Ocupado_y_pensionista','Parado_LD_pension_no_jubilacion','Parado_NoLD_pension_no_jubilacion','Pensionista') AND cobra_pension_2024_5 &lt;&gt; 'SI'</t>
         </is>
       </c>
+      <c r="Q215" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Desfase temporal entre Afiliación y Pensiones: el 99,8 % de las 2.346 tiene Baja_para_pension con causa 58 (paso a pensionista) y la última baja muy reciente (1.926 en 2025, 415 en 2024), pero la tabla de Pensiones de esta edición aún no recoge esa pensión. Cada columna está bien calculada desde su tabla de origen. </t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
@@ -16658,6 +16819,11 @@
           <t>situacion_paro_ocupacion = 'Pensionista' AND edad_actual_fecha_corte &gt; 100</t>
         </is>
       </c>
+      <c r="Q218" s="2" t="inlineStr">
+        <is>
+          <t>CASO RARO REAL. 1.048 pensionistas de más de 100 años: 366 fallecidos que murieron con más de 100 y 682 vivos con pensión en 2024 (cifra plausible: unos 560 esperables en una muestra del 4 %). 527 tienen jubilación; el resto, viudedad o incapacidad de mayores de 65. Con el corte el 1-5-2025, quien nació entre enero y abril de 1925 tiene entre 100,0 y 100,3 años: parte es efecto del umbral.</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
@@ -16732,6 +16898,11 @@
           <t>situacion_paro_ocupacion = 'Parado_LD' AND edad_actual_fecha_corte &gt; 100</t>
         </is>
       </c>
+      <c r="Q219" s="2" t="inlineStr">
+        <is>
+          <t>2 personas de más de 100 años en Parado_LD sin pensión: un desempleado de esa edad no es plausible (fecha de nacimiento errónea o registro sin cerrar).</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
@@ -16804,6 +16975,11 @@
       <c r="P220" s="2" t="inlineStr">
         <is>
           <t>situacion_paro_ocupacion = 'Parado_LD_pension_no_jubilacion' AND edad_actual_fecha_corte &gt; 100</t>
+        </is>
+      </c>
+      <c r="Q220" s="2" t="inlineStr">
+        <is>
+          <t>CASO RARO REAL. 83 personas de más de 100 años en Parado_LD_pension_no_jubilacion (19 fallecidas y 64 vivas) con viudedad o incapacidad, sin jubilación. La etiqueta 'parado' no mira la edad: 76 de las 83 dejaron de trabajar hace una mediana de 40,2 años. Las personas existen; lo raro es la etiqueta.</t>
         </is>
       </c>
     </row>
@@ -20218,6 +20394,11 @@
           <t>t_tot_reg_ppal &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) + 1 AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
         </is>
       </c>
+      <c r="Q272" s="2" t="inlineStr">
+        <is>
+          <t>Empezó a trabajar antes de la edad mínima legal (14 años hasta la cohorte 1965, 16 después; Ley 8/1980) y no en un régimen o sector de menores autorizados (régimen 0112 de artistas, cine/TV, artes, publicidad, deporte, casting: art. 6.4 ET). Del residuo de C-079 (397): 336 tienen el CNAE del primer empleo desconocido, 329 son del régimen general, 150 empezaron con 12-13 años, 133 con 14-15 y 114 con menos de 12. Pueden ser errores de fecha o menores autorizados sin CNAE; con los datos no se distinguen.</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
@@ -20292,6 +20473,11 @@
           <t>t_tot_grupo_ppal &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) + 1 AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
         </is>
       </c>
+      <c r="Q273" s="2" t="inlineStr">
+        <is>
+          <t>Empezó a trabajar antes de la edad mínima legal (14 años hasta la cohorte 1965, 16 después; Ley 8/1980) y no en un régimen o sector de menores autorizados (régimen 0112 de artistas, cine/TV, artes, publicidad, deporte, casting: art. 6.4 ET). Del residuo de C-079 (397): 336 tienen el CNAE del primer empleo desconocido, 329 son del régimen general, 150 empezaron con 12-13 años, 133 con 14-15 y 114 con menos de 12. Pueden ser errores de fecha o menores autorizados sin CNAE; con los datos no se distinguen.</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" s="2" t="inlineStr">
@@ -20366,6 +20552,11 @@
           <t>t_tot_tipo_contrato_ppal &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) + 1 AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
         </is>
       </c>
+      <c r="Q274" s="2" t="inlineStr">
+        <is>
+          <t>Empezó a trabajar antes de la edad mínima legal (14 años hasta la cohorte 1965, 16 después; Ley 8/1980) y no en un régimen o sector de menores autorizados (régimen 0112 de artistas, cine/TV, artes, publicidad, deporte, casting: art. 6.4 ET). Del residuo de C-079 (397): 336 tienen el CNAE del primer empleo desconocido, 329 son del régimen general, 150 empezaron con 12-13 años, 133 con 14-15 y 114 con menos de 12. Pueden ser errores de fecha o menores autorizados sin CNAE; con los datos no se distinguen.</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" s="2" t="inlineStr">
@@ -20440,6 +20631,11 @@
           <t>t_tot_prov_ppal &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) + 1 AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
         </is>
       </c>
+      <c r="Q275" s="2" t="inlineStr">
+        <is>
+          <t>Empezó a trabajar antes de la edad mínima legal (14 años hasta la cohorte 1965, 16 después; Ley 8/1980) y no en un régimen o sector de menores autorizados (régimen 0112 de artistas, cine/TV, artes, publicidad, deporte, casting: art. 6.4 ET). Del residuo de C-079 (397): 336 tienen el CNAE del primer empleo desconocido, 329 son del régimen general, 150 empezaron con 12-13 años, 133 con 14-15 y 114 con menos de 12. Pueden ser errores de fecha o menores autorizados sin CNAE; con los datos no se distinguen.</t>
+        </is>
+      </c>
     </row>
     <row r="276">
       <c r="A276" s="2" t="inlineStr">
@@ -20514,6 +20710,11 @@
           <t>t_tot_act_econ_ppal &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) + 1 AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
         </is>
       </c>
+      <c r="Q276" s="2" t="inlineStr">
+        <is>
+          <t>Empezó a trabajar antes de la edad mínima legal (14 años hasta la cohorte 1965, 16 después; Ley 8/1980) y no en un régimen o sector de menores autorizados (régimen 0112 de artistas, cine/TV, artes, publicidad, deporte, casting: art. 6.4 ET). Del residuo de C-079 (397): 336 tienen el CNAE del primer empleo desconocido, 329 son del régimen general, 150 empezaron con 12-13 años, 133 con 14-15 y 114 con menos de 12. Pueden ser errores de fecha o menores autorizados sin CNAE; con los datos no se distinguen.</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" s="2" t="inlineStr">
@@ -20588,6 +20789,11 @@
           <t>t_total_empleo &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) + 1 AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
         </is>
       </c>
+      <c r="Q277" s="2" t="inlineStr">
+        <is>
+          <t>Empezó a trabajar antes de la edad mínima legal (14 años hasta la cohorte 1965, 16 después; Ley 8/1980) y no en un régimen o sector de menores autorizados (régimen 0112 de artistas, cine/TV, artes, publicidad, deporte, casting: art. 6.4 ET). Del residuo de C-079 (397): 336 tienen el CNAE del primer empleo desconocido, 329 son del régimen general, 150 empezaron con 12-13 años, 133 con 14-15 y 114 con menos de 12. Pueden ser errores de fecha o menores autorizados sin CNAE; con los datos no se distinguen.</t>
+        </is>
+      </c>
     </row>
     <row r="278">
       <c r="A278" s="2" t="inlineStr">
@@ -20662,6 +20868,11 @@
           <t>t_contrato_mas_largo &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) + 1 AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
         </is>
       </c>
+      <c r="Q278" s="2" t="inlineStr">
+        <is>
+          <t>Empezó a trabajar antes de la edad mínima legal (14 años hasta la cohorte 1965, 16 después; Ley 8/1980) y no en un régimen o sector de menores autorizados (régimen 0112 de artistas, cine/TV, artes, publicidad, deporte, casting: art. 6.4 ET). Del residuo de C-079 (397): 336 tienen el CNAE del primer empleo desconocido, 329 son del régimen general, 150 empezaron con 12-13 años, 133 con 14-15 y 114 con menos de 12. Pueden ser errores de fecha o menores autorizados sin CNAE; con los datos no se distinguen.</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" s="2" t="inlineStr">
@@ -20734,6 +20945,11 @@
       <c r="P279" s="2" t="inlineStr">
         <is>
           <t>tiempo_total_desde_inicio_vl &gt; edad_actual_fecha_corte - (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) + 1 AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
+        </is>
+      </c>
+      <c r="Q279" s="2" t="inlineStr">
+        <is>
+          <t>Empezó a trabajar antes de la edad mínima legal (14 años hasta la cohorte 1965, 16 después; Ley 8/1980) y no en un régimen o sector de menores autorizados (régimen 0112 de artistas, cine/TV, artes, publicidad, deporte, casting: art. 6.4 ET). Del residuo de C-079 (397): 336 tienen el CNAE del primer empleo desconocido, 329 son del régimen general, 150 empezaron con 12-13 años, 133 con 14-15 y 114 con menos de 12. Pueden ser errores de fecha o menores autorizados sin CNAE; con los datos no se distinguen.</t>
         </is>
       </c>
     </row>
@@ -21458,6 +21674,11 @@
           <t>edad_actual_fecha_corte &gt; 105</t>
         </is>
       </c>
+      <c r="Q290" s="2" t="inlineStr">
+        <is>
+          <t>CASO RARO. 67 personas de más de 105 años (23 fallecidas con esa edad al morir y 44 vivas con pensión), nacidas entre 1913 y 1920: más de lo esperable (unas 15 en una muestra del 4 %); algunas reales y otras con fecha de nacimiento errónea o fallecimiento no comunicado.</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" s="2" t="inlineStr">
@@ -21598,6 +21819,11 @@
           <t>date_diff('year', fecha_nacimiento, fecha_ini_primer_empleo) &lt; (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
         </is>
       </c>
+      <c r="Q292" s="2" t="inlineStr">
+        <is>
+          <t>Empezó a trabajar antes de la edad mínima legal (14 años hasta la cohorte 1965, 16 después; Ley 8/1980) y no en un régimen o sector de menores autorizados (régimen 0112 de artistas, cine/TV, artes, publicidad, deporte, casting: art. 6.4 ET). Del residuo de C-079 (397): 336 tienen el CNAE del primer empleo desconocido, 329 son del régimen general, 150 empezaron con 12-13 años, 133 con 14-15 y 114 con menos de 12. Pueden ser errores de fecha o menores autorizados sin CNAE; con los datos no se distinguen.</t>
+        </is>
+      </c>
     </row>
     <row r="293">
       <c r="A293" s="2" t="inlineStr">
@@ -21670,6 +21896,11 @@
       <c r="P293" s="2" t="inlineStr">
         <is>
           <t>fecha_ultima_baja &lt; fecha_ini_primer_empleo AND ipf NOT IN (SELECT ipf FROM solo_prestaciones)</t>
+        </is>
+      </c>
+      <c r="Q293" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Episodios de 1979-1984 con la fecha de baja anterior a la de alta: la duración de empleo sale nula y arrastra t_total_empleo, el número de altas y el tiempo total. Afecta a 6-9 personas; dato de origen. </t>
         </is>
       </c>
     </row>
@@ -21870,6 +22101,11 @@
           <t>date_diff('year', fecha_nacimiento, fecha_ultima_baja) &lt; (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) AND (fecha_ultima_baja IS NULL OR year(fecha_ultima_baja) &lt;&gt; 2099) AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
         </is>
       </c>
+      <c r="Q296" s="2" t="inlineStr">
+        <is>
+          <t>Empezó a trabajar antes de la edad mínima legal (14 años hasta la cohorte 1965, 16 después; Ley 8/1980) y no en un régimen o sector de menores autorizados (régimen 0112 de artistas, cine/TV, artes, publicidad, deporte, casting: art. 6.4 ET). Del residuo de C-079 (397): 336 tienen el CNAE del primer empleo desconocido, 329 son del régimen general, 150 empezaron con 12-13 años, 133 con 14-15 y 114 con menos de 12. Pueden ser errores de fecha o menores autorizados sin CNAE; con los datos no se distinguen.</t>
+        </is>
+      </c>
     </row>
     <row r="297">
       <c r="A297" s="2" t="inlineStr">
@@ -22006,6 +22242,11 @@
           <t>date_diff('year', fecha_nacimiento, fecha_inicio_ultima_racha_sin_empleo) &lt; (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
         </is>
       </c>
+      <c r="Q298" s="2" t="inlineStr">
+        <is>
+          <t>Empezó a trabajar antes de la edad mínima legal (14 años hasta la cohorte 1965, 16 después; Ley 8/1980) y no en un régimen o sector de menores autorizados (régimen 0112 de artistas, cine/TV, artes, publicidad, deporte, casting: art. 6.4 ET). Del residuo de C-079 (397): 336 tienen el CNAE del primer empleo desconocido, 329 son del régimen general, 150 empezaron con 12-13 años, 133 con 14-15 y 114 con menos de 12. Pueden ser errores de fecha o menores autorizados sin CNAE; con los datos no se distinguen.</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" s="2" t="inlineStr">
@@ -22076,6 +22317,11 @@
           <t>fecha_inicio_ultima_racha_sin_empleo &gt; fecha_ultima_baja AND (fecha_ultima_baja IS NULL OR year(fecha_ultima_baja) &lt;&gt; 2099)</t>
         </is>
       </c>
+      <c r="Q299" s="2" t="inlineStr">
+        <is>
+          <t>4 personas con el inicio de la racha sin empleo posterior a la última baja: fechas incoherentes por episodios solapados; volumen insignificante.</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" s="2" t="inlineStr">
@@ -22125,7 +22371,7 @@
       </c>
       <c r="J300" s="5" t="inlineStr">
         <is>
-          <t>Baja calidad de los datos</t>
+          <t>Casos raros (reales)</t>
         </is>
       </c>
       <c r="K300" s="2" t="n">
@@ -22146,6 +22392,11 @@
           <t>fecha_inicio_ultima_racha_sin_empleo &lt; fecha_ini_primer_empleo</t>
         </is>
       </c>
+      <c r="Q300" s="2" t="inlineStr">
+        <is>
+          <t>CASO RARO REAL. 24 personas con la racha sin empleo antes de su primer empleo en Afiliación: cotización previa fuera de la muestra (igual que en G08) o subsidios sin cotización mínima.</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" s="2" t="inlineStr">
@@ -22195,7 +22446,7 @@
       </c>
       <c r="J301" s="5" t="inlineStr">
         <is>
-          <t>Baja calidad de los datos</t>
+          <t>Casos raros (reales)</t>
         </is>
       </c>
       <c r="K301" s="2" t="n">
@@ -22214,6 +22465,11 @@
       <c r="P301" s="2" t="inlineStr">
         <is>
           <t>fecha_inicio_ultima_racha_sin_empleo &lt; fecha_ini_primer_empleo + INTERVAL 360 DAY</t>
+        </is>
+      </c>
+      <c r="Q301" s="2" t="inlineStr">
+        <is>
+          <t>CASO RARO REAL. 1.088 personas con la racha sin empleo a menos de 360 días del primer empleo (mediana 184 días): el 88 % son subsidio o asimilado. Subsidios que no exigen la cotización mínima de la prestación contributiva, o cotización previa fuera de la muestra (igual que en G08).</t>
         </is>
       </c>
     </row>
@@ -22662,6 +22918,11 @@
           <t>fecha_ini_primer_empleo &lt; DATE '1967-01-01'</t>
         </is>
       </c>
+      <c r="Q308" s="2" t="inlineStr">
+        <is>
+          <t>Primer empleo anterior a 1967 (19.912 personas): la guía de la MCVL dice que los datos de afiliación empiezan en 1967; las fechas anteriores son de origen (posiblemente afiliaciones antiguas cargadas con su fecha real).</t>
+        </is>
+      </c>
     </row>
     <row r="309">
       <c r="A309" s="2" t="inlineStr">
@@ -22728,6 +22989,11 @@
           <t>fecha_ultima_baja &lt; DATE '1967-01-01'</t>
         </is>
       </c>
+      <c r="Q309" s="2" t="inlineStr">
+        <is>
+          <t>Última baja anterior a 1967: la guía de la MCVL dice que los datos de afiliación empiezan en 1967, así que fechas anteriores son de origen (133 personas).</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" s="2" t="inlineStr">
@@ -22792,6 +23058,11 @@
       <c r="P310" s="2" t="inlineStr">
         <is>
           <t>fecha_inicio_ultima_racha_sin_empleo &lt; DATE '1967-01-01'</t>
+        </is>
+      </c>
+      <c r="Q310" s="2" t="inlineStr">
+        <is>
+          <t>Inicio de racha sin empleo anterior a 1967 (5 personas): la guía dice que los datos empiezan en 1967; fechas de origen.</t>
         </is>
       </c>
     </row>
@@ -23330,6 +23601,11 @@
           <t>edad_primer_empleo_signif &lt; (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
         </is>
       </c>
+      <c r="Q318" s="2" t="inlineStr">
+        <is>
+          <t>Empezó a trabajar antes de la edad mínima legal (14 años hasta la cohorte 1965, 16 después; Ley 8/1980) y no en un régimen o sector de menores autorizados (régimen 0112 de artistas, cine/TV, artes, publicidad, deporte, casting: art. 6.4 ET). Del residuo de C-079 (397): 336 tienen el CNAE del primer empleo desconocido, 329 son del régimen general, 150 empezaron con 12-13 años, 133 con 14-15 y 114 con menos de 12. Pueden ser errores de fecha o menores autorizados sin CNAE; con los datos no se distinguen.</t>
+        </is>
+      </c>
     </row>
     <row r="319">
       <c r="A319" s="2" t="inlineStr">
@@ -23400,6 +23676,11 @@
           <t>edad_ultimo_empleo &lt; (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
         </is>
       </c>
+      <c r="Q319" s="2" t="inlineStr">
+        <is>
+          <t>Empezó a trabajar antes de la edad mínima legal (14 años hasta la cohorte 1965, 16 después; Ley 8/1980) y no en un régimen o sector de menores autorizados (régimen 0112 de artistas, cine/TV, artes, publicidad, deporte, casting: art. 6.4 ET). Del residuo de C-079 (397): 336 tienen el CNAE del primer empleo desconocido, 329 son del régimen general, 150 empezaron con 12-13 años, 133 con 14-15 y 114 con menos de 12. Pueden ser errores de fecha o menores autorizados sin CNAE; con los datos no se distinguen.</t>
+        </is>
+      </c>
     </row>
     <row r="320">
       <c r="A320" s="2" t="inlineStr">
@@ -23472,6 +23753,11 @@
       <c r="P320" s="2" t="inlineStr">
         <is>
           <t>edad_actual_fecha_corte - tiempo_total_desde_inicio_vl &lt; (CASE WHEN year(fecha_nacimiento) &lt;= 1965 THEN 14 ELSE 16 END) AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
+        </is>
+      </c>
+      <c r="Q320" s="2" t="inlineStr">
+        <is>
+          <t>Empezó a trabajar antes de la edad mínima legal (14 años hasta la cohorte 1965, 16 después; Ley 8/1980) y no en un régimen o sector de menores autorizados (régimen 0112 de artistas, cine/TV, artes, publicidad, deporte, casting: art. 6.4 ET). Del residuo de C-079 (397): 336 tienen el CNAE del primer empleo desconocido, 329 son del régimen general, 150 empezaron con 12-13 años, 133 con 14-15 y 114 con menos de 12. Pueden ser errores de fecha o menores autorizados sin CNAE; con los datos no se distinguen. C-107 sube respecto a antes porque la edad de los fallecidos ya se calcula a su fallecimiento y aflora quien empezó por debajo del mínimo.</t>
         </is>
       </c>
     </row>
@@ -23944,6 +24230,11 @@
           <t>edad_actual_fecha_corte &lt; 16 AND tiempo_total_desde_inicio_vl &gt; 0.1</t>
         </is>
       </c>
+      <c r="Q327" s="2" t="inlineStr">
+        <is>
+          <t>Menores de 16 años actuales con afiliación (287, los mismos en A-093, B-040, B-054, B-070, B-084, C-114 y C-115), nacidos sobre todo desde 2010. De los 262 que además tienen sueldo en 2024, 249 son menores autorizados en espectáculos (art. 6.4 ET); el resto son errores de fecha o afiliaciones de niños sin causa conocida.</t>
+        </is>
+      </c>
     </row>
     <row r="328">
       <c r="A328" s="2" t="inlineStr">
@@ -24012,6 +24303,11 @@
       <c r="P328" s="2" t="inlineStr">
         <is>
           <t>edad_actual_fecha_corte &lt; 16 AND situacion_actual_afiliacion &lt;&gt; 'Nunca_ha_cotizado'</t>
+        </is>
+      </c>
+      <c r="Q328" s="2" t="inlineStr">
+        <is>
+          <t>Menores de 16 años actuales con afiliación (287, los mismos en A-093, B-040, B-054, B-070, B-084, C-114 y C-115), nacidos sobre todo desde 2010. De los 262 que además tienen sueldo en 2024, 249 son menores autorizados en espectáculos (art. 6.4 ET); el resto son errores de fecha o afiliaciones de niños sin causa conocida.</t>
         </is>
       </c>
     </row>
@@ -25024,6 +25320,11 @@
           <t>t_total_empleo IS NULL AND tiempo_total_desde_inicio_vl IS NOT NULL AND ipf NOT IN (SELECT ipf FROM solo_prestaciones)</t>
         </is>
       </c>
+      <c r="Q343" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Episodios de 1979-1984 con la fecha de baja anterior a la de alta: la duración de empleo sale nula y arrastra t_total_empleo, el número de altas y el tiempo total. Afecta a 6-9 personas; dato de origen. </t>
+        </is>
+      </c>
     </row>
     <row r="344">
       <c r="A344" s="2" t="inlineStr">
@@ -25164,6 +25465,11 @@
           <t>num_altas_anual_promedio IS NULL AND tiempo_total_desde_inicio_vl IS NOT NULL AND ipf NOT IN (SELECT ipf FROM solo_prestaciones)</t>
         </is>
       </c>
+      <c r="Q345" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Episodios de 1979-1984 con la fecha de baja anterior a la de alta: la duración de empleo sale nula y arrastra t_total_empleo, el número de altas y el tiempo total. Afecta a 6-9 personas; dato de origen. </t>
+        </is>
+      </c>
     </row>
     <row r="346">
       <c r="A346" s="2" t="inlineStr">
@@ -25572,6 +25878,11 @@
           <t>t_total_desempleo IS NULL AND tiempo_total_desde_inicio_vl IS NOT NULL AND ipf NOT IN (SELECT ipf FROM solo_prestaciones)</t>
         </is>
       </c>
+      <c r="Q351" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Episodios de 1979-1984 con la fecha de baja anterior a la de alta: la duración de empleo sale nula y arrastra t_total_empleo, el número de altas y el tiempo total. Afecta a 6-9 personas; dato de origen. </t>
+        </is>
+      </c>
     </row>
     <row r="352">
       <c r="A352" s="2" t="inlineStr">
@@ -26108,6 +26419,11 @@
           <t>discap_pension AND (pension_todas_cobradas IS NULL OR array_to_string(pension_todas_cobradas, ',') NOT LIKE '%Incapacidad%')</t>
         </is>
       </c>
+      <c r="Q359" s="2" t="inlineStr">
+        <is>
+          <t>524 personas con discapacidad por pensión (Discap_pension) sin pensión de incapacidad en la tabla de pensiones. Pendiente de confirmar la definición de Discap_pension; probablemente el mismo desfase temporal que el resto de G07.</t>
+        </is>
+      </c>
     </row>
     <row r="360">
       <c r="A360" s="2" t="inlineStr">
@@ -26293,7 +26609,7 @@
       </c>
       <c r="J362" s="5" t="inlineStr">
         <is>
-          <t>Baja calidad de los datos</t>
+          <t>Casos raros (reales)</t>
         </is>
       </c>
       <c r="K362" s="2" t="n">
@@ -26316,6 +26632,11 @@
       <c r="P362" s="2" t="inlineStr">
         <is>
           <t>array_to_string(pension_actual, ',') LIKE '%Orfandad%' AND edad_actual_fecha_corte &gt; 60 AND ipf NOT IN (SELECT ipf FROM orfandad_vitalicia)</t>
+        </is>
+      </c>
+      <c r="Q362" s="2" t="inlineStr">
+        <is>
+          <t>CASO RARO REAL. 12 mujeres de más de 60 años con orfandad no vitalicia, nacidas entre 1946 y 1958, que cobran prestaciones complementarias de mutualidad (10 del régimen 68, Fondo de la Mutualidad de Previsión, y 2 del 38, Mutualidad de Funcionarios), con condiciones propias distintas de la LGSS.</t>
         </is>
       </c>
     </row>
@@ -26499,7 +26820,7 @@
       </c>
       <c r="J365" s="5" t="inlineStr">
         <is>
-          <t>Baja calidad de los datos</t>
+          <t>Casos raros (reales)</t>
         </is>
       </c>
       <c r="K365" s="2" t="n">
@@ -26520,6 +26841,11 @@
           <t>array_to_string(pension_actual, ',') LIKE '%Incapacidad&gt;65%' AND edad_actual_fecha_corte &lt; 65</t>
         </is>
       </c>
+      <c r="Q365" s="2" t="inlineStr">
+        <is>
+          <t>CASO RARO. 2 personas de 54 y 56 años con pensión 'Incapacidad&gt;65' (clave J, que se asigna al cumplir 65 años): clave anticipada o error de origen; caso aislado.</t>
+        </is>
+      </c>
     </row>
     <row r="366">
       <c r="A366" s="2" t="inlineStr">
@@ -26569,7 +26895,7 @@
       </c>
       <c r="J366" s="5" t="inlineStr">
         <is>
-          <t>Baja calidad de los datos</t>
+          <t>Casos raros (reales)</t>
         </is>
       </c>
       <c r="K366" s="2" t="n">
@@ -26590,6 +26916,11 @@
           <t>array_to_string(pension_actual, ',') LIKE '%Jubilaci%' AND array_to_string(pension_actual, ',') LIKE '%Incapacidad%'</t>
         </is>
       </c>
+      <c r="Q366" s="2" t="inlineStr">
+        <is>
+          <t>CASO RARO REAL. 1.108 personas con jubilación e incapacidad a la vez: 612 'Incapacidad&gt;65 + Jubilación' y 343 'Incapacidad + Jubilación'; solo 6 tienen SOVI. Posible pluripensión (pensiones de distintos regímenes); no se puede confirmar con los datos.</t>
+        </is>
+      </c>
     </row>
     <row r="367">
       <c r="A367" s="2" t="inlineStr">
@@ -26664,6 +26995,11 @@
           <t>array_to_string(pension_actual, ',') LIKE '%Jubilaci%' AND COALESCE(t_total_empleo,0) + COALESCE(t_total_mixto_empl_desempl,0) &lt; 10</t>
         </is>
       </c>
+      <c r="Q367" s="2" t="inlineStr">
+        <is>
+          <t>Jubilados con menos de 10 años de empleo afiliado (16.660), nacidos sobre todo entre 1920 y 1950 (edad mediana 82,7 años, 73 % mujeres). Tienen pensión SOVI (cotizaciones anteriores a 1967, que no están en Afiliación) 7.607 de los 16.660; el resto, carreras en parte anteriores a 1967 o en regímenes sin registro en la MCVL. Cobertura incompleta de origen.</t>
+        </is>
+      </c>
     </row>
     <row r="368">
       <c r="A368" s="2" t="inlineStr">
@@ -26736,6 +27072,11 @@
       <c r="P368" s="2" t="inlineStr">
         <is>
           <t>array_to_string(pension_actual, ',') LIKE '%Jubilaci%' AND edad_ultimo_empleo &lt; 30</t>
+        </is>
+      </c>
+      <c r="Q368" s="2" t="inlineStr">
+        <is>
+          <t>Jubilados cuyo último empleo afiliado fue antes de los 30 años (613): carreras anteriores a 1967 o sin registro en la MCVL; cobertura incompleta de origen.</t>
         </is>
       </c>
     </row>
@@ -27188,6 +27529,11 @@
           <t>ingresos_bruto_total_2024 &gt; 0 AND NOT (prov_fiscal_actual IS NOT NULL AND prov_fiscal_actual NOT IN ('NO CONSTA','No consta','0 NO CONSTA','00 No consta'))</t>
         </is>
       </c>
+      <c r="Q375" s="2" t="inlineStr">
+        <is>
+          <t>446 personas con ingresos fiscales y sin provincia fiscal: el código de provincia crudo del modelo 190 es 0 en 445 casos y 99 en 1; el modelo 190 no lo informa. Dato de origen.</t>
+        </is>
+      </c>
     </row>
     <row r="376">
       <c r="A376" s="2" t="inlineStr">
@@ -27303,7 +27649,7 @@
       </c>
       <c r="J377" s="5" t="inlineStr">
         <is>
-          <t>Baja calidad de los datos</t>
+          <t>Casos raros (reales)</t>
         </is>
       </c>
       <c r="K377" s="2" t="n">
@@ -27326,6 +27672,11 @@
       <c r="P377" s="2" t="inlineStr">
         <is>
           <t>ingresos_bruto_total_2024 &gt; 0 AND edad_actual_fecha_corte &lt; 16</t>
+        </is>
+      </c>
+      <c r="Q377" s="2" t="inlineStr">
+        <is>
+          <t>CASO RARO REAL. 1.626 personas con ingresos fiscales en 2024 y menos de 16 años: en su mayoría pensiones de orfandad (que constan como ingresos) y menores con sueldo autorizados en espectáculos (art. 6.4 ET). No es un error.</t>
         </is>
       </c>
     </row>
@@ -31161,7 +31512,7 @@
       </c>
       <c r="J438" s="4" t="inlineStr">
         <is>
-          <t>Baja calidad de los datos</t>
+          <t>Casos raros (reales)</t>
         </is>
       </c>
       <c r="K438" s="2" t="n">
@@ -31186,6 +31537,11 @@
           <t>reg_cotiz_ppal_agrupado LIKE '06 %' AND (act_econ_ppal IS NOT NULL AND act_econ_ppal NOT IN ('NO CONSTA','No consta','0 NO CONSTA','00 No consta')) AND NOT (act_econ_ppal LIKE '01%' OR act_econ_ppal LIKE '02%' OR act_econ_ppal LIKE '03%')</t>
         </is>
       </c>
+      <c r="Q438" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CASO RARO REAL. 8.906 agrarios por cuenta ajena con actividad principal no agraria. Desajuste estructural esperado: el régimen principal y la actividad principal son dos 'ganadores' calculados de forma independiente sobre la misma persona (la actividad puede ser de otro periodo) y no tienen por qué coincidir. Comprobado: la fusión de tramos no lo arregla (solo 3 de 6.000 casos cambian de actividad ganadora). Personas reales con combinaciones poco habituales, no datos erróneos. </t>
+        </is>
+      </c>
     </row>
     <row r="439">
       <c r="A439" s="2" t="inlineStr">
@@ -31235,7 +31591,7 @@
       </c>
       <c r="J439" s="4" t="inlineStr">
         <is>
-          <t>Baja calidad de los datos</t>
+          <t>Casos raros (reales)</t>
         </is>
       </c>
       <c r="K439" s="2" t="n">
@@ -31256,6 +31612,11 @@
           <t>reg_cotiz_ppal_agrupado LIKE '07 %' AND (act_econ_ppal IS NOT NULL AND act_econ_ppal NOT IN ('NO CONSTA','No consta','0 NO CONSTA','00 No consta')) AND NOT (act_econ_ppal LIKE '01%' OR act_econ_ppal LIKE '02%' OR act_econ_ppal LIKE '03%')</t>
         </is>
       </c>
+      <c r="Q439" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CASO RARO REAL. 1.450 del R.E. Agrario cuenta propia con actividad principal no agraria. Desajuste estructural esperado: el régimen principal y la actividad principal son dos 'ganadores' calculados de forma independiente sobre la misma persona (la actividad puede ser de otro periodo) y no tienen por qué coincidir. Comprobado: la fusión de tramos no lo arregla (solo 3 de 6.000 casos cambian de actividad ganadora). Personas reales con combinaciones poco habituales, no datos erróneos. </t>
+        </is>
+      </c>
     </row>
     <row r="440">
       <c r="A440" s="2" t="inlineStr">
@@ -31305,7 +31666,7 @@
       </c>
       <c r="J440" s="4" t="inlineStr">
         <is>
-          <t>Baja calidad de los datos</t>
+          <t>Casos raros (reales)</t>
         </is>
       </c>
       <c r="K440" s="2" t="n">
@@ -31326,6 +31687,11 @@
           <t>reg_cotiz_ppal_agrupado LIKE '12 %' AND (act_econ_ppal IS NOT NULL AND act_econ_ppal NOT IN ('NO CONSTA','No consta','0 NO CONSTA','00 No consta')) AND act_econ_ppal NOT LIKE '970%'</t>
         </is>
       </c>
+      <c r="Q440" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CASO RARO REAL. 2.310 del R.E. Empleados de Hogar con CNAE distinto de 970 (hogares como empleadores). Desajuste estructural esperado: el régimen principal y la actividad principal son dos 'ganadores' calculados de forma independiente sobre la misma persona (la actividad puede ser de otro periodo) y no tienen por qué coincidir. Comprobado: la fusión de tramos no lo arregla (solo 3 de 6.000 casos cambian de actividad ganadora). Personas reales con combinaciones poco habituales, no datos erróneos. </t>
+        </is>
+      </c>
     </row>
     <row r="441">
       <c r="A441" s="2" t="inlineStr">
@@ -31375,7 +31741,7 @@
       </c>
       <c r="J441" s="4" t="inlineStr">
         <is>
-          <t>Baja calidad de los datos</t>
+          <t>Casos raros (reales)</t>
         </is>
       </c>
       <c r="K441" s="2" t="n">
@@ -31400,6 +31766,11 @@
           <t>reg_cotiz_ppal_agrupado LIKE '0138 %' AND (act_econ_ppal IS NOT NULL AND act_econ_ppal NOT IN ('NO CONSTA','No consta','0 NO CONSTA','00 No consta')) AND act_econ_ppal NOT LIKE '970%'</t>
         </is>
       </c>
+      <c r="Q441" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CASO RARO REAL. 23 del Régimen General (S.E.C. Empleados de Hogar) con CNAE distinto de 970. Desajuste estructural esperado: el régimen principal y la actividad principal son dos 'ganadores' calculados de forma independiente sobre la misma persona (la actividad puede ser de otro periodo) y no tienen por qué coincidir. Comprobado: la fusión de tramos no lo arregla (solo 3 de 6.000 casos cambian de actividad ganadora). Personas reales con combinaciones poco habituales, no datos erróneos. </t>
+        </is>
+      </c>
     </row>
     <row r="442">
       <c r="A442" s="2" t="inlineStr">
@@ -31449,7 +31820,7 @@
       </c>
       <c r="J442" s="4" t="inlineStr">
         <is>
-          <t>Baja calidad de los datos</t>
+          <t>Casos raros (reales)</t>
         </is>
       </c>
       <c r="K442" s="2" t="n">
@@ -31470,6 +31841,11 @@
           <t>reg_cotiz_ppal_agrupado LIKE '08 %' AND (act_econ_ppal IS NOT NULL AND act_econ_ppal NOT IN ('NO CONSTA','No consta','0 NO CONSTA','00 No consta')) AND NOT (act_econ_ppal LIKE '03%' OR act_econ_ppal LIKE '50%')</t>
         </is>
       </c>
+      <c r="Q442" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CASO RARO REAL. 1.316 del R.E. del Mar con actividad principal distinta de pesca o transporte marítimo (p. ej. hostelería o servicios portuarios). Desajuste estructural esperado: el régimen principal y la actividad principal son dos 'ganadores' calculados de forma independiente sobre la misma persona (la actividad puede ser de otro periodo) y no tienen por qué coincidir. Comprobado: la fusión de tramos no lo arregla (solo 3 de 6.000 casos cambian de actividad ganadora). Personas reales con combinaciones poco habituales, no datos erróneos. </t>
+        </is>
+      </c>
     </row>
     <row r="443">
       <c r="A443" s="2" t="inlineStr">
@@ -31519,7 +31895,7 @@
       </c>
       <c r="J443" s="4" t="inlineStr">
         <is>
-          <t>Baja calidad de los datos</t>
+          <t>Casos raros (reales)</t>
         </is>
       </c>
       <c r="K443" s="2" t="n">
@@ -31540,6 +31916,11 @@
           <t>reg_cotiz_ppal_agrupado LIKE '09 %' AND (act_econ_ppal IS NOT NULL AND act_econ_ppal NOT IN ('NO CONSTA','No consta','0 NO CONSTA','00 No consta')) AND act_econ_ppal NOT LIKE '05%'</t>
         </is>
       </c>
+      <c r="Q443" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CASO RARO REAL. 112 del R.E. Minería del Carbón con actividad principal distinta de la extracción de carbón. Desajuste estructural esperado: el régimen principal y la actividad principal son dos 'ganadores' calculados de forma independiente sobre la misma persona (la actividad puede ser de otro periodo) y no tienen por qué coincidir. Comprobado: la fusión de tramos no lo arregla (solo 3 de 6.000 casos cambian de actividad ganadora). Personas reales con combinaciones poco habituales, no datos erróneos. </t>
+        </is>
+      </c>
     </row>
     <row r="444">
       <c r="A444" s="2" t="inlineStr">
@@ -31612,6 +31993,11 @@
       <c r="P444" s="2" t="inlineStr">
         <is>
           <t>reg_cotiz_ppal_agrupado LIKE '05 %' AND grupo_cotiz_ppal NOT IN ('0 NO CONSTA','NO CONSTA')</t>
+        </is>
+      </c>
+      <c r="Q444" s="2" t="inlineStr">
+        <is>
+          <t>162 autónomos con grupo de cotización: la guía (2.003) dice que en el R.E. de Autónomos no se asigna grupo; algunos registros de origen lo traen igualmente.</t>
         </is>
       </c>
     </row>
@@ -31684,6 +32070,11 @@
           <t>reg_cotiz_ppal_agrupado LIKE '12 %' AND grupo_cotiz_ppal NOT IN ('0 NO CONSTA','NO CONSTA')</t>
         </is>
       </c>
+      <c r="Q445" s="2" t="inlineStr">
+        <is>
+          <t>12 empleados de hogar con grupo de cotización, que la guía (2.003) dice que no se asigna en ese régimen; dato de origen.</t>
+        </is>
+      </c>
     </row>
     <row r="446">
       <c r="A446" s="2" t="inlineStr">
@@ -31758,6 +32149,11 @@
           <t>reg_cotiz_ppal_agrupado LIKE '05 %' AND tipo_contr_ppal_agrupado NOT IN ('No consta')</t>
         </is>
       </c>
+      <c r="Q446" s="2" t="inlineStr">
+        <is>
+          <t>12 autónomos con tipo de contrato distinto de 'No consta'; dato de origen.</t>
+        </is>
+      </c>
     </row>
     <row r="447">
       <c r="A447" s="2" t="inlineStr">
@@ -31807,7 +32203,7 @@
       </c>
       <c r="J447" s="5" t="inlineStr">
         <is>
-          <t>Baja calidad de los datos</t>
+          <t>Casos raros (reales)</t>
         </is>
       </c>
       <c r="K447" s="2" t="n">
@@ -31828,6 +32224,11 @@
           <t>reg_cotiz_ppal_agrupado LIKE '07 %' AND t_tot_reg_ppal &gt; 41.5</t>
         </is>
       </c>
+      <c r="Q447" s="2" t="inlineStr">
+        <is>
+          <t>CASO RARO REAL. 239 personas superan los 41,5 años en el R.E. Agrario cuenta propia (1967-2008, el máximo posible). Probable pluriactividad agraria o cuentas de cotización simultáneas que se cuentan por separado; son personas reales con historias poco habituales.</t>
+        </is>
+      </c>
     </row>
     <row r="448">
       <c r="A448" s="2" t="inlineStr">
@@ -31900,6 +32301,11 @@
       <c r="P448" s="2" t="inlineStr">
         <is>
           <t>reg_cotiz_ppal_agrupado LIKE '06 %' AND t_tot_reg_ppal &gt; 45.5</t>
+        </is>
+      </c>
+      <c r="Q448" s="2" t="inlineStr">
+        <is>
+          <t>21 personas con más de 45,5 años en el R.E. Agrario cuenta ajena integrado en 2012: posible por episodios simultáneos; volumen pequeño.</t>
         </is>
       </c>
     </row>
@@ -31972,6 +32378,11 @@
           <t>reg_cotiz_ppal_agrupado LIKE '12 %' AND t_tot_reg_ppal &gt; 45.5</t>
         </is>
       </c>
+      <c r="Q449" s="2" t="inlineStr">
+        <is>
+          <t>1 persona con más de 45,5 años en el régimen de Empleados de Hogar integrado en 2012: caso aislado.</t>
+        </is>
+      </c>
     </row>
     <row r="450">
       <c r="A450" s="2" t="inlineStr">
@@ -32116,6 +32527,11 @@
           <t>grupo_cotiz_ppal LIKE '11 %' AND t_tot_grupo_ppal &gt; 2.1</t>
         </is>
       </c>
+      <c r="Q451" s="2" t="inlineStr">
+        <is>
+          <t>El campo 03 GRU_COTIZACION de la MCVL no se actualiza al cumplir la edad: p. ej. un episodio único de 49,6 años seguidos codificado como grupo 11 (menores de 18) de principio a fin (el 76 % de C-243 tiene un único episodio así). El ETL reporta fielmente lo que trae el dato de origen; no hay cálculo propio que corregir. Aquí: más de 2,1 años en el grupo 11 (menores de 18), imposible entre los 16 y los 18 años.</t>
+        </is>
+      </c>
     </row>
     <row r="452">
       <c r="A452" s="2" t="inlineStr">
@@ -32188,6 +32604,11 @@
       <c r="P452" s="2" t="inlineStr">
         <is>
           <t>grupo_cotiz_ppal LIKE '12 %' AND t_tot_grupo_ppal &gt; 1.1</t>
+        </is>
+      </c>
+      <c r="Q452" s="2" t="inlineStr">
+        <is>
+          <t>El campo 03 GRU_COTIZACION de la MCVL no se actualiza al cumplir la edad: p. ej. un episodio único de 49,6 años seguidos codificado como grupo 11 (menores de 18) de principio a fin (el 76 % de C-243 tiene un único episodio así). El ETL reporta fielmente lo que trae el dato de origen; no hay cálculo propio que corregir. Aquí: más de 1,1 años en el grupo 12 (menores de 17).</t>
         </is>
       </c>
     </row>
@@ -32260,6 +32681,11 @@
           <t>grupo_ultimo_empleo LIKE '11 %' AND edad_ultimo_empleo &gt;= 18.1</t>
         </is>
       </c>
+      <c r="Q453" s="2" t="inlineStr">
+        <is>
+          <t>El campo 03 GRU_COTIZACION de la MCVL no se actualiza al cumplir la edad: p. ej. un episodio único de 49,6 años seguidos codificado como grupo 11 (menores de 18) de principio a fin (el 76 % de C-243 tiene un único episodio así). El ETL reporta fielmente lo que trae el dato de origen; no hay cálculo propio que corregir. Aquí: último empleo en el grupo 11 con edad del último empleo de 18 o más.</t>
+        </is>
+      </c>
     </row>
     <row r="454">
       <c r="A454" s="2" t="inlineStr">
@@ -32330,6 +32756,11 @@
           <t>grupo_ultimo_empleo LIKE '12 %' AND edad_ultimo_empleo &gt;= 17.1</t>
         </is>
       </c>
+      <c r="Q454" s="2" t="inlineStr">
+        <is>
+          <t>El campo 03 GRU_COTIZACION de la MCVL no se actualiza al cumplir la edad: p. ej. un episodio único de 49,6 años seguidos codificado como grupo 11 (menores de 18) de principio a fin (el 76 % de C-243 tiene un único episodio así). El ETL reporta fielmente lo que trae el dato de origen; no hay cálculo propio que corregir. Aquí: último empleo en el grupo 12 con edad del último empleo de 17 o más.</t>
+        </is>
+      </c>
     </row>
     <row r="455">
       <c r="A455" s="2" t="inlineStr">
@@ -32400,6 +32831,11 @@
           <t>grupo_cotiz_1er_empleo_signif LIKE '11 %' AND edad_primer_empleo_signif &gt;= 18.1</t>
         </is>
       </c>
+      <c r="Q455" s="2" t="inlineStr">
+        <is>
+          <t>El campo 03 GRU_COTIZACION de la MCVL no se actualiza al cumplir la edad: p. ej. un episodio único de 49,6 años seguidos codificado como grupo 11 (menores de 18) de principio a fin (el 76 % de C-243 tiene un único episodio así). El ETL reporta fielmente lo que trae el dato de origen; no hay cálculo propio que corregir. Aquí: primer empleo significativo en el grupo 11 (menores de 18) con 18 o más años.</t>
+        </is>
+      </c>
     </row>
     <row r="456">
       <c r="A456" s="2" t="inlineStr">
@@ -32470,6 +32906,11 @@
           <t>grupo_cotiz_1er_empleo_signif LIKE '12 %' AND edad_primer_empleo_signif &gt;= 17.1</t>
         </is>
       </c>
+      <c r="Q456" s="2" t="inlineStr">
+        <is>
+          <t>El campo 03 GRU_COTIZACION de la MCVL no se actualiza al cumplir la edad: p. ej. un episodio único de 49,6 años seguidos codificado como grupo 11 (menores de 18) de principio a fin (el 76 % de C-243 tiene un único episodio así). El ETL reporta fielmente lo que trae el dato de origen; no hay cálculo propio que corregir. Aquí: primer empleo significativo en el grupo 12 (menores de 17) con 17 o más años.</t>
+        </is>
+      </c>
     </row>
     <row r="457">
       <c r="A457" s="2" t="inlineStr">
@@ -32540,6 +32981,11 @@
           <t>grupo_ultimo_empleo LIKE '10 %' AND edad_ultimo_empleo &lt; 17.9</t>
         </is>
       </c>
+      <c r="Q457" s="2" t="inlineStr">
+        <is>
+          <t>El campo 03 GRU_COTIZACION de la MCVL no se actualiza al cumplir la edad: p. ej. un episodio único de 49,6 años seguidos codificado como grupo 11 (menores de 18) de principio a fin (el 76 % de C-243 tiene un único episodio así). El ETL reporta fielmente lo que trae el dato de origen; no hay cálculo propio que corregir. Aquí: último empleo en el grupo 10 ('mayores de 18') con menos de 18 años.</t>
+        </is>
+      </c>
     </row>
     <row r="458">
       <c r="A458" s="2" t="inlineStr">
@@ -32614,6 +33060,11 @@
           <t>grupo_cotiz_1er_empleo_signif LIKE '10 %' AND edad_primer_empleo_signif &lt; 17.9</t>
         </is>
       </c>
+      <c r="Q458" s="2" t="inlineStr">
+        <is>
+          <t>El campo 03 GRU_COTIZACION de la MCVL no se actualiza al cumplir la edad: p. ej. un episodio único de 49,6 años seguidos codificado como grupo 11 (menores de 18) de principio a fin (el 76 % de C-243 tiene un único episodio así). El ETL reporta fielmente lo que trae el dato de origen; no hay cálculo propio que corregir. Aquí: primer empleo en el grupo 10 ('mayores de 18 años') con menos de 18 años de edad.</t>
+        </is>
+      </c>
     </row>
     <row r="459">
       <c r="A459" s="2" t="inlineStr">
@@ -32663,7 +33114,7 @@
       </c>
       <c r="J459" s="5" t="inlineStr">
         <is>
-          <t>Baja calidad de los datos</t>
+          <t>Casos raros (reales)</t>
         </is>
       </c>
       <c r="K459" s="2" t="n">
@@ -32682,6 +33133,11 @@
       <c r="P459" s="2" t="inlineStr">
         <is>
           <t>grupo_cotiz_1er_empleo_signif LIKE '1 %' AND edad_primer_empleo_signif &lt; 18</t>
+        </is>
+      </c>
+      <c r="Q459" s="2" t="inlineStr">
+        <is>
+          <t>CASO RARO. 125 personas con primer empleo significativo como ingeniero o licenciado (grupo 1) con menos de 18 años: casos infrecuentes de jóvenes con esa cualificación o grupo mal asignado; no se distingue con los datos.</t>
         </is>
       </c>
     </row>
@@ -33824,6 +34280,11 @@
           <t>causa_ult_baja LIKE '56 %' AND fecha_fallecimiento = 0</t>
         </is>
       </c>
+      <c r="Q475" s="2" t="inlineStr">
+        <is>
+          <t>Baja por fallecimiento (causa 56) en Afiliación sin fecha de fallecimiento en Personas (7 personas): la guía admite retrasos en registrar el fallecimiento. Dato de origen.</t>
+        </is>
+      </c>
     </row>
     <row r="476">
       <c r="A476" s="2" t="inlineStr">
@@ -34430,6 +34891,11 @@
           <t>t_total_desempleo &gt; 0 AND num_bajas_anual_promedio IS NULL AND ipf NOT IN (SELECT ipf FROM solo_prestaciones) AND situacion_actual_afiliacion &lt;&gt; 'Alta_ocupado'</t>
         </is>
       </c>
+      <c r="Q484" s="2" t="inlineStr">
+        <is>
+          <t>8 personas con tiempo de desempleo y sin bajas de empleo, con empleo aún abierto: episodios sin cerrar; volumen pequeño.</t>
+        </is>
+      </c>
     </row>
     <row r="485">
       <c r="A485" s="2" t="inlineStr">
@@ -35758,6 +36224,11 @@
           <t>ingresos_sueldo_2024 &gt; 0 AND edad_actual_fecha_corte &lt; 16 AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
         </is>
       </c>
+      <c r="Q504" s="2" t="inlineStr">
+        <is>
+          <t>13 menores de 16 años con sueldo en 2024 que NO son menores autorizados (de 262 iniciales, 249 sí lo son: art. 6.4 ET). Fecha de nacimiento errónea o afiliación de niños sin causa conocida.</t>
+        </is>
+      </c>
     </row>
     <row r="505">
       <c r="A505" s="2" t="inlineStr">
@@ -36030,6 +36501,11 @@
           <t>ingresos_actividad_2024 &gt; 0 AND edad_actual_fecha_corte &lt; 16 AND ipf NOT IN (SELECT ipf FROM menor_autorizado)</t>
         </is>
       </c>
+      <c r="Q508" s="2" t="inlineStr">
+        <is>
+          <t>5 menores de 16 años con ingresos de actividad en 2024 que NO son menores autorizados (de 11 iniciales, 6 sí lo son). Fecha de nacimiento errónea o afiliación de niños sin causa conocida.</t>
+        </is>
+      </c>
     </row>
     <row r="509">
       <c r="A509" s="2" t="inlineStr">
@@ -36211,7 +36687,7 @@
       </c>
       <c r="J511" s="5" t="inlineStr">
         <is>
-          <t>Baja calidad de los datos</t>
+          <t>Casos raros (reales)</t>
         </is>
       </c>
       <c r="K511" s="2" t="n">
@@ -36236,6 +36712,11 @@
           <t>ingresos_prestacion_2024 &gt; 0 AND COALESCE(t_total_desempleo, 0) + COALESCE(t_total_mixto_empl_desempl, 0) = 0</t>
         </is>
       </c>
+      <c r="Q511" s="2" t="inlineStr">
+        <is>
+          <t>CASO RARO REAL. 383 personas con prestación por desempleo en 2024 y sin tiempo de desempleo en Afiliación: los subsidios pueden no figurar como desempleo en la tabla de afiliación.</t>
+        </is>
+      </c>
     </row>
     <row r="512">
       <c r="A512" s="2" t="inlineStr">
@@ -36285,7 +36766,7 @@
       </c>
       <c r="J512" s="5" t="inlineStr">
         <is>
-          <t>Baja calidad de los datos</t>
+          <t>Casos raros (reales)</t>
         </is>
       </c>
       <c r="K512" s="2" t="n">
@@ -36310,6 +36791,11 @@
           <t>ingresos_sueldo_2024 &gt; 0 AND fecha_ini_primer_empleo IS NULL</t>
         </is>
       </c>
+      <c r="Q512" s="2" t="inlineStr">
+        <is>
+          <t>CASO RARO REAL. 211 personas con sueldo en 2024 y sin primer empleo en Afiliación: los funcionarios de mutualidades (p. ej. MUFACE) no cotizan en el sistema de la MCVL.</t>
+        </is>
+      </c>
     </row>
     <row r="513">
       <c r="A513" s="2" t="inlineStr">
@@ -36359,7 +36845,7 @@
       </c>
       <c r="J513" s="5" t="inlineStr">
         <is>
-          <t>Baja calidad de los datos</t>
+          <t>Casos raros (reales)</t>
         </is>
       </c>
       <c r="K513" s="2" t="n">
@@ -36384,6 +36870,11 @@
           <t>ingresos_sueldo_2024 &gt; 0 AND fecha_ultima_baja IS NOT NULL AND year(fecha_ultima_baja) &lt; 2024</t>
         </is>
       </c>
+      <c r="Q513" s="2" t="inlineStr">
+        <is>
+          <t>CASO RARO REAL. 3.867 personas con sueldo en 2024 y última baja anterior a 2024: sueldo mediano de solo 328 €; 2.926 están en Baja_para_pension y 2.168 tienen la baja en 2023. Encaja con finiquitos, atrasos o indemnizaciones pagados después de la baja.</t>
+        </is>
+      </c>
     </row>
     <row r="514">
       <c r="A514" s="2" t="inlineStr">
@@ -36433,7 +36924,7 @@
       </c>
       <c r="J514" s="5" t="inlineStr">
         <is>
-          <t>Baja calidad de los datos</t>
+          <t>Casos raros (reales)</t>
         </is>
       </c>
       <c r="K514" s="2" t="n">
@@ -36456,6 +36947,11 @@
       <c r="P514" s="2" t="inlineStr">
         <is>
           <t>cobra_pension_2024_5 = 'SI' AND ingresos_bruto_total_2024 IS NOT NULL AND ingresos_pension_y_bajas_2024 = 0</t>
+        </is>
+      </c>
+      <c r="Q514" s="2" t="inlineStr">
+        <is>
+          <t>CASO RARO REAL. 2.030 personas que cobran pensión según la tabla de pensiones y no tienen importe de pensión en fiscal: pensión iniciada en 2025 (cobra_pension_2024/5 incluye 2025) o no declarada en el modelo 190 de 2024.</t>
         </is>
       </c>
     </row>
@@ -38079,7 +38575,7 @@
       </c>
       <c r="J539" s="5" t="inlineStr">
         <is>
-          <t>Baja calidad de los datos</t>
+          <t>Casos raros (reales)</t>
         </is>
       </c>
       <c r="K539" s="2" t="n">
@@ -38102,6 +38598,11 @@
       <c r="P539" s="2" t="inlineStr">
         <is>
           <t>(domic_resid_habitual IS NOT NULL AND domic_resid_habitual NOT IN ('NO CONSTA','No consta','0 NO CONSTA','00 No consta')) AND (prov_fiscal_actual IS NOT NULL AND prov_fiscal_actual NOT IN ('NO CONSTA','No consta','0 NO CONSTA','00 No consta')) AND CASE WHEN split_part(prov_fiscal_actual, ' ', 1) = '53' THEN '38' ELSE split_part(prov_fiscal_actual, ' ', 1) END &lt;&gt; left(domic_resid_habitual, 2) AND split_part(prov_fiscal_actual, ' ', 1) &lt;&gt; '98'</t>
+        </is>
+      </c>
+      <c r="Q539" s="2" t="inlineStr">
+        <is>
+          <t>CASO RARO REAL. La provincia de residencia (Padrón) no coincide con la fiscal (domicilio a 31-12-2024) en 61.583 personas (4,5 %): mudanzas y domicilios fiscales sin actualizar. La provincia fiscal 53 (Isla de La Palma) se compara como 38 y el 98 (residencia fiscal en el extranjero) se excluye. 1.354 de las 1.560 con fiscal 53 residen en Santa Cruz de Tenerife, que es su provincia INE.</t>
         </is>
       </c>
     </row>
@@ -38333,7 +38834,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>93</v>
+        <v>68</v>
       </c>
     </row>
     <row r="17">
@@ -38343,7 +38844,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>6</v>
+        <v>31</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
reglas: C-108, C-264 y C-265 (la misma persona) como baja calidad de los datos
Un fallecido con un episodio de empleo abierto al morir: la duracion del primer empleo significativo (2,17 anyos) supera su tiempo de empleo (1,08), cortado en el fallecimiento. Sin cambios en el ETL. No queda ninguna regla pendiente: 391 pasan, 45 corregidas, 71 baja calidad y 31 casos raros.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/reglas_consistencia_resultados_sin_ipf.xlsx
+++ b/tests/reglas_consistencia_resultados_sin_ipf.xlsx
@@ -1139,7 +1139,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Con las bajas reales (2026-09-21), C-255 (bajas &gt; altas) pasa a 0 y C-257/C-258 (enteros) se corrigieron (factor 365 vs 365,25). Siguen: 9.198 con más causas distintas que altas + 1,5 (C-260), ~2.100 con más de 20 altas/bajas por año (C-069/C-070). ACTUALIZACIÓN 2026-09-24: C-262 (120), C-264 (176), C-266 y C-267 pasan a 0 o 1 tras corregir los tramos de afiliación (ver G21). CERRADO 2026-09-25 (decisión del usuario): la variable causas_baja_distintas se ELIMINA (ETL, app y sus 11 reglas: A-018, A-044, C-026, C-077, C-139, C-140, C-144, C-145, C-259, C-260, C-261) porque contaba causas de todos los episodios y no era comparable con las altas de empleo; los umbrales de valores extremos C-069, C-070 (más de 20 altas o bajas por año: perfil real de contratación muy fragmentada, mediana 222 altas) y C-072 a C-076 se QUITAN por ser casos reales, no errores. C-268 (335): los grupos de cotización 21 y 23 son del R.E. Agrario Cuenta Propia (0721) y la guía dice que valores fuera de 00-12 = 'no consta'; el ETL asimila ahora TODA clave fuera de 00-12 (13, 14, 19, 20, 21, 23, 31, 63) al 00 NO CONSTA (335 -&gt; 0 en la prueba; en una muestra de 29.004 personas solo cambia el grupo principal de 38, el 0,13 %).</t>
+          <t>Con las bajas reales (2026-09-21), C-255 (bajas &gt; altas) pasa a 0 y C-257/C-258 (enteros) se corrigieron (factor 365 vs 365,25). Siguen: 9.198 con más causas distintas que altas + 1,5 (C-260), ~2.100 con más de 20 altas/bajas por año (C-069/C-070). ACTUALIZACIÓN 2026-09-24: C-262 (120), C-264 (176), C-266 y C-267 pasan a 0 o 1 tras corregir los tramos de afiliación (ver G21). CERRADO 2026-09-25 (decisión del usuario): la variable causas_baja_distintas se ELIMINA (ETL, app y sus 11 reglas: A-018, A-044, C-026, C-077, C-139, C-140, C-144, C-145, C-259, C-260, C-261) porque contaba causas de todos los episodios y no era comparable con las altas de empleo; los umbrales de valores extremos C-069, C-070 (más de 20 altas o bajas por año: perfil real de contratación muy fragmentada, mediana 222 altas) y C-072 a C-076 se QUITAN por ser casos reales, no errores. C-268 (335): los grupos de cotización 21 y 23 son del R.E. Agrario Cuenta Propia (0721) y la guía dice que valores fuera de 00-12 = 'no consta'; el ETL asimila ahora TODA clave fuera de 00-12 (13, 14, 19, 20, 21, 23, 31, 63) al 00 NO CONSTA (335 -&gt; 0 en la prueba; en una muestra de 29.004 personas solo cambia el grupo principal de 38, el 0,13 %). CLASIFICADO 2026-09-25 (decisión del usuario): C-264 (G11), C-265 (G21) y C-108 son la MISMA persona: un fallecido con un episodio de empleo abierto al morir (duración del primer empleo significativo 2,17 años frente a 1,08 años de tiempo de empleo). Baja calidad de los datos; ver la explicación en la hoja Resultados.</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Regenerado 2026-09-25: C-268 pasa de 335 a 0 (claves de grupo fuera de 00-12 al 00). Queda C-264 (1 persona), sin acción.</t>
+          <t>Regenerado 2026-09-25: C-268 pasa de 335 a 0 (claves de grupo fuera de 00-12 al 00). Queda C-264 (1 persona), sin acción. Sin acción sobre el ETL.</t>
         </is>
       </c>
     </row>
@@ -1691,7 +1691,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>C-265 (83): personas, casi todas agrarias con muchos episodios y episodios de empleo larguísimos (uno de 31,7 años) cuyo EMPLEO+MIXTO de tabla_afiliacion_tramos.parquet salía muy por debajo de sus propios episodios. B-046/B-076 (26+26): 52 personas Parado con t_total_empleo = 0 que sí trabajaron, siempre a la vez que cobraban prestación (tiempo en t_total_mixto_empl_desempl).</t>
+          <t>C-265 (83): personas, casi todas agrarias con muchos episodios y episodios de empleo larguísimos (uno de 31,7 años) cuyo EMPLEO+MIXTO de tabla_afiliacion_tramos.parquet salía muy por debajo de sus propios episodios. B-046/B-076 (26+26): 52 personas Parado con t_total_empleo = 0 que sí trabajaron, siempre a la vez que cobraban prestación (tiempo en t_total_mixto_empl_desempl). CLASIFICADO 2026-09-25 (decisión del usuario): C-264 (G11), C-265 (G21) y C-108 son la MISMA persona: un fallecido con un episodio de empleo abierto al morir (duración del primer empleo significativo 2,17 años frente a 1,08 años de tiempo de empleo). Baja calidad de los datos; ver la explicación en la hoja Resultados.</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -1711,7 +1711,7 @@
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>ARREGLADO: ORDER BY fecha_alta, fecha_baja, rn (file_row_number) en las dos ventanas de ambas funciones (commit 3ec2fe5); acción 'tramos' en ejecutar_paso.py (f00acb7); etl/verificar_tramos.py comprueba determinismo y violaciones. Verificado a escala completa en el PC corporativo: 0 diferencias entre ejecuciones y 0 violaciones. Tramos, parcial y final regenerados. Resultado: C-265 83 -&gt; 1, C-264 176 -&gt; 1, C-262 120 -&gt; 0, C-266/C-267 -&gt; 0, C-252 186 -&gt; 112. B-046/B-076 reformuladas (suman t_total_mixto_empl_desempl): 0.</t>
+          <t>ARREGLADO: ORDER BY fecha_alta, fecha_baja, rn (file_row_number) en las dos ventanas de ambas funciones (commit 3ec2fe5); acción 'tramos' en ejecutar_paso.py (f00acb7); etl/verificar_tramos.py comprueba determinismo y violaciones. Verificado a escala completa en el PC corporativo: 0 diferencias entre ejecuciones y 0 violaciones. Tramos, parcial y final regenerados. Resultado: C-265 83 -&gt; 1, C-264 176 -&gt; 1, C-262 120 -&gt; 0, C-266/C-267 -&gt; 0, C-252 186 -&gt; 112. B-046/B-076 reformuladas (suman t_total_mixto_empl_desempl): 0. Sin acción sobre el ETL.</t>
         </is>
       </c>
     </row>
@@ -23809,7 +23809,7 @@
       </c>
       <c r="J321" s="6" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K321" s="2" t="n">
@@ -23822,12 +23822,17 @@
       <c r="N321" s="2" t="n"/>
       <c r="O321" s="2" t="inlineStr">
         <is>
-          <t>Actualizado 2026-09-25 tras regenerar con: Edad_Actual_Fecha_Corte de fallecidos a su fecha de fallecimiento, claves de grupo fuera de 00-12 al 00 y sin causas_baja_distintas.</t>
+          <t>Clasificada como baja calidad 2026-09-25 (decisión del usuario): fallecido con un episodio de empleo abierto al morir.</t>
         </is>
       </c>
       <c r="P321" s="2" t="inlineStr">
         <is>
           <t>edad_primer_empleo_signif + duracion_1er_empleo_signif &gt; edad_actual_fecha_corte + 1</t>
+        </is>
+      </c>
+      <c r="Q321" s="2" t="inlineStr">
+        <is>
+          <t>Es la MISMA persona en C-108, C-264 y C-265: un fallecido (murió a los 57,25 años) con un episodio de empleo abierto al morir. Su primer empleo significativo empezó a los 56,25 años y dura 2,17 años, pero solo vivió 1,08 años después: la duración del episodio se cuenta hasta la fecha de corte, mientras que su tiempo total de empleo sí está cortado en el fallecimiento. Con una tolerancia de 1 día solo esta persona viola (duracion_1er_empleo_signif y t_contrato_mas_largo); hay 14 fallecidos con episodio abierto, pero en los otros 13 las duraciones no superan el tiempo total. Afiliación sin cerrar en un fallecido: dato de origen. Corrección posible y no aplicada (decisión del usuario): limitar esas dos duraciones al tiempo de empleo más mixto en el Grupo H, como ya se hace con T_total_*, la edad actual y Edad_Ultimo_Empleo.</t>
         </is>
       </c>
     </row>
@@ -33815,7 +33820,7 @@
       </c>
       <c r="J469" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K469" s="2" t="n">
@@ -33832,12 +33837,17 @@
       <c r="N469" s="2" t="n"/>
       <c r="O469" s="2" t="inlineStr">
         <is>
-          <t>Actualizado 2026-09-24: tramos de afiliación regenerados con orden total en las ventanas (la fusión anterior no era determinista: 2.476 personas cambian).</t>
+          <t>Clasificada como baja calidad 2026-09-25 (decisión del usuario): fallecido con un episodio de empleo abierto al morir.</t>
         </is>
       </c>
       <c r="P469" s="2" t="inlineStr">
         <is>
           <t>t_contrato_mas_largo &gt; COALESCE(t_total_empleo,0) + COALESCE(t_total_mixto_empl_desempl,0) + 1</t>
+        </is>
+      </c>
+      <c r="Q469" s="2" t="inlineStr">
+        <is>
+          <t>Es la MISMA persona en C-108, C-264 y C-265: un fallecido (murió a los 57,25 años) con un episodio de empleo abierto al morir. Su primer empleo significativo empezó a los 56,25 años y dura 2,17 años, pero solo vivió 1,08 años después: la duración del episodio se cuenta hasta la fecha de corte, mientras que su tiempo total de empleo sí está cortado en el fallecimiento. Con una tolerancia de 1 día solo esta persona viola (duracion_1er_empleo_signif y t_contrato_mas_largo); hay 14 fallecidos con episodio abierto, pero en los otros 13 las duraciones no superan el tiempo total. Afiliación sin cerrar en un fallecido: dato de origen. Corrección posible y no aplicada (decisión del usuario): limitar esas dos duraciones al tiempo de empleo más mixto en el Grupo H, como ya se hace con T_total_*, la edad actual y Edad_Ultimo_Empleo.</t>
         </is>
       </c>
     </row>
@@ -33889,7 +33899,7 @@
       </c>
       <c r="J470" s="5" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Baja calidad de los datos</t>
         </is>
       </c>
       <c r="K470" s="2" t="n">
@@ -33906,12 +33916,17 @@
       <c r="N470" s="2" t="n"/>
       <c r="O470" s="2" t="inlineStr">
         <is>
-          <t>Regla ajustada 2026-09-24 (G08): excluye a quien solo tiene episodios TRL 7xx/400 (dato de origen, p. ej. agrarios con trabajo temporal mal registrado). | Actualizado 2026-09-24: tramos de afiliación regenerados con orden total en las ventanas (la fusión anterior no era determinista: 2.476 personas cambian).</t>
+          <t>Clasificada como baja calidad 2026-09-25 (decisión del usuario): fallecido con un episodio de empleo abierto al morir.</t>
         </is>
       </c>
       <c r="P470" s="2" t="inlineStr">
         <is>
           <t>duracion_1er_empleo_signif &gt; COALESCE(t_total_empleo,0) + COALESCE(t_total_mixto_empl_desempl,0) + 1 AND ipf NOT IN (SELECT ipf FROM solo_prestaciones)</t>
+        </is>
+      </c>
+      <c r="Q470" s="2" t="inlineStr">
+        <is>
+          <t>Es la MISMA persona en C-108, C-264 y C-265: un fallecido (murió a los 57,25 años) con un episodio de empleo abierto al morir. Su primer empleo significativo empezó a los 56,25 años y dura 2,17 años, pero solo vivió 1,08 años después: la duración del episodio se cuenta hasta la fecha de corte, mientras que su tiempo total de empleo sí está cortado en el fallecimiento. Con una tolerancia de 1 día solo esta persona viola (duracion_1er_empleo_signif y t_contrato_mas_largo); hay 14 fallecidos con episodio abierto, pero en los otros 13 las duraciones no superan el tiempo total. Afiliación sin cerrar en un fallecido: dato de origen. Corrección posible y no aplicada (decisión del usuario): limitar esas dos duraciones al tiempo de empleo más mixto en el Grupo H, como ya se hace con T_total_*, la edad actual y Edad_Ultimo_Empleo.</t>
         </is>
       </c>
     </row>
@@ -38824,7 +38839,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -38834,7 +38849,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
reglas: C-119, C-120, C-187..189 adaptadas a la categoria unica '0 NO CONSTA' de los grupos de cotizacion
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/reglas_consistencia_resultados_sin_ipf.xlsx
+++ b/tests/reglas_consistencia_resultados_sin_ipf.xlsx
@@ -24576,7 +24576,7 @@
       <c r="O332" s="2" t="inlineStr"/>
       <c r="P332" s="2" t="inlineStr">
         <is>
-          <t>t_tot_grupo_ppal IS NULL AND NOT (grupo_cotiz_ppal = 'NO CONSTA')</t>
+          <t>t_tot_grupo_ppal IS NULL AND NOT (grupo_cotiz_ppal = '0 NO CONSTA')</t>
         </is>
       </c>
     </row>
@@ -24608,7 +24608,7 @@
       </c>
       <c r="F333" s="2" t="inlineStr">
         <is>
-          <t>grupo_cotiz_ppal sin valor ⇒ t_tot_grupo_ppal vacío</t>
+          <t>Sin primer empleo ⇒ t_tot_grupo_ppal vacío</t>
         </is>
       </c>
       <c r="G333" s="2" t="inlineStr">
@@ -24642,7 +24642,7 @@
       <c r="O333" s="2" t="inlineStr"/>
       <c r="P333" s="2" t="inlineStr">
         <is>
-          <t>t_tot_grupo_ppal IS NOT NULL AND (grupo_cotiz_ppal = 'NO CONSTA') AND t_tot_grupo_ppal &gt; 0</t>
+          <t>fecha_ini_primer_empleo IS NULL AND t_tot_grupo_ppal IS NOT NULL</t>
         </is>
       </c>
     </row>
@@ -28861,7 +28861,7 @@
       <c r="O395" s="2" t="inlineStr"/>
       <c r="P395" s="2" t="inlineStr">
         <is>
-          <t>split_part(grupo_cotiz_ppal, ' ', 1) IN (SELECT split_part(grupo_cotiz_ppal, ' ', 1) FROM personas WHERE grupo_cotiz_ppal &lt;&gt; 'NO CONSTA' GROUP BY 1 HAVING COUNT(DISTINCT grupo_cotiz_ppal) &gt; 1)</t>
+          <t>split_part(grupo_cotiz_ppal, ' ', 1) IN (SELECT split_part(grupo_cotiz_ppal, ' ', 1) FROM personas WHERE grupo_cotiz_ppal &lt;&gt; '0 NO CONSTA' GROUP BY 1 HAVING COUNT(DISTINCT grupo_cotiz_ppal) &gt; 1)</t>
         </is>
       </c>
     </row>
@@ -28923,7 +28923,7 @@
       <c r="O396" s="2" t="inlineStr"/>
       <c r="P396" s="2" t="inlineStr">
         <is>
-          <t>split_part(grupo_ultimo_empleo, ' ', 1) IN (SELECT split_part(grupo_ultimo_empleo, ' ', 1) FROM personas WHERE grupo_ultimo_empleo &lt;&gt; 'NO CONSTA' GROUP BY 1 HAVING COUNT(DISTINCT grupo_ultimo_empleo) &gt; 1)</t>
+          <t>split_part(grupo_ultimo_empleo, ' ', 1) IN (SELECT split_part(grupo_ultimo_empleo, ' ', 1) FROM personas WHERE grupo_ultimo_empleo &lt;&gt; '0 NO CONSTA' GROUP BY 1 HAVING COUNT(DISTINCT grupo_ultimo_empleo) &gt; 1)</t>
         </is>
       </c>
     </row>
@@ -28985,7 +28985,7 @@
       <c r="O397" s="2" t="inlineStr"/>
       <c r="P397" s="2" t="inlineStr">
         <is>
-          <t>split_part(grupo_cotiz_1er_empleo_signif, ' ', 1) IN (SELECT split_part(grupo_cotiz_1er_empleo_signif, ' ', 1) FROM personas WHERE grupo_cotiz_1er_empleo_signif &lt;&gt; 'NO CONSTA' GROUP BY 1 HAVING COUNT(DISTINCT grupo_cotiz_1er_empleo_signif) &gt; 1)</t>
+          <t>split_part(grupo_cotiz_1er_empleo_signif, ' ', 1) IN (SELECT split_part(grupo_cotiz_1er_empleo_signif, ' ', 1) FROM personas WHERE grupo_cotiz_1er_empleo_signif &lt;&gt; '0 NO CONSTA' GROUP BY 1 HAVING COUNT(DISTINCT grupo_cotiz_1er_empleo_signif) &gt; 1)</t>
         </is>
       </c>
     </row>
@@ -38633,7 +38633,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -38728,7 +38728,6 @@
         <v>124</v>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
@@ -38799,7 +38798,6 @@
         <v>28</v>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -38869,7 +38867,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>